<commit_message>
Add initial database migration
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R328cdbfd5bcb4662"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R332d6f1101ae4917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R7d39e43e3ad84ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc9cf09a812d54608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1162,7 +1162,7 @@
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
         <x:f>COUNTIF(I9:I998,"Pass")</x:f>
-        <x:v>34</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
         <x:f>COUNTA(A9:A998)</x:f>
-        <x:v>35</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -3652,21 +3652,45 @@
       <x:c r="Z43" s="75" t="n"/>
     </x:row>
     <x:row r="44" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A44" s="75" t="n"/>
-      <x:c r="B44" s="76" t="n"/>
-      <x:c r="C44" s="75" t="n"/>
-      <x:c r="D44" s="75" t="n"/>
-      <x:c r="E44" s="75" t="n"/>
-      <x:c r="F44" s="76" t="n"/>
-      <x:c r="G44" s="75" t="n"/>
-      <x:c r="H44" s="75" t="n"/>
-      <x:c r="I44" s="75" t="n"/>
-      <x:c r="J44" s="75" t="n"/>
-      <x:c r="K44" s="75" t="n"/>
-      <x:c r="L44" s="75" t="n"/>
-      <x:c r="M44" s="75" t="n"/>
-      <x:c r="N44" s="75" t="n"/>
-      <x:c r="O44" s="75" t="n"/>
+      <x:c r="A44" s="75" t="str">
+        <x:v>TC_VIZI_036</x:v>
+      </x:c>
+      <x:c r="B44" s="76" t="str">
+        <x:v>Unit/static test migration SQL an toàn</x:v>
+      </x:c>
+      <x:c r="C44" s="75" t="str">
+        <x:v>Xác nhận file V1 dùng PostgreSQL đúng chuẩn và không chứa câu lệnh phá dữ liệu.</x:v>
+      </x:c>
+      <x:c r="D44" s="75" t="str">
+        <x:v>B1: Đọc V1__initial_schema.sql trong test.
+B2: Assert có timestamptz, jsonb, FK users.
+B3: Assert không có drop/truncate/delete destructive.</x:v>
+      </x:c>
+      <x:c r="E44" s="75" t="str">
+        <x:v>backend/src/main/resources/db/migration/V1__initial_schema.sql</x:v>
+      </x:c>
+      <x:c r="F44" s="76" t="str">
+        <x:v>SQL có jsonb/timestamptz/FK/index; không có lệnh destructive.</x:v>
+      </x:c>
+      <x:c r="G44" s="75" t="str">
+        <x:v>InitialSchemaMigrationTests.migrationSqlKeepsPostgreSqlSafeDefaults pass.</x:v>
+      </x:c>
+      <x:c r="H44" s="75" t="str">
+        <x:v>TC_VIZI_035</x:v>
+      </x:c>
+      <x:c r="I44" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J44" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K44" s="75" t="str">
+        <x:v>Loại test: unit/static/security baseline.</x:v>
+      </x:c>
+      <x:c r="L44" s="75"/>
+      <x:c r="M44" s="75"/>
+      <x:c r="N44" s="75"/>
+      <x:c r="O44" s="75"/>
       <x:c r="P44" s="75" t="n"/>
       <x:c r="Q44" s="75" t="n"/>
       <x:c r="R44" s="75" t="n"/>
@@ -3680,21 +3704,46 @@
       <x:c r="Z44" s="75" t="n"/>
     </x:row>
     <x:row r="45" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A45" s="75" t="n"/>
-      <x:c r="B45" s="76" t="n"/>
-      <x:c r="C45" s="75" t="n"/>
-      <x:c r="D45" s="75" t="n"/>
-      <x:c r="E45" s="75" t="n"/>
-      <x:c r="F45" s="76" t="n"/>
-      <x:c r="G45" s="75" t="n"/>
-      <x:c r="H45" s="75" t="n"/>
-      <x:c r="I45" s="75" t="n"/>
-      <x:c r="J45" s="75" t="n"/>
-      <x:c r="K45" s="75" t="n"/>
-      <x:c r="L45" s="75" t="n"/>
-      <x:c r="M45" s="75" t="n"/>
-      <x:c r="N45" s="75" t="n"/>
-      <x:c r="O45" s="75" t="n"/>
+      <x:c r="A45" s="75" t="str">
+        <x:v>TC_VIZI_037</x:v>
+      </x:c>
+      <x:c r="B45" s="76" t="str">
+        <x:v>Integration test Flyway migrate DB rỗng</x:v>
+      </x:c>
+      <x:c r="C45" s="75" t="str">
+        <x:v>Xác nhận Flyway chạy sạch trên PostgreSQL database rỗng tạm thời.</x:v>
+      </x:c>
+      <x:c r="D45" s="75" t="str">
+        <x:v>B1: Tạo database vizi_schema_test_*.
+B2: Chạy Flyway migrate.
+B3: Kiểm tra flyway_schema_history.
+B4: Drop database tạm.</x:v>
+      </x:c>
+      <x:c r="E45" s="75" t="str">
+        <x:v>PostgreSQL local 17.10, database tạm vizi_schema_test_*</x:v>
+      </x:c>
+      <x:c r="F45" s="76" t="str">
+        <x:v>Migration V1 apply thành công và cleanup DB test không để sót database.</x:v>
+      </x:c>
+      <x:c r="G45" s="75" t="str">
+        <x:v>mvnw test pass; Flyway log Successfully applied 1 migration; kiểm tra sau test không còn vizi_schema_test_*.</x:v>
+      </x:c>
+      <x:c r="H45" s="75" t="str">
+        <x:v>TC_VIZI_036</x:v>
+      </x:c>
+      <x:c r="I45" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J45" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K45" s="75" t="str">
+        <x:v>Loại test: integration/database.</x:v>
+      </x:c>
+      <x:c r="L45" s="75"/>
+      <x:c r="M45" s="75"/>
+      <x:c r="N45" s="75"/>
+      <x:c r="O45" s="75"/>
       <x:c r="P45" s="75" t="n"/>
       <x:c r="Q45" s="75" t="n"/>
       <x:c r="R45" s="75" t="n"/>
@@ -3708,21 +3757,45 @@
       <x:c r="Z45" s="75" t="n"/>
     </x:row>
     <x:row r="46" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A46" s="75" t="n"/>
-      <x:c r="B46" s="76" t="n"/>
-      <x:c r="C46" s="75" t="n"/>
-      <x:c r="D46" s="75" t="n"/>
-      <x:c r="E46" s="75" t="n"/>
-      <x:c r="F46" s="76" t="n"/>
-      <x:c r="G46" s="75" t="n"/>
-      <x:c r="H46" s="75" t="n"/>
-      <x:c r="I46" s="75" t="n"/>
-      <x:c r="J46" s="75" t="n"/>
-      <x:c r="K46" s="75" t="n"/>
-      <x:c r="L46" s="75" t="n"/>
-      <x:c r="M46" s="75" t="n"/>
-      <x:c r="N46" s="75" t="n"/>
-      <x:c r="O46" s="75" t="n"/>
+      <x:c r="A46" s="75" t="str">
+        <x:v>TC_VIZI_038</x:v>
+      </x:c>
+      <x:c r="B46" s="76" t="str">
+        <x:v>Schema test đủ bảng MVP</x:v>
+      </x:c>
+      <x:c r="C46" s="75" t="str">
+        <x:v>Xác nhận migration tạo đủ các bảng nền users/templates/designs/design_snapshots/assets/orders/order_items.</x:v>
+      </x:c>
+      <x:c r="D46" s="75" t="str">
+        <x:v>B1: Query information_schema.tables sau migrate.
+B2: So sánh danh sách bảng public với schema MVP.
+B3: Fail nếu thiếu bảng.</x:v>
+      </x:c>
+      <x:c r="E46" s="75" t="str">
+        <x:v>Database tạm sau Flyway migrate</x:v>
+      </x:c>
+      <x:c r="F46" s="76" t="str">
+        <x:v>Có đủ 7 bảng MVP và flyway_schema_history.</x:v>
+      </x:c>
+      <x:c r="G46" s="75" t="str">
+        <x:v>InitialSchemaMigrationTests.assertTables pass với users, templates, designs, design_snapshots, assets, orders, order_items.</x:v>
+      </x:c>
+      <x:c r="H46" s="75" t="str">
+        <x:v>TC_VIZI_037</x:v>
+      </x:c>
+      <x:c r="I46" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J46" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K46" s="75" t="str">
+        <x:v>Loại test: integration/schema.</x:v>
+      </x:c>
+      <x:c r="L46" s="75"/>
+      <x:c r="M46" s="75"/>
+      <x:c r="N46" s="75"/>
+      <x:c r="O46" s="75"/>
       <x:c r="P46" s="75" t="n"/>
       <x:c r="Q46" s="75" t="n"/>
       <x:c r="R46" s="75" t="n"/>
@@ -3736,21 +3809,45 @@
       <x:c r="Z46" s="75" t="n"/>
     </x:row>
     <x:row r="47" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A47" s="75" t="n"/>
-      <x:c r="B47" s="76" t="n"/>
-      <x:c r="C47" s="75" t="n"/>
-      <x:c r="D47" s="75" t="n"/>
-      <x:c r="E47" s="75" t="n"/>
-      <x:c r="F47" s="76" t="n"/>
-      <x:c r="G47" s="75" t="n"/>
-      <x:c r="H47" s="75" t="n"/>
-      <x:c r="I47" s="75" t="n"/>
-      <x:c r="J47" s="75" t="n"/>
-      <x:c r="K47" s="75" t="n"/>
-      <x:c r="L47" s="75" t="n"/>
-      <x:c r="M47" s="75" t="n"/>
-      <x:c r="N47" s="75" t="n"/>
-      <x:c r="O47" s="75" t="n"/>
+      <x:c r="A47" s="75" t="str">
+        <x:v>TC_VIZI_039</x:v>
+      </x:c>
+      <x:c r="B47" s="76" t="str">
+        <x:v>Schema test kiểu dữ liệu và index</x:v>
+      </x:c>
+      <x:c r="C47" s="75" t="str">
+        <x:v>Xác nhận canvas/snapshot dùng jsonb, thời gian dùng timestamptz, tiền dùng numeric và các FK/index chính tồn tại.</x:v>
+      </x:c>
+      <x:c r="D47" s="75" t="str">
+        <x:v>B1: Query information_schema.columns.
+B2: Query pg_indexes.
+B3: Assert jsonb/timestamptz/numeric/index user_id/template_id/design_id/order_id.</x:v>
+      </x:c>
+      <x:c r="E47" s="75" t="str">
+        <x:v>Database tạm sau Flyway migrate</x:v>
+      </x:c>
+      <x:c r="F47" s="76" t="str">
+        <x:v>Đúng kiểu dữ liệu PostgreSQL và đủ index chính theo guardrail.</x:v>
+      </x:c>
+      <x:c r="G47" s="75" t="str">
+        <x:v>InitialSchemaMigrationTests.assertColumnTypes và assertIndexes pass.</x:v>
+      </x:c>
+      <x:c r="H47" s="75" t="str">
+        <x:v>TC_VIZI_038</x:v>
+      </x:c>
+      <x:c r="I47" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J47" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K47" s="75" t="str">
+        <x:v>Loại test: integration/performance foundation.</x:v>
+      </x:c>
+      <x:c r="L47" s="75"/>
+      <x:c r="M47" s="75"/>
+      <x:c r="N47" s="75"/>
+      <x:c r="O47" s="75"/>
       <x:c r="P47" s="75" t="n"/>
       <x:c r="Q47" s="75" t="n"/>
       <x:c r="R47" s="75" t="n"/>
@@ -3764,21 +3861,48 @@
       <x:c r="Z47" s="75" t="n"/>
     </x:row>
     <x:row r="48" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A48" s="75" t="n"/>
-      <x:c r="B48" s="76" t="n"/>
-      <x:c r="C48" s="75" t="n"/>
-      <x:c r="D48" s="75" t="n"/>
-      <x:c r="E48" s="75" t="n"/>
-      <x:c r="F48" s="76" t="n"/>
-      <x:c r="G48" s="75" t="n"/>
-      <x:c r="H48" s="75" t="n"/>
-      <x:c r="I48" s="75" t="n"/>
-      <x:c r="J48" s="75" t="n"/>
-      <x:c r="K48" s="75" t="n"/>
-      <x:c r="L48" s="75" t="n"/>
-      <x:c r="M48" s="75" t="n"/>
-      <x:c r="N48" s="75" t="n"/>
-      <x:c r="O48" s="75" t="n"/>
+      <x:c r="A48" s="75" t="str">
+        <x:v>TC_VIZI_040</x:v>
+      </x:c>
+      <x:c r="B48" s="76" t="str">
+        <x:v>UAT acceptance flow dữ liệu MVP</x:v>
+      </x:c>
+      <x:c r="C48" s="75" t="str">
+        <x:v>Xác nhận luồng mẫu user -&gt; template -&gt; design -&gt; snapshot -&gt; order -&gt; order item lưu và đọc lại được.</x:v>
+      </x:c>
+      <x:c r="D48" s="75" t="str">
+        <x:v>B1: Insert user mẫu.
+B2: Insert template card 90x54.
+B3: Insert design từ template.
+B4: Insert snapshot.
+B5: Insert order và order_item.
+B6: Join đọc lại status, quantity, design name.</x:v>
+      </x:c>
+      <x:c r="E48" s="75" t="str">
+        <x:v>Database tạm sau Flyway migrate</x:v>
+      </x:c>
+      <x:c r="F48" s="76" t="str">
+        <x:v>Luồng dữ liệu MVP cơ bản chạy được, output join đúng.</x:v>
+      </x:c>
+      <x:c r="G48" s="75" t="str">
+        <x:v>InitialSchemaMigrationTests.assertMvpAcceptanceFlow pass; đọc lại status PENDING_PAYMENT, quantity 100, design Bao card.</x:v>
+      </x:c>
+      <x:c r="H48" s="75" t="str">
+        <x:v>TC_VIZI_039</x:v>
+      </x:c>
+      <x:c r="I48" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J48" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K48" s="75" t="str">
+        <x:v>Loại test: UAT acceptance/system database.</x:v>
+      </x:c>
+      <x:c r="L48" s="75"/>
+      <x:c r="M48" s="75"/>
+      <x:c r="N48" s="75"/>
+      <x:c r="O48" s="75"/>
       <x:c r="P48" s="75" t="n"/>
       <x:c r="Q48" s="75" t="n"/>
       <x:c r="R48" s="75" t="n"/>
@@ -3792,21 +3916,45 @@
       <x:c r="Z48" s="75" t="n"/>
     </x:row>
     <x:row r="49" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A49" s="75" t="n"/>
-      <x:c r="B49" s="76" t="n"/>
-      <x:c r="C49" s="75" t="n"/>
-      <x:c r="D49" s="75" t="n"/>
-      <x:c r="E49" s="75" t="n"/>
-      <x:c r="F49" s="76" t="n"/>
-      <x:c r="G49" s="75" t="n"/>
-      <x:c r="H49" s="75" t="n"/>
-      <x:c r="I49" s="75" t="n"/>
-      <x:c r="J49" s="75" t="n"/>
-      <x:c r="K49" s="75" t="n"/>
-      <x:c r="L49" s="75" t="n"/>
-      <x:c r="M49" s="75" t="n"/>
-      <x:c r="N49" s="75" t="n"/>
-      <x:c r="O49" s="75" t="n"/>
+      <x:c r="A49" s="75" t="str">
+        <x:v>TC_VIZI_041</x:v>
+      </x:c>
+      <x:c r="B49" s="76" t="str">
+        <x:v>Security test FK owner bắt lỗi dữ liệu mồ côi</x:v>
+      </x:c>
+      <x:c r="C49" s="75" t="str">
+        <x:v>Xác nhận bảng user-owned data không nhận design với user_id không tồn tại.</x:v>
+      </x:c>
+      <x:c r="D49" s="75" t="str">
+        <x:v>B1: Insert designs với user_id=999999.
+B2: Kỳ vọng PostgreSQL reject bằng FK.
+B3: Assert message có violates foreign key constraint.</x:v>
+      </x:c>
+      <x:c r="E49" s="75" t="str">
+        <x:v>Database tạm sau Flyway migrate</x:v>
+      </x:c>
+      <x:c r="F49" s="76" t="str">
+        <x:v>DB chặn dữ liệu mồ côi, làm nền chống IDOR ở tầng API sau này.</x:v>
+      </x:c>
+      <x:c r="G49" s="75" t="str">
+        <x:v>InitialSchemaMigrationTests.assertForeignKeysRejectMissingOwners pass.</x:v>
+      </x:c>
+      <x:c r="H49" s="75" t="str">
+        <x:v>TC_VIZI_040</x:v>
+      </x:c>
+      <x:c r="I49" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J49" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K49" s="75" t="str">
+        <x:v>Loại test: security/database constraint.</x:v>
+      </x:c>
+      <x:c r="L49" s="75"/>
+      <x:c r="M49" s="75"/>
+      <x:c r="N49" s="75"/>
+      <x:c r="O49" s="75"/>
       <x:c r="P49" s="75" t="n"/>
       <x:c r="Q49" s="75" t="n"/>
       <x:c r="R49" s="75" t="n"/>
@@ -3820,21 +3968,45 @@
       <x:c r="Z49" s="75" t="n"/>
     </x:row>
     <x:row r="50" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A50" s="75" t="n"/>
-      <x:c r="B50" s="76" t="n"/>
-      <x:c r="C50" s="75" t="n"/>
-      <x:c r="D50" s="75" t="n"/>
-      <x:c r="E50" s="75" t="n"/>
-      <x:c r="F50" s="76" t="n"/>
-      <x:c r="G50" s="75" t="n"/>
-      <x:c r="H50" s="75" t="n"/>
-      <x:c r="I50" s="75" t="n"/>
-      <x:c r="J50" s="75" t="n"/>
-      <x:c r="K50" s="75" t="n"/>
-      <x:c r="L50" s="75" t="n"/>
-      <x:c r="M50" s="75" t="n"/>
-      <x:c r="N50" s="75" t="n"/>
-      <x:c r="O50" s="75" t="n"/>
+      <x:c r="A50" s="75" t="str">
+        <x:v>TC_VIZI_042</x:v>
+      </x:c>
+      <x:c r="B50" s="76" t="str">
+        <x:v>Performance test query active templates</x:v>
+      </x:c>
+      <x:c r="C50" s="75" t="str">
+        <x:v>Xác nhận query template active/category có index và chạy nhanh với dữ liệu mẫu nhỏ.</x:v>
+      </x:c>
+      <x:c r="D50" s="75" t="str">
+        <x:v>B1: Insert 100 template active.
+B2: Query active=true and category='business' limit 20.
+B3: Assert trả 20 dòng dưới 500ms.</x:v>
+      </x:c>
+      <x:c r="E50" s="75" t="str">
+        <x:v>Database tạm sau Flyway migrate</x:v>
+      </x:c>
+      <x:c r="F50" s="76" t="str">
+        <x:v>Query trả đúng 20 dòng và dưới ngưỡng 500ms.</x:v>
+      </x:c>
+      <x:c r="G50" s="75" t="str">
+        <x:v>InitialSchemaMigrationTests.assertActiveTemplateQueryIsFastEnough pass.</x:v>
+      </x:c>
+      <x:c r="H50" s="75" t="str">
+        <x:v>TC_VIZI_041</x:v>
+      </x:c>
+      <x:c r="I50" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J50" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K50" s="75" t="str">
+        <x:v>Loại test: performance smoke, chưa thay thế load test lớn.</x:v>
+      </x:c>
+      <x:c r="L50" s="75"/>
+      <x:c r="M50" s="75"/>
+      <x:c r="N50" s="75"/>
+      <x:c r="O50" s="75"/>
       <x:c r="P50" s="75" t="n"/>
       <x:c r="Q50" s="75" t="n"/>
       <x:c r="R50" s="75" t="n"/>
@@ -3848,21 +4020,46 @@
       <x:c r="Z50" s="75" t="n"/>
     </x:row>
     <x:row r="51" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A51" s="75" t="n"/>
-      <x:c r="B51" s="76" t="n"/>
-      <x:c r="C51" s="75" t="n"/>
-      <x:c r="D51" s="75" t="n"/>
-      <x:c r="E51" s="75" t="n"/>
-      <x:c r="F51" s="76" t="n"/>
-      <x:c r="G51" s="75" t="n"/>
-      <x:c r="H51" s="75" t="n"/>
-      <x:c r="I51" s="75" t="n"/>
-      <x:c r="J51" s="75" t="n"/>
-      <x:c r="K51" s="75" t="n"/>
-      <x:c r="L51" s="75" t="n"/>
-      <x:c r="M51" s="75" t="n"/>
-      <x:c r="N51" s="75" t="n"/>
-      <x:c r="O51" s="75" t="n"/>
+      <x:c r="A51" s="75" t="str">
+        <x:v>TC_VIZI_043</x:v>
+      </x:c>
+      <x:c r="B51" s="76" t="str">
+        <x:v>Smoke/system test Flyway tự chạy khi backend local start</x:v>
+      </x:c>
+      <x:c r="C51" s="75" t="str">
+        <x:v>Xác nhận backend profile local tự chạy Flyway trên database vizi thật khi app khởi động.</x:v>
+      </x:c>
+      <x:c r="D51" s="75" t="str">
+        <x:v>B1: Chạy mvnw spring-boot:run profile local.
+B2: Quan sát log Flyway.
+B3: Query flyway_schema_history.
+B4: Query danh sách 7 bảng MVP.</x:v>
+      </x:c>
+      <x:c r="E51" s="75" t="str">
+        <x:v>Database vizi thật trên 127.0.0.1:55432</x:v>
+      </x:c>
+      <x:c r="F51" s="76" t="str">
+        <x:v>Startup log có Flyway migrate; DB thật có version 1 và 7 bảng MVP.</x:v>
+      </x:c>
+      <x:c r="G51" s="75" t="str">
+        <x:v>Ban đầu fail vì thiếu spring-boot-starter-flyway; đã thêm starter, retest log Successfully applied 1 migration, flyway_schema_history version 1 success=true.</x:v>
+      </x:c>
+      <x:c r="H51" s="75" t="str">
+        <x:v>TC_VIZI_037</x:v>
+      </x:c>
+      <x:c r="I51" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J51" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K51" s="75" t="str">
+        <x:v>Loại test: smoke/system; có bug được sửa và retest pass.</x:v>
+      </x:c>
+      <x:c r="L51" s="75"/>
+      <x:c r="M51" s="75"/>
+      <x:c r="N51" s="75"/>
+      <x:c r="O51" s="75"/>
       <x:c r="P51" s="75" t="n"/>
       <x:c r="Q51" s="75" t="n"/>
       <x:c r="R51" s="75" t="n"/>
@@ -3876,21 +4073,46 @@
       <x:c r="Z51" s="75" t="n"/>
     </x:row>
     <x:row r="52" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A52" s="75" t="n"/>
-      <x:c r="B52" s="76" t="n"/>
-      <x:c r="C52" s="75" t="n"/>
-      <x:c r="D52" s="75" t="n"/>
-      <x:c r="E52" s="75" t="n"/>
-      <x:c r="F52" s="76" t="n"/>
-      <x:c r="G52" s="75" t="n"/>
-      <x:c r="H52" s="75" t="n"/>
-      <x:c r="I52" s="75" t="n"/>
-      <x:c r="J52" s="75" t="n"/>
-      <x:c r="K52" s="75" t="n"/>
-      <x:c r="L52" s="75" t="n"/>
-      <x:c r="M52" s="75" t="n"/>
-      <x:c r="N52" s="75" t="n"/>
-      <x:c r="O52" s="75" t="n"/>
+      <x:c r="A52" s="75" t="str">
+        <x:v>TC_VIZI_044</x:v>
+      </x:c>
+      <x:c r="B52" s="76" t="str">
+        <x:v>Regression test backend và API lỗi</x:v>
+      </x:c>
+      <x:c r="C52" s="75" t="str">
+        <x:v>Xác nhận thay đổi Flyway/schema không làm hỏng health API, JSON 404 và test backend cũ.</x:v>
+      </x:c>
+      <x:c r="D52" s="75" t="str">
+        <x:v>B1: Chạy mvnw test.
+B2: Gọi /api/health khi backend local chạy.
+B3: Gọi /api/not-found.
+B4: Kiểm tra JSON response.</x:v>
+      </x:c>
+      <x:c r="E52" s="75" t="str">
+        <x:v>Backend Spring Boot local</x:v>
+      </x:c>
+      <x:c r="F52" s="76" t="str">
+        <x:v>Test pass 7/7; health UP; 404 trả application/json.</x:v>
+      </x:c>
+      <x:c r="G52" s="75" t="str">
+        <x:v>mvnw test BUILD SUCCESS Tests run 7; /api/health status UP; /api/not-found trả HTTP 404 Content-Type application/json.</x:v>
+      </x:c>
+      <x:c r="H52" s="75" t="str">
+        <x:v>TC_VIZI_043</x:v>
+      </x:c>
+      <x:c r="I52" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J52" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K52" s="75" t="str">
+        <x:v>Loại test: regression/smoke API.</x:v>
+      </x:c>
+      <x:c r="L52" s="75"/>
+      <x:c r="M52" s="75"/>
+      <x:c r="N52" s="75"/>
+      <x:c r="O52" s="75"/>
       <x:c r="P52" s="75" t="n"/>
       <x:c r="Q52" s="75" t="n"/>
       <x:c r="R52" s="75" t="n"/>
@@ -3904,21 +4126,45 @@
       <x:c r="Z52" s="75" t="n"/>
     </x:row>
     <x:row r="53" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A53" s="75" t="n"/>
-      <x:c r="B53" s="76" t="n"/>
-      <x:c r="C53" s="75" t="n"/>
-      <x:c r="D53" s="75" t="n"/>
-      <x:c r="E53" s="75" t="n"/>
-      <x:c r="F53" s="76" t="n"/>
-      <x:c r="G53" s="75" t="n"/>
-      <x:c r="H53" s="75" t="n"/>
-      <x:c r="I53" s="75" t="n"/>
-      <x:c r="J53" s="75" t="n"/>
-      <x:c r="K53" s="75" t="n"/>
-      <x:c r="L53" s="75" t="n"/>
-      <x:c r="M53" s="75" t="n"/>
-      <x:c r="N53" s="75" t="n"/>
-      <x:c r="O53" s="75" t="n"/>
+      <x:c r="A53" s="75" t="str">
+        <x:v>TC_VIZI_045</x:v>
+      </x:c>
+      <x:c r="B53" s="76" t="str">
+        <x:v>Regression test frontend build và secret scan</x:v>
+      </x:c>
+      <x:c r="C53" s="75" t="str">
+        <x:v>Xác nhận thay đổi backend/schema không làm hỏng frontend build và không thêm secret thật vào repo.</x:v>
+      </x:c>
+      <x:c r="D53" s="75" t="str">
+        <x:v>B1: Chạy npm run build trong frontend.
+B2: Chạy rg secret pattern loại trừ node_modules/dist/target/.agents/.codex-work.
+B3: Kiểm tra git status/staged trước commit.</x:v>
+      </x:c>
+      <x:c r="E53" s="75" t="str">
+        <x:v>Frontend Vite, toàn repo source</x:v>
+      </x:c>
+      <x:c r="F53" s="76" t="str">
+        <x:v>Frontend build pass; secret scan chỉ có placeholder/env references/tài liệu, không có secret thật.</x:v>
+      </x:c>
+      <x:c r="G53" s="75" t="str">
+        <x:v>npm run build pass; secret scan chỉ match change-me, env var reference, docs và wrapper Maven; không có API key/token/password thật.</x:v>
+      </x:c>
+      <x:c r="H53" s="75" t="str">
+        <x:v>TC_VIZI_044</x:v>
+      </x:c>
+      <x:c r="I53" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J53" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K53" s="75" t="str">
+        <x:v>Loại test: regression/security.</x:v>
+      </x:c>
+      <x:c r="L53" s="75"/>
+      <x:c r="M53" s="75"/>
+      <x:c r="N53" s="75"/>
+      <x:c r="O53" s="75"/>
       <x:c r="P53" s="75" t="n"/>
       <x:c r="Q53" s="75" t="n"/>
       <x:c r="R53" s="75" t="n"/>
@@ -30496,7 +30742,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cd02055834743c5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86f28c35692b47f5"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add template read API
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R7d39e43e3ad84ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc9cf09a812d54608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R3ee08e9e8b3149d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R9502e49c24184253"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1162,7 +1162,7 @@
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
         <x:f>COUNTIF(I9:I998,"Pass")</x:f>
-        <x:v>44</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
         <x:f>COUNTA(A9:A998)</x:f>
-        <x:v>45</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -4178,21 +4178,45 @@
       <x:c r="Z53" s="75" t="n"/>
     </x:row>
     <x:row r="54" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A54" s="75" t="n"/>
-      <x:c r="B54" s="76" t="n"/>
-      <x:c r="C54" s="75" t="n"/>
-      <x:c r="D54" s="75" t="n"/>
-      <x:c r="E54" s="75" t="n"/>
-      <x:c r="F54" s="76" t="n"/>
-      <x:c r="G54" s="75" t="n"/>
-      <x:c r="H54" s="75" t="n"/>
-      <x:c r="I54" s="75" t="n"/>
-      <x:c r="J54" s="75" t="n"/>
-      <x:c r="K54" s="75" t="n"/>
-      <x:c r="L54" s="75" t="n"/>
-      <x:c r="M54" s="75" t="n"/>
-      <x:c r="N54" s="75" t="n"/>
-      <x:c r="O54" s="75" t="n"/>
+      <x:c r="A54" s="75" t="str">
+        <x:v>TC_VIZI_046</x:v>
+      </x:c>
+      <x:c r="B54" s="76" t="str">
+        <x:v>Unit/compile test Template entity và repository</x:v>
+      </x:c>
+      <x:c r="C54" s="75" t="str">
+        <x:v>Xác nhận backend có Template entity map bảng templates và repository query active templates.</x:v>
+      </x:c>
+      <x:c r="D54" s="75" t="str">
+        <x:v>B1: Thêm Template entity map id/name/category/preview_url/width_mm/height_mm/canvas_json/active.
+B2: Thêm TemplateRepository.
+B3: Chạy mvnw test.</x:v>
+      </x:c>
+      <x:c r="E54" s="75" t="str">
+        <x:v>backend/src/main/java/com/example/vizi/Template.java, TemplateRepository.java</x:v>
+      </x:c>
+      <x:c r="F54" s="76" t="str">
+        <x:v>Compile pass; Spring context scan được 1 JPA repository.</x:v>
+      </x:c>
+      <x:c r="G54" s="75" t="str">
+        <x:v>mvnw test pass; log TemplateApiIntegrationTests Found 1 JPA repository interface.</x:v>
+      </x:c>
+      <x:c r="H54" s="75" t="str">
+        <x:v>TC_VIZI_045</x:v>
+      </x:c>
+      <x:c r="I54" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J54" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K54" s="75" t="str">
+        <x:v>Loại test: compile/unit foundation.</x:v>
+      </x:c>
+      <x:c r="L54" s="75"/>
+      <x:c r="M54" s="75"/>
+      <x:c r="N54" s="75"/>
+      <x:c r="O54" s="75"/>
       <x:c r="P54" s="75" t="n"/>
       <x:c r="Q54" s="75" t="n"/>
       <x:c r="R54" s="75" t="n"/>
@@ -4206,21 +4230,46 @@
       <x:c r="Z54" s="75" t="n"/>
     </x:row>
     <x:row r="55" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A55" s="75" t="n"/>
-      <x:c r="B55" s="76" t="n"/>
-      <x:c r="C55" s="75" t="n"/>
-      <x:c r="D55" s="75" t="n"/>
-      <x:c r="E55" s="75" t="n"/>
-      <x:c r="F55" s="76" t="n"/>
-      <x:c r="G55" s="75" t="n"/>
-      <x:c r="H55" s="75" t="n"/>
-      <x:c r="I55" s="75" t="n"/>
-      <x:c r="J55" s="75" t="n"/>
-      <x:c r="K55" s="75" t="n"/>
-      <x:c r="L55" s="75" t="n"/>
-      <x:c r="M55" s="75" t="n"/>
-      <x:c r="N55" s="75" t="n"/>
-      <x:c r="O55" s="75" t="n"/>
+      <x:c r="A55" s="75" t="str">
+        <x:v>TC_VIZI_047</x:v>
+      </x:c>
+      <x:c r="B55" s="76" t="str">
+        <x:v>Unit test TemplateService</x:v>
+      </x:c>
+      <x:c r="C55" s="75" t="str">
+        <x:v>Xác nhận service map entity sang DTO và trả 404 khi template không active/không tồn tại.</x:v>
+      </x:c>
+      <x:c r="D55" s="75" t="str">
+        <x:v>B1: Mock TemplateRepository.
+B2: Test listActiveTemplates.
+B3: Test getActiveTemplate success.
+B4: Test missing id ném ResponseStatusException 404.</x:v>
+      </x:c>
+      <x:c r="E55" s="75" t="str">
+        <x:v>TemplateServiceTests</x:v>
+      </x:c>
+      <x:c r="F55" s="76" t="str">
+        <x:v>Service trả list item đúng; detail có canvasJson; missing trả 404 Template not found.</x:v>
+      </x:c>
+      <x:c r="G55" s="75" t="str">
+        <x:v>TemplateServiceTests pass 2/2.</x:v>
+      </x:c>
+      <x:c r="H55" s="75" t="str">
+        <x:v>TC_VIZI_046</x:v>
+      </x:c>
+      <x:c r="I55" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J55" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K55" s="75" t="str">
+        <x:v>Loại test: unit/service/security behavior.</x:v>
+      </x:c>
+      <x:c r="L55" s="75"/>
+      <x:c r="M55" s="75"/>
+      <x:c r="N55" s="75"/>
+      <x:c r="O55" s="75"/>
       <x:c r="P55" s="75" t="n"/>
       <x:c r="Q55" s="75" t="n"/>
       <x:c r="R55" s="75" t="n"/>
@@ -4234,21 +4283,47 @@
       <x:c r="Z55" s="75" t="n"/>
     </x:row>
     <x:row r="56" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A56" s="75" t="n"/>
-      <x:c r="B56" s="76" t="n"/>
-      <x:c r="C56" s="75" t="n"/>
-      <x:c r="D56" s="75" t="n"/>
-      <x:c r="E56" s="75" t="n"/>
-      <x:c r="F56" s="76" t="n"/>
-      <x:c r="G56" s="75" t="n"/>
-      <x:c r="H56" s="75" t="n"/>
-      <x:c r="I56" s="75" t="n"/>
-      <x:c r="J56" s="75" t="n"/>
-      <x:c r="K56" s="75" t="n"/>
-      <x:c r="L56" s="75" t="n"/>
-      <x:c r="M56" s="75" t="n"/>
-      <x:c r="N56" s="75" t="n"/>
-      <x:c r="O56" s="75" t="n"/>
+      <x:c r="A56" s="75" t="str">
+        <x:v>TC_VIZI_048</x:v>
+      </x:c>
+      <x:c r="B56" s="76" t="str">
+        <x:v>Integration/API test GET /api/templates</x:v>
+      </x:c>
+      <x:c r="C56" s="75" t="str">
+        <x:v>Xác nhận API list chỉ trả active templates và sort theo id trên PostgreSQL DB tạm.</x:v>
+      </x:c>
+      <x:c r="D56" s="75" t="str">
+        <x:v>B1: SpringBootTest random port.
+B2: Tạo DB PostgreSQL tạm.
+B3: Flyway migrate.
+B4: Seed 2 active + 1 inactive.
+B5: Gọi GET /api/templates bằng HttpClient.</x:v>
+      </x:c>
+      <x:c r="E56" s="75" t="str">
+        <x:v>TemplateApiIntegrationTests.listTemplatesReturnsOnlyActiveTemplatesSortedById</x:v>
+      </x:c>
+      <x:c r="F56" s="76" t="str">
+        <x:v>HTTP 200; response có active templates theo id; không có Hidden Card.</x:v>
+      </x:c>
+      <x:c r="G56" s="75" t="str">
+        <x:v>TemplateApiIntegrationTests pass; list API không trả inactive template.</x:v>
+      </x:c>
+      <x:c r="H56" s="75" t="str">
+        <x:v>TC_VIZI_047</x:v>
+      </x:c>
+      <x:c r="I56" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J56" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K56" s="75" t="str">
+        <x:v>Loại test: integration/API/security filter.</x:v>
+      </x:c>
+      <x:c r="L56" s="75"/>
+      <x:c r="M56" s="75"/>
+      <x:c r="N56" s="75"/>
+      <x:c r="O56" s="75"/>
       <x:c r="P56" s="75" t="n"/>
       <x:c r="Q56" s="75" t="n"/>
       <x:c r="R56" s="75" t="n"/>
@@ -4262,21 +4337,47 @@
       <x:c r="Z56" s="75" t="n"/>
     </x:row>
     <x:row r="57" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A57" s="75" t="n"/>
-      <x:c r="B57" s="76" t="n"/>
-      <x:c r="C57" s="75" t="n"/>
-      <x:c r="D57" s="75" t="n"/>
-      <x:c r="E57" s="75" t="n"/>
-      <x:c r="F57" s="76" t="n"/>
-      <x:c r="G57" s="75" t="n"/>
-      <x:c r="H57" s="75" t="n"/>
-      <x:c r="I57" s="75" t="n"/>
-      <x:c r="J57" s="75" t="n"/>
-      <x:c r="K57" s="75" t="n"/>
-      <x:c r="L57" s="75" t="n"/>
-      <x:c r="M57" s="75" t="n"/>
-      <x:c r="N57" s="75" t="n"/>
-      <x:c r="O57" s="75" t="n"/>
+      <x:c r="A57" s="75" t="str">
+        <x:v>TC_VIZI_049</x:v>
+      </x:c>
+      <x:c r="B57" s="76" t="str">
+        <x:v>Integration/API test GET /api/templates/{id}</x:v>
+      </x:c>
+      <x:c r="C57" s="75" t="str">
+        <x:v>Xác nhận API detail trả active template và ẩn inactive/missing bằng 404 JSON.</x:v>
+      </x:c>
+      <x:c r="D57" s="75" t="str">
+        <x:v>B1: Seed active template.
+B2: Seed inactive template.
+B3: GET active id.
+B4: GET inactive id.
+B5: GET missing id.</x:v>
+      </x:c>
+      <x:c r="E57" s="75" t="str">
+        <x:v>TemplateApiIntegrationTests.getTemplateReturnsActiveTemplateDetailAndHidesInactiveTemplates</x:v>
+      </x:c>
+      <x:c r="F57" s="76" t="str">
+        <x:v>Active trả 200 có canvasJson; inactive và missing trả 404 Template not found.</x:v>
+      </x:c>
+      <x:c r="G57" s="75" t="str">
+        <x:v>TemplateApiIntegrationTests pass; inactive id và id 999999 đều trả 404.</x:v>
+      </x:c>
+      <x:c r="H57" s="75" t="str">
+        <x:v>TC_VIZI_048</x:v>
+      </x:c>
+      <x:c r="I57" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J57" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K57" s="75" t="str">
+        <x:v>Loại test: integration/API/security no inactive exposure.</x:v>
+      </x:c>
+      <x:c r="L57" s="75"/>
+      <x:c r="M57" s="75"/>
+      <x:c r="N57" s="75"/>
+      <x:c r="O57" s="75"/>
       <x:c r="P57" s="75" t="n"/>
       <x:c r="Q57" s="75" t="n"/>
       <x:c r="R57" s="75" t="n"/>
@@ -4290,21 +4391,48 @@
       <x:c r="Z57" s="75" t="n"/>
     </x:row>
     <x:row r="58" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A58" s="75" t="n"/>
-      <x:c r="B58" s="76" t="n"/>
-      <x:c r="C58" s="75" t="n"/>
-      <x:c r="D58" s="75" t="n"/>
-      <x:c r="E58" s="75" t="n"/>
-      <x:c r="F58" s="76" t="n"/>
-      <x:c r="G58" s="75" t="n"/>
-      <x:c r="H58" s="75" t="n"/>
-      <x:c r="I58" s="75" t="n"/>
-      <x:c r="J58" s="75" t="n"/>
-      <x:c r="K58" s="75" t="n"/>
-      <x:c r="L58" s="75" t="n"/>
-      <x:c r="M58" s="75" t="n"/>
-      <x:c r="N58" s="75" t="n"/>
-      <x:c r="O58" s="75" t="n"/>
+      <x:c r="A58" s="75" t="str">
+        <x:v>TC_VIZI_050</x:v>
+      </x:c>
+      <x:c r="B58" s="76" t="str">
+        <x:v>Smoke/system test Template API trên DB local thật</x:v>
+      </x:c>
+      <x:c r="C58" s="75" t="str">
+        <x:v>Xác nhận backend local profile chạy với DB vizi thật và API template hoạt động với seed tạm.</x:v>
+      </x:c>
+      <x:c r="D58" s="75" t="str">
+        <x:v>B1: Insert Smoke Active Template và Smoke Hidden Template vào DB vizi.
+B2: Start backend local.
+B3: GET /api/templates.
+B4: GET /api/templates/1.
+B5: GET inactive/missing.
+B6: Xóa seed tạm.</x:v>
+      </x:c>
+      <x:c r="E58" s="75" t="str">
+        <x:v>PostgreSQL local 127.0.0.1:55432, backend port 8080</x:v>
+      </x:c>
+      <x:c r="F58" s="76" t="str">
+        <x:v>List trả 1 active, không trả hidden; detail active có canvasJson; inactive/missing 404; seed tạm được xóa.</x:v>
+      </x:c>
+      <x:c r="G58" s="75" t="str">
+        <x:v>Smoke list Count=1 FirstName=Smoke Active Template ContainsHidden=false; detail active 200; inactive/missing 404; delete seed count còn 0.</x:v>
+      </x:c>
+      <x:c r="H58" s="75" t="str">
+        <x:v>TC_VIZI_049</x:v>
+      </x:c>
+      <x:c r="I58" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J58" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K58" s="75" t="str">
+        <x:v>Loại test: smoke/system/UAT nhỏ.</x:v>
+      </x:c>
+      <x:c r="L58" s="75"/>
+      <x:c r="M58" s="75"/>
+      <x:c r="N58" s="75"/>
+      <x:c r="O58" s="75"/>
       <x:c r="P58" s="75" t="n"/>
       <x:c r="Q58" s="75" t="n"/>
       <x:c r="R58" s="75" t="n"/>
@@ -4318,21 +4446,45 @@
       <x:c r="Z58" s="75" t="n"/>
     </x:row>
     <x:row r="59" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A59" s="75" t="n"/>
-      <x:c r="B59" s="76" t="n"/>
-      <x:c r="C59" s="75" t="n"/>
-      <x:c r="D59" s="75" t="n"/>
-      <x:c r="E59" s="75" t="n"/>
-      <x:c r="F59" s="76" t="n"/>
-      <x:c r="G59" s="75" t="n"/>
-      <x:c r="H59" s="75" t="n"/>
-      <x:c r="I59" s="75" t="n"/>
-      <x:c r="J59" s="75" t="n"/>
-      <x:c r="K59" s="75" t="n"/>
-      <x:c r="L59" s="75" t="n"/>
-      <x:c r="M59" s="75" t="n"/>
-      <x:c r="N59" s="75" t="n"/>
-      <x:c r="O59" s="75" t="n"/>
+      <x:c r="A59" s="75" t="str">
+        <x:v>TC_VIZI_051</x:v>
+      </x:c>
+      <x:c r="B59" s="76" t="str">
+        <x:v>Performance smoke Template API</x:v>
+      </x:c>
+      <x:c r="C59" s="75" t="str">
+        <x:v>Đo thời gian GET /api/templates sau warm-up trên máy local.</x:v>
+      </x:c>
+      <x:c r="D59" s="75" t="str">
+        <x:v>B1: Gọi /api/templates 5 lần sau khi backend đã warm.
+B2: Đo min/avg/max bằng Stopwatch.
+B3: So với ngưỡng smoke local.</x:v>
+      </x:c>
+      <x:c r="E59" s="75" t="str">
+        <x:v>GET /api/templates local</x:v>
+      </x:c>
+      <x:c r="F59" s="76" t="str">
+        <x:v>Average dưới 500ms trên local smoke.</x:v>
+      </x:c>
+      <x:c r="G59" s="75" t="str">
+        <x:v>5 requests: average 8.8ms, max 34ms, min 2ms.</x:v>
+      </x:c>
+      <x:c r="H59" s="75" t="str">
+        <x:v>TC_VIZI_050</x:v>
+      </x:c>
+      <x:c r="I59" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J59" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K59" s="75" t="str">
+        <x:v>Loại test: performance smoke, chưa phải load test sản xuất.</x:v>
+      </x:c>
+      <x:c r="L59" s="75"/>
+      <x:c r="M59" s="75"/>
+      <x:c r="N59" s="75"/>
+      <x:c r="O59" s="75"/>
       <x:c r="P59" s="75" t="n"/>
       <x:c r="Q59" s="75" t="n"/>
       <x:c r="R59" s="75" t="n"/>
@@ -4346,21 +4498,45 @@
       <x:c r="Z59" s="75" t="n"/>
     </x:row>
     <x:row r="60" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A60" s="75" t="n"/>
-      <x:c r="B60" s="76" t="n"/>
-      <x:c r="C60" s="75" t="n"/>
-      <x:c r="D60" s="75" t="n"/>
-      <x:c r="E60" s="75" t="n"/>
-      <x:c r="F60" s="76" t="n"/>
-      <x:c r="G60" s="75" t="n"/>
-      <x:c r="H60" s="75" t="n"/>
-      <x:c r="I60" s="75" t="n"/>
-      <x:c r="J60" s="75" t="n"/>
-      <x:c r="K60" s="75" t="n"/>
-      <x:c r="L60" s="75" t="n"/>
-      <x:c r="M60" s="75" t="n"/>
-      <x:c r="N60" s="75" t="n"/>
-      <x:c r="O60" s="75" t="n"/>
+      <x:c r="A60" s="75" t="str">
+        <x:v>TC_VIZI_052</x:v>
+      </x:c>
+      <x:c r="B60" s="76" t="str">
+        <x:v>Regression test backend và frontend sau Template API</x:v>
+      </x:c>
+      <x:c r="C60" s="75" t="str">
+        <x:v>Xác nhận thêm Template API không làm hỏng backend test suite và frontend build.</x:v>
+      </x:c>
+      <x:c r="D60" s="75" t="str">
+        <x:v>B1: Chạy backend mvnw test.
+B2: Chạy frontend npm run build.
+B3: Kiểm tra không còn DB test tạm và port 8080 đóng sau smoke.</x:v>
+      </x:c>
+      <x:c r="E60" s="75" t="str">
+        <x:v>Backend Maven tests, frontend Vite build</x:v>
+      </x:c>
+      <x:c r="F60" s="76" t="str">
+        <x:v>Backend pass 11/11; frontend build pass; không còn vizi_template_api_test_* hoặc vizi_schema_test_*.</x:v>
+      </x:c>
+      <x:c r="G60" s="75" t="str">
+        <x:v>mvnw test BUILD SUCCESS Tests run 11; npm run build pass; DB test tạm không còn; port 8080 closed.</x:v>
+      </x:c>
+      <x:c r="H60" s="75" t="str">
+        <x:v>TC_VIZI_051</x:v>
+      </x:c>
+      <x:c r="I60" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J60" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K60" s="75" t="str">
+        <x:v>Loại test: regression/system cleanup.</x:v>
+      </x:c>
+      <x:c r="L60" s="75"/>
+      <x:c r="M60" s="75"/>
+      <x:c r="N60" s="75"/>
+      <x:c r="O60" s="75"/>
       <x:c r="P60" s="75" t="n"/>
       <x:c r="Q60" s="75" t="n"/>
       <x:c r="R60" s="75" t="n"/>
@@ -4374,21 +4550,45 @@
       <x:c r="Z60" s="75" t="n"/>
     </x:row>
     <x:row r="61" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A61" s="75" t="n"/>
-      <x:c r="B61" s="76" t="n"/>
-      <x:c r="C61" s="75" t="n"/>
-      <x:c r="D61" s="75" t="n"/>
-      <x:c r="E61" s="75" t="n"/>
-      <x:c r="F61" s="76" t="n"/>
-      <x:c r="G61" s="75" t="n"/>
-      <x:c r="H61" s="75" t="n"/>
-      <x:c r="I61" s="75" t="n"/>
-      <x:c r="J61" s="75" t="n"/>
-      <x:c r="K61" s="75" t="n"/>
-      <x:c r="L61" s="75" t="n"/>
-      <x:c r="M61" s="75" t="n"/>
-      <x:c r="N61" s="75" t="n"/>
-      <x:c r="O61" s="75" t="n"/>
+      <x:c r="A61" s="75" t="str">
+        <x:v>TC_VIZI_053</x:v>
+      </x:c>
+      <x:c r="B61" s="76" t="str">
+        <x:v>Security scan Template API changes</x:v>
+      </x:c>
+      <x:c r="C61" s="75" t="str">
+        <x:v>Xác nhận thay đổi API template không thêm secret thật và không expose entity trực tiếp.</x:v>
+      </x:c>
+      <x:c r="D61" s="75" t="str">
+        <x:v>B1: Kiểm tra staged/source files.
+B2: Chạy rg secret pattern loại trừ node_modules/dist/target/.agents/.codex-work.
+B3: Kiểm tra controller trả DTO records thay vì entity.</x:v>
+      </x:c>
+      <x:c r="E61" s="75" t="str">
+        <x:v>TemplateController, TemplateResponse, toàn repo source</x:v>
+      </x:c>
+      <x:c r="F61" s="76" t="str">
+        <x:v>Không có API key/token/password thật; API trả DTO; inactive templates bị ẩn.</x:v>
+      </x:c>
+      <x:c r="G61" s="75" t="str">
+        <x:v>Secret scan chỉ thấy placeholder/env references/tài liệu/wrapper Maven; TemplateController trả TemplateListItem/TemplateDetail DTO.</x:v>
+      </x:c>
+      <x:c r="H61" s="75" t="str">
+        <x:v>TC_VIZI_052</x:v>
+      </x:c>
+      <x:c r="I61" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J61" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K61" s="75" t="str">
+        <x:v>Loại test: security/API design.</x:v>
+      </x:c>
+      <x:c r="L61" s="75"/>
+      <x:c r="M61" s="75"/>
+      <x:c r="N61" s="75"/>
+      <x:c r="O61" s="75"/>
       <x:c r="P61" s="75" t="n"/>
       <x:c r="Q61" s="75" t="n"/>
       <x:c r="R61" s="75" t="n"/>
@@ -30742,7 +30942,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86f28c35692b47f5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9373c7c1dfac463a"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add template list UI
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R3ee08e9e8b3149d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R9502e49c24184253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R9d8db3f9e69f4a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R0332a7e890e54641"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1162,7 +1162,7 @@
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
         <x:f>COUNTIF(I9:I998,"Pass")</x:f>
-        <x:v>52</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1170,7 +1170,7 @@
       </x:c>
       <x:c r="C5" s="90" t="n">
         <x:f>G5-E5-B5-A5</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="91" t="n"/>
       <x:c r="E5" s="90" t="n">
@@ -1180,7 +1180,7 @@
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
         <x:f>COUNTA(A9:A998)</x:f>
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -4602,21 +4602,45 @@
       <x:c r="Z61" s="75" t="n"/>
     </x:row>
     <x:row r="62" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A62" s="75" t="n"/>
-      <x:c r="B62" s="76" t="n"/>
-      <x:c r="C62" s="75" t="n"/>
-      <x:c r="D62" s="75" t="n"/>
-      <x:c r="E62" s="75" t="n"/>
-      <x:c r="F62" s="76" t="n"/>
-      <x:c r="G62" s="75" t="n"/>
-      <x:c r="H62" s="75" t="n"/>
-      <x:c r="I62" s="75" t="n"/>
-      <x:c r="J62" s="75" t="n"/>
-      <x:c r="K62" s="75" t="n"/>
-      <x:c r="L62" s="75" t="n"/>
-      <x:c r="M62" s="75" t="n"/>
-      <x:c r="N62" s="75" t="n"/>
-      <x:c r="O62" s="75" t="n"/>
+      <x:c r="A62" s="75" t="str">
+        <x:v>TC_VIZI_054</x:v>
+      </x:c>
+      <x:c r="B62" s="76" t="str">
+        <x:v>Frontend build sau khi them Template UI</x:v>
+      </x:c>
+      <x:c r="C62" s="75" t="str">
+        <x:v>Xac nhan FE typecheck/build thanh cong sau khi them getTemplates va template list tren HomeView.</x:v>
+      </x:c>
+      <x:c r="D62" s="75" t="str">
+        <x:v>B1: Them type TemplateListItem va getTemplates trong api.ts.
+B2: Them template loading/error/empty/list state trong HomeView.
+B3: Chay npm run build.</x:v>
+      </x:c>
+      <x:c r="E62" s="75" t="str">
+        <x:v>frontend/src/api.ts, HomeView.vue, styles.css</x:v>
+      </x:c>
+      <x:c r="F62" s="76" t="str">
+        <x:v>vue-tsc pass; Vite build pass; khong them dependency moi.</x:v>
+      </x:c>
+      <x:c r="G62" s="75" t="str">
+        <x:v>npm run build pass; Vite built 31 modules; dist assets sinh thanh cong.</x:v>
+      </x:c>
+      <x:c r="H62" s="75" t="str">
+        <x:v>TC_VIZI_053</x:v>
+      </x:c>
+      <x:c r="I62" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J62" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K62" s="75" t="str">
+        <x:v>Loai test: frontend typecheck/build regression.</x:v>
+      </x:c>
+      <x:c r="L62" s="75"/>
+      <x:c r="M62" s="75"/>
+      <x:c r="N62" s="75"/>
+      <x:c r="O62" s="75"/>
       <x:c r="P62" s="75" t="n"/>
       <x:c r="Q62" s="75" t="n"/>
       <x:c r="R62" s="75" t="n"/>
@@ -4630,21 +4654,47 @@
       <x:c r="Z62" s="75" t="n"/>
     </x:row>
     <x:row r="63" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A63" s="75" t="n"/>
-      <x:c r="B63" s="76" t="n"/>
-      <x:c r="C63" s="75" t="n"/>
-      <x:c r="D63" s="75" t="n"/>
-      <x:c r="E63" s="75" t="n"/>
-      <x:c r="F63" s="76" t="n"/>
-      <x:c r="G63" s="75" t="n"/>
-      <x:c r="H63" s="75" t="n"/>
-      <x:c r="I63" s="75" t="n"/>
-      <x:c r="J63" s="75" t="n"/>
-      <x:c r="K63" s="75" t="n"/>
-      <x:c r="L63" s="75" t="n"/>
-      <x:c r="M63" s="75" t="n"/>
-      <x:c r="N63" s="75" t="n"/>
-      <x:c r="O63" s="75" t="n"/>
+      <x:c r="A63" s="75" t="str">
+        <x:v>TC_VIZI_055</x:v>
+      </x:c>
+      <x:c r="B63" s="76" t="str">
+        <x:v>API smoke cho FE Template UI voi seed tam</x:v>
+      </x:c>
+      <x:c r="C63" s="75" t="str">
+        <x:v>Xac nhan backend /api/templates tra du lieu dung de FE render danh sach template.</x:v>
+      </x:c>
+      <x:c r="D63" s="75" t="str">
+        <x:v>B1: Insert FE Smoke Active Template active=true.
+B2: Insert FE Smoke Hidden Template active=false.
+B3: Start backend local.
+B4: Goi GET /api/templates.
+B5: Kiem tra hidden khong xuat hien.</x:v>
+      </x:c>
+      <x:c r="E63" s="75" t="str">
+        <x:v>PostgreSQL local 127.0.0.1:55432, backend port 8080</x:v>
+      </x:c>
+      <x:c r="F63" s="76" t="str">
+        <x:v>HTTP 200; Count=1; FirstName=FE Smoke Active Template; ContainsHidden=false.</x:v>
+      </x:c>
+      <x:c r="G63" s="75" t="str">
+        <x:v>API smoke output: {Count:1, FirstName:FE Smoke Active Template, ContainsHidden:false}.</x:v>
+      </x:c>
+      <x:c r="H63" s="75" t="str">
+        <x:v>TC_VIZI_054</x:v>
+      </x:c>
+      <x:c r="I63" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J63" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K63" s="75" t="str">
+        <x:v>Loai test: API smoke/data filter.</x:v>
+      </x:c>
+      <x:c r="L63" s="75"/>
+      <x:c r="M63" s="75"/>
+      <x:c r="N63" s="75"/>
+      <x:c r="O63" s="75"/>
       <x:c r="P63" s="75" t="n"/>
       <x:c r="Q63" s="75" t="n"/>
       <x:c r="R63" s="75" t="n"/>
@@ -4658,21 +4708,45 @@
       <x:c r="Z63" s="75" t="n"/>
     </x:row>
     <x:row r="64" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A64" s="75" t="n"/>
-      <x:c r="B64" s="76" t="n"/>
-      <x:c r="C64" s="75" t="n"/>
-      <x:c r="D64" s="75" t="n"/>
-      <x:c r="E64" s="75" t="n"/>
-      <x:c r="F64" s="76" t="n"/>
-      <x:c r="G64" s="75" t="n"/>
-      <x:c r="H64" s="75" t="n"/>
-      <x:c r="I64" s="75" t="n"/>
-      <x:c r="J64" s="75" t="n"/>
-      <x:c r="K64" s="75" t="n"/>
-      <x:c r="L64" s="75" t="n"/>
-      <x:c r="M64" s="75" t="n"/>
-      <x:c r="N64" s="75" t="n"/>
-      <x:c r="O64" s="75" t="n"/>
+      <x:c r="A64" s="75" t="str">
+        <x:v>TC_VIZI_056</x:v>
+      </x:c>
+      <x:c r="B64" s="76" t="str">
+        <x:v>CORS smoke tu frontend dev origin</x:v>
+      </x:c>
+      <x:c r="C64" s="75" t="str">
+        <x:v>Xac nhan backend cho FE dev server doc template API qua origin 127.0.0.1:5173.</x:v>
+      </x:c>
+      <x:c r="D64" s="75" t="str">
+        <x:v>B1: Start FE dev server 127.0.0.1:5173.
+B2: Goi curl GET /api/templates voi Origin http://127.0.0.1:5173.
+B3: Kiem tra header CORS va body.</x:v>
+      </x:c>
+      <x:c r="E64" s="75" t="str">
+        <x:v>curl.exe -H Origin:http://127.0.0.1:5173 /api/templates</x:v>
+      </x:c>
+      <x:c r="F64" s="76" t="str">
+        <x:v>Access-Control-Allow-Origin=http://127.0.0.1:5173; body co active template, khong co hidden template.</x:v>
+      </x:c>
+      <x:c r="G64" s="75" t="str">
+        <x:v>curl response HTTP 200 co Access-Control-Allow-Origin dung FE origin va JSON chi co FE Smoke Active Template.</x:v>
+      </x:c>
+      <x:c r="H64" s="75" t="str">
+        <x:v>TC_VIZI_055</x:v>
+      </x:c>
+      <x:c r="I64" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J64" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K64" s="75" t="str">
+        <x:v>Loai test: integration/CORS/security.</x:v>
+      </x:c>
+      <x:c r="L64" s="75"/>
+      <x:c r="M64" s="75"/>
+      <x:c r="N64" s="75"/>
+      <x:c r="O64" s="75"/>
       <x:c r="P64" s="75" t="n"/>
       <x:c r="Q64" s="75" t="n"/>
       <x:c r="R64" s="75" t="n"/>
@@ -4686,21 +4760,45 @@
       <x:c r="Z64" s="75" t="n"/>
     </x:row>
     <x:row r="65" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A65" s="75" t="n"/>
-      <x:c r="B65" s="76" t="n"/>
-      <x:c r="C65" s="75" t="n"/>
-      <x:c r="D65" s="75" t="n"/>
-      <x:c r="E65" s="75" t="n"/>
-      <x:c r="F65" s="76" t="n"/>
-      <x:c r="G65" s="75" t="n"/>
-      <x:c r="H65" s="75" t="n"/>
-      <x:c r="I65" s="75" t="n"/>
-      <x:c r="J65" s="75" t="n"/>
-      <x:c r="K65" s="75" t="n"/>
-      <x:c r="L65" s="75" t="n"/>
-      <x:c r="M65" s="75" t="n"/>
-      <x:c r="N65" s="75" t="n"/>
-      <x:c r="O65" s="75" t="n"/>
+      <x:c r="A65" s="75" t="str">
+        <x:v>TC_VIZI_057</x:v>
+      </x:c>
+      <x:c r="B65" s="76" t="str">
+        <x:v>Frontend dev server smoke</x:v>
+      </x:c>
+      <x:c r="C65" s="75" t="str">
+        <x:v>Xac nhan Vite dev server phuc vu app shell sau khi them Template UI.</x:v>
+      </x:c>
+      <x:c r="D65" s="75" t="str">
+        <x:v>B1: Start npm run dev -- --host 127.0.0.1.
+B2: curl http://127.0.0.1:5173/.
+B3: Kiem tra status va HTML root.</x:v>
+      </x:c>
+      <x:c r="E65" s="75" t="str">
+        <x:v>frontend dev server port 5173</x:v>
+      </x:c>
+      <x:c r="F65" s="76" t="str">
+        <x:v>HTTP 200; HTML co div id=app va /@vite/client.</x:v>
+      </x:c>
+      <x:c r="G65" s="75" t="str">
+        <x:v>curl response HTTP 200 OK; Content-Type text/html; co &lt;div id="app"&gt;&lt;/div&gt; va script /src/main.ts.</x:v>
+      </x:c>
+      <x:c r="H65" s="75" t="str">
+        <x:v>TC_VIZI_056</x:v>
+      </x:c>
+      <x:c r="I65" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J65" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K65" s="75" t="str">
+        <x:v>Loai test: smoke/system app shell.</x:v>
+      </x:c>
+      <x:c r="L65" s="75"/>
+      <x:c r="M65" s="75"/>
+      <x:c r="N65" s="75"/>
+      <x:c r="O65" s="75"/>
       <x:c r="P65" s="75" t="n"/>
       <x:c r="Q65" s="75" t="n"/>
       <x:c r="R65" s="75" t="n"/>
@@ -4714,21 +4812,46 @@
       <x:c r="Z65" s="75" t="n"/>
     </x:row>
     <x:row r="66" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A66" s="75" t="n"/>
-      <x:c r="B66" s="76" t="n"/>
-      <x:c r="C66" s="75" t="n"/>
-      <x:c r="D66" s="75" t="n"/>
-      <x:c r="E66" s="75" t="n"/>
-      <x:c r="F66" s="76" t="n"/>
-      <x:c r="G66" s="75" t="n"/>
-      <x:c r="H66" s="75" t="n"/>
-      <x:c r="I66" s="75" t="n"/>
-      <x:c r="J66" s="75" t="n"/>
-      <x:c r="K66" s="75" t="n"/>
-      <x:c r="L66" s="75" t="n"/>
-      <x:c r="M66" s="75" t="n"/>
-      <x:c r="N66" s="75" t="n"/>
-      <x:c r="O66" s="75" t="n"/>
+      <x:c r="A66" s="75" t="str">
+        <x:v>TC_VIZI_058</x:v>
+      </x:c>
+      <x:c r="B66" s="76" t="str">
+        <x:v>Browser automation visual check cho Template UI</x:v>
+      </x:c>
+      <x:c r="C66" s="75" t="str">
+        <x:v>Ghi nhan tinh trang visual browser automation trong moi truong hien tai.</x:v>
+      </x:c>
+      <x:c r="D66" s="75" t="str">
+        <x:v>B1: Thu Playwright bundled qua Node REPL.
+B2: Thu Chrome channel headless.
+B3: Thu npx playwright tam thoi.
+B4: Neu moi truong chan, khong danh dau visual screenshot la pass.</x:v>
+      </x:c>
+      <x:c r="E66" s="75" t="str">
+        <x:v>Playwright/Chrome local automation</x:v>
+      </x:c>
+      <x:c r="F66" s="76" t="str">
+        <x:v>Neu browser automation kha dung thi DOM co Backend UP, active template, khong co hidden template, console khong error.</x:v>
+      </x:c>
+      <x:c r="G66" s="75" t="str">
+        <x:v>Blocked by environment: bundled browser missing; Chrome spawn EPERM under sandbox; npx playwright returned exit 1 without usable output.</x:v>
+      </x:c>
+      <x:c r="H66" s="75" t="str">
+        <x:v>TC_VIZI_057</x:v>
+      </x:c>
+      <x:c r="I66" s="75" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J66" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K66" s="75" t="str">
+        <x:v>Khong phai bug product da verify; can re-run visual screenshot khi browser automation kha dung.</x:v>
+      </x:c>
+      <x:c r="L66" s="75"/>
+      <x:c r="M66" s="75"/>
+      <x:c r="N66" s="75"/>
+      <x:c r="O66" s="75"/>
       <x:c r="P66" s="75" t="n"/>
       <x:c r="Q66" s="75" t="n"/>
       <x:c r="R66" s="75" t="n"/>
@@ -4742,21 +4865,46 @@
       <x:c r="Z66" s="75" t="n"/>
     </x:row>
     <x:row r="67" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A67" s="75" t="n"/>
-      <x:c r="B67" s="76" t="n"/>
-      <x:c r="C67" s="75" t="n"/>
-      <x:c r="D67" s="75" t="n"/>
-      <x:c r="E67" s="75" t="n"/>
-      <x:c r="F67" s="76" t="n"/>
-      <x:c r="G67" s="75" t="n"/>
-      <x:c r="H67" s="75" t="n"/>
-      <x:c r="I67" s="75" t="n"/>
-      <x:c r="J67" s="75" t="n"/>
-      <x:c r="K67" s="75" t="n"/>
-      <x:c r="L67" s="75" t="n"/>
-      <x:c r="M67" s="75" t="n"/>
-      <x:c r="N67" s="75" t="n"/>
-      <x:c r="O67" s="75" t="n"/>
+      <x:c r="A67" s="75" t="str">
+        <x:v>TC_VIZI_059</x:v>
+      </x:c>
+      <x:c r="B67" s="76" t="str">
+        <x:v>Cleanup smoke data va server ports</x:v>
+      </x:c>
+      <x:c r="C67" s="75" t="str">
+        <x:v>Xac nhan seed tam duoc xoa va backend/frontend dev server khong con chay sau smoke.</x:v>
+      </x:c>
+      <x:c r="D67" s="75" t="str">
+        <x:v>B1: Delete templates co name FE Smoke Active/Hidden Template.
+B2: Select count name like FE Smoke%.
+B3: Stop backend/frontend PID.
+B4: Test port 8080 va 5173.</x:v>
+      </x:c>
+      <x:c r="E67" s="75" t="str">
+        <x:v>PostgreSQL local, ports 8080/5173</x:v>
+      </x:c>
+      <x:c r="F67" s="76" t="str">
+        <x:v>DELETE 2; remaining_smoke_templates=0; port 8080 false; port 5173 false.</x:v>
+      </x:c>
+      <x:c r="G67" s="75" t="str">
+        <x:v>Cleanup pass: xoa 2 rows; count con 0; Test-NetConnection 8080/5173 TcpTestSucceeded=False.</x:v>
+      </x:c>
+      <x:c r="H67" s="75" t="str">
+        <x:v>TC_VIZI_058</x:v>
+      </x:c>
+      <x:c r="I67" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J67" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K67" s="75" t="str">
+        <x:v>Loai test: cleanup/regression environment.</x:v>
+      </x:c>
+      <x:c r="L67" s="75"/>
+      <x:c r="M67" s="75"/>
+      <x:c r="N67" s="75"/>
+      <x:c r="O67" s="75"/>
       <x:c r="P67" s="75" t="n"/>
       <x:c r="Q67" s="75" t="n"/>
       <x:c r="R67" s="75" t="n"/>
@@ -4770,21 +4918,44 @@
       <x:c r="Z67" s="75" t="n"/>
     </x:row>
     <x:row r="68" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A68" s="75" t="n"/>
-      <x:c r="B68" s="76" t="n"/>
-      <x:c r="C68" s="75" t="n"/>
-      <x:c r="D68" s="75" t="n"/>
-      <x:c r="E68" s="75" t="n"/>
-      <x:c r="F68" s="76" t="n"/>
-      <x:c r="G68" s="75" t="n"/>
-      <x:c r="H68" s="75" t="n"/>
-      <x:c r="I68" s="75" t="n"/>
-      <x:c r="J68" s="75" t="n"/>
-      <x:c r="K68" s="75" t="n"/>
-      <x:c r="L68" s="75" t="n"/>
-      <x:c r="M68" s="75" t="n"/>
-      <x:c r="N68" s="75" t="n"/>
-      <x:c r="O68" s="75" t="n"/>
+      <x:c r="A68" s="75" t="str">
+        <x:v>TC_VIZI_060</x:v>
+      </x:c>
+      <x:c r="B68" s="76" t="str">
+        <x:v>Regression backend sau FE Template UI</x:v>
+      </x:c>
+      <x:c r="C68" s="75" t="str">
+        <x:v>Xac nhan thay doi FE khong lam lech API contract backend va test suite backend van xanh.</x:v>
+      </x:c>
+      <x:c r="D68" s="75" t="str">
+        <x:v>B1: Sau khi cleanup smoke, chay backend mvnw test.
+B2: Kiem tra temp DB duoc migrate va test API van pass.</x:v>
+      </x:c>
+      <x:c r="E68" s="75" t="str">
+        <x:v>backend Maven test suite</x:v>
+      </x:c>
+      <x:c r="F68" s="76" t="str">
+        <x:v>BUILD SUCCESS; Tests run 11, Failures 0, Errors 0, Skipped 0.</x:v>
+      </x:c>
+      <x:c r="G68" s="75" t="str">
+        <x:v>mvnw test pass 11/11; TemplateApiIntegrationTests va TemplateServiceTests pass.</x:v>
+      </x:c>
+      <x:c r="H68" s="75" t="str">
+        <x:v>TC_VIZI_059</x:v>
+      </x:c>
+      <x:c r="I68" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J68" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K68" s="75" t="str">
+        <x:v>Loai test: backend regression/integration.</x:v>
+      </x:c>
+      <x:c r="L68" s="75"/>
+      <x:c r="M68" s="75"/>
+      <x:c r="N68" s="75"/>
+      <x:c r="O68" s="75"/>
       <x:c r="P68" s="75" t="n"/>
       <x:c r="Q68" s="75" t="n"/>
       <x:c r="R68" s="75" t="n"/>
@@ -30942,7 +31113,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9373c7c1dfac463a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48390e8ddbbc4540"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add template detail route
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R9d8db3f9e69f4a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R0332a7e890e54641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R6a1271ce89eb41f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5779240e2a12440c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1162,7 +1162,7 @@
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
         <x:f>COUNTIF(I9:I998,"Pass")</x:f>
-        <x:v>58</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
         <x:f>COUNTA(A9:A998)</x:f>
-        <x:v>60</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -4969,21 +4969,46 @@
       <x:c r="Z68" s="75" t="n"/>
     </x:row>
     <x:row r="69" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A69" s="75" t="n"/>
-      <x:c r="B69" s="76" t="n"/>
-      <x:c r="C69" s="75" t="n"/>
-      <x:c r="D69" s="75" t="n"/>
-      <x:c r="E69" s="75" t="n"/>
-      <x:c r="F69" s="76" t="n"/>
-      <x:c r="G69" s="75" t="n"/>
-      <x:c r="H69" s="75" t="n"/>
-      <x:c r="I69" s="75" t="n"/>
-      <x:c r="J69" s="75" t="n"/>
-      <x:c r="K69" s="75" t="n"/>
-      <x:c r="L69" s="75" t="n"/>
-      <x:c r="M69" s="75" t="n"/>
-      <x:c r="N69" s="75" t="n"/>
-      <x:c r="O69" s="75" t="n"/>
+      <x:c r="A69" s="75" t="str">
+        <x:v>TC_VIZI_061</x:v>
+      </x:c>
+      <x:c r="B69" s="76" t="str">
+        <x:v>Frontend build cho route chi tiet template</x:v>
+      </x:c>
+      <x:c r="C69" s="75" t="str">
+        <x:v>Xac nhan them getTemplate, route /templates/:id va TemplateDetailView khong gay loi typecheck/build.</x:v>
+      </x:c>
+      <x:c r="D69" s="75" t="str">
+        <x:v>B1: Them TemplateDetail type va getTemplate(id).
+B2: Them route /templates/:id.
+B3: Them TemplateDetailView.
+B4: Chay npm run build.</x:v>
+      </x:c>
+      <x:c r="E69" s="75" t="str">
+        <x:v>frontend/src/api.ts, router.ts, TemplateDetailView.vue</x:v>
+      </x:c>
+      <x:c r="F69" s="76" t="str">
+        <x:v>vue-tsc pass; Vite build pass; 33 modules transformed.</x:v>
+      </x:c>
+      <x:c r="G69" s="75" t="str">
+        <x:v>npm run build pass; dist JS/CSS sinh thanh cong.</x:v>
+      </x:c>
+      <x:c r="H69" s="75" t="str">
+        <x:v>TC_VIZI_060</x:v>
+      </x:c>
+      <x:c r="I69" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J69" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K69" s="75" t="str">
+        <x:v>Loai test: frontend build/typecheck.</x:v>
+      </x:c>
+      <x:c r="L69" s="75"/>
+      <x:c r="M69" s="75"/>
+      <x:c r="N69" s="75"/>
+      <x:c r="O69" s="75"/>
       <x:c r="P69" s="75" t="n"/>
       <x:c r="Q69" s="75" t="n"/>
       <x:c r="R69" s="75" t="n"/>
@@ -4997,21 +5022,45 @@
       <x:c r="Z69" s="75" t="n"/>
     </x:row>
     <x:row r="70" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A70" s="75" t="n"/>
-      <x:c r="B70" s="76" t="n"/>
-      <x:c r="C70" s="75" t="n"/>
-      <x:c r="D70" s="75" t="n"/>
-      <x:c r="E70" s="75" t="n"/>
-      <x:c r="F70" s="76" t="n"/>
-      <x:c r="G70" s="75" t="n"/>
-      <x:c r="H70" s="75" t="n"/>
-      <x:c r="I70" s="75" t="n"/>
-      <x:c r="J70" s="75" t="n"/>
-      <x:c r="K70" s="75" t="n"/>
-      <x:c r="L70" s="75" t="n"/>
-      <x:c r="M70" s="75" t="n"/>
-      <x:c r="N70" s="75" t="n"/>
-      <x:c r="O70" s="75" t="n"/>
+      <x:c r="A70" s="75" t="str">
+        <x:v>TC_VIZI_062</x:v>
+      </x:c>
+      <x:c r="B70" s="76" t="str">
+        <x:v>Home template card link den detail route</x:v>
+      </x:c>
+      <x:c r="C70" s="75" t="str">
+        <x:v>Xac nhan card template tren Home la RouterLink toi route template-detail theo id.</x:v>
+      </x:c>
+      <x:c r="D70" s="75" t="str">
+        <x:v>B1: Render danh sach template tu /api/templates.
+B2: Moi card dung :to name=template-detail params id.
+B3: Kiem tra build typecheck.</x:v>
+      </x:c>
+      <x:c r="E70" s="75" t="str">
+        <x:v>frontend/src/views/HomeView.vue</x:v>
+      </x:c>
+      <x:c r="F70" s="76" t="str">
+        <x:v>Template card co the dieu huong den /templates/:id va van giu loading/error/empty state.</x:v>
+      </x:c>
+      <x:c r="G70" s="75" t="str">
+        <x:v>Build pass; HomeView compile thanh cong voi RouterLink va params id.</x:v>
+      </x:c>
+      <x:c r="H70" s="75" t="str">
+        <x:v>TC_VIZI_061</x:v>
+      </x:c>
+      <x:c r="I70" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J70" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K70" s="75" t="str">
+        <x:v>Loai test: navigation/static regression.</x:v>
+      </x:c>
+      <x:c r="L70" s="75"/>
+      <x:c r="M70" s="75"/>
+      <x:c r="N70" s="75"/>
+      <x:c r="O70" s="75"/>
       <x:c r="P70" s="75" t="n"/>
       <x:c r="Q70" s="75" t="n"/>
       <x:c r="R70" s="75" t="n"/>
@@ -5025,21 +5074,47 @@
       <x:c r="Z70" s="75" t="n"/>
     </x:row>
     <x:row r="71" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A71" s="75" t="n"/>
-      <x:c r="B71" s="76" t="n"/>
-      <x:c r="C71" s="75" t="n"/>
-      <x:c r="D71" s="75" t="n"/>
-      <x:c r="E71" s="75" t="n"/>
-      <x:c r="F71" s="76" t="n"/>
-      <x:c r="G71" s="75" t="n"/>
-      <x:c r="H71" s="75" t="n"/>
-      <x:c r="I71" s="75" t="n"/>
-      <x:c r="J71" s="75" t="n"/>
-      <x:c r="K71" s="75" t="n"/>
-      <x:c r="L71" s="75" t="n"/>
-      <x:c r="M71" s="75" t="n"/>
-      <x:c r="N71" s="75" t="n"/>
-      <x:c r="O71" s="75" t="n"/>
+      <x:c r="A71" s="75" t="str">
+        <x:v>TC_VIZI_063</x:v>
+      </x:c>
+      <x:c r="B71" s="76" t="str">
+        <x:v>API smoke detail template cho route moi</x:v>
+      </x:c>
+      <x:c r="C71" s="75" t="str">
+        <x:v>Xac nhan FE detail route co API detail hop dong dung tu backend.</x:v>
+      </x:c>
+      <x:c r="D71" s="75" t="str">
+        <x:v>B1: Seed Luxury Step31 Template active=true co canvas 1 layer.
+B2: Seed hidden template active=false.
+B3: Start backend local.
+B4: GET /api/templates/5.
+B5: GET inactive id 6.</x:v>
+      </x:c>
+      <x:c r="E71" s="75" t="str">
+        <x:v>backend /api/templates/{id}</x:v>
+      </x:c>
+      <x:c r="F71" s="76" t="str">
+        <x:v>Active detail HTTP 200 co name/category/dimension/canvasJson; inactive id tra 404.</x:v>
+      </x:c>
+      <x:c r="G71" s="75" t="str">
+        <x:v>Detail output Name=Luxury Step31 Template, Category=executive, LayerCount=1; inactive id 6 tra 404.</x:v>
+      </x:c>
+      <x:c r="H71" s="75" t="str">
+        <x:v>TC_VIZI_062</x:v>
+      </x:c>
+      <x:c r="I71" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J71" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K71" s="75" t="str">
+        <x:v>Loai test: API smoke/security inactive hidden.</x:v>
+      </x:c>
+      <x:c r="L71" s="75"/>
+      <x:c r="M71" s="75"/>
+      <x:c r="N71" s="75"/>
+      <x:c r="O71" s="75"/>
       <x:c r="P71" s="75" t="n"/>
       <x:c r="Q71" s="75" t="n"/>
       <x:c r="R71" s="75" t="n"/>
@@ -5053,21 +5128,46 @@
       <x:c r="Z71" s="75" t="n"/>
     </x:row>
     <x:row r="72" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A72" s="75" t="n"/>
-      <x:c r="B72" s="76" t="n"/>
-      <x:c r="C72" s="75" t="n"/>
-      <x:c r="D72" s="75" t="n"/>
-      <x:c r="E72" s="75" t="n"/>
-      <x:c r="F72" s="76" t="n"/>
-      <x:c r="G72" s="75" t="n"/>
-      <x:c r="H72" s="75" t="n"/>
-      <x:c r="I72" s="75" t="n"/>
-      <x:c r="J72" s="75" t="n"/>
-      <x:c r="K72" s="75" t="n"/>
-      <x:c r="L72" s="75" t="n"/>
-      <x:c r="M72" s="75" t="n"/>
-      <x:c r="N72" s="75" t="n"/>
-      <x:c r="O72" s="75" t="n"/>
+      <x:c r="A72" s="75" t="str">
+        <x:v>TC_VIZI_064</x:v>
+      </x:c>
+      <x:c r="B72" s="76" t="str">
+        <x:v>Frontend dev server route detail</x:v>
+      </x:c>
+      <x:c r="C72" s="75" t="str">
+        <x:v>Xac nhan Vite dev server phuc vu route /templates/:id cho Vue Router history mode.</x:v>
+      </x:c>
+      <x:c r="D72" s="75" t="str">
+        <x:v>B1: Start frontend dev server voi VITE_API_BASE_URL.
+B2: curl /.
+B3: curl /templates/5.
+B4: Kiem tra app shell.</x:v>
+      </x:c>
+      <x:c r="E72" s="75" t="str">
+        <x:v>frontend dev server port 5173</x:v>
+      </x:c>
+      <x:c r="F72" s="76" t="str">
+        <x:v>HTTP 200 cho / va /templates/5; HTML co div id=app va /src/main.ts.</x:v>
+      </x:c>
+      <x:c r="G72" s="75" t="str">
+        <x:v>curl /templates/5 tra HTTP 200 OK app shell; detail API CORS cung tra 200.</x:v>
+      </x:c>
+      <x:c r="H72" s="75" t="str">
+        <x:v>TC_VIZI_063</x:v>
+      </x:c>
+      <x:c r="I72" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J72" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K72" s="75" t="str">
+        <x:v>Loai test: SPA route smoke.</x:v>
+      </x:c>
+      <x:c r="L72" s="75"/>
+      <x:c r="M72" s="75"/>
+      <x:c r="N72" s="75"/>
+      <x:c r="O72" s="75"/>
       <x:c r="P72" s="75" t="n"/>
       <x:c r="Q72" s="75" t="n"/>
       <x:c r="R72" s="75" t="n"/>
@@ -5081,21 +5181,45 @@
       <x:c r="Z72" s="75" t="n"/>
     </x:row>
     <x:row r="73" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A73" s="75" t="n"/>
-      <x:c r="B73" s="76" t="n"/>
-      <x:c r="C73" s="75" t="n"/>
-      <x:c r="D73" s="75" t="n"/>
-      <x:c r="E73" s="75" t="n"/>
-      <x:c r="F73" s="76" t="n"/>
-      <x:c r="G73" s="75" t="n"/>
-      <x:c r="H73" s="75" t="n"/>
-      <x:c r="I73" s="75" t="n"/>
-      <x:c r="J73" s="75" t="n"/>
-      <x:c r="K73" s="75" t="n"/>
-      <x:c r="L73" s="75" t="n"/>
-      <x:c r="M73" s="75" t="n"/>
-      <x:c r="N73" s="75" t="n"/>
-      <x:c r="O73" s="75" t="n"/>
+      <x:c r="A73" s="75" t="str">
+        <x:v>TC_VIZI_065</x:v>
+      </x:c>
+      <x:c r="B73" s="76" t="str">
+        <x:v>Luxury light UI static regression</x:v>
+      </x:c>
+      <x:c r="C73" s="75" t="str">
+        <x:v>Xac nhan UI duoc chuyen sang phong cach sang mau, chuyen nghiep, luxury ma khong them package.</x:v>
+      </x:c>
+      <x:c r="D73" s="75" t="str">
+        <x:v>B1: Cap nhat palette warm ivory/champagne.
+B2: Them serif heading, card hover/focus, detail shell.
+B3: Kiem tra CSS khong dung secret hoac external asset.</x:v>
+      </x:c>
+      <x:c r="E73" s="75" t="str">
+        <x:v>frontend/src/styles.css, App.vue, HomeView.vue, TemplateDetailView.vue</x:v>
+      </x:c>
+      <x:c r="F73" s="76" t="str">
+        <x:v>UI van la light theme; khong them dependency; CSS responsive co mobile fallback.</x:v>
+      </x:c>
+      <x:c r="G73" s="75" t="str">
+        <x:v>Build pass; git diff chi gom CSS/Vue/API/router va workbook.</x:v>
+      </x:c>
+      <x:c r="H73" s="75" t="str">
+        <x:v>TC_VIZI_064</x:v>
+      </x:c>
+      <x:c r="I73" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J73" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K73" s="75" t="str">
+        <x:v>Loai test: visual/static/style regression.</x:v>
+      </x:c>
+      <x:c r="L73" s="75"/>
+      <x:c r="M73" s="75"/>
+      <x:c r="N73" s="75"/>
+      <x:c r="O73" s="75"/>
       <x:c r="P73" s="75" t="n"/>
       <x:c r="Q73" s="75" t="n"/>
       <x:c r="R73" s="75" t="n"/>
@@ -5109,21 +5233,46 @@
       <x:c r="Z73" s="75" t="n"/>
     </x:row>
     <x:row r="74" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A74" s="75" t="n"/>
-      <x:c r="B74" s="76" t="n"/>
-      <x:c r="C74" s="75" t="n"/>
-      <x:c r="D74" s="75" t="n"/>
-      <x:c r="E74" s="75" t="n"/>
-      <x:c r="F74" s="76" t="n"/>
-      <x:c r="G74" s="75" t="n"/>
-      <x:c r="H74" s="75" t="n"/>
-      <x:c r="I74" s="75" t="n"/>
-      <x:c r="J74" s="75" t="n"/>
-      <x:c r="K74" s="75" t="n"/>
-      <x:c r="L74" s="75" t="n"/>
-      <x:c r="M74" s="75" t="n"/>
-      <x:c r="N74" s="75" t="n"/>
-      <x:c r="O74" s="75" t="n"/>
+      <x:c r="A74" s="75" t="str">
+        <x:v>TC_VIZI_066</x:v>
+      </x:c>
+      <x:c r="B74" s="76" t="str">
+        <x:v>Cleanup Step31 smoke data va ports</x:v>
+      </x:c>
+      <x:c r="C74" s="75" t="str">
+        <x:v>Xac nhan seed tam Step31 duoc xoa va server local da dung.</x:v>
+      </x:c>
+      <x:c r="D74" s="75" t="str">
+        <x:v>B1: Delete templates name Luxury Step31 Template/Hidden.
+B2: Count name like Luxury Step31%.
+B3: Stop backend/frontend PID.
+B4: Test port 8080 va 5173.</x:v>
+      </x:c>
+      <x:c r="E74" s="75" t="str">
+        <x:v>PostgreSQL local, ports 8080/5173</x:v>
+      </x:c>
+      <x:c r="F74" s="76" t="str">
+        <x:v>DELETE 2; remaining_step31_templates=0; ports 8080/5173 closed.</x:v>
+      </x:c>
+      <x:c r="G74" s="75" t="str">
+        <x:v>Cleanup pass: remaining_step31_templates=0; TcpTestSucceeded=False cho 8080 va 5173.</x:v>
+      </x:c>
+      <x:c r="H74" s="75" t="str">
+        <x:v>TC_VIZI_065</x:v>
+      </x:c>
+      <x:c r="I74" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J74" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K74" s="75" t="str">
+        <x:v>Loai test: cleanup/environment regression.</x:v>
+      </x:c>
+      <x:c r="L74" s="75"/>
+      <x:c r="M74" s="75"/>
+      <x:c r="N74" s="75"/>
+      <x:c r="O74" s="75"/>
       <x:c r="P74" s="75" t="n"/>
       <x:c r="Q74" s="75" t="n"/>
       <x:c r="R74" s="75" t="n"/>
@@ -5137,21 +5286,46 @@
       <x:c r="Z74" s="75" t="n"/>
     </x:row>
     <x:row r="75" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A75" s="75" t="n"/>
-      <x:c r="B75" s="76" t="n"/>
-      <x:c r="C75" s="75" t="n"/>
-      <x:c r="D75" s="75" t="n"/>
-      <x:c r="E75" s="75" t="n"/>
-      <x:c r="F75" s="76" t="n"/>
-      <x:c r="G75" s="75" t="n"/>
-      <x:c r="H75" s="75" t="n"/>
-      <x:c r="I75" s="75" t="n"/>
-      <x:c r="J75" s="75" t="n"/>
-      <x:c r="K75" s="75" t="n"/>
-      <x:c r="L75" s="75" t="n"/>
-      <x:c r="M75" s="75" t="n"/>
-      <x:c r="N75" s="75" t="n"/>
-      <x:c r="O75" s="75" t="n"/>
+      <x:c r="A75" s="75" t="str">
+        <x:v>TC_VIZI_067</x:v>
+      </x:c>
+      <x:c r="B75" s="76" t="str">
+        <x:v>Regression sau Step31</x:v>
+      </x:c>
+      <x:c r="C75" s="75" t="str">
+        <x:v>Xac nhan sau route detail va luxury UI, backend/frontend van xanh.</x:v>
+      </x:c>
+      <x:c r="D75" s="75" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Chay backend mvnw test.
+B3: Kiem tra khong con DB test tam.
+B4: Secret scan truoc commit.</x:v>
+      </x:c>
+      <x:c r="E75" s="75" t="str">
+        <x:v>Frontend build, backend Maven tests, repo secret scan</x:v>
+      </x:c>
+      <x:c r="F75" s="76" t="str">
+        <x:v>FE build pass; backend tests run 11 fail 0 error 0; secret scan khong co secret that.</x:v>
+      </x:c>
+      <x:c r="G75" s="75" t="str">
+        <x:v>npm run build pass; mvnw test BUILD SUCCESS Tests run 11; secret scan chi thay placeholder/env references.</x:v>
+      </x:c>
+      <x:c r="H75" s="75" t="str">
+        <x:v>TC_VIZI_066</x:v>
+      </x:c>
+      <x:c r="I75" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J75" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K75" s="75" t="str">
+        <x:v>Loai test: regression/security pre-commit.</x:v>
+      </x:c>
+      <x:c r="L75" s="75"/>
+      <x:c r="M75" s="75"/>
+      <x:c r="N75" s="75"/>
+      <x:c r="O75" s="75"/>
       <x:c r="P75" s="75" t="n"/>
       <x:c r="Q75" s="75" t="n"/>
       <x:c r="R75" s="75" t="n"/>
@@ -31113,7 +31287,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48390e8ddbbc4540"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0f990541eb94c23"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Render template canvas preview
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R6a1271ce89eb41f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5779240e2a12440c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R0706674046134872"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc930892ee2a848e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1162,7 +1162,7 @@
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
         <x:f>COUNTIF(I9:I998,"Pass")</x:f>
-        <x:v>65</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
         <x:f>COUNTA(A9:A998)</x:f>
-        <x:v>67</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -5339,21 +5339,46 @@
       <x:c r="Z75" s="75" t="n"/>
     </x:row>
     <x:row r="76" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A76" s="75" t="n"/>
-      <x:c r="B76" s="76" t="n"/>
-      <x:c r="C76" s="75" t="n"/>
-      <x:c r="D76" s="75" t="n"/>
-      <x:c r="E76" s="75" t="n"/>
-      <x:c r="F76" s="76" t="n"/>
-      <x:c r="G76" s="75" t="n"/>
-      <x:c r="H76" s="75" t="n"/>
-      <x:c r="I76" s="75" t="n"/>
-      <x:c r="J76" s="75" t="n"/>
-      <x:c r="K76" s="75" t="n"/>
-      <x:c r="L76" s="75" t="n"/>
-      <x:c r="M76" s="75" t="n"/>
-      <x:c r="N76" s="75" t="n"/>
-      <x:c r="O76" s="75" t="n"/>
+      <x:c r="A76" s="75" t="str">
+        <x:v>TC_VIZI_068</x:v>
+      </x:c>
+      <x:c r="B76" s="76" t="str">
+        <x:v>Frontend build cho canvas renderer</x:v>
+      </x:c>
+      <x:c r="C76" s="75" t="str">
+        <x:v>Xac nhan TemplateDetailView render canvasJson bang CSS layers ma khong loi typecheck/build.</x:v>
+      </x:c>
+      <x:c r="D76" s="75" t="str">
+        <x:v>B1: Them parser canvasJson.
+B2: Them canvasLayers, canvasFrameStyle, layerStyle.
+B3: Them CSS canvas-frame/canvas-layer.
+B4: Chay npm run build.</x:v>
+      </x:c>
+      <x:c r="E76" s="75" t="str">
+        <x:v>frontend/src/views/TemplateDetailView.vue, styles.css</x:v>
+      </x:c>
+      <x:c r="F76" s="76" t="str">
+        <x:v>vue-tsc pass; Vite build pass; 33 modules transformed.</x:v>
+      </x:c>
+      <x:c r="G76" s="75" t="str">
+        <x:v>npm run build pass; dist CSS/JS sinh thanh cong.</x:v>
+      </x:c>
+      <x:c r="H76" s="75" t="str">
+        <x:v>TC_VIZI_067</x:v>
+      </x:c>
+      <x:c r="I76" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J76" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K76" s="75" t="str">
+        <x:v>Loai test: frontend build/typecheck.</x:v>
+      </x:c>
+      <x:c r="L76" s="75"/>
+      <x:c r="M76" s="75"/>
+      <x:c r="N76" s="75"/>
+      <x:c r="O76" s="75"/>
       <x:c r="P76" s="75" t="n"/>
       <x:c r="Q76" s="75" t="n"/>
       <x:c r="R76" s="75" t="n"/>
@@ -5367,21 +5392,45 @@
       <x:c r="Z76" s="75" t="n"/>
     </x:row>
     <x:row r="77" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A77" s="75" t="n"/>
-      <x:c r="B77" s="76" t="n"/>
-      <x:c r="C77" s="75" t="n"/>
-      <x:c r="D77" s="75" t="n"/>
-      <x:c r="E77" s="75" t="n"/>
-      <x:c r="F77" s="76" t="n"/>
-      <x:c r="G77" s="75" t="n"/>
-      <x:c r="H77" s="75" t="n"/>
-      <x:c r="I77" s="75" t="n"/>
-      <x:c r="J77" s="75" t="n"/>
-      <x:c r="K77" s="75" t="n"/>
-      <x:c r="L77" s="75" t="n"/>
-      <x:c r="M77" s="75" t="n"/>
-      <x:c r="N77" s="75" t="n"/>
-      <x:c r="O77" s="75" t="n"/>
+      <x:c r="A77" s="75" t="str">
+        <x:v>TC_VIZI_069</x:v>
+      </x:c>
+      <x:c r="B77" s="76" t="str">
+        <x:v>Canvas renderer static security</x:v>
+      </x:c>
+      <x:c r="C77" s="75" t="str">
+        <x:v>Xac nhan renderer khong render HTML raw tu canvasJson va khong them secret vao FE.</x:v>
+      </x:c>
+      <x:c r="D77" s="75" t="str">
+        <x:v>B1: Search v-html/innerHTML/outerHTML/dangerously trong frontend/src.
+B2: Search secret pattern trong frontend/src.
+B3: Search font-size theo vw va negative letter-spacing.</x:v>
+      </x:c>
+      <x:c r="E77" s="75" t="str">
+        <x:v>frontend/src</x:v>
+      </x:c>
+      <x:c r="F77" s="76" t="str">
+        <x:v>Khong co v-html/innerHTML/outerHTML; khong co secret pattern; khong co font-size theo vw.</x:v>
+      </x:c>
+      <x:c r="G77" s="75" t="str">
+        <x:v>rg scan tra 0 match cho raw HTML/secret/font-size vw/negative letter-spacing.</x:v>
+      </x:c>
+      <x:c r="H77" s="75" t="str">
+        <x:v>TC_VIZI_068</x:v>
+      </x:c>
+      <x:c r="I77" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J77" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K77" s="75" t="str">
+        <x:v>Loai test: security/static regression.</x:v>
+      </x:c>
+      <x:c r="L77" s="75"/>
+      <x:c r="M77" s="75"/>
+      <x:c r="N77" s="75"/>
+      <x:c r="O77" s="75"/>
       <x:c r="P77" s="75" t="n"/>
       <x:c r="Q77" s="75" t="n"/>
       <x:c r="R77" s="75" t="n"/>
@@ -5395,21 +5444,47 @@
       <x:c r="Z77" s="75" t="n"/>
     </x:row>
     <x:row r="78" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A78" s="75" t="n"/>
-      <x:c r="B78" s="76" t="n"/>
-      <x:c r="C78" s="75" t="n"/>
-      <x:c r="D78" s="75" t="n"/>
-      <x:c r="E78" s="75" t="n"/>
-      <x:c r="F78" s="76" t="n"/>
-      <x:c r="G78" s="75" t="n"/>
-      <x:c r="H78" s="75" t="n"/>
-      <x:c r="I78" s="75" t="n"/>
-      <x:c r="J78" s="75" t="n"/>
-      <x:c r="K78" s="75" t="n"/>
-      <x:c r="L78" s="75" t="n"/>
-      <x:c r="M78" s="75" t="n"/>
-      <x:c r="N78" s="75" t="n"/>
-      <x:c r="O78" s="75" t="n"/>
+      <x:c r="A78" s="75" t="str">
+        <x:v>TC_VIZI_070</x:v>
+      </x:c>
+      <x:c r="B78" s="76" t="str">
+        <x:v>API smoke canvasJson nhieu layer</x:v>
+      </x:c>
+      <x:c r="C78" s="75" t="str">
+        <x:v>Xac nhan backend detail API tra canvasJson co nhieu layer de FE renderer dung.</x:v>
+      </x:c>
+      <x:c r="D78" s="75" t="str">
+        <x:v>B1: Seed Canvas Step32 Template active=true co rect/text/text layers.
+B2: Seed hidden template active=false.
+B3: Start backend local.
+B4: GET /api/templates/7.
+B5: GET inactive id 8.</x:v>
+      </x:c>
+      <x:c r="E78" s="75" t="str">
+        <x:v>backend /api/templates/{id}</x:v>
+      </x:c>
+      <x:c r="F78" s="76" t="str">
+        <x:v>Active detail HTTP 200 co 3 layers type rect,text,text; inactive id tra 404.</x:v>
+      </x:c>
+      <x:c r="G78" s="75" t="str">
+        <x:v>Detail output Name=Canvas Step32 Template, LayerCount=3, Types=rect,text,text, Text=Bao Studio; inactive id 8 tra 404.</x:v>
+      </x:c>
+      <x:c r="H78" s="75" t="str">
+        <x:v>TC_VIZI_069</x:v>
+      </x:c>
+      <x:c r="I78" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J78" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K78" s="75" t="str">
+        <x:v>Loai test: API smoke/data contract/security inactive hidden.</x:v>
+      </x:c>
+      <x:c r="L78" s="75"/>
+      <x:c r="M78" s="75"/>
+      <x:c r="N78" s="75"/>
+      <x:c r="O78" s="75"/>
       <x:c r="P78" s="75" t="n"/>
       <x:c r="Q78" s="75" t="n"/>
       <x:c r="R78" s="75" t="n"/>
@@ -5423,21 +5498,46 @@
       <x:c r="Z78" s="75" t="n"/>
     </x:row>
     <x:row r="79" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A79" s="75" t="n"/>
-      <x:c r="B79" s="76" t="n"/>
-      <x:c r="C79" s="75" t="n"/>
-      <x:c r="D79" s="75" t="n"/>
-      <x:c r="E79" s="75" t="n"/>
-      <x:c r="F79" s="76" t="n"/>
-      <x:c r="G79" s="75" t="n"/>
-      <x:c r="H79" s="75" t="n"/>
-      <x:c r="I79" s="75" t="n"/>
-      <x:c r="J79" s="75" t="n"/>
-      <x:c r="K79" s="75" t="n"/>
-      <x:c r="L79" s="75" t="n"/>
-      <x:c r="M79" s="75" t="n"/>
-      <x:c r="N79" s="75" t="n"/>
-      <x:c r="O79" s="75" t="n"/>
+      <x:c r="A79" s="75" t="str">
+        <x:v>TC_VIZI_071</x:v>
+      </x:c>
+      <x:c r="B79" s="76" t="str">
+        <x:v>Frontend dev route cho canvas preview</x:v>
+      </x:c>
+      <x:c r="C79" s="75" t="str">
+        <x:v>Xac nhan Vite dev server phuc vu route detail dung cho preview canvas Step32.</x:v>
+      </x:c>
+      <x:c r="D79" s="75" t="str">
+        <x:v>B1: Start FE dev server voi VITE_API_BASE_URL.
+B2: curl /templates/7.
+B3: curl /.
+B4: Kiem tra app shell.</x:v>
+      </x:c>
+      <x:c r="E79" s="75" t="str">
+        <x:v>frontend dev server port 5173</x:v>
+      </x:c>
+      <x:c r="F79" s="76" t="str">
+        <x:v>HTTP 200 cho /templates/7 va /; HTML co div id=app va /src/main.ts.</x:v>
+      </x:c>
+      <x:c r="G79" s="75" t="str">
+        <x:v>curl /templates/7 va / deu tra HTTP 200 OK app shell.</x:v>
+      </x:c>
+      <x:c r="H79" s="75" t="str">
+        <x:v>TC_VIZI_070</x:v>
+      </x:c>
+      <x:c r="I79" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J79" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K79" s="75" t="str">
+        <x:v>Loai test: SPA route smoke.</x:v>
+      </x:c>
+      <x:c r="L79" s="75"/>
+      <x:c r="M79" s="75"/>
+      <x:c r="N79" s="75"/>
+      <x:c r="O79" s="75"/>
       <x:c r="P79" s="75" t="n"/>
       <x:c r="Q79" s="75" t="n"/>
       <x:c r="R79" s="75" t="n"/>
@@ -5451,21 +5551,46 @@
       <x:c r="Z79" s="75" t="n"/>
     </x:row>
     <x:row r="80" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A80" s="75" t="n"/>
-      <x:c r="B80" s="76" t="n"/>
-      <x:c r="C80" s="75" t="n"/>
-      <x:c r="D80" s="75" t="n"/>
-      <x:c r="E80" s="75" t="n"/>
-      <x:c r="F80" s="76" t="n"/>
-      <x:c r="G80" s="75" t="n"/>
-      <x:c r="H80" s="75" t="n"/>
-      <x:c r="I80" s="75" t="n"/>
-      <x:c r="J80" s="75" t="n"/>
-      <x:c r="K80" s="75" t="n"/>
-      <x:c r="L80" s="75" t="n"/>
-      <x:c r="M80" s="75" t="n"/>
-      <x:c r="N80" s="75" t="n"/>
-      <x:c r="O80" s="75" t="n"/>
+      <x:c r="A80" s="75" t="str">
+        <x:v>TC_VIZI_072</x:v>
+      </x:c>
+      <x:c r="B80" s="76" t="str">
+        <x:v>Cleanup Step32 smoke data va ports</x:v>
+      </x:c>
+      <x:c r="C80" s="75" t="str">
+        <x:v>Xac nhan seed tam Step32 duoc xoa va server local da dung sau smoke.</x:v>
+      </x:c>
+      <x:c r="D80" s="75" t="str">
+        <x:v>B1: Delete templates Canvas Step32 Template/Hidden.
+B2: Count name like Canvas Step32%.
+B3: Stop backend/frontend PID.
+B4: Test port 8080 va 5173.</x:v>
+      </x:c>
+      <x:c r="E80" s="75" t="str">
+        <x:v>PostgreSQL local, ports 8080/5173</x:v>
+      </x:c>
+      <x:c r="F80" s="76" t="str">
+        <x:v>DELETE 2; remaining_step32_templates=0; ports 8080/5173 closed.</x:v>
+      </x:c>
+      <x:c r="G80" s="75" t="str">
+        <x:v>Cleanup pass: remaining_step32_templates=0; TcpTestSucceeded=False cho 8080 va 5173.</x:v>
+      </x:c>
+      <x:c r="H80" s="75" t="str">
+        <x:v>TC_VIZI_071</x:v>
+      </x:c>
+      <x:c r="I80" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J80" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K80" s="75" t="str">
+        <x:v>Loai test: cleanup/environment regression.</x:v>
+      </x:c>
+      <x:c r="L80" s="75"/>
+      <x:c r="M80" s="75"/>
+      <x:c r="N80" s="75"/>
+      <x:c r="O80" s="75"/>
       <x:c r="P80" s="75" t="n"/>
       <x:c r="Q80" s="75" t="n"/>
       <x:c r="R80" s="75" t="n"/>
@@ -5479,21 +5604,46 @@
       <x:c r="Z80" s="75" t="n"/>
     </x:row>
     <x:row r="81" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A81" s="75" t="n"/>
-      <x:c r="B81" s="76" t="n"/>
-      <x:c r="C81" s="75" t="n"/>
-      <x:c r="D81" s="75" t="n"/>
-      <x:c r="E81" s="75" t="n"/>
-      <x:c r="F81" s="76" t="n"/>
-      <x:c r="G81" s="75" t="n"/>
-      <x:c r="H81" s="75" t="n"/>
-      <x:c r="I81" s="75" t="n"/>
-      <x:c r="J81" s="75" t="n"/>
-      <x:c r="K81" s="75" t="n"/>
-      <x:c r="L81" s="75" t="n"/>
-      <x:c r="M81" s="75" t="n"/>
-      <x:c r="N81" s="75" t="n"/>
-      <x:c r="O81" s="75" t="n"/>
+      <x:c r="A81" s="75" t="str">
+        <x:v>TC_VIZI_073</x:v>
+      </x:c>
+      <x:c r="B81" s="76" t="str">
+        <x:v>Regression sau Step32</x:v>
+      </x:c>
+      <x:c r="C81" s="75" t="str">
+        <x:v>Xac nhan sau canvas renderer, backend/frontend van xanh.</x:v>
+      </x:c>
+      <x:c r="D81" s="75" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Chay backend mvnw test.
+B3: Kiem tra khong con DB test tam.
+B4: Kiem tra ports closed.</x:v>
+      </x:c>
+      <x:c r="E81" s="75" t="str">
+        <x:v>Frontend build, backend Maven tests, PostgreSQL temp DB cleanup</x:v>
+      </x:c>
+      <x:c r="F81" s="76" t="str">
+        <x:v>FE build pass; backend tests run 11 fail 0 error 0; khong con vizi_*_test DB.</x:v>
+      </x:c>
+      <x:c r="G81" s="75" t="str">
+        <x:v>npm run build pass; mvnw test BUILD SUCCESS Tests run 11; ports 8080/5173 closed.</x:v>
+      </x:c>
+      <x:c r="H81" s="75" t="str">
+        <x:v>TC_VIZI_072</x:v>
+      </x:c>
+      <x:c r="I81" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J81" s="103" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K81" s="75" t="str">
+        <x:v>Loai test: regression/system cleanup.</x:v>
+      </x:c>
+      <x:c r="L81" s="75"/>
+      <x:c r="M81" s="75"/>
+      <x:c r="N81" s="75"/>
+      <x:c r="O81" s="75"/>
       <x:c r="P81" s="75" t="n"/>
       <x:c r="Q81" s="75" t="n"/>
       <x:c r="R81" s="75" t="n"/>
@@ -31287,7 +31437,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0f990541eb94c23"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5142ed301ff943f5"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add first text layer editor
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R0706674046134872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc930892ee2a848e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rfdf36a34859f4aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R9c4e60bb0cff4eed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1073,10 +1073,8 @@
           <x:t xml:space="preserve">Tester(Người thực hiện kiểm thử)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="87" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bao</x:t>
-        </x:is>
+      <x:c r="B3" s="87" t="str">
+        <x:v>Tester</x:v>
       </x:c>
       <x:c r="C3" s="85" t="n"/>
       <x:c r="D3" s="85" t="n"/>
@@ -1161,8 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:f>COUNTIF(I9:I998,"Pass")</x:f>
-        <x:v>71</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1179,8 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:f>COUNTA(A9:A998)</x:f>
-        <x:v>73</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -1428,10 +1424,8 @@
 B2: Kiểm tra backend/, frontend/, docs/.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E10" s="97" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Root project C:\Users\Bao\IdeaProjects\Vizi</x:t>
-        </x:is>
+      <x:c r="E10" s="97" t="str">
+        <x:v>Root project workspace Vizi</x:v>
       </x:c>
       <x:c r="F10" s="98" t="inlineStr">
         <x:is>
@@ -1564,10 +1558,8 @@
 B3: Kiểm tra số lượng .ttf/.otf.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E12" s="97" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">C:\Users\Bao\Downloads\1570 Font</x:t>
-        </x:is>
+      <x:c r="E12" s="97" t="str">
+        <x:v>Local font sample folder</x:v>
       </x:c>
       <x:c r="F12" s="98" t="inlineStr">
         <x:is>
@@ -3885,7 +3877,7 @@
         <x:v>Luồng dữ liệu MVP cơ bản chạy được, output join đúng.</x:v>
       </x:c>
       <x:c r="G48" s="75" t="str">
-        <x:v>InitialSchemaMigrationTests.assertMvpAcceptanceFlow pass; đọc lại status PENDING_PAYMENT, quantity 100, design Bao card.</x:v>
+        <x:v>InitialSchemaMigrationTests.assertMvpAcceptanceFlow pass; đọc lại status PENDING_PAYMENT, quantity 100, sample design card.</x:v>
       </x:c>
       <x:c r="H48" s="75" t="str">
         <x:v>TC_VIZI_039</x:v>
@@ -5467,7 +5459,7 @@
         <x:v>Active detail HTTP 200 co 3 layers type rect,text,text; inactive id tra 404.</x:v>
       </x:c>
       <x:c r="G78" s="75" t="str">
-        <x:v>Detail output Name=Canvas Step32 Template, LayerCount=3, Types=rect,text,text, Text=Bao Studio; inactive id 8 tra 404.</x:v>
+        <x:v>Detail output Name=Canvas Step32 Template, LayerCount=3, Types=rect,text,text, Text=Sample Studio; inactive id 8 trả 404.</x:v>
       </x:c>
       <x:c r="H78" s="75" t="str">
         <x:v>TC_VIZI_069</x:v>
@@ -5657,21 +5649,44 @@
       <x:c r="Z81" s="75" t="n"/>
     </x:row>
     <x:row r="82" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A82" s="75" t="n"/>
-      <x:c r="B82" s="76" t="n"/>
-      <x:c r="C82" s="75" t="n"/>
-      <x:c r="D82" s="75" t="n"/>
-      <x:c r="E82" s="75" t="n"/>
-      <x:c r="F82" s="76" t="n"/>
-      <x:c r="G82" s="75" t="n"/>
-      <x:c r="H82" s="75" t="n"/>
-      <x:c r="I82" s="75" t="n"/>
-      <x:c r="J82" s="75" t="n"/>
-      <x:c r="K82" s="75" t="n"/>
-      <x:c r="L82" s="75" t="n"/>
-      <x:c r="M82" s="75" t="n"/>
-      <x:c r="N82" s="75" t="n"/>
-      <x:c r="O82" s="75" t="n"/>
+      <x:c r="A82" s="75" t="str">
+        <x:v>TC_VIZI_074</x:v>
+      </x:c>
+      <x:c r="B82" s="76" t="str">
+        <x:v>Build frontend sau khi thêm editor text layer</x:v>
+      </x:c>
+      <x:c r="C82" s="75" t="str">
+        <x:v>Xác nhận TypeScript và Vite build thành công sau khi thêm textarea chỉnh text layer đầu tiên.</x:v>
+      </x:c>
+      <x:c r="D82" s="75" t="str">
+        <x:v>B1: Chạy npm run build trong frontend.
+B2: Quan sát vue-tsc và Vite build.</x:v>
+      </x:c>
+      <x:c r="E82" s="75" t="str">
+        <x:v>frontend/src/views/TemplateDetailView.vue; frontend/src/styles.css</x:v>
+      </x:c>
+      <x:c r="F82" s="76" t="str">
+        <x:v>Build pass, không có lỗi TypeScript hoặc Vite.</x:v>
+      </x:c>
+      <x:c r="G82" s="75" t="str">
+        <x:v>Pass: vue-tsc --noEmit và vite build thành công.</x:v>
+      </x:c>
+      <x:c r="H82" s="75" t="str">
+        <x:v>TC_VIZI_073</x:v>
+      </x:c>
+      <x:c r="I82" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J82" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K82" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L82" s="75"/>
+      <x:c r="M82" s="75"/>
+      <x:c r="N82" s="75"/>
+      <x:c r="O82" s="75"/>
       <x:c r="P82" s="75" t="n"/>
       <x:c r="Q82" s="75" t="n"/>
       <x:c r="R82" s="75" t="n"/>
@@ -5685,21 +5700,44 @@
       <x:c r="Z82" s="75" t="n"/>
     </x:row>
     <x:row r="83" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A83" s="75" t="n"/>
-      <x:c r="B83" s="76" t="n"/>
-      <x:c r="C83" s="75" t="n"/>
-      <x:c r="D83" s="75" t="n"/>
-      <x:c r="E83" s="75" t="n"/>
-      <x:c r="F83" s="76" t="n"/>
-      <x:c r="G83" s="75" t="n"/>
-      <x:c r="H83" s="75" t="n"/>
-      <x:c r="I83" s="75" t="n"/>
-      <x:c r="J83" s="75" t="n"/>
-      <x:c r="K83" s="75" t="n"/>
-      <x:c r="L83" s="75" t="n"/>
-      <x:c r="M83" s="75" t="n"/>
-      <x:c r="N83" s="75" t="n"/>
-      <x:c r="O83" s="75" t="n"/>
+      <x:c r="A83" s="75" t="str">
+        <x:v>TC_VIZI_075</x:v>
+      </x:c>
+      <x:c r="B83" s="76" t="str">
+        <x:v>Static scan editor text layer</x:v>
+      </x:c>
+      <x:c r="C83" s="75" t="str">
+        <x:v>Kiểm tra FE không render raw HTML, không có pattern secret và không dùng rule responsive rủi ro.</x:v>
+      </x:c>
+      <x:c r="D83" s="75" t="str">
+        <x:v>B1: Chạy rg v-html/innerHTML/secret pattern.
+B2: Chạy rg font-size vw/letter-spacing âm.</x:v>
+      </x:c>
+      <x:c r="E83" s="75" t="str">
+        <x:v>frontend/src</x:v>
+      </x:c>
+      <x:c r="F83" s="76" t="str">
+        <x:v>Không có match nguy hiểm.</x:v>
+      </x:c>
+      <x:c r="G83" s="75" t="str">
+        <x:v>Pass: không có match cho raw HTML/secret pattern/font-size vw/letter-spacing âm.</x:v>
+      </x:c>
+      <x:c r="H83" s="75" t="str">
+        <x:v>TC_VIZI_074</x:v>
+      </x:c>
+      <x:c r="I83" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J83" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K83" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L83" s="75"/>
+      <x:c r="M83" s="75"/>
+      <x:c r="N83" s="75"/>
+      <x:c r="O83" s="75"/>
       <x:c r="P83" s="75" t="n"/>
       <x:c r="Q83" s="75" t="n"/>
       <x:c r="R83" s="75" t="n"/>
@@ -5713,21 +5751,47 @@
       <x:c r="Z83" s="75" t="n"/>
     </x:row>
     <x:row r="84" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A84" s="75" t="n"/>
-      <x:c r="B84" s="76" t="n"/>
-      <x:c r="C84" s="75" t="n"/>
-      <x:c r="D84" s="75" t="n"/>
-      <x:c r="E84" s="75" t="n"/>
-      <x:c r="F84" s="76" t="n"/>
-      <x:c r="G84" s="75" t="n"/>
-      <x:c r="H84" s="75" t="n"/>
-      <x:c r="I84" s="75" t="n"/>
-      <x:c r="J84" s="75" t="n"/>
-      <x:c r="K84" s="75" t="n"/>
-      <x:c r="L84" s="75" t="n"/>
-      <x:c r="M84" s="75" t="n"/>
-      <x:c r="N84" s="75" t="n"/>
-      <x:c r="O84" s="75" t="n"/>
+      <x:c r="A84" s="75" t="str">
+        <x:v>TC_VIZI_076</x:v>
+      </x:c>
+      <x:c r="B84" s="76" t="str">
+        <x:v>Browser smoke editor cập nhật preview</x:v>
+      </x:c>
+      <x:c r="C84" s="75" t="str">
+        <x:v>Xác nhận textarea của text layer đầu tiên cập nhật preview canvas ngay trên route detail.</x:v>
+      </x:c>
+      <x:c r="D84" s="75" t="str">
+        <x:v>B1: Chạy Vite dev server.
+B2: Chạy mock API template id 33.
+B3: Mở /templates/33.
+B4: Fill textarea bằng Luxury card text.
+B5: Đọc DOM canvas layer.</x:v>
+      </x:c>
+      <x:c r="E84" s="75" t="str">
+        <x:v>Template mock có rect + 2 text layers</x:v>
+      </x:c>
+      <x:c r="F84" s="76" t="str">
+        <x:v>Textarea và text layer đầu tiên cùng đổi sang nội dung mới; text layer thứ hai giữ nguyên.</x:v>
+      </x:c>
+      <x:c r="G84" s="75" t="str">
+        <x:v>Pass: textareaValue và canvas text layer đầu tiên là Luxury card text; text layer thứ hai giữ nguyên.</x:v>
+      </x:c>
+      <x:c r="H84" s="75" t="str">
+        <x:v>TC_VIZI_074</x:v>
+      </x:c>
+      <x:c r="I84" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J84" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K84" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L84" s="75"/>
+      <x:c r="M84" s="75"/>
+      <x:c r="N84" s="75"/>
+      <x:c r="O84" s="75"/>
       <x:c r="P84" s="75" t="n"/>
       <x:c r="Q84" s="75" t="n"/>
       <x:c r="R84" s="75" t="n"/>
@@ -5741,21 +5805,45 @@
       <x:c r="Z84" s="75" t="n"/>
     </x:row>
     <x:row r="85" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A85" s="75" t="n"/>
-      <x:c r="B85" s="76" t="n"/>
-      <x:c r="C85" s="75" t="n"/>
-      <x:c r="D85" s="75" t="n"/>
-      <x:c r="E85" s="75" t="n"/>
-      <x:c r="F85" s="76" t="n"/>
-      <x:c r="G85" s="75" t="n"/>
-      <x:c r="H85" s="75" t="n"/>
-      <x:c r="I85" s="75" t="n"/>
-      <x:c r="J85" s="75" t="n"/>
-      <x:c r="K85" s="75" t="n"/>
-      <x:c r="L85" s="75" t="n"/>
-      <x:c r="M85" s="75" t="n"/>
-      <x:c r="N85" s="75" t="n"/>
-      <x:c r="O85" s="75" t="n"/>
+      <x:c r="A85" s="75" t="str">
+        <x:v>TC_VIZI_077</x:v>
+      </x:c>
+      <x:c r="B85" s="76" t="str">
+        <x:v>Security smoke XSS trong text editor</x:v>
+      </x:c>
+      <x:c r="C85" s="75" t="str">
+        <x:v>Xác nhận input HTML/script chỉ hiển thị dạng text trong canvas, không tạo DOM node nguy hiểm.</x:v>
+      </x:c>
+      <x:c r="D85" s="75" t="str">
+        <x:v>B1: Fill textarea bằng chuỗi img/script.
+B2: Kiểm tra textContent.
+B3: Đếm img/script node trong canvas.</x:v>
+      </x:c>
+      <x:c r="E85" s="75" t="str">
+        <x:v>&lt;img src=x onerror=alert(1)&gt;&lt;script&gt;alert(2)&lt;/script&gt;</x:v>
+      </x:c>
+      <x:c r="F85" s="76" t="str">
+        <x:v>Canvas chứa text literal; không có img/script node phát sinh.</x:v>
+      </x:c>
+      <x:c r="G85" s="75" t="str">
+        <x:v>Pass: imgCountInCanvas = 0, scriptCountInCanvas = 0, textContent giữ chuỗi literal.</x:v>
+      </x:c>
+      <x:c r="H85" s="75" t="str">
+        <x:v>TC_VIZI_076</x:v>
+      </x:c>
+      <x:c r="I85" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J85" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K85" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L85" s="75"/>
+      <x:c r="M85" s="75"/>
+      <x:c r="N85" s="75"/>
+      <x:c r="O85" s="75"/>
       <x:c r="P85" s="75" t="n"/>
       <x:c r="Q85" s="75" t="n"/>
       <x:c r="R85" s="75" t="n"/>
@@ -5769,21 +5857,46 @@
       <x:c r="Z85" s="75" t="n"/>
     </x:row>
     <x:row r="86" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A86" s="75" t="n"/>
-      <x:c r="B86" s="76" t="n"/>
-      <x:c r="C86" s="75" t="n"/>
-      <x:c r="D86" s="75" t="n"/>
-      <x:c r="E86" s="75" t="n"/>
-      <x:c r="F86" s="76" t="n"/>
-      <x:c r="G86" s="75" t="n"/>
-      <x:c r="H86" s="75" t="n"/>
-      <x:c r="I86" s="75" t="n"/>
-      <x:c r="J86" s="75" t="n"/>
-      <x:c r="K86" s="75" t="n"/>
-      <x:c r="L86" s="75" t="n"/>
-      <x:c r="M86" s="75" t="n"/>
-      <x:c r="N86" s="75" t="n"/>
-      <x:c r="O86" s="75" t="n"/>
+      <x:c r="A86" s="75" t="str">
+        <x:v>TC_VIZI_078</x:v>
+      </x:c>
+      <x:c r="B86" s="76" t="str">
+        <x:v>Responsive smoke editor mobile</x:v>
+      </x:c>
+      <x:c r="C86" s="75" t="str">
+        <x:v>Kiểm tra editor ở viewport mobile không tạo horizontal scroll và preview vẫn cập nhật.</x:v>
+      </x:c>
+      <x:c r="D86" s="75" t="str">
+        <x:v>B1: Đặt viewport 390x844.
+B2: Reload /templates/33.
+B3: Fill textarea bằng chuỗi dài.
+B4: So sánh scrollWidth và clientWidth.</x:v>
+      </x:c>
+      <x:c r="E86" s="75" t="str">
+        <x:v>390x844; long word text</x:v>
+      </x:c>
+      <x:c r="F86" s="76" t="str">
+        <x:v>Không có horizontal scroll; textarea nằm trong panel; preview cập nhật text mới.</x:v>
+      </x:c>
+      <x:c r="G86" s="75" t="str">
+        <x:v>Pass: scrollWidth = clientWidth; textareaWidth = panelWidth; layer text đổi đúng.</x:v>
+      </x:c>
+      <x:c r="H86" s="75" t="str">
+        <x:v>TC_VIZI_076</x:v>
+      </x:c>
+      <x:c r="I86" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J86" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K86" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L86" s="75"/>
+      <x:c r="M86" s="75"/>
+      <x:c r="N86" s="75"/>
+      <x:c r="O86" s="75"/>
       <x:c r="P86" s="75" t="n"/>
       <x:c r="Q86" s="75" t="n"/>
       <x:c r="R86" s="75" t="n"/>
@@ -5797,21 +5910,44 @@
       <x:c r="Z86" s="75" t="n"/>
     </x:row>
     <x:row r="87" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A87" s="75" t="n"/>
-      <x:c r="B87" s="76" t="n"/>
-      <x:c r="C87" s="75" t="n"/>
-      <x:c r="D87" s="75" t="n"/>
-      <x:c r="E87" s="75" t="n"/>
-      <x:c r="F87" s="76" t="n"/>
-      <x:c r="G87" s="75" t="n"/>
-      <x:c r="H87" s="75" t="n"/>
-      <x:c r="I87" s="75" t="n"/>
-      <x:c r="J87" s="75" t="n"/>
-      <x:c r="K87" s="75" t="n"/>
-      <x:c r="L87" s="75" t="n"/>
-      <x:c r="M87" s="75" t="n"/>
-      <x:c r="N87" s="75" t="n"/>
-      <x:c r="O87" s="75" t="n"/>
+      <x:c r="A87" s="75" t="str">
+        <x:v>TC_VIZI_079</x:v>
+      </x:c>
+      <x:c r="B87" s="76" t="str">
+        <x:v>Regression backend sau bước 33</x:v>
+      </x:c>
+      <x:c r="C87" s="75" t="str">
+        <x:v>Đảm bảo thay đổi FE không làm hỏng regression backend hiện có.</x:v>
+      </x:c>
+      <x:c r="D87" s="75" t="str">
+        <x:v>B1: Chạy .\mvnw.cmd test trong backend.
+B2: Kiểm tra tổng kết test.</x:v>
+      </x:c>
+      <x:c r="E87" s="75" t="str">
+        <x:v>backend Maven test suite</x:v>
+      </x:c>
+      <x:c r="F87" s="76" t="str">
+        <x:v>Build success; test không fail/error.</x:v>
+      </x:c>
+      <x:c r="G87" s="75" t="str">
+        <x:v>Pass: 11 tests, 0 failures, 0 errors; 3 PostgreSQL-local tests skipped do session thiếu datasource env.</x:v>
+      </x:c>
+      <x:c r="H87" s="75" t="str">
+        <x:v>TC_VIZI_074</x:v>
+      </x:c>
+      <x:c r="I87" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J87" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K87" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L87" s="75"/>
+      <x:c r="M87" s="75"/>
+      <x:c r="N87" s="75"/>
+      <x:c r="O87" s="75"/>
       <x:c r="P87" s="75" t="n"/>
       <x:c r="Q87" s="75" t="n"/>
       <x:c r="R87" s="75" t="n"/>
@@ -5825,21 +5961,45 @@
       <x:c r="Z87" s="75" t="n"/>
     </x:row>
     <x:row r="88" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A88" s="75" t="n"/>
-      <x:c r="B88" s="76" t="n"/>
-      <x:c r="C88" s="75" t="n"/>
-      <x:c r="D88" s="75" t="n"/>
-      <x:c r="E88" s="75" t="n"/>
-      <x:c r="F88" s="76" t="n"/>
-      <x:c r="G88" s="75" t="n"/>
-      <x:c r="H88" s="75" t="n"/>
-      <x:c r="I88" s="75" t="n"/>
-      <x:c r="J88" s="75" t="n"/>
-      <x:c r="K88" s="75" t="n"/>
-      <x:c r="L88" s="75" t="n"/>
-      <x:c r="M88" s="75" t="n"/>
-      <x:c r="N88" s="75" t="n"/>
-      <x:c r="O88" s="75" t="n"/>
+      <x:c r="A88" s="75" t="str">
+        <x:v>TC_VIZI_080</x:v>
+      </x:c>
+      <x:c r="B88" s="76" t="str">
+        <x:v>Visual smoke editor luxury light</x:v>
+      </x:c>
+      <x:c r="C88" s="75" t="str">
+        <x:v>Kiểm tra UI detail/editor vẫn giữ phong cách sáng, chuyên nghiệp, luxury sau khi thêm control.</x:v>
+      </x:c>
+      <x:c r="D88" s="75" t="str">
+        <x:v>B1: Mở /templates/33.
+B2: Chụp full-page screenshot.
+B3: Quan sát canvas, panel detail, textarea và typography.</x:v>
+      </x:c>
+      <x:c r="E88" s="75" t="str">
+        <x:v>Browser screenshot sau browser smoke</x:v>
+      </x:c>
+      <x:c r="F88" s="76" t="str">
+        <x:v>Editor hiển thị rõ, không che layout chính; phong cách light luxury được giữ.</x:v>
+      </x:c>
+      <x:c r="G88" s="75" t="str">
+        <x:v>Pass: screenshot cho thấy canvas, detail panel, Save draft disabled và textarea hiển thị đúng.</x:v>
+      </x:c>
+      <x:c r="H88" s="75" t="str">
+        <x:v>TC_VIZI_076</x:v>
+      </x:c>
+      <x:c r="I88" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J88" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K88" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L88" s="75"/>
+      <x:c r="M88" s="75"/>
+      <x:c r="N88" s="75"/>
+      <x:c r="O88" s="75"/>
       <x:c r="P88" s="75" t="n"/>
       <x:c r="Q88" s="75" t="n"/>
       <x:c r="R88" s="75" t="n"/>
@@ -5853,21 +6013,45 @@
       <x:c r="Z88" s="75" t="n"/>
     </x:row>
     <x:row r="89" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A89" s="75" t="n"/>
-      <x:c r="B89" s="76" t="n"/>
-      <x:c r="C89" s="75" t="n"/>
-      <x:c r="D89" s="75" t="n"/>
-      <x:c r="E89" s="75" t="n"/>
-      <x:c r="F89" s="76" t="n"/>
-      <x:c r="G89" s="75" t="n"/>
-      <x:c r="H89" s="75" t="n"/>
-      <x:c r="I89" s="75" t="n"/>
-      <x:c r="J89" s="75" t="n"/>
-      <x:c r="K89" s="75" t="n"/>
-      <x:c r="L89" s="75" t="n"/>
-      <x:c r="M89" s="75" t="n"/>
-      <x:c r="N89" s="75" t="n"/>
-      <x:c r="O89" s="75" t="n"/>
+      <x:c r="A89" s="75" t="str">
+        <x:v>TC_VIZI_081</x:v>
+      </x:c>
+      <x:c r="B89" s="76" t="str">
+        <x:v>Cleanup test runtime bước 33</x:v>
+      </x:c>
+      <x:c r="C89" s="75" t="str">
+        <x:v>Xác nhận server/mock test được dừng sau kiểm thử và không để process dev chiếm port.</x:v>
+      </x:c>
+      <x:c r="D89" s="75" t="str">
+        <x:v>B1: Dừng Vite dev server.
+B2: Dừng mock API.
+B3: Kiểm tra port 5173 và 8080.</x:v>
+      </x:c>
+      <x:c r="E89" s="75" t="str">
+        <x:v>Ports 5173, 8080</x:v>
+      </x:c>
+      <x:c r="F89" s="76" t="str">
+        <x:v>Không còn process listen trên port test.</x:v>
+      </x:c>
+      <x:c r="G89" s="75" t="str">
+        <x:v>Pass: port 5173 và 8080 được kiểm tra sau khi dừng session.</x:v>
+      </x:c>
+      <x:c r="H89" s="75" t="str">
+        <x:v>TC_VIZI_076</x:v>
+      </x:c>
+      <x:c r="I89" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J89" s="75" t="n">
+        <x:v>46208</x:v>
+      </x:c>
+      <x:c r="K89" s="75" t="str">
+        <x:v>Bước 33</x:v>
+      </x:c>
+      <x:c r="L89" s="75"/>
+      <x:c r="M89" s="75"/>
+      <x:c r="N89" s="75"/>
+      <x:c r="O89" s="75"/>
       <x:c r="P89" s="75" t="n"/>
       <x:c r="Q89" s="75" t="n"/>
       <x:c r="R89" s="75" t="n"/>
@@ -31437,7 +31621,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5142ed301ff943f5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79a039d788424cce"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add session authentication foundation
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rfdf36a34859f4aee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R9c4e60bb0cff4eed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R14db4008c5b14014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5cd9eea25119452e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>79</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>81</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -6065,21 +6065,44 @@
       <x:c r="Z89" s="75" t="n"/>
     </x:row>
     <x:row r="90" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A90" s="75" t="n"/>
-      <x:c r="B90" s="76" t="n"/>
-      <x:c r="C90" s="75" t="n"/>
-      <x:c r="D90" s="75" t="n"/>
-      <x:c r="E90" s="75" t="n"/>
-      <x:c r="F90" s="76" t="n"/>
-      <x:c r="G90" s="75" t="n"/>
-      <x:c r="H90" s="75" t="n"/>
-      <x:c r="I90" s="75" t="n"/>
-      <x:c r="J90" s="75" t="n"/>
-      <x:c r="K90" s="75" t="n"/>
-      <x:c r="L90" s="75" t="n"/>
-      <x:c r="M90" s="75" t="n"/>
-      <x:c r="N90" s="75" t="n"/>
-      <x:c r="O90" s="75" t="n"/>
+      <x:c r="A90" s="75" t="str">
+        <x:v>TC_VIZI_082</x:v>
+      </x:c>
+      <x:c r="B90" s="76" t="str">
+        <x:v>CSRF chặn đăng ký thiếu token</x:v>
+      </x:c>
+      <x:c r="C90" s="75" t="str">
+        <x:v>Xác nhận endpoint ghi dữ liệu không chấp nhận request thiếu CSRF token.</x:v>
+      </x:c>
+      <x:c r="D90" s="75" t="str">
+        <x:v>B1: POST /api/auth/register không kèm CSRF.
+B2: Kiểm tra status.</x:v>
+      </x:c>
+      <x:c r="E90" s="75" t="str">
+        <x:v>JSON đăng ký hợp lệ nhưng không có CSRF</x:v>
+      </x:c>
+      <x:c r="F90" s="76" t="str">
+        <x:v>HTTP 403; không tạo tài khoản.</x:v>
+      </x:c>
+      <x:c r="G90" s="75" t="str">
+        <x:v>Pass: integration test trả 403.</x:v>
+      </x:c>
+      <x:c r="H90" s="75" t="str">
+        <x:v>TC_VIZI_081</x:v>
+      </x:c>
+      <x:c r="I90" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J90" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K90" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L90" s="75"/>
+      <x:c r="M90" s="75"/>
+      <x:c r="N90" s="75"/>
+      <x:c r="O90" s="75"/>
       <x:c r="P90" s="75" t="n"/>
       <x:c r="Q90" s="75" t="n"/>
       <x:c r="R90" s="75" t="n"/>
@@ -6093,21 +6116,45 @@
       <x:c r="Z90" s="75" t="n"/>
     </x:row>
     <x:row r="91" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A91" s="75" t="n"/>
-      <x:c r="B91" s="76" t="n"/>
-      <x:c r="C91" s="75" t="n"/>
-      <x:c r="D91" s="75" t="n"/>
-      <x:c r="E91" s="75" t="n"/>
-      <x:c r="F91" s="76" t="n"/>
-      <x:c r="G91" s="75" t="n"/>
-      <x:c r="H91" s="75" t="n"/>
-      <x:c r="I91" s="75" t="n"/>
-      <x:c r="J91" s="75" t="n"/>
-      <x:c r="K91" s="75" t="n"/>
-      <x:c r="L91" s="75" t="n"/>
-      <x:c r="M91" s="75" t="n"/>
-      <x:c r="N91" s="75" t="n"/>
-      <x:c r="O91" s="75" t="n"/>
+      <x:c r="A91" s="75" t="str">
+        <x:v>TC_VIZI_083</x:v>
+      </x:c>
+      <x:c r="B91" s="76" t="str">
+        <x:v>Đăng ký hợp lệ và không lộ mật khẩu</x:v>
+      </x:c>
+      <x:c r="C91" s="75" t="str">
+        <x:v>Kiểm tra đăng ký tạo user, chuẩn hóa email và response không chứa password/hash.</x:v>
+      </x:c>
+      <x:c r="D91" s="75" t="str">
+        <x:v>B1: Lấy CSRF.
+B2: POST dữ liệu hợp lệ.
+B3: Kiểm tra response.</x:v>
+      </x:c>
+      <x:c r="E91" s="75" t="str">
+        <x:v>Customer@Example.Test; mật khẩu đủ 8 ký tự</x:v>
+      </x:c>
+      <x:c r="F91" s="76" t="str">
+        <x:v>HTTP 201; email chữ thường; không có password hoặc passwordHash.</x:v>
+      </x:c>
+      <x:c r="G91" s="75" t="str">
+        <x:v>Pass: account được tạo, response chỉ có id/email/fullName/role.</x:v>
+      </x:c>
+      <x:c r="H91" s="75" t="str">
+        <x:v>TC_VIZI_082</x:v>
+      </x:c>
+      <x:c r="I91" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J91" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K91" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L91" s="75"/>
+      <x:c r="M91" s="75"/>
+      <x:c r="N91" s="75"/>
+      <x:c r="O91" s="75"/>
       <x:c r="P91" s="75" t="n"/>
       <x:c r="Q91" s="75" t="n"/>
       <x:c r="R91" s="75" t="n"/>
@@ -6121,21 +6168,44 @@
       <x:c r="Z91" s="75" t="n"/>
     </x:row>
     <x:row r="92" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A92" s="75" t="n"/>
-      <x:c r="B92" s="76" t="n"/>
-      <x:c r="C92" s="75" t="n"/>
-      <x:c r="D92" s="75" t="n"/>
-      <x:c r="E92" s="75" t="n"/>
-      <x:c r="F92" s="76" t="n"/>
-      <x:c r="G92" s="75" t="n"/>
-      <x:c r="H92" s="75" t="n"/>
-      <x:c r="I92" s="75" t="n"/>
-      <x:c r="J92" s="75" t="n"/>
-      <x:c r="K92" s="75" t="n"/>
-      <x:c r="L92" s="75" t="n"/>
-      <x:c r="M92" s="75" t="n"/>
-      <x:c r="N92" s="75" t="n"/>
-      <x:c r="O92" s="75" t="n"/>
+      <x:c r="A92" s="75" t="str">
+        <x:v>TC_VIZI_084</x:v>
+      </x:c>
+      <x:c r="B92" s="76" t="str">
+        <x:v>Validation auth trả 400 an toàn</x:v>
+      </x:c>
+      <x:c r="C92" s="75" t="str">
+        <x:v>Email sai và mật khẩu ngắn phải bị reject, không rơi vào 500 và không echo mật khẩu.</x:v>
+      </x:c>
+      <x:c r="D92" s="75" t="str">
+        <x:v>B1: POST email sai + password ngắn có CSRF.
+B2: Kiểm tra JSON lỗi.</x:v>
+      </x:c>
+      <x:c r="E92" s="75" t="str">
+        <x:v>not-an-email; short</x:v>
+      </x:c>
+      <x:c r="F92" s="76" t="str">
+        <x:v>HTTP 400; response không chứa password.</x:v>
+      </x:c>
+      <x:c r="G92" s="75" t="str">
+        <x:v>Pass: trả 400 Validation failed, không lộ dữ liệu nhạy cảm.</x:v>
+      </x:c>
+      <x:c r="H92" s="75" t="str">
+        <x:v>TC_VIZI_083</x:v>
+      </x:c>
+      <x:c r="I92" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J92" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K92" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L92" s="75"/>
+      <x:c r="M92" s="75"/>
+      <x:c r="N92" s="75"/>
+      <x:c r="O92" s="75"/>
       <x:c r="P92" s="75" t="n"/>
       <x:c r="Q92" s="75" t="n"/>
       <x:c r="R92" s="75" t="n"/>
@@ -6149,21 +6219,44 @@
       <x:c r="Z92" s="75" t="n"/>
     </x:row>
     <x:row r="93" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A93" s="75" t="n"/>
-      <x:c r="B93" s="76" t="n"/>
-      <x:c r="C93" s="75" t="n"/>
-      <x:c r="D93" s="75" t="n"/>
-      <x:c r="E93" s="75" t="n"/>
-      <x:c r="F93" s="76" t="n"/>
-      <x:c r="G93" s="75" t="n"/>
-      <x:c r="H93" s="75" t="n"/>
-      <x:c r="I93" s="75" t="n"/>
-      <x:c r="J93" s="75" t="n"/>
-      <x:c r="K93" s="75" t="n"/>
-      <x:c r="L93" s="75" t="n"/>
-      <x:c r="M93" s="75" t="n"/>
-      <x:c r="N93" s="75" t="n"/>
-      <x:c r="O93" s="75" t="n"/>
+      <x:c r="A93" s="75" t="str">
+        <x:v>TC_VIZI_085</x:v>
+      </x:c>
+      <x:c r="B93" s="76" t="str">
+        <x:v>Chặn email trùng không phân biệt hoa thường</x:v>
+      </x:c>
+      <x:c r="C93" s="75" t="str">
+        <x:v>Không cho tạo hai tài khoản cùng email với khác biệt chữ hoa/chữ thường.</x:v>
+      </x:c>
+      <x:c r="D93" s="75" t="str">
+        <x:v>B1: Đăng ký email thường.
+B2: Đăng ký lại email viết hoa.</x:v>
+      </x:c>
+      <x:c r="E93" s="75" t="str">
+        <x:v>customer@example.test và CUSTOMER@example.test</x:v>
+      </x:c>
+      <x:c r="F93" s="76" t="str">
+        <x:v>Lần hai trả HTTP 409.</x:v>
+      </x:c>
+      <x:c r="G93" s="75" t="str">
+        <x:v>Pass: trả 409 Email already registered.</x:v>
+      </x:c>
+      <x:c r="H93" s="75" t="str">
+        <x:v>TC_VIZI_083</x:v>
+      </x:c>
+      <x:c r="I93" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J93" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K93" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L93" s="75"/>
+      <x:c r="M93" s="75"/>
+      <x:c r="N93" s="75"/>
+      <x:c r="O93" s="75"/>
       <x:c r="P93" s="75" t="n"/>
       <x:c r="Q93" s="75" t="n"/>
       <x:c r="R93" s="75" t="n"/>
@@ -6177,21 +6270,45 @@
       <x:c r="Z93" s="75" t="n"/>
     </x:row>
     <x:row r="94" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A94" s="75" t="n"/>
-      <x:c r="B94" s="76" t="n"/>
-      <x:c r="C94" s="75" t="n"/>
-      <x:c r="D94" s="75" t="n"/>
-      <x:c r="E94" s="75" t="n"/>
-      <x:c r="F94" s="76" t="n"/>
-      <x:c r="G94" s="75" t="n"/>
-      <x:c r="H94" s="75" t="n"/>
-      <x:c r="I94" s="75" t="n"/>
-      <x:c r="J94" s="75" t="n"/>
-      <x:c r="K94" s="75" t="n"/>
-      <x:c r="L94" s="75" t="n"/>
-      <x:c r="M94" s="75" t="n"/>
-      <x:c r="N94" s="75" t="n"/>
-      <x:c r="O94" s="75" t="n"/>
+      <x:c r="A94" s="75" t="str">
+        <x:v>TC_VIZI_086</x:v>
+      </x:c>
+      <x:c r="B94" s="76" t="str">
+        <x:v>Đăng nhập tạo session và đọc current user</x:v>
+      </x:c>
+      <x:c r="C94" s="75" t="str">
+        <x:v>Xác nhận BCrypt credential hợp lệ tạo session dùng được cho /api/auth/me.</x:v>
+      </x:c>
+      <x:c r="D94" s="75" t="str">
+        <x:v>B1: Đăng ký.
+B2: POST login có CSRF.
+B3: GET /api/auth/me bằng session.</x:v>
+      </x:c>
+      <x:c r="E94" s="75" t="str">
+        <x:v>Tài khoản test hợp lệ</x:v>
+      </x:c>
+      <x:c r="F94" s="76" t="str">
+        <x:v>Login 204; /me 200 trả đúng email và role USER.</x:v>
+      </x:c>
+      <x:c r="G94" s="75" t="str">
+        <x:v>Pass: session xác thực đọc được current user.</x:v>
+      </x:c>
+      <x:c r="H94" s="75" t="str">
+        <x:v>TC_VIZI_083</x:v>
+      </x:c>
+      <x:c r="I94" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J94" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K94" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L94" s="75"/>
+      <x:c r="M94" s="75"/>
+      <x:c r="N94" s="75"/>
+      <x:c r="O94" s="75"/>
       <x:c r="P94" s="75" t="n"/>
       <x:c r="Q94" s="75" t="n"/>
       <x:c r="R94" s="75" t="n"/>
@@ -6205,21 +6322,44 @@
       <x:c r="Z94" s="75" t="n"/>
     </x:row>
     <x:row r="95" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A95" s="75" t="n"/>
-      <x:c r="B95" s="76" t="n"/>
-      <x:c r="C95" s="75" t="n"/>
-      <x:c r="D95" s="75" t="n"/>
-      <x:c r="E95" s="75" t="n"/>
-      <x:c r="F95" s="76" t="n"/>
-      <x:c r="G95" s="75" t="n"/>
-      <x:c r="H95" s="75" t="n"/>
-      <x:c r="I95" s="75" t="n"/>
-      <x:c r="J95" s="75" t="n"/>
-      <x:c r="K95" s="75" t="n"/>
-      <x:c r="L95" s="75" t="n"/>
-      <x:c r="M95" s="75" t="n"/>
-      <x:c r="N95" s="75" t="n"/>
-      <x:c r="O95" s="75" t="n"/>
+      <x:c r="A95" s="75" t="str">
+        <x:v>TC_VIZI_087</x:v>
+      </x:c>
+      <x:c r="B95" s="76" t="str">
+        <x:v>Sai mật khẩu và anonymous bị từ chối</x:v>
+      </x:c>
+      <x:c r="C95" s="75" t="str">
+        <x:v>Kiểm tra negative authentication không cấp session và endpoint private không mở cho anonymous.</x:v>
+      </x:c>
+      <x:c r="D95" s="75" t="str">
+        <x:v>B1: Login bằng password sai.
+B2: GET /api/auth/me không session.</x:v>
+      </x:c>
+      <x:c r="E95" s="75" t="str">
+        <x:v>WrongPass123</x:v>
+      </x:c>
+      <x:c r="F95" s="76" t="str">
+        <x:v>Cả hai request trả HTTP 401.</x:v>
+      </x:c>
+      <x:c r="G95" s="75" t="str">
+        <x:v>Pass: sai mật khẩu và anonymous đều trả 401.</x:v>
+      </x:c>
+      <x:c r="H95" s="75" t="str">
+        <x:v>TC_VIZI_086</x:v>
+      </x:c>
+      <x:c r="I95" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J95" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K95" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L95" s="75"/>
+      <x:c r="M95" s="75"/>
+      <x:c r="N95" s="75"/>
+      <x:c r="O95" s="75"/>
       <x:c r="P95" s="75" t="n"/>
       <x:c r="Q95" s="75" t="n"/>
       <x:c r="R95" s="75" t="n"/>
@@ -6233,21 +6373,46 @@
       <x:c r="Z95" s="75" t="n"/>
     </x:row>
     <x:row r="96" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A96" s="75" t="n"/>
-      <x:c r="B96" s="76" t="n"/>
-      <x:c r="C96" s="75" t="n"/>
-      <x:c r="D96" s="75" t="n"/>
-      <x:c r="E96" s="75" t="n"/>
-      <x:c r="F96" s="76" t="n"/>
-      <x:c r="G96" s="75" t="n"/>
-      <x:c r="H96" s="75" t="n"/>
-      <x:c r="I96" s="75" t="n"/>
-      <x:c r="J96" s="75" t="n"/>
-      <x:c r="K96" s="75" t="n"/>
-      <x:c r="L96" s="75" t="n"/>
-      <x:c r="M96" s="75" t="n"/>
-      <x:c r="N96" s="75" t="n"/>
-      <x:c r="O96" s="75" t="n"/>
+      <x:c r="A96" s="75" t="str">
+        <x:v>TC_VIZI_088</x:v>
+      </x:c>
+      <x:c r="B96" s="76" t="str">
+        <x:v>CSRF token và logout hủy session</x:v>
+      </x:c>
+      <x:c r="C96" s="75" t="str">
+        <x:v>Xác nhận browser lấy được CSRF token và logout làm session không còn truy cập /me.</x:v>
+      </x:c>
+      <x:c r="D96" s="75" t="str">
+        <x:v>B1: GET /api/auth/csrf.
+B2: Login.
+B3: Logout có CSRF.
+B4: GET /me.</x:v>
+      </x:c>
+      <x:c r="E96" s="75" t="str">
+        <x:v>X-CSRF-TOKEN; session hợp lệ</x:v>
+      </x:c>
+      <x:c r="F96" s="76" t="str">
+        <x:v>CSRF trả token; logout 204; /me sau logout trả 401.</x:v>
+      </x:c>
+      <x:c r="G96" s="75" t="str">
+        <x:v>Pass: toàn bộ lifecycle session đúng.</x:v>
+      </x:c>
+      <x:c r="H96" s="75" t="str">
+        <x:v>TC_VIZI_086</x:v>
+      </x:c>
+      <x:c r="I96" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J96" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K96" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L96" s="75"/>
+      <x:c r="M96" s="75"/>
+      <x:c r="N96" s="75"/>
+      <x:c r="O96" s="75"/>
       <x:c r="P96" s="75" t="n"/>
       <x:c r="Q96" s="75" t="n"/>
       <x:c r="R96" s="75" t="n"/>
@@ -6261,21 +6426,44 @@
       <x:c r="Z96" s="75" t="n"/>
     </x:row>
     <x:row r="97" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A97" s="75" t="n"/>
-      <x:c r="B97" s="76" t="n"/>
-      <x:c r="C97" s="75" t="n"/>
-      <x:c r="D97" s="75" t="n"/>
-      <x:c r="E97" s="75" t="n"/>
-      <x:c r="F97" s="76" t="n"/>
-      <x:c r="G97" s="75" t="n"/>
-      <x:c r="H97" s="75" t="n"/>
-      <x:c r="I97" s="75" t="n"/>
-      <x:c r="J97" s="75" t="n"/>
-      <x:c r="K97" s="75" t="n"/>
-      <x:c r="L97" s="75" t="n"/>
-      <x:c r="M97" s="75" t="n"/>
-      <x:c r="N97" s="75" t="n"/>
-      <x:c r="O97" s="75" t="n"/>
+      <x:c r="A97" s="75" t="str">
+        <x:v>TC_VIZI_089</x:v>
+      </x:c>
+      <x:c r="B97" s="76" t="str">
+        <x:v>Regression backend và PostgreSQL thật</x:v>
+      </x:c>
+      <x:c r="C97" s="75" t="str">
+        <x:v>Chạy toàn bộ test suite sau khi thêm security, gồm migration/schema và template API trên PostgreSQL 17.</x:v>
+      </x:c>
+      <x:c r="D97" s="75" t="str">
+        <x:v>B1: Chạy .\mvnw.cmd test.
+B2: Kiểm tra tổng kết.</x:v>
+      </x:c>
+      <x:c r="E97" s="75" t="str">
+        <x:v>Backend Maven test suite</x:v>
+      </x:c>
+      <x:c r="F97" s="76" t="str">
+        <x:v>Không có failure/error/skip.</x:v>
+      </x:c>
+      <x:c r="G97" s="75" t="str">
+        <x:v>Pass: 21 tests, 0 failures, 0 errors, 0 skipped.</x:v>
+      </x:c>
+      <x:c r="H97" s="75" t="str">
+        <x:v>TC_VIZI_088</x:v>
+      </x:c>
+      <x:c r="I97" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J97" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K97" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L97" s="75"/>
+      <x:c r="M97" s="75"/>
+      <x:c r="N97" s="75"/>
+      <x:c r="O97" s="75"/>
       <x:c r="P97" s="75" t="n"/>
       <x:c r="Q97" s="75" t="n"/>
       <x:c r="R97" s="75" t="n"/>
@@ -6289,21 +6477,44 @@
       <x:c r="Z97" s="75" t="n"/>
     </x:row>
     <x:row r="98" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A98" s="75" t="n"/>
-      <x:c r="B98" s="76" t="n"/>
-      <x:c r="C98" s="75" t="n"/>
-      <x:c r="D98" s="75" t="n"/>
-      <x:c r="E98" s="75" t="n"/>
-      <x:c r="F98" s="76" t="n"/>
-      <x:c r="G98" s="75" t="n"/>
-      <x:c r="H98" s="75" t="n"/>
-      <x:c r="I98" s="75" t="n"/>
-      <x:c r="J98" s="75" t="n"/>
-      <x:c r="K98" s="75" t="n"/>
-      <x:c r="L98" s="75" t="n"/>
-      <x:c r="M98" s="75" t="n"/>
-      <x:c r="N98" s="75" t="n"/>
-      <x:c r="O98" s="75" t="n"/>
+      <x:c r="A98" s="75" t="str">
+        <x:v>TC_VIZI_090</x:v>
+      </x:c>
+      <x:c r="B98" s="76" t="str">
+        <x:v>Build frontend có Account flow</x:v>
+      </x:c>
+      <x:c r="C98" s="75" t="str">
+        <x:v>Xác nhận TypeScript và Vite build sau khi thêm API client auth và AccountView.</x:v>
+      </x:c>
+      <x:c r="D98" s="75" t="str">
+        <x:v>B1: Chạy npm run build trong frontend.
+B2: Kiểm tra vue-tsc và Vite.</x:v>
+      </x:c>
+      <x:c r="E98" s="75" t="str">
+        <x:v>frontend/src/api.ts; AccountView.vue</x:v>
+      </x:c>
+      <x:c r="F98" s="76" t="str">
+        <x:v>Build production thành công.</x:v>
+      </x:c>
+      <x:c r="G98" s="75" t="str">
+        <x:v>Pass: vue-tsc --noEmit và Vite build pass.</x:v>
+      </x:c>
+      <x:c r="H98" s="75" t="str">
+        <x:v>TC_VIZI_089</x:v>
+      </x:c>
+      <x:c r="I98" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J98" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K98" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L98" s="75"/>
+      <x:c r="M98" s="75"/>
+      <x:c r="N98" s="75"/>
+      <x:c r="O98" s="75"/>
       <x:c r="P98" s="75" t="n"/>
       <x:c r="Q98" s="75" t="n"/>
       <x:c r="R98" s="75" t="n"/>
@@ -6317,21 +6528,47 @@
       <x:c r="Z98" s="75" t="n"/>
     </x:row>
     <x:row r="99" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A99" s="75" t="n"/>
-      <x:c r="B99" s="76" t="n"/>
-      <x:c r="C99" s="75" t="n"/>
-      <x:c r="D99" s="75" t="n"/>
-      <x:c r="E99" s="75" t="n"/>
-      <x:c r="F99" s="76" t="n"/>
-      <x:c r="G99" s="75" t="n"/>
-      <x:c r="H99" s="75" t="n"/>
-      <x:c r="I99" s="75" t="n"/>
-      <x:c r="J99" s="75" t="n"/>
-      <x:c r="K99" s="75" t="n"/>
-      <x:c r="L99" s="75" t="n"/>
-      <x:c r="M99" s="75" t="n"/>
-      <x:c r="N99" s="75" t="n"/>
-      <x:c r="O99" s="75" t="n"/>
+      <x:c r="A99" s="75" t="str">
+        <x:v>TC_VIZI_091</x:v>
+      </x:c>
+      <x:c r="B99" s="76" t="str">
+        <x:v>Browser UAT đăng ký, logout và login</x:v>
+      </x:c>
+      <x:c r="C99" s="75" t="str">
+        <x:v>Kiểm thử hành trình account trên FE/BE/PostgreSQL chạy thật.</x:v>
+      </x:c>
+      <x:c r="D99" s="75" t="str">
+        <x:v>B1: Mở /account.
+B2: Tạo account.
+B3: Logout.
+B4: Login sai.
+B5: Login đúng.</x:v>
+      </x:c>
+      <x:c r="E99" s="75" t="str">
+        <x:v>Tài khoản QA tạm trên PostgreSQL local</x:v>
+      </x:c>
+      <x:c r="F99" s="76" t="str">
+        <x:v>Đăng ký tự login; logout về form; sai password có lỗi; đúng password vào account.</x:v>
+      </x:c>
+      <x:c r="G99" s="75" t="str">
+        <x:v>Pass sau retest: session hoạt động end-to-end, không console error.</x:v>
+      </x:c>
+      <x:c r="H99" s="75" t="str">
+        <x:v>TC_VIZI_090</x:v>
+      </x:c>
+      <x:c r="I99" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J99" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K99" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L99" s="75"/>
+      <x:c r="M99" s="75"/>
+      <x:c r="N99" s="75"/>
+      <x:c r="O99" s="75"/>
       <x:c r="P99" s="75" t="n"/>
       <x:c r="Q99" s="75" t="n"/>
       <x:c r="R99" s="75" t="n"/>
@@ -6345,21 +6582,45 @@
       <x:c r="Z99" s="75" t="n"/>
     </x:row>
     <x:row r="100" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A100" s="75" t="n"/>
-      <x:c r="B100" s="76" t="n"/>
-      <x:c r="C100" s="75" t="n"/>
-      <x:c r="D100" s="75" t="n"/>
-      <x:c r="E100" s="75" t="n"/>
-      <x:c r="F100" s="76" t="n"/>
-      <x:c r="G100" s="75" t="n"/>
-      <x:c r="H100" s="75" t="n"/>
-      <x:c r="I100" s="75" t="n"/>
-      <x:c r="J100" s="75" t="n"/>
-      <x:c r="K100" s="75" t="n"/>
-      <x:c r="L100" s="75" t="n"/>
-      <x:c r="M100" s="75" t="n"/>
-      <x:c r="N100" s="75" t="n"/>
-      <x:c r="O100" s="75" t="n"/>
+      <x:c r="A100" s="75" t="str">
+        <x:v>TC_VIZI_092</x:v>
+      </x:c>
+      <x:c r="B100" s="76" t="str">
+        <x:v>Regression bug hostname làm mất session cookie</x:v>
+      </x:c>
+      <x:c r="C100" s="75" t="str">
+        <x:v>Xác nhận sửa lỗi FE chạy 127.0.0.1 nhưng API mặc định gọi localhost khiến đăng ký trả 401.</x:v>
+      </x:c>
+      <x:c r="D100" s="75" t="str">
+        <x:v>B1: Tái hiện POST register 401.
+B2: Dùng hostname hiện tại cho API mặc định.
+B3: Build và browser retest.</x:v>
+      </x:c>
+      <x:c r="E100" s="75" t="str">
+        <x:v>FE 127.0.0.1:5173; BE port 8080</x:v>
+      </x:c>
+      <x:c r="F100" s="76" t="str">
+        <x:v>FE và API cùng hostname; cookie session được gửi; đăng ký thành công.</x:v>
+      </x:c>
+      <x:c r="G100" s="75" t="str">
+        <x:v>Pass: lỗi 401 đã tái hiện, sửa root cause và retest thành công.</x:v>
+      </x:c>
+      <x:c r="H100" s="75" t="str">
+        <x:v>TC_VIZI_091</x:v>
+      </x:c>
+      <x:c r="I100" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J100" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K100" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L100" s="75"/>
+      <x:c r="M100" s="75"/>
+      <x:c r="N100" s="75"/>
+      <x:c r="O100" s="75"/>
       <x:c r="P100" s="75" t="n"/>
       <x:c r="Q100" s="75" t="n"/>
       <x:c r="R100" s="75" t="n"/>
@@ -6373,21 +6634,45 @@
       <x:c r="Z100" s="75" t="n"/>
     </x:row>
     <x:row r="101" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A101" s="75" t="n"/>
-      <x:c r="B101" s="76" t="n"/>
-      <x:c r="C101" s="75" t="n"/>
-      <x:c r="D101" s="75" t="n"/>
-      <x:c r="E101" s="75" t="n"/>
-      <x:c r="F101" s="76" t="n"/>
-      <x:c r="G101" s="75" t="n"/>
-      <x:c r="H101" s="75" t="n"/>
-      <x:c r="I101" s="75" t="n"/>
-      <x:c r="J101" s="75" t="n"/>
-      <x:c r="K101" s="75" t="n"/>
-      <x:c r="L101" s="75" t="n"/>
-      <x:c r="M101" s="75" t="n"/>
-      <x:c r="N101" s="75" t="n"/>
-      <x:c r="O101" s="75" t="n"/>
+      <x:c r="A101" s="75" t="str">
+        <x:v>TC_VIZI_093</x:v>
+      </x:c>
+      <x:c r="B101" s="76" t="str">
+        <x:v>Responsive, visual và performance smoke</x:v>
+      </x:c>
+      <x:c r="C101" s="75" t="str">
+        <x:v>Kiểm tra Account UI desktop/mobile và độ trễ health API local.</x:v>
+      </x:c>
+      <x:c r="D101" s="75" t="str">
+        <x:v>B1: Chụp desktop.
+B2: Test 390x844.
+B3: Gọi health 25 lần và tính p95.</x:v>
+      </x:c>
+      <x:c r="E101" s="75" t="str">
+        <x:v>Viewport 1280x720, 390x844; 25 requests</x:v>
+      </x:c>
+      <x:c r="F101" s="76" t="str">
+        <x:v>Không overlay/tràn ngang; UI rõ; health p95 dưới 100 ms.</x:v>
+      </x:c>
+      <x:c r="G101" s="75" t="str">
+        <x:v>Pass: mobile scrollWidth=390; console sạch; health p95=11.91 ms.</x:v>
+      </x:c>
+      <x:c r="H101" s="75" t="str">
+        <x:v>TC_VIZI_091</x:v>
+      </x:c>
+      <x:c r="I101" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J101" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K101" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L101" s="75"/>
+      <x:c r="M101" s="75"/>
+      <x:c r="N101" s="75"/>
+      <x:c r="O101" s="75"/>
       <x:c r="P101" s="75" t="n"/>
       <x:c r="Q101" s="75" t="n"/>
       <x:c r="R101" s="75" t="n"/>
@@ -6401,21 +6686,46 @@
       <x:c r="Z101" s="75" t="n"/>
     </x:row>
     <x:row r="102" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A102" s="75" t="n"/>
-      <x:c r="B102" s="76" t="n"/>
-      <x:c r="C102" s="75" t="n"/>
-      <x:c r="D102" s="75" t="n"/>
-      <x:c r="E102" s="75" t="n"/>
-      <x:c r="F102" s="76" t="n"/>
-      <x:c r="G102" s="75" t="n"/>
-      <x:c r="H102" s="75" t="n"/>
-      <x:c r="I102" s="75" t="n"/>
-      <x:c r="J102" s="75" t="n"/>
-      <x:c r="K102" s="75" t="n"/>
-      <x:c r="L102" s="75" t="n"/>
-      <x:c r="M102" s="75" t="n"/>
-      <x:c r="N102" s="75" t="n"/>
-      <x:c r="O102" s="75" t="n"/>
+      <x:c r="A102" s="75" t="str">
+        <x:v>TC_VIZI_094</x:v>
+      </x:c>
+      <x:c r="B102" s="76" t="str">
+        <x:v>Security static scan và cleanup runtime</x:v>
+      </x:c>
+      <x:c r="C102" s="75" t="str">
+        <x:v>Kiểm tra raw HTML, wildcard CORS, hardcoded secret; dọn account/process test trước commit.</x:v>
+      </x:c>
+      <x:c r="D102" s="75" t="str">
+        <x:v>B1: Chạy rg security patterns.
+B2: Xóa dữ liệu QA local.
+B3: Dừng port 5173/8080.
+B4: Scan staged diff.</x:v>
+      </x:c>
+      <x:c r="E102" s="75" t="str">
+        <x:v>backend/src; frontend/src; staged files</x:v>
+      </x:c>
+      <x:c r="F102" s="76" t="str">
+        <x:v>Không có raw HTML/wildcard CORS/secret thật; runtime test được dọn.</x:v>
+      </x:c>
+      <x:c r="G102" s="75" t="str">
+        <x:v>Pass sau bước verify cuối trước commit.</x:v>
+      </x:c>
+      <x:c r="H102" s="75" t="str">
+        <x:v>TC_VIZI_089</x:v>
+      </x:c>
+      <x:c r="I102" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J102" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K102" s="75" t="str">
+        <x:v>Bước 34</x:v>
+      </x:c>
+      <x:c r="L102" s="75"/>
+      <x:c r="M102" s="75"/>
+      <x:c r="N102" s="75"/>
+      <x:c r="O102" s="75"/>
       <x:c r="P102" s="75" t="n"/>
       <x:c r="Q102" s="75" t="n"/>
       <x:c r="R102" s="75" t="n"/>
@@ -31621,7 +31931,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79a039d788424cce"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafae9c16f3524067"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add owned design draft saving
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R14db4008c5b14014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5cd9eea25119452e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R479e3d9a8f9f40b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1d0233696fac44f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>92</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>94</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -6739,21 +6739,45 @@
       <x:c r="Z102" s="75" t="n"/>
     </x:row>
     <x:row r="103" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A103" s="75" t="n"/>
-      <x:c r="B103" s="76" t="n"/>
-      <x:c r="C103" s="75" t="n"/>
-      <x:c r="D103" s="75" t="n"/>
-      <x:c r="E103" s="75" t="n"/>
-      <x:c r="F103" s="76" t="n"/>
-      <x:c r="G103" s="75" t="n"/>
-      <x:c r="H103" s="75" t="n"/>
-      <x:c r="I103" s="75" t="n"/>
-      <x:c r="J103" s="75" t="n"/>
-      <x:c r="K103" s="75" t="n"/>
-      <x:c r="L103" s="75" t="n"/>
-      <x:c r="M103" s="75" t="n"/>
-      <x:c r="N103" s="75" t="n"/>
-      <x:c r="O103" s="75" t="n"/>
+      <x:c r="A103" s="75" t="str">
+        <x:v>TC_VIZI_095</x:v>
+      </x:c>
+      <x:c r="B103" s="76" t="str">
+        <x:v>API tạo design từ template active</x:v>
+      </x:c>
+      <x:c r="C103" s="75" t="str">
+        <x:v>Xác nhận user đã đăng nhập có thể tạo draft design từ template active và response trả đúng canvas ban đầu.</x:v>
+      </x:c>
+      <x:c r="D103" s="75" t="str">
+        <x:v>B1: Tạo user và template active.
+B2: POST /api/designs/from-template/{templateId} có CSRF.
+B3: Kiểm tra response.</x:v>
+      </x:c>
+      <x:c r="E103" s="75" t="str">
+        <x:v>Template có canvas_json gồm text layer Studio.</x:v>
+      </x:c>
+      <x:c r="F103" s="76" t="str">
+        <x:v>HTTP 201; trả id, templateId, name, widthMm, heightMm, canvasJson.</x:v>
+      </x:c>
+      <x:c r="G103" s="75" t="str">
+        <x:v>Pass: DesignApiIntegrationTests tạo design và canvas readback đúng Studio.</x:v>
+      </x:c>
+      <x:c r="H103" s="75" t="str">
+        <x:v>TC_VIZI_094</x:v>
+      </x:c>
+      <x:c r="I103" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J103" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K103" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L103" s="75"/>
+      <x:c r="M103" s="75"/>
+      <x:c r="N103" s="75"/>
+      <x:c r="O103" s="75"/>
       <x:c r="P103" s="75" t="n"/>
       <x:c r="Q103" s="75" t="n"/>
       <x:c r="R103" s="75" t="n"/>
@@ -6767,21 +6791,45 @@
       <x:c r="Z103" s="75" t="n"/>
     </x:row>
     <x:row r="104" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A104" s="75" t="n"/>
-      <x:c r="B104" s="76" t="n"/>
-      <x:c r="C104" s="75" t="n"/>
-      <x:c r="D104" s="75" t="n"/>
-      <x:c r="E104" s="75" t="n"/>
-      <x:c r="F104" s="76" t="n"/>
-      <x:c r="G104" s="75" t="n"/>
-      <x:c r="H104" s="75" t="n"/>
-      <x:c r="I104" s="75" t="n"/>
-      <x:c r="J104" s="75" t="n"/>
-      <x:c r="K104" s="75" t="n"/>
-      <x:c r="L104" s="75" t="n"/>
-      <x:c r="M104" s="75" t="n"/>
-      <x:c r="N104" s="75" t="n"/>
-      <x:c r="O104" s="75" t="n"/>
+      <x:c r="A104" s="75" t="str">
+        <x:v>TC_VIZI_096</x:v>
+      </x:c>
+      <x:c r="B104" s="76" t="str">
+        <x:v>API đọc design thuộc owner</x:v>
+      </x:c>
+      <x:c r="C104" s="75" t="str">
+        <x:v>Xác nhận endpoint GET /api/designs/{id} chỉ trả design thuộc current user và giữ đúng metadata template.</x:v>
+      </x:c>
+      <x:c r="D104" s="75" t="str">
+        <x:v>B1: Tạo design từ template.
+B2: GET /api/designs/{id} bằng cùng user.
+B3: Kiểm tra JSON.</x:v>
+      </x:c>
+      <x:c r="E104" s="75" t="str">
+        <x:v>Session owner@example.test; design vừa tạo.</x:v>
+      </x:c>
+      <x:c r="F104" s="76" t="str">
+        <x:v>HTTP 200; templateId, kích thước và canvasJson đúng dữ liệu đã lưu.</x:v>
+      </x:c>
+      <x:c r="G104" s="75" t="str">
+        <x:v>Pass: owner đọc lại design và canvas layer text đúng.</x:v>
+      </x:c>
+      <x:c r="H104" s="75" t="str">
+        <x:v>TC_VIZI_095</x:v>
+      </x:c>
+      <x:c r="I104" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J104" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K104" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L104" s="75"/>
+      <x:c r="M104" s="75"/>
+      <x:c r="N104" s="75"/>
+      <x:c r="O104" s="75"/>
       <x:c r="P104" s="75" t="n"/>
       <x:c r="Q104" s="75" t="n"/>
       <x:c r="R104" s="75" t="n"/>
@@ -6795,21 +6843,45 @@
       <x:c r="Z104" s="75" t="n"/>
     </x:row>
     <x:row r="105" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A105" s="75" t="n"/>
-      <x:c r="B105" s="76" t="n"/>
-      <x:c r="C105" s="75" t="n"/>
-      <x:c r="D105" s="75" t="n"/>
-      <x:c r="E105" s="75" t="n"/>
-      <x:c r="F105" s="76" t="n"/>
-      <x:c r="G105" s="75" t="n"/>
-      <x:c r="H105" s="75" t="n"/>
-      <x:c r="I105" s="75" t="n"/>
-      <x:c r="J105" s="75" t="n"/>
-      <x:c r="K105" s="75" t="n"/>
-      <x:c r="L105" s="75" t="n"/>
-      <x:c r="M105" s="75" t="n"/>
-      <x:c r="N105" s="75" t="n"/>
-      <x:c r="O105" s="75" t="n"/>
+      <x:c r="A105" s="75" t="str">
+        <x:v>TC_VIZI_097</x:v>
+      </x:c>
+      <x:c r="B105" s="76" t="str">
+        <x:v>API lưu canvas draft và đọc lại</x:v>
+      </x:c>
+      <x:c r="C105" s="75" t="str">
+        <x:v>Kiểm tra PUT /api/designs/{id} cập nhật tên/canvas và GET sau đó trả nội dung mới.</x:v>
+      </x:c>
+      <x:c r="D105" s="75" t="str">
+        <x:v>B1: Tạo design.
+B2: PUT canvasJson mới có CSRF.
+B3: GET lại design.</x:v>
+      </x:c>
+      <x:c r="E105" s="75" t="str">
+        <x:v>canvasJson mới có text Saved Studio.</x:v>
+      </x:c>
+      <x:c r="F105" s="76" t="str">
+        <x:v>HTTP 200; GET sau save trả text Saved Studio.</x:v>
+      </x:c>
+      <x:c r="G105" s="75" t="str">
+        <x:v>Pass: update và readback qua API đều đúng.</x:v>
+      </x:c>
+      <x:c r="H105" s="75" t="str">
+        <x:v>TC_VIZI_096</x:v>
+      </x:c>
+      <x:c r="I105" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J105" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K105" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L105" s="75"/>
+      <x:c r="M105" s="75"/>
+      <x:c r="N105" s="75"/>
+      <x:c r="O105" s="75"/>
       <x:c r="P105" s="75" t="n"/>
       <x:c r="Q105" s="75" t="n"/>
       <x:c r="R105" s="75" t="n"/>
@@ -6823,21 +6895,45 @@
       <x:c r="Z105" s="75" t="n"/>
     </x:row>
     <x:row r="106" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A106" s="75" t="n"/>
-      <x:c r="B106" s="76" t="n"/>
-      <x:c r="C106" s="75" t="n"/>
-      <x:c r="D106" s="75" t="n"/>
-      <x:c r="E106" s="75" t="n"/>
-      <x:c r="F106" s="76" t="n"/>
-      <x:c r="G106" s="75" t="n"/>
-      <x:c r="H106" s="75" t="n"/>
-      <x:c r="I106" s="75" t="n"/>
-      <x:c r="J106" s="75" t="n"/>
-      <x:c r="K106" s="75" t="n"/>
-      <x:c r="L106" s="75" t="n"/>
-      <x:c r="M106" s="75" t="n"/>
-      <x:c r="N106" s="75" t="n"/>
-      <x:c r="O106" s="75" t="n"/>
+      <x:c r="A106" s="75" t="str">
+        <x:v>TC_VIZI_098</x:v>
+      </x:c>
+      <x:c r="B106" s="76" t="str">
+        <x:v>Chặn IDOR đọc/sửa design</x:v>
+      </x:c>
+      <x:c r="C106" s="75" t="str">
+        <x:v>Xác nhận user khác không thể đọc hoặc sửa design không thuộc mình.</x:v>
+      </x:c>
+      <x:c r="D106" s="75" t="str">
+        <x:v>B1: Owner tạo design.
+B2: Other user GET design.
+B3: Other user PUT design.</x:v>
+      </x:c>
+      <x:c r="E106" s="75" t="str">
+        <x:v>owner@example.test và other@example.test.</x:v>
+      </x:c>
+      <x:c r="F106" s="76" t="str">
+        <x:v>Cả GET và PUT bằng other user trả HTTP 404.</x:v>
+      </x:c>
+      <x:c r="G106" s="75" t="str">
+        <x:v>Pass: repository filter theo id + user_id, không expose dữ liệu owner.</x:v>
+      </x:c>
+      <x:c r="H106" s="75" t="str">
+        <x:v>TC_VIZI_097</x:v>
+      </x:c>
+      <x:c r="I106" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J106" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K106" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L106" s="75"/>
+      <x:c r="M106" s="75"/>
+      <x:c r="N106" s="75"/>
+      <x:c r="O106" s="75"/>
       <x:c r="P106" s="75" t="n"/>
       <x:c r="Q106" s="75" t="n"/>
       <x:c r="R106" s="75" t="n"/>
@@ -6851,21 +6947,45 @@
       <x:c r="Z106" s="75" t="n"/>
     </x:row>
     <x:row r="107" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A107" s="75" t="n"/>
-      <x:c r="B107" s="76" t="n"/>
-      <x:c r="C107" s="75" t="n"/>
-      <x:c r="D107" s="75" t="n"/>
-      <x:c r="E107" s="75" t="n"/>
-      <x:c r="F107" s="76" t="n"/>
-      <x:c r="G107" s="75" t="n"/>
-      <x:c r="H107" s="75" t="n"/>
-      <x:c r="I107" s="75" t="n"/>
-      <x:c r="J107" s="75" t="n"/>
-      <x:c r="K107" s="75" t="n"/>
-      <x:c r="L107" s="75" t="n"/>
-      <x:c r="M107" s="75" t="n"/>
-      <x:c r="N107" s="75" t="n"/>
-      <x:c r="O107" s="75" t="n"/>
+      <x:c r="A107" s="75" t="str">
+        <x:v>TC_VIZI_099</x:v>
+      </x:c>
+      <x:c r="B107" s="76" t="str">
+        <x:v>Reject canvas JSON không hợp lệ</x:v>
+      </x:c>
+      <x:c r="C107" s="75" t="str">
+        <x:v>Canvas update thiếu layers array phải bị reject và không overwrite bản đang lưu.</x:v>
+      </x:c>
+      <x:c r="D107" s="75" t="str">
+        <x:v>B1: Tạo design có canvas Original.
+B2: PUT canvasJson = {}.
+B3: GET lại design.</x:v>
+      </x:c>
+      <x:c r="E107" s="75" t="str">
+        <x:v>canvasJson thiếu layers.</x:v>
+      </x:c>
+      <x:c r="F107" s="76" t="str">
+        <x:v>HTTP 400; tên và text Original vẫn được giữ.</x:v>
+      </x:c>
+      <x:c r="G107" s="75" t="str">
+        <x:v>Pass: invalid canvas bị chặn, dữ liệu cũ không mất.</x:v>
+      </x:c>
+      <x:c r="H107" s="75" t="str">
+        <x:v>TC_VIZI_097</x:v>
+      </x:c>
+      <x:c r="I107" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J107" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K107" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L107" s="75"/>
+      <x:c r="M107" s="75"/>
+      <x:c r="N107" s="75"/>
+      <x:c r="O107" s="75"/>
       <x:c r="P107" s="75" t="n"/>
       <x:c r="Q107" s="75" t="n"/>
       <x:c r="R107" s="75" t="n"/>
@@ -6879,21 +6999,45 @@
       <x:c r="Z107" s="75" t="n"/>
     </x:row>
     <x:row r="108" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A108" s="75" t="n"/>
-      <x:c r="B108" s="76" t="n"/>
-      <x:c r="C108" s="75" t="n"/>
-      <x:c r="D108" s="75" t="n"/>
-      <x:c r="E108" s="75" t="n"/>
-      <x:c r="F108" s="76" t="n"/>
-      <x:c r="G108" s="75" t="n"/>
-      <x:c r="H108" s="75" t="n"/>
-      <x:c r="I108" s="75" t="n"/>
-      <x:c r="J108" s="75" t="n"/>
-      <x:c r="K108" s="75" t="n"/>
-      <x:c r="L108" s="75" t="n"/>
-      <x:c r="M108" s="75" t="n"/>
-      <x:c r="N108" s="75" t="n"/>
-      <x:c r="O108" s="75" t="n"/>
+      <x:c r="A108" s="75" t="str">
+        <x:v>TC_VIZI_100</x:v>
+      </x:c>
+      <x:c r="B108" s="76" t="str">
+        <x:v>Không tạo design từ template inactive/missing</x:v>
+      </x:c>
+      <x:c r="C108" s="75" t="str">
+        <x:v>Template inactive hoặc id không tồn tại không được dùng để tạo design draft.</x:v>
+      </x:c>
+      <x:c r="D108" s="75" t="str">
+        <x:v>B1: Tạo template inactive.
+B2: POST từ template inactive.
+B3: POST từ id không tồn tại.</x:v>
+      </x:c>
+      <x:c r="E108" s="75" t="str">
+        <x:v>inactive.id và 999999.</x:v>
+      </x:c>
+      <x:c r="F108" s="76" t="str">
+        <x:v>Cả hai request trả HTTP 404.</x:v>
+      </x:c>
+      <x:c r="G108" s="75" t="str">
+        <x:v>Pass: service chỉ dùng findByIdAndActiveTrue.</x:v>
+      </x:c>
+      <x:c r="H108" s="75" t="str">
+        <x:v>TC_VIZI_095</x:v>
+      </x:c>
+      <x:c r="I108" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J108" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K108" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L108" s="75"/>
+      <x:c r="M108" s="75"/>
+      <x:c r="N108" s="75"/>
+      <x:c r="O108" s="75"/>
       <x:c r="P108" s="75" t="n"/>
       <x:c r="Q108" s="75" t="n"/>
       <x:c r="R108" s="75" t="n"/>
@@ -6907,21 +7051,45 @@
       <x:c r="Z108" s="75" t="n"/>
     </x:row>
     <x:row r="109" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A109" s="75" t="n"/>
-      <x:c r="B109" s="76" t="n"/>
-      <x:c r="C109" s="75" t="n"/>
-      <x:c r="D109" s="75" t="n"/>
-      <x:c r="E109" s="75" t="n"/>
-      <x:c r="F109" s="76" t="n"/>
-      <x:c r="G109" s="75" t="n"/>
-      <x:c r="H109" s="75" t="n"/>
-      <x:c r="I109" s="75" t="n"/>
-      <x:c r="J109" s="75" t="n"/>
-      <x:c r="K109" s="75" t="n"/>
-      <x:c r="L109" s="75" t="n"/>
-      <x:c r="M109" s="75" t="n"/>
-      <x:c r="N109" s="75" t="n"/>
-      <x:c r="O109" s="75" t="n"/>
+      <x:c r="A109" s="75" t="str">
+        <x:v>TC_VIZI_101</x:v>
+      </x:c>
+      <x:c r="B109" s="76" t="str">
+        <x:v>Regression full backend test</x:v>
+      </x:c>
+      <x:c r="C109" s="75" t="str">
+        <x:v>Chạy toàn bộ backend test sau khi thêm design API, entity và repository.</x:v>
+      </x:c>
+      <x:c r="D109" s="75" t="str">
+        <x:v>B1: Start PostgreSQL local.
+B2: Chạy .\mvnw.cmd test trong backend.
+B3: Kiểm tra tổng kết.</x:v>
+      </x:c>
+      <x:c r="E109" s="75" t="str">
+        <x:v>Backend Maven test suite + PostgreSQL 17 local.</x:v>
+      </x:c>
+      <x:c r="F109" s="76" t="str">
+        <x:v>Không có failure/error/skip.</x:v>
+      </x:c>
+      <x:c r="G109" s="75" t="str">
+        <x:v>Pass: 26 tests, 0 failures, 0 errors, 0 skipped.</x:v>
+      </x:c>
+      <x:c r="H109" s="75" t="str">
+        <x:v>TC_VIZI_100</x:v>
+      </x:c>
+      <x:c r="I109" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J109" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K109" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L109" s="75"/>
+      <x:c r="M109" s="75"/>
+      <x:c r="N109" s="75"/>
+      <x:c r="O109" s="75"/>
       <x:c r="P109" s="75" t="n"/>
       <x:c r="Q109" s="75" t="n"/>
       <x:c r="R109" s="75" t="n"/>
@@ -6935,21 +7103,44 @@
       <x:c r="Z109" s="75" t="n"/>
     </x:row>
     <x:row r="110" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A110" s="75" t="n"/>
-      <x:c r="B110" s="76" t="n"/>
-      <x:c r="C110" s="75" t="n"/>
-      <x:c r="D110" s="75" t="n"/>
-      <x:c r="E110" s="75" t="n"/>
-      <x:c r="F110" s="76" t="n"/>
-      <x:c r="G110" s="75" t="n"/>
-      <x:c r="H110" s="75" t="n"/>
-      <x:c r="I110" s="75" t="n"/>
-      <x:c r="J110" s="75" t="n"/>
-      <x:c r="K110" s="75" t="n"/>
-      <x:c r="L110" s="75" t="n"/>
-      <x:c r="M110" s="75" t="n"/>
-      <x:c r="N110" s="75" t="n"/>
-      <x:c r="O110" s="75" t="n"/>
+      <x:c r="A110" s="75" t="str">
+        <x:v>TC_VIZI_102</x:v>
+      </x:c>
+      <x:c r="B110" s="76" t="str">
+        <x:v>Build frontend có Save draft thật</x:v>
+      </x:c>
+      <x:c r="C110" s="75" t="str">
+        <x:v>Xác nhận TypeScript và Vite build sau khi thêm create/update design client và nút Save draft.</x:v>
+      </x:c>
+      <x:c r="D110" s="75" t="str">
+        <x:v>B1: Chạy npm run build trong frontend.
+B2: Kiểm tra vue-tsc và Vite.</x:v>
+      </x:c>
+      <x:c r="E110" s="75" t="str">
+        <x:v>frontend/src/api.ts; TemplateDetailView.vue.</x:v>
+      </x:c>
+      <x:c r="F110" s="76" t="str">
+        <x:v>Build production thành công.</x:v>
+      </x:c>
+      <x:c r="G110" s="75" t="str">
+        <x:v>Pass: vue-tsc --noEmit và Vite build pass.</x:v>
+      </x:c>
+      <x:c r="H110" s="75" t="str">
+        <x:v>TC_VIZI_101</x:v>
+      </x:c>
+      <x:c r="I110" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J110" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K110" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L110" s="75"/>
+      <x:c r="M110" s="75"/>
+      <x:c r="N110" s="75"/>
+      <x:c r="O110" s="75"/>
       <x:c r="P110" s="75" t="n"/>
       <x:c r="Q110" s="75" t="n"/>
       <x:c r="R110" s="75" t="n"/>
@@ -6963,21 +7154,45 @@
       <x:c r="Z110" s="75" t="n"/>
     </x:row>
     <x:row r="111" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A111" s="75" t="n"/>
-      <x:c r="B111" s="76" t="n"/>
-      <x:c r="C111" s="75" t="n"/>
-      <x:c r="D111" s="75" t="n"/>
-      <x:c r="E111" s="75" t="n"/>
-      <x:c r="F111" s="76" t="n"/>
-      <x:c r="G111" s="75" t="n"/>
-      <x:c r="H111" s="75" t="n"/>
-      <x:c r="I111" s="75" t="n"/>
-      <x:c r="J111" s="75" t="n"/>
-      <x:c r="K111" s="75" t="n"/>
-      <x:c r="L111" s="75" t="n"/>
-      <x:c r="M111" s="75" t="n"/>
-      <x:c r="N111" s="75" t="n"/>
-      <x:c r="O111" s="75" t="n"/>
+      <x:c r="A111" s="75" t="str">
+        <x:v>TC_VIZI_103</x:v>
+      </x:c>
+      <x:c r="B111" s="76" t="str">
+        <x:v>Browser UAT chưa login không được save</x:v>
+      </x:c>
+      <x:c r="C111" s="75" t="str">
+        <x:v>Người dùng anonymous bấm Save draft phải thấy yêu cầu đăng nhập thay vì tạo design.</x:v>
+      </x:c>
+      <x:c r="D111" s="75" t="str">
+        <x:v>B1: Mở /templates/9 chưa login.
+B2: Bấm Save draft.
+B3: Kiểm tra alert và link Account.</x:v>
+      </x:c>
+      <x:c r="E111" s="75" t="str">
+        <x:v>Template smoke id 9.</x:v>
+      </x:c>
+      <x:c r="F111" s="76" t="str">
+        <x:v>Hiển thị Sign in to save your draft và link Open account.</x:v>
+      </x:c>
+      <x:c r="G111" s="75" t="str">
+        <x:v>Pass: không tạo draft khi anonymous, UI hiển thị đúng hướng xử lý.</x:v>
+      </x:c>
+      <x:c r="H111" s="75" t="str">
+        <x:v>TC_VIZI_102</x:v>
+      </x:c>
+      <x:c r="I111" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J111" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K111" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L111" s="75"/>
+      <x:c r="M111" s="75"/>
+      <x:c r="N111" s="75"/>
+      <x:c r="O111" s="75"/>
       <x:c r="P111" s="75" t="n"/>
       <x:c r="Q111" s="75" t="n"/>
       <x:c r="R111" s="75" t="n"/>
@@ -6991,21 +7206,46 @@
       <x:c r="Z111" s="75" t="n"/>
     </x:row>
     <x:row r="112" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A112" s="75" t="n"/>
-      <x:c r="B112" s="76" t="n"/>
-      <x:c r="C112" s="75" t="n"/>
-      <x:c r="D112" s="75" t="n"/>
-      <x:c r="E112" s="75" t="n"/>
-      <x:c r="F112" s="76" t="n"/>
-      <x:c r="G112" s="75" t="n"/>
-      <x:c r="H112" s="75" t="n"/>
-      <x:c r="I112" s="75" t="n"/>
-      <x:c r="J112" s="75" t="n"/>
-      <x:c r="K112" s="75" t="n"/>
-      <x:c r="L112" s="75" t="n"/>
-      <x:c r="M112" s="75" t="n"/>
-      <x:c r="N112" s="75" t="n"/>
-      <x:c r="O112" s="75" t="n"/>
+      <x:c r="A112" s="75" t="str">
+        <x:v>TC_VIZI_104</x:v>
+      </x:c>
+      <x:c r="B112" s="76" t="str">
+        <x:v>Browser UAT save draft sau login</x:v>
+      </x:c>
+      <x:c r="C112" s="75" t="str">
+        <x:v>Người dùng đăng ký local, sửa text layer và bấm Save draft tạo design thật.</x:v>
+      </x:c>
+      <x:c r="D112" s="75" t="str">
+        <x:v>B1: Tạo account QA.
+B2: Quay lại template.
+B3: Sửa text layer.
+B4: Bấm Save draft.</x:v>
+      </x:c>
+      <x:c r="E112" s="75" t="str">
+        <x:v>Text layer chứa Saved Studio Step 35.</x:v>
+      </x:c>
+      <x:c r="F112" s="76" t="str">
+        <x:v>UI hiển thị Draft #id saved; không có alert lỗi.</x:v>
+      </x:c>
+      <x:c r="G112" s="75" t="str">
+        <x:v>Pass: account QA tạo session và Save draft trả Draft #1 saved.</x:v>
+      </x:c>
+      <x:c r="H112" s="75" t="str">
+        <x:v>TC_VIZI_103</x:v>
+      </x:c>
+      <x:c r="I112" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J112" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K112" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L112" s="75"/>
+      <x:c r="M112" s="75"/>
+      <x:c r="N112" s="75"/>
+      <x:c r="O112" s="75"/>
       <x:c r="P112" s="75" t="n"/>
       <x:c r="Q112" s="75" t="n"/>
       <x:c r="R112" s="75" t="n"/>
@@ -7019,21 +7259,45 @@
       <x:c r="Z112" s="75" t="n"/>
     </x:row>
     <x:row r="113" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A113" s="75" t="n"/>
-      <x:c r="B113" s="76" t="n"/>
-      <x:c r="C113" s="75" t="n"/>
-      <x:c r="D113" s="75" t="n"/>
-      <x:c r="E113" s="75" t="n"/>
-      <x:c r="F113" s="76" t="n"/>
-      <x:c r="G113" s="75" t="n"/>
-      <x:c r="H113" s="75" t="n"/>
-      <x:c r="I113" s="75" t="n"/>
-      <x:c r="J113" s="75" t="n"/>
-      <x:c r="K113" s="75" t="n"/>
-      <x:c r="L113" s="75" t="n"/>
-      <x:c r="M113" s="75" t="n"/>
-      <x:c r="N113" s="75" t="n"/>
-      <x:c r="O113" s="75" t="n"/>
+      <x:c r="A113" s="75" t="str">
+        <x:v>TC_VIZI_105</x:v>
+      </x:c>
+      <x:c r="B113" s="76" t="str">
+        <x:v>Browser UAT save lần hai update cùng draft</x:v>
+      </x:c>
+      <x:c r="C113" s="75" t="str">
+        <x:v>Save lần hai trên cùng màn template phải cập nhật draft hiện tại, không tạo duplicate.</x:v>
+      </x:c>
+      <x:c r="D113" s="75" t="str">
+        <x:v>B1: Sau save lần 1, sửa text thành Updated Studio Step 35.
+B2: Bấm Save draft lần hai.
+B3: Readback DB.</x:v>
+      </x:c>
+      <x:c r="E113" s="75" t="str">
+        <x:v>QA user và design vừa tạo.</x:v>
+      </x:c>
+      <x:c r="F113" s="76" t="str">
+        <x:v>Status vẫn là Draft #1 saved; DB chỉ có 1 design của QA user.</x:v>
+      </x:c>
+      <x:c r="G113" s="75" t="str">
+        <x:v>Pass: DB saved_text=Updated Studio Step 35, qa_design_count=1.</x:v>
+      </x:c>
+      <x:c r="H113" s="75" t="str">
+        <x:v>TC_VIZI_104</x:v>
+      </x:c>
+      <x:c r="I113" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J113" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K113" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L113" s="75"/>
+      <x:c r="M113" s="75"/>
+      <x:c r="N113" s="75"/>
+      <x:c r="O113" s="75"/>
       <x:c r="P113" s="75" t="n"/>
       <x:c r="Q113" s="75" t="n"/>
       <x:c r="R113" s="75" t="n"/>
@@ -7047,21 +7311,46 @@
       <x:c r="Z113" s="75" t="n"/>
     </x:row>
     <x:row r="114" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A114" s="75" t="n"/>
-      <x:c r="B114" s="76" t="n"/>
-      <x:c r="C114" s="75" t="n"/>
-      <x:c r="D114" s="75" t="n"/>
-      <x:c r="E114" s="75" t="n"/>
-      <x:c r="F114" s="76" t="n"/>
-      <x:c r="G114" s="75" t="n"/>
-      <x:c r="H114" s="75" t="n"/>
-      <x:c r="I114" s="75" t="n"/>
-      <x:c r="J114" s="75" t="n"/>
-      <x:c r="K114" s="75" t="n"/>
-      <x:c r="L114" s="75" t="n"/>
-      <x:c r="M114" s="75" t="n"/>
-      <x:c r="N114" s="75" t="n"/>
-      <x:c r="O114" s="75" t="n"/>
+      <x:c r="A114" s="75" t="str">
+        <x:v>TC_VIZI_106</x:v>
+      </x:c>
+      <x:c r="B114" s="76" t="str">
+        <x:v>XSS và responsive smoke cho editor</x:v>
+      </x:c>
+      <x:c r="C114" s="75" t="str">
+        <x:v>Text layer nhập chuỗi HTML phải render như text; mobile không tràn ngang và console không có error.</x:v>
+      </x:c>
+      <x:c r="D114" s="75" t="str">
+        <x:v>B1: Nhập &lt;img src=x onerror=alert(1)&gt; vào textarea.
+B2: Save.
+B3: Kiểm tra DOM canvas.
+B4: Test viewport 390x844.</x:v>
+      </x:c>
+      <x:c r="E114" s="75" t="str">
+        <x:v>Viewport desktop và 390x844.</x:v>
+      </x:c>
+      <x:c r="F114" s="76" t="str">
+        <x:v>Không có img/script trong .canvas-layer; scrollWidth bằng clientWidth; console error rỗng.</x:v>
+      </x:c>
+      <x:c r="G114" s="75" t="str">
+        <x:v>Pass: renderedImgInCanvas=0, mobile overflow=false, consoleErrors=[]</x:v>
+      </x:c>
+      <x:c r="H114" s="75" t="str">
+        <x:v>TC_VIZI_105</x:v>
+      </x:c>
+      <x:c r="I114" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J114" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K114" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L114" s="75"/>
+      <x:c r="M114" s="75"/>
+      <x:c r="N114" s="75"/>
+      <x:c r="O114" s="75"/>
       <x:c r="P114" s="75" t="n"/>
       <x:c r="Q114" s="75" t="n"/>
       <x:c r="R114" s="75" t="n"/>
@@ -7075,21 +7364,46 @@
       <x:c r="Z114" s="75" t="n"/>
     </x:row>
     <x:row r="115" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A115" s="75" t="n"/>
-      <x:c r="B115" s="76" t="n"/>
-      <x:c r="C115" s="75" t="n"/>
-      <x:c r="D115" s="75" t="n"/>
-      <x:c r="E115" s="75" t="n"/>
-      <x:c r="F115" s="76" t="n"/>
-      <x:c r="G115" s="75" t="n"/>
-      <x:c r="H115" s="75" t="n"/>
-      <x:c r="I115" s="75" t="n"/>
-      <x:c r="J115" s="75" t="n"/>
-      <x:c r="K115" s="75" t="n"/>
-      <x:c r="L115" s="75" t="n"/>
-      <x:c r="M115" s="75" t="n"/>
-      <x:c r="N115" s="75" t="n"/>
-      <x:c r="O115" s="75" t="n"/>
+      <x:c r="A115" s="75" t="str">
+        <x:v>TC_VIZI_107</x:v>
+      </x:c>
+      <x:c r="B115" s="76" t="str">
+        <x:v>Security scan, cleanup và staged diff</x:v>
+      </x:c>
+      <x:c r="C115" s="75" t="str">
+        <x:v>Kiểm tra không có raw HTML/wildcard CORS/secret trong thay đổi; dọn dữ liệu QA/log/runtime trước commit.</x:v>
+      </x:c>
+      <x:c r="D115" s="75" t="str">
+        <x:v>B1: Chạy rg security patterns.
+B2: Xóa QA user/template smoke local.
+B3: Stop BE/FE.
+B4: git diff --check và scan staged files.</x:v>
+      </x:c>
+      <x:c r="E115" s="75" t="str">
+        <x:v>backend, frontend, Template_TestCase.xlsx, staged diff.</x:v>
+      </x:c>
+      <x:c r="F115" s="76" t="str">
+        <x:v>Không stage .agents/.codex-work/.env/log; không có secret hoặc thông tin cá nhân.</x:v>
+      </x:c>
+      <x:c r="G115" s="75" t="str">
+        <x:v>Pass sau vòng verify cuối trước commit.</x:v>
+      </x:c>
+      <x:c r="H115" s="75" t="str">
+        <x:v>TC_VIZI_101</x:v>
+      </x:c>
+      <x:c r="I115" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J115" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K115" s="75" t="str">
+        <x:v>Bước 35</x:v>
+      </x:c>
+      <x:c r="L115" s="75"/>
+      <x:c r="M115" s="75"/>
+      <x:c r="N115" s="75"/>
+      <x:c r="O115" s="75"/>
       <x:c r="P115" s="75" t="n"/>
       <x:c r="Q115" s="75" t="n"/>
       <x:c r="R115" s="75" t="n"/>
@@ -31931,7 +32245,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafae9c16f3524067"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51eb3e20601b4e2d"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add draft workspace views
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R479e3d9a8f9f40b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1d0233696fac44f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R90f65733aa8c4367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc0e80ff0a1f44c38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>105</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>107</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -7417,21 +7417,45 @@
       <x:c r="Z115" s="75" t="n"/>
     </x:row>
     <x:row r="116" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A116" s="75" t="n"/>
-      <x:c r="B116" s="76" t="n"/>
-      <x:c r="C116" s="75" t="n"/>
-      <x:c r="D116" s="75" t="n"/>
-      <x:c r="E116" s="75" t="n"/>
-      <x:c r="F116" s="76" t="n"/>
-      <x:c r="G116" s="75" t="n"/>
-      <x:c r="H116" s="75" t="n"/>
-      <x:c r="I116" s="75" t="n"/>
-      <x:c r="J116" s="75" t="n"/>
-      <x:c r="K116" s="75" t="n"/>
-      <x:c r="L116" s="75" t="n"/>
-      <x:c r="M116" s="75" t="n"/>
-      <x:c r="N116" s="75" t="n"/>
-      <x:c r="O116" s="75" t="n"/>
+      <x:c r="A116" s="75" t="str">
+        <x:v>TC_VIZI_108</x:v>
+      </x:c>
+      <x:c r="B116" s="76" t="str">
+        <x:v>API list draft cua owner</x:v>
+      </x:c>
+      <x:c r="C116" s="75" t="str">
+        <x:v>GET /api/designs phai tra danh sach draft cua current user va khong tra canvasJson nang.</x:v>
+      </x:c>
+      <x:c r="D116" s="75" t="str">
+        <x:v>B1: Tao 2 design cho owner.
+B2: Tao 1 design cho other user.
+B3: GET /api/designs bang owner.</x:v>
+      </x:c>
+      <x:c r="E116" s="75" t="str">
+        <x:v>owner@example.test, other@example.test, PostgreSQL local.</x:v>
+      </x:c>
+      <x:c r="F116" s="76" t="str">
+        <x:v>HTTP 200; chi co 2 draft cua owner; response list khong co canvasJson.</x:v>
+      </x:c>
+      <x:c r="G116" s="75" t="str">
+        <x:v>Pass: DesignApiIntegrationTests list 2 item va canvasJson khong ton tai.</x:v>
+      </x:c>
+      <x:c r="H116" s="75" t="str">
+        <x:v>TC_VIZI_107</x:v>
+      </x:c>
+      <x:c r="I116" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J116" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K116" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L116" s="75"/>
+      <x:c r="M116" s="75"/>
+      <x:c r="N116" s="75"/>
+      <x:c r="O116" s="75"/>
       <x:c r="P116" s="75" t="n"/>
       <x:c r="Q116" s="75" t="n"/>
       <x:c r="R116" s="75" t="n"/>
@@ -7445,21 +7469,45 @@
       <x:c r="Z116" s="75" t="n"/>
     </x:row>
     <x:row r="117" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A117" s="75" t="n"/>
-      <x:c r="B117" s="76" t="n"/>
-      <x:c r="C117" s="75" t="n"/>
-      <x:c r="D117" s="75" t="n"/>
-      <x:c r="E117" s="75" t="n"/>
-      <x:c r="F117" s="76" t="n"/>
-      <x:c r="G117" s="75" t="n"/>
-      <x:c r="H117" s="75" t="n"/>
-      <x:c r="I117" s="75" t="n"/>
-      <x:c r="J117" s="75" t="n"/>
-      <x:c r="K117" s="75" t="n"/>
-      <x:c r="L117" s="75" t="n"/>
-      <x:c r="M117" s="75" t="n"/>
-      <x:c r="N117" s="75" t="n"/>
-      <x:c r="O117" s="75" t="n"/>
+      <x:c r="A117" s="75" t="str">
+        <x:v>TC_VIZI_109</x:v>
+      </x:c>
+      <x:c r="B117" s="76" t="str">
+        <x:v>API list draft sap xep moi nhat</x:v>
+      </x:c>
+      <x:c r="C117" s="75" t="str">
+        <x:v>Draft vua update phai len dau danh sach de My drafts uu tien ban dang lam.</x:v>
+      </x:c>
+      <x:c r="D117" s="75" t="str">
+        <x:v>B1: Tao 2 draft.
+B2: PUT draft dau tien.
+B3: GET /api/designs.</x:v>
+      </x:c>
+      <x:c r="E117" s="75" t="str">
+        <x:v>Draft dau tien duoc update thanh Newest Owner Draft.</x:v>
+      </x:c>
+      <x:c r="F117" s="76" t="str">
+        <x:v>Item dau tien trong list co name Newest Owner Draft.</x:v>
+      </x:c>
+      <x:c r="G117" s="75" t="str">
+        <x:v>Pass: sort theo updatedAt desc dung trong integration test.</x:v>
+      </x:c>
+      <x:c r="H117" s="75" t="str">
+        <x:v>TC_VIZI_108</x:v>
+      </x:c>
+      <x:c r="I117" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J117" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K117" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L117" s="75"/>
+      <x:c r="M117" s="75"/>
+      <x:c r="N117" s="75"/>
+      <x:c r="O117" s="75"/>
       <x:c r="P117" s="75" t="n"/>
       <x:c r="Q117" s="75" t="n"/>
       <x:c r="R117" s="75" t="n"/>
@@ -7473,21 +7521,45 @@
       <x:c r="Z117" s="75" t="n"/>
     </x:row>
     <x:row r="118" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A118" s="75" t="n"/>
-      <x:c r="B118" s="76" t="n"/>
-      <x:c r="C118" s="75" t="n"/>
-      <x:c r="D118" s="75" t="n"/>
-      <x:c r="E118" s="75" t="n"/>
-      <x:c r="F118" s="76" t="n"/>
-      <x:c r="G118" s="75" t="n"/>
-      <x:c r="H118" s="75" t="n"/>
-      <x:c r="I118" s="75" t="n"/>
-      <x:c r="J118" s="75" t="n"/>
-      <x:c r="K118" s="75" t="n"/>
-      <x:c r="L118" s="75" t="n"/>
-      <x:c r="M118" s="75" t="n"/>
-      <x:c r="N118" s="75" t="n"/>
-      <x:c r="O118" s="75" t="n"/>
+      <x:c r="A118" s="75" t="str">
+        <x:v>TC_VIZI_110</x:v>
+      </x:c>
+      <x:c r="B118" s="76" t="str">
+        <x:v>Regression backend sau list API</x:v>
+      </x:c>
+      <x:c r="C118" s="75" t="str">
+        <x:v>Chay full backend suite sau khi them repository query, DTO list va controller GET /api/designs.</x:v>
+      </x:c>
+      <x:c r="D118" s="75" t="str">
+        <x:v>B1: Kiem tra PostgreSQL local dang chay.
+B2: Chay .\mvnw.cmd test.
+B3: Kiem tra tong ket.</x:v>
+      </x:c>
+      <x:c r="E118" s="75" t="str">
+        <x:v>Backend Maven test suite.</x:v>
+      </x:c>
+      <x:c r="F118" s="76" t="str">
+        <x:v>Khong co failure/error/skip.</x:v>
+      </x:c>
+      <x:c r="G118" s="75" t="str">
+        <x:v>Pass: 27 tests, 0 failures, 0 errors, 0 skipped.</x:v>
+      </x:c>
+      <x:c r="H118" s="75" t="str">
+        <x:v>TC_VIZI_109</x:v>
+      </x:c>
+      <x:c r="I118" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J118" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K118" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L118" s="75"/>
+      <x:c r="M118" s="75"/>
+      <x:c r="N118" s="75"/>
+      <x:c r="O118" s="75"/>
       <x:c r="P118" s="75" t="n"/>
       <x:c r="Q118" s="75" t="n"/>
       <x:c r="R118" s="75" t="n"/>
@@ -7501,21 +7573,44 @@
       <x:c r="Z118" s="75" t="n"/>
     </x:row>
     <x:row r="119" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A119" s="75" t="n"/>
-      <x:c r="B119" s="76" t="n"/>
-      <x:c r="C119" s="75" t="n"/>
-      <x:c r="D119" s="75" t="n"/>
-      <x:c r="E119" s="75" t="n"/>
-      <x:c r="F119" s="76" t="n"/>
-      <x:c r="G119" s="75" t="n"/>
-      <x:c r="H119" s="75" t="n"/>
-      <x:c r="I119" s="75" t="n"/>
-      <x:c r="J119" s="75" t="n"/>
-      <x:c r="K119" s="75" t="n"/>
-      <x:c r="L119" s="75" t="n"/>
-      <x:c r="M119" s="75" t="n"/>
-      <x:c r="N119" s="75" t="n"/>
-      <x:c r="O119" s="75" t="n"/>
+      <x:c r="A119" s="75" t="str">
+        <x:v>TC_VIZI_111</x:v>
+      </x:c>
+      <x:c r="B119" s="76" t="str">
+        <x:v>Build frontend My drafts</x:v>
+      </x:c>
+      <x:c r="C119" s="75" t="str">
+        <x:v>Xac nhan TypeScript va Vite build sau khi them route /designs va /designs/:id.</x:v>
+      </x:c>
+      <x:c r="D119" s="75" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Kiem tra vue-tsc va Vite.</x:v>
+      </x:c>
+      <x:c r="E119" s="75" t="str">
+        <x:v>DesignsView.vue, DesignDetailView.vue, router.ts, api.ts.</x:v>
+      </x:c>
+      <x:c r="F119" s="76" t="str">
+        <x:v>Build production thanh cong.</x:v>
+      </x:c>
+      <x:c r="G119" s="75" t="str">
+        <x:v>Pass: vue-tsc --noEmit va Vite build pass.</x:v>
+      </x:c>
+      <x:c r="H119" s="75" t="str">
+        <x:v>TC_VIZI_110</x:v>
+      </x:c>
+      <x:c r="I119" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J119" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K119" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L119" s="75"/>
+      <x:c r="M119" s="75"/>
+      <x:c r="N119" s="75"/>
+      <x:c r="O119" s="75"/>
       <x:c r="P119" s="75" t="n"/>
       <x:c r="Q119" s="75" t="n"/>
       <x:c r="R119" s="75" t="n"/>
@@ -7529,21 +7624,44 @@
       <x:c r="Z119" s="75" t="n"/>
     </x:row>
     <x:row r="120" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A120" s="75" t="n"/>
-      <x:c r="B120" s="76" t="n"/>
-      <x:c r="C120" s="75" t="n"/>
-      <x:c r="D120" s="75" t="n"/>
-      <x:c r="E120" s="75" t="n"/>
-      <x:c r="F120" s="76" t="n"/>
-      <x:c r="G120" s="75" t="n"/>
-      <x:c r="H120" s="75" t="n"/>
-      <x:c r="I120" s="75" t="n"/>
-      <x:c r="J120" s="75" t="n"/>
-      <x:c r="K120" s="75" t="n"/>
-      <x:c r="L120" s="75" t="n"/>
-      <x:c r="M120" s="75" t="n"/>
-      <x:c r="N120" s="75" t="n"/>
-      <x:c r="O120" s="75" t="n"/>
+      <x:c r="A120" s="75" t="str">
+        <x:v>TC_VIZI_112</x:v>
+      </x:c>
+      <x:c r="B120" s="76" t="str">
+        <x:v>Browser UAT /designs anonymous</x:v>
+      </x:c>
+      <x:c r="C120" s="75" t="str">
+        <x:v>Nguoi dung chua login vao My drafts phai duoc yeu cau dang nhap.</x:v>
+      </x:c>
+      <x:c r="D120" s="75" t="str">
+        <x:v>B1: Mo /designs khi chua login.
+B2: Doc alert va link.</x:v>
+      </x:c>
+      <x:c r="E120" s="75" t="str">
+        <x:v>Browser local 127.0.0.1:5173.</x:v>
+      </x:c>
+      <x:c r="F120" s="76" t="str">
+        <x:v>Hien thi Sign in to view your drafts va Open account.</x:v>
+      </x:c>
+      <x:c r="G120" s="75" t="str">
+        <x:v>Pass: unauth /designs khong hien draft va co link account.</x:v>
+      </x:c>
+      <x:c r="H120" s="75" t="str">
+        <x:v>TC_VIZI_111</x:v>
+      </x:c>
+      <x:c r="I120" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J120" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K120" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L120" s="75"/>
+      <x:c r="M120" s="75"/>
+      <x:c r="N120" s="75"/>
+      <x:c r="O120" s="75"/>
       <x:c r="P120" s="75" t="n"/>
       <x:c r="Q120" s="75" t="n"/>
       <x:c r="R120" s="75" t="n"/>
@@ -7557,21 +7675,46 @@
       <x:c r="Z120" s="75" t="n"/>
     </x:row>
     <x:row r="121" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A121" s="75" t="n"/>
-      <x:c r="B121" s="76" t="n"/>
-      <x:c r="C121" s="75" t="n"/>
-      <x:c r="D121" s="75" t="n"/>
-      <x:c r="E121" s="75" t="n"/>
-      <x:c r="F121" s="76" t="n"/>
-      <x:c r="G121" s="75" t="n"/>
-      <x:c r="H121" s="75" t="n"/>
-      <x:c r="I121" s="75" t="n"/>
-      <x:c r="J121" s="75" t="n"/>
-      <x:c r="K121" s="75" t="n"/>
-      <x:c r="L121" s="75" t="n"/>
-      <x:c r="M121" s="75" t="n"/>
-      <x:c r="N121" s="75" t="n"/>
-      <x:c r="O121" s="75" t="n"/>
+      <x:c r="A121" s="75" t="str">
+        <x:v>TC_VIZI_113</x:v>
+      </x:c>
+      <x:c r="B121" s="76" t="str">
+        <x:v>Browser UAT tao draft tu template</x:v>
+      </x:c>
+      <x:c r="C121" s="75" t="str">
+        <x:v>Sau khi dang ky QA, user tao draft tu template smoke va thay status saved.</x:v>
+      </x:c>
+      <x:c r="D121" s="75" t="str">
+        <x:v>B1: Dang ky QA.
+B2: Mo /templates/10.
+B3: Sua text layer.
+B4: Save draft.</x:v>
+      </x:c>
+      <x:c r="E121" s="75" t="str">
+        <x:v>Template Step36 Draft Smoke Card.</x:v>
+      </x:c>
+      <x:c r="F121" s="76" t="str">
+        <x:v>UI hien Draft #id saved, canvas preview co text moi.</x:v>
+      </x:c>
+      <x:c r="G121" s="75" t="str">
+        <x:v>Pass: Draft #2 saved va preview co Draft From Template Step 36.</x:v>
+      </x:c>
+      <x:c r="H121" s="75" t="str">
+        <x:v>TC_VIZI_112</x:v>
+      </x:c>
+      <x:c r="I121" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J121" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K121" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L121" s="75"/>
+      <x:c r="M121" s="75"/>
+      <x:c r="N121" s="75"/>
+      <x:c r="O121" s="75"/>
       <x:c r="P121" s="75" t="n"/>
       <x:c r="Q121" s="75" t="n"/>
       <x:c r="R121" s="75" t="n"/>
@@ -7585,21 +7728,44 @@
       <x:c r="Z121" s="75" t="n"/>
     </x:row>
     <x:row r="122" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A122" s="75" t="n"/>
-      <x:c r="B122" s="76" t="n"/>
-      <x:c r="C122" s="75" t="n"/>
-      <x:c r="D122" s="75" t="n"/>
-      <x:c r="E122" s="75" t="n"/>
-      <x:c r="F122" s="76" t="n"/>
-      <x:c r="G122" s="75" t="n"/>
-      <x:c r="H122" s="75" t="n"/>
-      <x:c r="I122" s="75" t="n"/>
-      <x:c r="J122" s="75" t="n"/>
-      <x:c r="K122" s="75" t="n"/>
-      <x:c r="L122" s="75" t="n"/>
-      <x:c r="M122" s="75" t="n"/>
-      <x:c r="N122" s="75" t="n"/>
-      <x:c r="O122" s="75" t="n"/>
+      <x:c r="A122" s="75" t="str">
+        <x:v>TC_VIZI_114</x:v>
+      </x:c>
+      <x:c r="B122" s="76" t="str">
+        <x:v>Browser UAT My drafts list</x:v>
+      </x:c>
+      <x:c r="C122" s="75" t="str">
+        <x:v>My drafts phai hien draft vua tao voi link mo lai dung id.</x:v>
+      </x:c>
+      <x:c r="D122" s="75" t="str">
+        <x:v>B1: Mo /designs sau khi save.
+B2: Kiem tra card va href.</x:v>
+      </x:c>
+      <x:c r="E122" s="75" t="str">
+        <x:v>QA session co 1 draft.</x:v>
+      </x:c>
+      <x:c r="F122" s="76" t="str">
+        <x:v>Card hien Step36 Draft Smoke Card, Draft #id va href /designs/{id}.</x:v>
+      </x:c>
+      <x:c r="G122" s="75" t="str">
+        <x:v>Pass: list co 1 card href /designs/2.</x:v>
+      </x:c>
+      <x:c r="H122" s="75" t="str">
+        <x:v>TC_VIZI_113</x:v>
+      </x:c>
+      <x:c r="I122" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J122" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K122" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L122" s="75"/>
+      <x:c r="M122" s="75"/>
+      <x:c r="N122" s="75"/>
+      <x:c r="O122" s="75"/>
       <x:c r="P122" s="75" t="n"/>
       <x:c r="Q122" s="75" t="n"/>
       <x:c r="R122" s="75" t="n"/>
@@ -7613,21 +7779,46 @@
       <x:c r="Z122" s="75" t="n"/>
     </x:row>
     <x:row r="123" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A123" s="75" t="n"/>
-      <x:c r="B123" s="76" t="n"/>
-      <x:c r="C123" s="75" t="n"/>
-      <x:c r="D123" s="75" t="n"/>
-      <x:c r="E123" s="75" t="n"/>
-      <x:c r="F123" s="76" t="n"/>
-      <x:c r="G123" s="75" t="n"/>
-      <x:c r="H123" s="75" t="n"/>
-      <x:c r="I123" s="75" t="n"/>
-      <x:c r="J123" s="75" t="n"/>
-      <x:c r="K123" s="75" t="n"/>
-      <x:c r="L123" s="75" t="n"/>
-      <x:c r="M123" s="75" t="n"/>
-      <x:c r="N123" s="75" t="n"/>
-      <x:c r="O123" s="75" t="n"/>
+      <x:c r="A123" s="75" t="str">
+        <x:v>TC_VIZI_115</x:v>
+      </x:c>
+      <x:c r="B123" s="76" t="str">
+        <x:v>Browser UAT mo lai va save draft</x:v>
+      </x:c>
+      <x:c r="C123" s="75" t="str">
+        <x:v>User mo /designs/{id}, thay noi dung da save, sua text va save cap nhat draft hien tai.</x:v>
+      </x:c>
+      <x:c r="D123" s="75" t="str">
+        <x:v>B1: Mo /designs/{id}.
+B2: Kiem tra textarea.
+B3: Sua text.
+B4: Save.</x:v>
+      </x:c>
+      <x:c r="E123" s="75" t="str">
+        <x:v>Text moi Reopened Draft Step 36.</x:v>
+      </x:c>
+      <x:c r="F123" s="76" t="str">
+        <x:v>Status Draft #id saved; DB saved_text la text moi; chi co 1 draft QA.</x:v>
+      </x:c>
+      <x:c r="G123" s="75" t="str">
+        <x:v>Pass: DB readback saved_text moi va qa_design_count=1.</x:v>
+      </x:c>
+      <x:c r="H123" s="75" t="str">
+        <x:v>TC_VIZI_114</x:v>
+      </x:c>
+      <x:c r="I123" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J123" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K123" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L123" s="75"/>
+      <x:c r="M123" s="75"/>
+      <x:c r="N123" s="75"/>
+      <x:c r="O123" s="75"/>
       <x:c r="P123" s="75" t="n"/>
       <x:c r="Q123" s="75" t="n"/>
       <x:c r="R123" s="75" t="n"/>
@@ -7641,21 +7832,46 @@
       <x:c r="Z123" s="75" t="n"/>
     </x:row>
     <x:row r="124" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A124" s="75" t="n"/>
-      <x:c r="B124" s="76" t="n"/>
-      <x:c r="C124" s="75" t="n"/>
-      <x:c r="D124" s="75" t="n"/>
-      <x:c r="E124" s="75" t="n"/>
-      <x:c r="F124" s="76" t="n"/>
-      <x:c r="G124" s="75" t="n"/>
-      <x:c r="H124" s="75" t="n"/>
-      <x:c r="I124" s="75" t="n"/>
-      <x:c r="J124" s="75" t="n"/>
-      <x:c r="K124" s="75" t="n"/>
-      <x:c r="L124" s="75" t="n"/>
-      <x:c r="M124" s="75" t="n"/>
-      <x:c r="N124" s="75" t="n"/>
-      <x:c r="O124" s="75" t="n"/>
+      <x:c r="A124" s="75" t="str">
+        <x:v>TC_VIZI_116</x:v>
+      </x:c>
+      <x:c r="B124" s="76" t="str">
+        <x:v>XSS, mobile va performance smoke</x:v>
+      </x:c>
+      <x:c r="C124" s="75" t="str">
+        <x:v>Text HTML trong draft detail phai render nhu text; mobile khong tran ngang; health API nhanh.</x:v>
+      </x:c>
+      <x:c r="D124" s="75" t="str">
+        <x:v>B1: Nhap &lt;script&gt;alert(1)&lt;/script&gt; vao text layer.
+B2: Save.
+B3: Test viewport 390x844.
+B4: Goi health 25 lan.</x:v>
+      </x:c>
+      <x:c r="E124" s="75" t="str">
+        <x:v>Viewport desktop va 390x844; 25 health requests.</x:v>
+      </x:c>
+      <x:c r="F124" s="76" t="str">
+        <x:v>Khong co script/img trong canvas; overflow=false; console error rong; p95 duoi 100 ms.</x:v>
+      </x:c>
+      <x:c r="G124" s="75" t="str">
+        <x:v>Pass: renderedScriptInCanvas=0, mobile overflow=false, consoleErrors=[], health p95=1.59 ms.</x:v>
+      </x:c>
+      <x:c r="H124" s="75" t="str">
+        <x:v>TC_VIZI_115</x:v>
+      </x:c>
+      <x:c r="I124" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J124" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K124" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L124" s="75"/>
+      <x:c r="M124" s="75"/>
+      <x:c r="N124" s="75"/>
+      <x:c r="O124" s="75"/>
       <x:c r="P124" s="75" t="n"/>
       <x:c r="Q124" s="75" t="n"/>
       <x:c r="R124" s="75" t="n"/>
@@ -7669,21 +7885,46 @@
       <x:c r="Z124" s="75" t="n"/>
     </x:row>
     <x:row r="125" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A125" s="75" t="n"/>
-      <x:c r="B125" s="76" t="n"/>
-      <x:c r="C125" s="75" t="n"/>
-      <x:c r="D125" s="75" t="n"/>
-      <x:c r="E125" s="75" t="n"/>
-      <x:c r="F125" s="76" t="n"/>
-      <x:c r="G125" s="75" t="n"/>
-      <x:c r="H125" s="75" t="n"/>
-      <x:c r="I125" s="75" t="n"/>
-      <x:c r="J125" s="75" t="n"/>
-      <x:c r="K125" s="75" t="n"/>
-      <x:c r="L125" s="75" t="n"/>
-      <x:c r="M125" s="75" t="n"/>
-      <x:c r="N125" s="75" t="n"/>
-      <x:c r="O125" s="75" t="n"/>
+      <x:c r="A125" s="75" t="str">
+        <x:v>TC_VIZI_117</x:v>
+      </x:c>
+      <x:c r="B125" s="76" t="str">
+        <x:v>Security scan, cleanup va staged diff buoc 36</x:v>
+      </x:c>
+      <x:c r="C125" s="75" t="str">
+        <x:v>Kiem tra khong co raw HTML/wildcard CORS/secret; xoa QA data va khong stage file agent/log.</x:v>
+      </x:c>
+      <x:c r="D125" s="75" t="str">
+        <x:v>B1: Xoa design/user/template smoke.
+B2: Stop BE/FE.
+B3: Chay security rg va git diff --check.
+B4: Scan staged files.</x:v>
+      </x:c>
+      <x:c r="E125" s="75" t="str">
+        <x:v>backend, frontend, Template_TestCase.xlsx, staged diff.</x:v>
+      </x:c>
+      <x:c r="F125" s="76" t="str">
+        <x:v>Khong co secret/thong tin ca nhan; khong stage .agents/.codex-work/.env/log.</x:v>
+      </x:c>
+      <x:c r="G125" s="75" t="str">
+        <x:v>Pass sau vong verify cuoi truoc commit.</x:v>
+      </x:c>
+      <x:c r="H125" s="75" t="str">
+        <x:v>TC_VIZI_110</x:v>
+      </x:c>
+      <x:c r="I125" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J125" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K125" s="75" t="str">
+        <x:v>Bước 36</x:v>
+      </x:c>
+      <x:c r="L125" s="75"/>
+      <x:c r="M125" s="75"/>
+      <x:c r="N125" s="75"/>
+      <x:c r="O125" s="75"/>
       <x:c r="P125" s="75" t="n"/>
       <x:c r="Q125" s="75" t="n"/>
       <x:c r="R125" s="75" t="n"/>
@@ -32245,7 +32486,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51eb3e20601b4e2d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec08c99b8c664094"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Persist design save snapshots
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R2053ee2117f144ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rd774792a332d4fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R3c7e7fda04a14a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R9ac9b2436bd14c02"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>124</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>126</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -8408,21 +8408,45 @@
       <x:c r="Z134" s="75" t="n"/>
     </x:row>
     <x:row r="135" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A135" s="75" t="n"/>
-      <x:c r="B135" s="76" t="n"/>
-      <x:c r="C135" s="75" t="n"/>
-      <x:c r="D135" s="75" t="n"/>
-      <x:c r="E135" s="75" t="n"/>
-      <x:c r="F135" s="76" t="n"/>
-      <x:c r="G135" s="75" t="n"/>
-      <x:c r="H135" s="75" t="n"/>
-      <x:c r="I135" s="75" t="n"/>
-      <x:c r="J135" s="75" t="n"/>
-      <x:c r="K135" s="75" t="n"/>
-      <x:c r="L135" s="75" t="n"/>
-      <x:c r="M135" s="75" t="n"/>
-      <x:c r="N135" s="75" t="n"/>
-      <x:c r="O135" s="75" t="n"/>
+      <x:c r="A135" s="75" t="str">
+        <x:v>TC_VIZI_127</x:v>
+      </x:c>
+      <x:c r="B135" s="76" t="str">
+        <x:v>Entity va repository design snapshot</x:v>
+      </x:c>
+      <x:c r="C135" s="75" t="str">
+        <x:v>Backend map bang design_snapshots bang JPA entity va repository de luu lich su canvas.</x:v>
+      </x:c>
+      <x:c r="D135" s="75" t="str">
+        <x:v>B1: Them DesignSnapshot entity.
+B2: Them DesignSnapshotRepository.
+B3: Compile backend.</x:v>
+      </x:c>
+      <x:c r="E135" s="75" t="str">
+        <x:v>Bang design_snapshots trong migration V1.</x:v>
+      </x:c>
+      <x:c r="F135" s="76" t="str">
+        <x:v>JPA context load duoc repository moi va schema hien tai khong can migration moi.</x:v>
+      </x:c>
+      <x:c r="G135" s="75" t="str">
+        <x:v>Pass: full backend compile va context tests load 4 repositories.</x:v>
+      </x:c>
+      <x:c r="H135" s="75" t="str">
+        <x:v>TC_VIZI_022</x:v>
+      </x:c>
+      <x:c r="I135" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J135" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K135" s="75" t="str">
+        <x:v>Bước 38</x:v>
+      </x:c>
+      <x:c r="L135" s="75"/>
+      <x:c r="M135" s="75"/>
+      <x:c r="N135" s="75"/>
+      <x:c r="O135" s="75"/>
       <x:c r="P135" s="75" t="n"/>
       <x:c r="Q135" s="75" t="n"/>
       <x:c r="R135" s="75" t="n"/>
@@ -8436,21 +8460,45 @@
       <x:c r="Z135" s="75" t="n"/>
     </x:row>
     <x:row r="136" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A136" s="75" t="n"/>
-      <x:c r="B136" s="76" t="n"/>
-      <x:c r="C136" s="75" t="n"/>
-      <x:c r="D136" s="75" t="n"/>
-      <x:c r="E136" s="75" t="n"/>
-      <x:c r="F136" s="76" t="n"/>
-      <x:c r="G136" s="75" t="n"/>
-      <x:c r="H136" s="75" t="n"/>
-      <x:c r="I136" s="75" t="n"/>
-      <x:c r="J136" s="75" t="n"/>
-      <x:c r="K136" s="75" t="n"/>
-      <x:c r="L136" s="75" t="n"/>
-      <x:c r="M136" s="75" t="n"/>
-      <x:c r="N136" s="75" t="n"/>
-      <x:c r="O136" s="75" t="n"/>
+      <x:c r="A136" s="75" t="str">
+        <x:v>TC_VIZI_128</x:v>
+      </x:c>
+      <x:c r="B136" s="76" t="str">
+        <x:v>Save draft tao snapshot</x:v>
+      </x:c>
+      <x:c r="C136" s="75" t="str">
+        <x:v>Moi lan PUT /api/designs/{id} thanh cong phai luu snapshot canvas voi reason save.</x:v>
+      </x:c>
+      <x:c r="D136" s="75" t="str">
+        <x:v>B1: Owner tao draft tu template.
+B2: PUT canvas moi.
+B3: Doc design_snapshots theo design_id.</x:v>
+      </x:c>
+      <x:c r="E136" s="75" t="str">
+        <x:v>Canvas co text Saved Studio.</x:v>
+      </x:c>
+      <x:c r="F136" s="76" t="str">
+        <x:v>Co 1 snapshot; reason=save; canvas_json trong snapshot co text Saved Studio.</x:v>
+      </x:c>
+      <x:c r="G136" s="75" t="str">
+        <x:v>Pass: DesignApiIntegrationTests xac nhan snapshot size=1, reason=save va canvas dung.</x:v>
+      </x:c>
+      <x:c r="H136" s="75" t="str">
+        <x:v>TC_VIZI_033</x:v>
+      </x:c>
+      <x:c r="I136" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J136" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K136" s="75" t="str">
+        <x:v>Bước 38</x:v>
+      </x:c>
+      <x:c r="L136" s="75"/>
+      <x:c r="M136" s="75"/>
+      <x:c r="N136" s="75"/>
+      <x:c r="O136" s="75"/>
       <x:c r="P136" s="75" t="n"/>
       <x:c r="Q136" s="75" t="n"/>
       <x:c r="R136" s="75" t="n"/>
@@ -8464,21 +8512,45 @@
       <x:c r="Z136" s="75" t="n"/>
     </x:row>
     <x:row r="137" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A137" s="75" t="n"/>
-      <x:c r="B137" s="76" t="n"/>
-      <x:c r="C137" s="75" t="n"/>
-      <x:c r="D137" s="75" t="n"/>
-      <x:c r="E137" s="75" t="n"/>
-      <x:c r="F137" s="76" t="n"/>
-      <x:c r="G137" s="75" t="n"/>
-      <x:c r="H137" s="75" t="n"/>
-      <x:c r="I137" s="75" t="n"/>
-      <x:c r="J137" s="75" t="n"/>
-      <x:c r="K137" s="75" t="n"/>
-      <x:c r="L137" s="75" t="n"/>
-      <x:c r="M137" s="75" t="n"/>
-      <x:c r="N137" s="75" t="n"/>
-      <x:c r="O137" s="75" t="n"/>
+      <x:c r="A137" s="75" t="str">
+        <x:v>TC_VIZI_129</x:v>
+      </x:c>
+      <x:c r="B137" s="76" t="str">
+        <x:v>Invalid canvas khong tao snapshot</x:v>
+      </x:c>
+      <x:c r="C137" s="75" t="str">
+        <x:v>Neu save bi reject do canvas JSON sai schema, backend khong duoc tao snapshot moi.</x:v>
+      </x:c>
+      <x:c r="D137" s="75" t="str">
+        <x:v>B1: Owner tao draft.
+B2: PUT canvasJson = {}.
+B3: Doc lai design va count snapshot.</x:v>
+      </x:c>
+      <x:c r="E137" s="75" t="str">
+        <x:v>canvasJson invalid thieu layers.</x:v>
+      </x:c>
+      <x:c r="F137" s="76" t="str">
+        <x:v>HTTP 400; design giu canvas cu; snapshot count = 0.</x:v>
+      </x:c>
+      <x:c r="G137" s="75" t="str">
+        <x:v>Pass: invalid canvas tra 400, content cu con nguyen, snapshot count zero.</x:v>
+      </x:c>
+      <x:c r="H137" s="75" t="str">
+        <x:v>TC_VIZI_128</x:v>
+      </x:c>
+      <x:c r="I137" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J137" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K137" s="75" t="str">
+        <x:v>Bước 38</x:v>
+      </x:c>
+      <x:c r="L137" s="75"/>
+      <x:c r="M137" s="75"/>
+      <x:c r="N137" s="75"/>
+      <x:c r="O137" s="75"/>
       <x:c r="P137" s="75" t="n"/>
       <x:c r="Q137" s="75" t="n"/>
       <x:c r="R137" s="75" t="n"/>
@@ -8492,21 +8564,46 @@
       <x:c r="Z137" s="75" t="n"/>
     </x:row>
     <x:row r="138" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A138" s="75" t="n"/>
-      <x:c r="B138" s="76" t="n"/>
-      <x:c r="C138" s="75" t="n"/>
-      <x:c r="D138" s="75" t="n"/>
-      <x:c r="E138" s="75" t="n"/>
-      <x:c r="F138" s="76" t="n"/>
-      <x:c r="G138" s="75" t="n"/>
-      <x:c r="H138" s="75" t="n"/>
-      <x:c r="I138" s="75" t="n"/>
-      <x:c r="J138" s="75" t="n"/>
-      <x:c r="K138" s="75" t="n"/>
-      <x:c r="L138" s="75" t="n"/>
-      <x:c r="M138" s="75" t="n"/>
-      <x:c r="N138" s="75" t="n"/>
-      <x:c r="O138" s="75" t="n"/>
+      <x:c r="A138" s="75" t="str">
+        <x:v>TC_VIZI_130</x:v>
+      </x:c>
+      <x:c r="B138" s="76" t="str">
+        <x:v>Delete draft xoa cascade snapshot</x:v>
+      </x:c>
+      <x:c r="C138" s="75" t="str">
+        <x:v>Khi draft co snapshot bi xoa, snapshot lien quan phai bien mat theo FK cascade.</x:v>
+      </x:c>
+      <x:c r="D138" s="75" t="str">
+        <x:v>B1: Owner tao draft.
+B2: PUT de tao snapshot.
+B3: DELETE design.
+B4: Count snapshot theo design_id.</x:v>
+      </x:c>
+      <x:c r="E138" s="75" t="str">
+        <x:v>Draft co 1 snapshot truoc khi delete.</x:v>
+      </x:c>
+      <x:c r="F138" s="76" t="str">
+        <x:v>Owner DELETE tra 204; GET design tra 404; snapshot count = 0.</x:v>
+      </x:c>
+      <x:c r="G138" s="75" t="str">
+        <x:v>Pass: before delete snapshot count=1, after owner delete snapshot count=0.</x:v>
+      </x:c>
+      <x:c r="H138" s="75" t="str">
+        <x:v>TC_VIZI_118</x:v>
+      </x:c>
+      <x:c r="I138" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J138" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K138" s="75" t="str">
+        <x:v>Bước 38</x:v>
+      </x:c>
+      <x:c r="L138" s="75"/>
+      <x:c r="M138" s="75"/>
+      <x:c r="N138" s="75"/>
+      <x:c r="O138" s="75"/>
       <x:c r="P138" s="75" t="n"/>
       <x:c r="Q138" s="75" t="n"/>
       <x:c r="R138" s="75" t="n"/>
@@ -8520,21 +8617,44 @@
       <x:c r="Z138" s="75" t="n"/>
     </x:row>
     <x:row r="139" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A139" s="75" t="n"/>
-      <x:c r="B139" s="76" t="n"/>
-      <x:c r="C139" s="75" t="n"/>
-      <x:c r="D139" s="75" t="n"/>
-      <x:c r="E139" s="75" t="n"/>
-      <x:c r="F139" s="76" t="n"/>
-      <x:c r="G139" s="75" t="n"/>
-      <x:c r="H139" s="75" t="n"/>
-      <x:c r="I139" s="75" t="n"/>
-      <x:c r="J139" s="75" t="n"/>
-      <x:c r="K139" s="75" t="n"/>
-      <x:c r="L139" s="75" t="n"/>
-      <x:c r="M139" s="75" t="n"/>
-      <x:c r="N139" s="75" t="n"/>
-      <x:c r="O139" s="75" t="n"/>
+      <x:c r="A139" s="75" t="str">
+        <x:v>TC_VIZI_131</x:v>
+      </x:c>
+      <x:c r="B139" s="76" t="str">
+        <x:v>Regression backend sau snapshot</x:v>
+      </x:c>
+      <x:c r="C139" s="75" t="str">
+        <x:v>Chay full backend suite sau khi them DesignSnapshot entity va ghi snapshot khi save.</x:v>
+      </x:c>
+      <x:c r="D139" s="75" t="str">
+        <x:v>B1: Chay .\mvnw.cmd -Dtest=DesignApiIntegrationTests test.
+B2: Chay .\mvnw.cmd test.</x:v>
+      </x:c>
+      <x:c r="E139" s="75" t="str">
+        <x:v>Backend Maven test suite voi PostgreSQL local.</x:v>
+      </x:c>
+      <x:c r="F139" s="76" t="str">
+        <x:v>Khong co failure/error/skip.</x:v>
+      </x:c>
+      <x:c r="G139" s="75" t="str">
+        <x:v>Pass: DesignApiIntegrationTests 7/0/0/0; full backend 28/0/0/0.</x:v>
+      </x:c>
+      <x:c r="H139" s="75" t="str">
+        <x:v>TC_VIZI_127</x:v>
+      </x:c>
+      <x:c r="I139" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J139" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K139" s="75" t="str">
+        <x:v>Bước 38</x:v>
+      </x:c>
+      <x:c r="L139" s="75"/>
+      <x:c r="M139" s="75"/>
+      <x:c r="N139" s="75"/>
+      <x:c r="O139" s="75"/>
       <x:c r="P139" s="75" t="n"/>
       <x:c r="Q139" s="75" t="n"/>
       <x:c r="R139" s="75" t="n"/>
@@ -8548,21 +8668,45 @@
       <x:c r="Z139" s="75" t="n"/>
     </x:row>
     <x:row r="140" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A140" s="75" t="n"/>
-      <x:c r="B140" s="76" t="n"/>
-      <x:c r="C140" s="75" t="n"/>
-      <x:c r="D140" s="75" t="n"/>
-      <x:c r="E140" s="75" t="n"/>
-      <x:c r="F140" s="76" t="n"/>
-      <x:c r="G140" s="75" t="n"/>
-      <x:c r="H140" s="75" t="n"/>
-      <x:c r="I140" s="75" t="n"/>
-      <x:c r="J140" s="75" t="n"/>
-      <x:c r="K140" s="75" t="n"/>
-      <x:c r="L140" s="75" t="n"/>
-      <x:c r="M140" s="75" t="n"/>
-      <x:c r="N140" s="75" t="n"/>
-      <x:c r="O140" s="75" t="n"/>
+      <x:c r="A140" s="75" t="str">
+        <x:v>TC_VIZI_132</x:v>
+      </x:c>
+      <x:c r="B140" s="76" t="str">
+        <x:v>Build FE va security scan buoc 38</x:v>
+      </x:c>
+      <x:c r="C140" s="75" t="str">
+        <x:v>Doi backend snapshot khong pha FE build va staged diff khong co secret/agent file.</x:v>
+      </x:c>
+      <x:c r="D140" s="75" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Chay security grep.
+B3: Chay git diff --check va scan staged files.</x:v>
+      </x:c>
+      <x:c r="E140" s="75" t="str">
+        <x:v>frontend build, backend/src, frontend/src, staged diff.</x:v>
+      </x:c>
+      <x:c r="F140" s="76" t="str">
+        <x:v>FE build pass; khong raw HTML/wildcard CORS/secret; khong stage .agents/.codex-work/.env/log.</x:v>
+      </x:c>
+      <x:c r="G140" s="75" t="str">
+        <x:v>Pass: vue-tsc va Vite pass; security scan chi co hit benign trong test/env docs.</x:v>
+      </x:c>
+      <x:c r="H140" s="75" t="str">
+        <x:v>TC_VIZI_131</x:v>
+      </x:c>
+      <x:c r="I140" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J140" s="75" t="n">
+        <x:v>46209</x:v>
+      </x:c>
+      <x:c r="K140" s="75" t="str">
+        <x:v>Bước 38</x:v>
+      </x:c>
+      <x:c r="L140" s="75"/>
+      <x:c r="M140" s="75"/>
+      <x:c r="N140" s="75"/>
+      <x:c r="O140" s="75"/>
       <x:c r="P140" s="75" t="n"/>
       <x:c r="Q140" s="75" t="n"/>
       <x:c r="R140" s="75" t="n"/>
@@ -32704,7 +32848,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e5c543266a346d0"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378fe59e46ef4588"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Require sign-in before draft creation
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R3c7e7fda04a14a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R9ac9b2436bd14c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R125fafe4c11c4276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R456b3cafd5044b01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>130</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>132</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -8720,17 +8720,44 @@
       <x:c r="Z140" s="75" t="n"/>
     </x:row>
     <x:row r="141" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A141" s="75" t="n"/>
-      <x:c r="B141" s="76" t="n"/>
-      <x:c r="C141" s="75" t="n"/>
-      <x:c r="D141" s="75" t="n"/>
-      <x:c r="E141" s="75" t="n"/>
-      <x:c r="F141" s="76" t="n"/>
-      <x:c r="G141" s="75" t="n"/>
-      <x:c r="H141" s="75" t="n"/>
-      <x:c r="I141" s="75" t="n"/>
-      <x:c r="J141" s="75" t="n"/>
-      <x:c r="K141" s="75" t="n"/>
+      <x:c r="A141" s="75" t="str">
+        <x:v>TC_VIZI_133</x:v>
+      </x:c>
+      <x:c r="B141" s="76" t="str">
+        <x:v>Bat buoc dang nhap truoc khi tao draft</x:v>
+      </x:c>
+      <x:c r="C141" s="75" t="str">
+        <x:v>Khi nguoi dung anonymous muon tao/save draft tu template, FE phai chuyen sang account truoc; login/register xong quay lai template moi tao draft.</x:v>
+      </x:c>
+      <x:c r="D141" s="75" t="str">
+        <x:v>B1: Mo /templates/12 khi chua dang nhap.
+B2: Bam Save draft.
+B3: Kiem tra URL chuyen sang /account?redirect=/templates/12.
+B4: Tao account/login.
+B5: Kiem tra quay lai /templates/12.
+B6: Bam Save draft va doc status.</x:v>
+      </x:c>
+      <x:c r="E141" s="75" t="str">
+        <x:v>Template #12; user test step39-*@example.test.</x:v>
+      </x:c>
+      <x:c r="F141" s="76" t="str">
+        <x:v>Anonymous khong tao draft truc tiep; FE bat dang nhap truoc; sau auth quay lai template va tao draft thanh cong.</x:v>
+      </x:c>
+      <x:c r="G141" s="75" t="str">
+        <x:v>Pass: Browser smoke redirect dung, quay lai /templates/12, hien Draft #6 saved, consoleIssues=[]; API anonymous POST /api/designs/from-template/12 tra 401; data test da don.</x:v>
+      </x:c>
+      <x:c r="H141" s="75" t="str">
+        <x:v>TC_VIZI_102; TC_VIZI_126</x:v>
+      </x:c>
+      <x:c r="I141" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J141" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K141" s="75" t="str">
+        <x:v>Bước 39</x:v>
+      </x:c>
       <x:c r="L141" s="75" t="n"/>
       <x:c r="M141" s="75" t="n"/>
       <x:c r="N141" s="75" t="n"/>
@@ -32848,7 +32875,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378fe59e46ef4588"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21190bb60e2a4d58"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Record home route verification
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R125fafe4c11c4276"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R456b3cafd5044b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Ra5d6d2cf88e74330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R6e23f40ddd904422"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>131</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1176,7 +1176,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>133</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -8775,17 +8775,43 @@
       <x:c r="Z141" s="75" t="n"/>
     </x:row>
     <x:row r="142" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A142" s="75" t="n"/>
-      <x:c r="B142" s="76" t="n"/>
-      <x:c r="C142" s="75" t="n"/>
-      <x:c r="D142" s="75" t="n"/>
-      <x:c r="E142" s="75" t="n"/>
-      <x:c r="F142" s="76" t="n"/>
-      <x:c r="G142" s="75" t="n"/>
-      <x:c r="H142" s="75" t="n"/>
-      <x:c r="I142" s="75" t="n"/>
-      <x:c r="J142" s="75" t="n"/>
-      <x:c r="K142" s="75" t="n"/>
+      <x:c r="A142" s="75" t="str">
+        <x:v>TC_VIZI_134</x:v>
+      </x:c>
+      <x:c r="B142" s="76" t="str">
+        <x:v>Route Home vao duoc</x:v>
+      </x:c>
+      <x:c r="C142" s="75" t="str">
+        <x:v>Xac nhan route Home `/` render dung man hinh dau tien, goi backend health/templates va co the di sang template detail.</x:v>
+      </x:c>
+      <x:c r="D142" s="75" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Mo http://127.0.0.1:5173/.
+B3: Cho status Backend vizi-backend: UP.
+B4: Kiem tra noi dung Home va template card.
+B5: Click template card.</x:v>
+      </x:c>
+      <x:c r="E142" s="75" t="str">
+        <x:v>Local FE 127.0.0.1:5173; BE 127.0.0.1:8080; template #12.</x:v>
+      </x:c>
+      <x:c r="F142" s="76" t="str">
+        <x:v>URL `/` hien Home khong blank/overlay; backend status UP; co template card; click card vao `/templates/12`; console khong co warning/error.</x:v>
+      </x:c>
+      <x:c r="G142" s="75" t="str">
+        <x:v>Pass: npm run build pass; browser smoke homeOk=true, overlayOk=true, cardCount=1, href=/templates/12, detailLoaded=true, consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H142" s="75" t="str">
+        <x:v>TC_VIZI_038; TC_VIZI_039</x:v>
+      </x:c>
+      <x:c r="I142" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J142" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K142" s="75" t="str">
+        <x:v>Bước 40</x:v>
+      </x:c>
       <x:c r="L142" s="75" t="n"/>
       <x:c r="M142" s="75" t="n"/>
       <x:c r="N142" s="75" t="n"/>
@@ -32875,7 +32901,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21190bb60e2a4d58"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2fb725ee6e4756"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor route for drafts
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re4ae86f729e24b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R2f554f69c1bb47a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R0ec4c3f585764be2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rdb8ac71171d042e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>133</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>135</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -8888,17 +8888,42 @@
       <x:c r="Z143" s="75" t="n"/>
     </x:row>
     <x:row r="144" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A144" s="75" t="n"/>
-      <x:c r="B144" s="76" t="n"/>
-      <x:c r="C144" s="75" t="n"/>
-      <x:c r="D144" s="75" t="n"/>
-      <x:c r="E144" s="75" t="n"/>
-      <x:c r="F144" s="76" t="n"/>
-      <x:c r="G144" s="75" t="n"/>
-      <x:c r="H144" s="75" t="n"/>
-      <x:c r="I144" s="75" t="n"/>
-      <x:c r="J144" s="75" t="n"/>
-      <x:c r="K144" s="75" t="n"/>
+      <x:c r="A144" s="75" t="str">
+        <x:v>TC_VIZI_136</x:v>
+      </x:c>
+      <x:c r="B144" s="76" t="str">
+        <x:v>Route Editor load dung draft</x:v>
+      </x:c>
+      <x:c r="C144" s="75" t="str">
+        <x:v>Xac nhan route /editor/:designId ton tai, dung component draft detail hien co va load design bang designId.</x:v>
+      </x:c>
+      <x:c r="D144" s="75" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Chay Vite dev server tam thoi.
+B3: Goi /editor/1 va /designs/1 bang HTTP smoke.
+B4: Kiem tra router source va link tu draft/template sang editor.</x:v>
+      </x:c>
+      <x:c r="E144" s="75" t="str">
+        <x:v>Local FE 127.0.0.1:5174; route /editor/1; source router/views.</x:v>
+      </x:c>
+      <x:c r="F144" s="76" t="str">
+        <x:v>/editor/:designId tra app shell 200; router co name editor; draft list va template saved link tro den editor.</x:v>
+      </x:c>
+      <x:c r="G144" s="75" t="str">
+        <x:v>Pass: npm run build pass; HTTP /editor/1=200 va /designs/1=200; source check thay route editor, DesignsView link designId, TemplateDetail Open editor.</x:v>
+      </x:c>
+      <x:c r="H144" s="75" t="str">
+        <x:v>TC_VIZI_135</x:v>
+      </x:c>
+      <x:c r="I144" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J144" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K144" s="75" t="str">
+        <x:v>Buoc 42A</x:v>
+      </x:c>
       <x:c r="L144" s="75" t="n"/>
       <x:c r="M144" s="75" t="n"/>
       <x:c r="N144" s="75" t="n"/>
@@ -32932,7 +32957,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R975a9844fe6a4aee"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9272a61d2464055"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Extract shared canvas preview
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R0ec4c3f585764be2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rdb8ac71171d042e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R13483daa54fa43a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rdb5f373ee0674446"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>136</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -8941,21 +8941,45 @@
       <x:c r="Z144" s="75" t="n"/>
     </x:row>
     <x:row r="145" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A145" s="75" t="n"/>
-      <x:c r="B145" s="76" t="n"/>
-      <x:c r="C145" s="75" t="n"/>
-      <x:c r="D145" s="75" t="n"/>
-      <x:c r="E145" s="75" t="n"/>
-      <x:c r="F145" s="76" t="n"/>
-      <x:c r="G145" s="75" t="n"/>
-      <x:c r="H145" s="75" t="n"/>
-      <x:c r="I145" s="75" t="n"/>
-      <x:c r="J145" s="75" t="n"/>
-      <x:c r="K145" s="75" t="n"/>
-      <x:c r="L145" s="75" t="n"/>
-      <x:c r="M145" s="75" t="n"/>
-      <x:c r="N145" s="75" t="n"/>
-      <x:c r="O145" s="75" t="n"/>
+      <x:c r="A145" s="75" t="str">
+        <x:v>TC_VIZI_137</x:v>
+      </x:c>
+      <x:c r="B145" s="76" t="str">
+        <x:v>Canvas preview dùng chung</x:v>
+      </x:c>
+      <x:c r="C145" s="75" t="str">
+        <x:v>Xác minh template và editor dùng chung canvas renderer, text scale theo khổ card</x:v>
+      </x:c>
+      <x:c r="D145" s="75" t="str">
+        <x:v>Frontend và backend local đang chạy; template 12 có 3 layers</x:v>
+      </x:c>
+      <x:c r="E145" s="75" t="str">
+        <x:v>1. Mở /templates/12
+2. Nhập Shared canvas renderer
+3. Kiểm tra desktop và mobile 390x844</x:v>
+      </x:c>
+      <x:c r="F145" s="76" t="str">
+        <x:v>Canvas render 3 layers, giữ tỷ lệ 90/54, text cập nhật tức thời, không clipping hoặc tràn ngang</x:v>
+      </x:c>
+      <x:c r="G145" s="75" t="str">
+        <x:v>Canvas render 3 layers; text cập nhật; mobile font 10.50px, scrollHeight=clientHeight=29; không tràn ngang; console 0 lỗi</x:v>
+      </x:c>
+      <x:c r="H145" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I145" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J145" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K145" s="75" t="str">
+        <x:v>Build, source scan, Playwright desktop/mobile</x:v>
+      </x:c>
+      <x:c r="L145" s="75"/>
+      <x:c r="M145" s="75"/>
+      <x:c r="N145" s="75"/>
+      <x:c r="O145" s="75"/>
       <x:c r="P145" s="75" t="n"/>
       <x:c r="Q145" s="75" t="n"/>
       <x:c r="R145" s="75" t="n"/>
@@ -32957,7 +32981,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9272a61d2464055"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe01a718030c4b0a"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add three-panel editor shell
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R13483daa54fa43a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rdb5f373ee0674446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R35435cbf15e44782"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R035db5e1428546da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>135</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>137</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -8993,21 +8993,47 @@
       <x:c r="Z145" s="75" t="n"/>
     </x:row>
     <x:row r="146" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A146" s="75" t="n"/>
-      <x:c r="B146" s="76" t="n"/>
-      <x:c r="C146" s="75" t="n"/>
-      <x:c r="D146" s="75" t="n"/>
-      <x:c r="E146" s="75" t="n"/>
-      <x:c r="F146" s="76" t="n"/>
-      <x:c r="G146" s="75" t="n"/>
-      <x:c r="H146" s="75" t="n"/>
-      <x:c r="I146" s="75" t="n"/>
-      <x:c r="J146" s="75" t="n"/>
-      <x:c r="K146" s="75" t="n"/>
-      <x:c r="L146" s="75" t="n"/>
-      <x:c r="M146" s="75" t="n"/>
-      <x:c r="N146" s="75" t="n"/>
-      <x:c r="O146" s="75" t="n"/>
+      <x:c r="A146" s="75" t="str">
+        <x:v>TC_VIZI_138</x:v>
+      </x:c>
+      <x:c r="B146" s="76" t="str">
+        <x:v>Editor shell ba vùng</x:v>
+      </x:c>
+      <x:c r="C146" s="75" t="str">
+        <x:v>Xác minh route editor có sidebar trái, canvas giữa và properties bên phải</x:v>
+      </x:c>
+      <x:c r="D146" s="75" t="str">
+        <x:v>Frontend và backend local đang chạy; tài khoản và draft QA tạm</x:v>
+      </x:c>
+      <x:c r="E146" s="75" t="str">
+        <x:v>1. Đăng nhập và mở draft từ My drafts
+2. Kiểm tra ba vùng editor
+3. Sửa text và save
+4. Kiểm tra desktop/mobile
+5. Xóa dữ liệu QA</x:v>
+      </x:c>
+      <x:c r="F146" s="76" t="str">
+        <x:v>Editor render đủ left/center/right; canvas cập nhật và save; desktop ba cột; mobile xếp dọc không tràn ngang</x:v>
+      </x:c>
+      <x:c r="G146" s="75" t="str">
+        <x:v>Pass: left=1, center=1, right=1; 3 layers; ratio 90/54; text save thành công; mobile 390x844 overflow=0; dữ liệu QA đã dọn</x:v>
+      </x:c>
+      <x:c r="H146" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I146" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J146" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K146" s="75" t="str">
+        <x:v>Build, Playwright desktop/mobile, API save/delete, DB readback</x:v>
+      </x:c>
+      <x:c r="L146" s="75"/>
+      <x:c r="M146" s="75"/>
+      <x:c r="N146" s="75"/>
+      <x:c r="O146" s="75"/>
       <x:c r="P146" s="75" t="n"/>
       <x:c r="Q146" s="75" t="n"/>
       <x:c r="R146" s="75" t="n"/>
@@ -32981,7 +33007,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe01a718030c4b0a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fbc5664e1b04f34"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add floating editor toolbar
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R35435cbf15e44782"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R035db5e1428546da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re37dc23338674404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5b900ab76faa49cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>136</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>138</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -9047,21 +9047,46 @@
       <x:c r="Z146" s="75" t="n"/>
     </x:row>
     <x:row r="147" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A147" s="75" t="n"/>
-      <x:c r="B147" s="76" t="n"/>
-      <x:c r="C147" s="75" t="n"/>
-      <x:c r="D147" s="75" t="n"/>
-      <x:c r="E147" s="75" t="n"/>
-      <x:c r="F147" s="76" t="n"/>
-      <x:c r="G147" s="75" t="n"/>
-      <x:c r="H147" s="75" t="n"/>
-      <x:c r="I147" s="75" t="n"/>
-      <x:c r="J147" s="75" t="n"/>
-      <x:c r="K147" s="75" t="n"/>
-      <x:c r="L147" s="75" t="n"/>
-      <x:c r="M147" s="75" t="n"/>
-      <x:c r="N147" s="75" t="n"/>
-      <x:c r="O147" s="75" t="n"/>
+      <x:c r="A147" s="75" t="str">
+        <x:v>TC_VIZI_139</x:v>
+      </x:c>
+      <x:c r="B147" s="76" t="str">
+        <x:v>Floating toolbar ban dau</x:v>
+      </x:c>
+      <x:c r="C147" s="75" t="str">
+        <x:v>Xac minh editor hien thi toolbar noi voi Select, Text, Shape, Image, QR va Icon</x:v>
+      </x:c>
+      <x:c r="D147" s="75" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E147" s="75" t="str">
+        <x:v>1. Dang nhap va mo draft tu My drafts
+2. Kiem tra toolbar noi tren canvas
+3. Kiem tra desktop va mobile 390x844
+4. Xoa du lieu QA</x:v>
+      </x:c>
+      <x:c r="F147" s="76" t="str">
+        <x:v>Toolbar co 6 cong cu dung nhan, nam trong workspace, khong che canvas, mobile khong tran ngang</x:v>
+      </x:c>
+      <x:c r="G147" s="75" t="str">
+        <x:v>Pass: buttonCount=6, labels Select/Text/Shape/Image/QR/Icon; role toolbar; toolbarAboveCanvas=true; mobile overflow=0; toolbarFullyVisible=true; du lieu QA da don</x:v>
+      </x:c>
+      <x:c r="H147" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I147" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J147" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K147" s="75" t="str">
+        <x:v>Build, Playwright desktop/mobile, DB readback</x:v>
+      </x:c>
+      <x:c r="L147" s="75"/>
+      <x:c r="M147" s="75"/>
+      <x:c r="N147" s="75"/>
+      <x:c r="O147" s="75"/>
       <x:c r="P147" s="75" t="n"/>
       <x:c r="Q147" s="75" t="n"/>
       <x:c r="R147" s="75" t="n"/>
@@ -33007,7 +33032,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fbc5664e1b04f34"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35e7361e757445d0"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add fixed editor page switch
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re37dc23338674404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5b900ab76faa49cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf9857fb6957e44d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R47f844cc5c514aaf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>137</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>139</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -9100,21 +9100,47 @@
       <x:c r="Z147" s="75" t="n"/>
     </x:row>
     <x:row r="148" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A148" s="75" t="n"/>
-      <x:c r="B148" s="76" t="n"/>
-      <x:c r="C148" s="75" t="n"/>
-      <x:c r="D148" s="75" t="n"/>
-      <x:c r="E148" s="75" t="n"/>
-      <x:c r="F148" s="76" t="n"/>
-      <x:c r="G148" s="75" t="n"/>
-      <x:c r="H148" s="75" t="n"/>
-      <x:c r="I148" s="75" t="n"/>
-      <x:c r="J148" s="75" t="n"/>
-      <x:c r="K148" s="75" t="n"/>
-      <x:c r="L148" s="75" t="n"/>
-      <x:c r="M148" s="75" t="n"/>
-      <x:c r="N148" s="75" t="n"/>
-      <x:c r="O148" s="75" t="n"/>
+      <x:c r="A148" s="75" t="str">
+        <x:v>TC_VIZI_140</x:v>
+      </x:c>
+      <x:c r="B148" s="76" t="str">
+        <x:v>Page switch Front Back co dinh</x:v>
+      </x:c>
+      <x:c r="C148" s="75" t="str">
+        <x:v>Xac minh editor chi co hai mat Front va Back, chuyen mat duoc va khong co nut them page</x:v>
+      </x:c>
+      <x:c r="D148" s="75" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E148" s="75" t="str">
+        <x:v>1. Dang nhap va mo draft editor
+2. Kiem tra Pages chi co Front/Back
+3. Chuyen Front -&gt; Back -&gt; Front
+4. Kiem tra desktop va mobile 390x844
+5. Xoa du lieu QA</x:v>
+      </x:c>
+      <x:c r="F148" s="76" t="str">
+        <x:v>Page switch co dung 2 nut Front/Back, khong co Add page; Front hien layers hien co, Back hien mat rong va properties cap nhat</x:v>
+      </x:c>
+      <x:c r="G148" s="75" t="str">
+        <x:v>Pass: pageCount=2, labels Front/Back, addButtonCount=0, Front layers=3, Back layers=0, Side property doi dung, mobile overflow=0, console error=0, du lieu QA da don</x:v>
+      </x:c>
+      <x:c r="H148" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I148" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J148" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K148" s="75" t="str">
+        <x:v>Build, Playwright desktop/mobile, DB readback</x:v>
+      </x:c>
+      <x:c r="L148" s="75"/>
+      <x:c r="M148" s="75"/>
+      <x:c r="N148" s="75"/>
+      <x:c r="O148" s="75"/>
       <x:c r="P148" s="75" t="n"/>
       <x:c r="Q148" s="75" t="n"/>
       <x:c r="R148" s="75" t="n"/>
@@ -33032,7 +33058,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35e7361e757445d0"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff54f8e35699467c"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Scale editor card from design size
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf9857fb6957e44d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R47f844cc5c514aaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf07e70cad39748d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rda250586a7514f17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>138</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>140</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -9154,21 +9154,47 @@
       <x:c r="Z148" s="75" t="n"/>
     </x:row>
     <x:row r="149" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A149" s="75" t="n"/>
-      <x:c r="B149" s="76" t="n"/>
-      <x:c r="C149" s="75" t="n"/>
-      <x:c r="D149" s="75" t="n"/>
-      <x:c r="E149" s="75" t="n"/>
-      <x:c r="F149" s="76" t="n"/>
-      <x:c r="G149" s="75" t="n"/>
-      <x:c r="H149" s="75" t="n"/>
-      <x:c r="I149" s="75" t="n"/>
-      <x:c r="J149" s="75" t="n"/>
-      <x:c r="K149" s="75" t="n"/>
-      <x:c r="L149" s="75" t="n"/>
-      <x:c r="M149" s="75" t="n"/>
-      <x:c r="N149" s="75" t="n"/>
-      <x:c r="O149" s="75" t="n"/>
+      <x:c r="A149" s="75" t="str">
+        <x:v>TC_VIZI_141</x:v>
+      </x:c>
+      <x:c r="B149" s="76" t="str">
+        <x:v>Card size theo widthMm heightMm</x:v>
+      </x:c>
+      <x:c r="C149" s="75" t="str">
+        <x:v>Xac minh card editor nam giua workspace va kich thuoc hien thi duoc tinh tu widthMm/heightMm</x:v>
+      </x:c>
+      <x:c r="D149" s="75" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E149" s="75" t="str">
+        <x:v>1. Dang nhap va mo draft editor
+2. Kiem tra CSS vars widthMm/heightMm
+3. Kiem tra wide desktop 1600x950 dat widthMm*8px
+4. Kiem tra mobile 390x844 co lai trong workspace
+5. Xoa du lieu QA</x:v>
+      </x:c>
+      <x:c r="F149" s="76" t="str">
+        <x:v>Card dung ti le 90/54, wide desktop dat width 720px tu 90mm, mobile co lai nhung van giu ratio va can giua</x:v>
+      </x:c>
+      <x:c r="G149" s="75" t="str">
+        <x:v>Pass: cssWidthMm=90, cssHeightMm=54, desktop width=720px, ratio=90/54, centerDelta&lt;=1, toolbarAboveCanvas=true, mobile overflow=0, du lieu QA da don</x:v>
+      </x:c>
+      <x:c r="H149" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I149" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J149" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K149" s="75" t="str">
+        <x:v>Build, Playwright desktop/mobile, DB readback</x:v>
+      </x:c>
+      <x:c r="L149" s="75"/>
+      <x:c r="M149" s="75"/>
+      <x:c r="N149" s="75"/>
+      <x:c r="O149" s="75"/>
       <x:c r="P149" s="75" t="n"/>
       <x:c r="Q149" s="75" t="n"/>
       <x:c r="R149" s="75" t="n"/>
@@ -33058,7 +33084,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff54f8e35699467c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4852edfcc5f14e52"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Record editor text save verification
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf07e70cad39748d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rda250586a7514f17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R21249d1b40734a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1ecd443029774c03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>139</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>141</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -9208,21 +9208,48 @@
       <x:c r="Z149" s="75" t="n"/>
     </x:row>
     <x:row r="150" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A150" s="75" t="n"/>
-      <x:c r="B150" s="76" t="n"/>
-      <x:c r="C150" s="75" t="n"/>
-      <x:c r="D150" s="75" t="n"/>
-      <x:c r="E150" s="75" t="n"/>
-      <x:c r="F150" s="76" t="n"/>
-      <x:c r="G150" s="75" t="n"/>
-      <x:c r="H150" s="75" t="n"/>
-      <x:c r="I150" s="75" t="n"/>
-      <x:c r="J150" s="75" t="n"/>
-      <x:c r="K150" s="75" t="n"/>
-      <x:c r="L150" s="75" t="n"/>
-      <x:c r="M150" s="75" t="n"/>
-      <x:c r="N150" s="75" t="n"/>
-      <x:c r="O150" s="75" t="n"/>
+      <x:c r="A150" s="75" t="str">
+        <x:v>TC_VIZI_142</x:v>
+      </x:c>
+      <x:c r="B150" s="76" t="str">
+        <x:v>Luu text edit qua design API</x:v>
+      </x:c>
+      <x:c r="C150" s="75" t="str">
+        <x:v>Xac minh editor luu noi dung text layer bang PUT /api/designs va reload van giu text da sua</x:v>
+      </x:c>
+      <x:c r="D150" s="75" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E150" s="75" t="str">
+        <x:v>1. Dang nhap va tao draft tu template
+2. Mo /editor/:designId
+3. Sua #editor-text-layer
+4. Bam Save draft
+5. Reload editor va doc API
+6. Kiem tra mobile 390x844 va cleanup QA</x:v>
+      </x:c>
+      <x:c r="F150" s="76" t="str">
+        <x:v>Text layer cap nhat tren canvas, save hien Draft saved, reload editor va API tra canvasJson co text moi</x:v>
+      </x:c>
+      <x:c r="G150" s="75" t="str">
+        <x:v>Pass: edited text=Editor saved text 42G, save status Draft #16 saved, reload UI/API giu text, mobile overflow=0, console error=0, DB cleanup users/designs=0</x:v>
+      </x:c>
+      <x:c r="H150" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I150" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J150" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K150" s="75" t="str">
+        <x:v>Build, Browser fallback, Playwright desktop/mobile/API, DB readback</x:v>
+      </x:c>
+      <x:c r="L150" s="75"/>
+      <x:c r="M150" s="75"/>
+      <x:c r="N150" s="75"/>
+      <x:c r="O150" s="75"/>
       <x:c r="P150" s="75" t="n"/>
       <x:c r="Q150" s="75" t="n"/>
       <x:c r="R150" s="75" t="n"/>
@@ -33084,7 +33111,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4852edfcc5f14e52"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b580de1c4e4c2a"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Record editor shell verification
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R21249d1b40734a1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1ecd443029774c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Refbeafd1a4e34e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R94b485d0e77445f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,7 +1163,7 @@
     </x:row>
     <x:row r="5" s="83" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="23" t="n">
-        <x:v>140</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -1180,7 +1180,7 @@
       </x:c>
       <x:c r="F5" s="91" t="n"/>
       <x:c r="G5" s="92" t="n">
-        <x:v>142</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="H5" s="93" t="n"/>
       <x:c r="I5" s="94" t="n"/>
@@ -9263,21 +9263,48 @@
       <x:c r="Z150" s="75" t="n"/>
     </x:row>
     <x:row r="151" s="83" customFormat="1" ht="12.75" customHeight="1">
-      <x:c r="A151" s="75" t="n"/>
-      <x:c r="B151" s="76" t="n"/>
-      <x:c r="C151" s="75" t="n"/>
-      <x:c r="D151" s="75" t="n"/>
-      <x:c r="E151" s="75" t="n"/>
-      <x:c r="F151" s="76" t="n"/>
-      <x:c r="G151" s="75" t="n"/>
-      <x:c r="H151" s="75" t="n"/>
-      <x:c r="I151" s="75" t="n"/>
-      <x:c r="J151" s="75" t="n"/>
-      <x:c r="K151" s="75" t="n"/>
-      <x:c r="L151" s="75" t="n"/>
-      <x:c r="M151" s="75" t="n"/>
-      <x:c r="N151" s="75" t="n"/>
-      <x:c r="O151" s="75" t="n"/>
+      <x:c r="A151" s="75" t="str">
+        <x:v>TC_VIZI_143</x:v>
+      </x:c>
+      <x:c r="B151" s="76" t="str">
+        <x:v>Verify editor shell</x:v>
+      </x:c>
+      <x:c r="C151" s="75" t="str">
+        <x:v>Xac minh editor shell tong the build pass, vao /editor/:designId khong loi console va cac vung chinh hoat dong</x:v>
+      </x:c>
+      <x:c r="D151" s="75" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E151" s="75" t="str">
+        <x:v>1. Chay npm run build
+2. Browser mo /editor/1 lay URL/title/console
+3. Playwright tao draft va mo /editor/:designId
+4. Kiem tra left/center/right, toolbar, Front/Back, canvas size
+5. Sua text, save, reload, API readback
+6. Kiem tra mobile va cleanup QA</x:v>
+      </x:c>
+      <x:c r="F151" s="76" t="str">
+        <x:v>Build pass; editor render day du shell, toolbar, page switch, save/reload duoc, desktop/mobile khong tran ngang va khong console error</x:v>
+      </x:c>
+      <x:c r="G151" s="75" t="str">
+        <x:v>Pass: build pass, Browser URL/title=Vizi va console=0, Playwright /editor/17 notBlank=true, shell 2 sidebars + workspace, 6 toolbar tools, Front/Back no Add page, ratio=90/54, save/reload/API giu text, mobile overflow=0, DB cleanup users/designs=0</x:v>
+      </x:c>
+      <x:c r="H151" s="75" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I151" s="75" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J151" s="75" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K151" s="75" t="str">
+        <x:v>Build, Browser URL/title/console, Playwright shell desktop/mobile/API, DB readback</x:v>
+      </x:c>
+      <x:c r="L151" s="75"/>
+      <x:c r="M151" s="75"/>
+      <x:c r="N151" s="75"/>
+      <x:c r="O151" s="75"/>
       <x:c r="P151" s="75" t="n"/>
       <x:c r="Q151" s="75" t="n"/>
       <x:c r="R151" s="75" t="n"/>
@@ -33111,7 +33138,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b580de1c4e4c2a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd7edd8252d1425b"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor toolbar active tool state
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R445fbf0910ab48c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R052146fa50334b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R64aa9f795ed94d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rfed02493e4aa4731"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>142</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -4479,7 +4479,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>144</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -11749,17 +11749,44 @@
       <x:c r="Z152" s="5"/>
     </x:row>
     <x:row r="153">
-      <x:c r="A153" s="5"/>
-      <x:c r="B153" s="39"/>
-      <x:c r="C153" s="5"/>
-      <x:c r="D153" s="5"/>
-      <x:c r="E153" s="5"/>
-      <x:c r="F153" s="39"/>
-      <x:c r="G153" s="5"/>
-      <x:c r="H153" s="5"/>
-      <x:c r="I153" s="5"/>
-      <x:c r="J153" s="5"/>
-      <x:c r="K153" s="5"/>
+      <x:c r="A153" s="5" t="str">
+        <x:v>TC_VIZI_145</x:v>
+      </x:c>
+      <x:c r="B153" s="39" t="str">
+        <x:v>Floating toolbar tool state 56B</x:v>
+      </x:c>
+      <x:c r="C153" s="5" t="str">
+        <x:v>Xac minh toolbar editor co state chon tool cho Select, Text, Shape, Image, QR va Icon</x:v>
+      </x:c>
+      <x:c r="D153" s="5" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E153" s="5" t="str">
+        <x:v>1. Chay npm run build
+2. Browser mo /editor/1 lay URL/title/console
+3. Playwright tao draft va mo /editor/:designId
+4. Kiem tra mac dinh Select active
+5. Click lan luot Select/Text/Shape/Image/QR/Icon
+6. Kiem tra aria-pressed, class active, Properties Tool, Front/Back, mobile va cleanup QA</x:v>
+      </x:c>
+      <x:c r="F153" s="39" t="str">
+        <x:v>Toolbar co dung mot active tool; moi tool click duoc va Properties Tool cap nhat dung tren desktop/mobile</x:v>
+      </x:c>
+      <x:c r="G153" s="5" t="str">
+        <x:v>Pass: build pass; Browser URL/title=Vizi console=0, DOM snapshot fallback do incrementalAriaSnapshot; Playwright /editor/20 mac dinh Select active, click du 6 tool cap nhat aria/class/Properties Tool, Shape giu active qua Front/Back, mobile Icon active, overflow=0, console error=0, DB cleanup users/designs=0</x:v>
+      </x:c>
+      <x:c r="H153" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I153" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J153" s="5" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K153" s="5" t="str">
+        <x:v>Build, Browser URL/title/console, Playwright toolbar desktop/mobile, DB readback</x:v>
+      </x:c>
       <x:c r="L153" s="5"/>
       <x:c r="M153" s="5"/>
       <x:c r="N153" s="5"/>
@@ -35541,8 +35568,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc45e58a923df4794"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc65e253a037c47b5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3599752219064538"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16f595869d104957"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor quick color bar
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R64aa9f795ed94d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rfed02493e4aa4731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R4d886bcf0e7a4b93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R30b7b473cada480b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>143</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -4479,7 +4479,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>145</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -11804,17 +11804,44 @@
       <x:c r="Z153" s="5"/>
     </x:row>
     <x:row r="154">
-      <x:c r="A154" s="5"/>
-      <x:c r="B154" s="39"/>
-      <x:c r="C154" s="5"/>
-      <x:c r="D154" s="5"/>
-      <x:c r="E154" s="5"/>
-      <x:c r="F154" s="39"/>
-      <x:c r="G154" s="5"/>
-      <x:c r="H154" s="5"/>
-      <x:c r="I154" s="5"/>
-      <x:c r="J154" s="5"/>
-      <x:c r="K154" s="5"/>
+      <x:c r="A154" s="5" t="str">
+        <x:v>TC_VIZI_146</x:v>
+      </x:c>
+      <x:c r="B154" s="39" t="str">
+        <x:v>Bottom quick color bar 56C</x:v>
+      </x:c>
+      <x:c r="C154" s="5" t="str">
+        <x:v>Xac minh thanh mau nhanh doi duoc fill/stroke tu recent colors va luu vao design JSON</x:v>
+      </x:c>
+      <x:c r="D154" s="5" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E154" s="5" t="str">
+        <x:v>1. Chay npm run build
+2. Browser mo /editor/1 lay URL/title/console
+3. Playwright tao draft va mo /editor/:designId
+4. Kiem tra quick color bar co Fill/Stroke va 6 swatch
+5. Doi fill #A87F33 va stroke #2F281C cho layer 1
+6. Save, reload, API readback, mobile va cleanup QA</x:v>
+      </x:c>
+      <x:c r="F154" s="39" t="str">
+        <x:v>Quick color bar hien o day workspace; doi fill/stroke layer 1, render cap nhat, save/reload va API giu mau</x:v>
+      </x:c>
+      <x:c r="G154" s="5" t="str">
+        <x:v>Pass: build pass; Browser URL/title=Vizi console=0, DOM snapshot fallback do incrementalAriaSnapshot; Playwright /editor/21 co Fill/Stroke + 6 swatch, layer 1 label 1. rect, fill #A87F33 va stroke #2F281C render dung, save/reload/API readback dung, mobile overflow=0, console error=0, DB cleanup users/designs=0</x:v>
+      </x:c>
+      <x:c r="H154" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I154" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J154" s="5" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K154" s="5" t="str">
+        <x:v>Build, Browser URL/title/console, Playwright quick color desktop/mobile/API, DB readback</x:v>
+      </x:c>
       <x:c r="L154" s="5"/>
       <x:c r="M154" s="5"/>
       <x:c r="N154" s="5"/>
@@ -35568,8 +35595,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3599752219064538"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16f595869d104957"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R388e131cd81449e9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576d6af8c0e04b75"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor layer selection
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R4d886bcf0e7a4b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R30b7b473cada480b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R2ae696e19bbe48a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1c212736851943ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>144</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -4479,7 +4479,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>146</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -11859,17 +11859,44 @@
       <x:c r="Z154" s="5"/>
     </x:row>
     <x:row r="155">
-      <x:c r="A155" s="5"/>
-      <x:c r="B155" s="39"/>
-      <x:c r="C155" s="5"/>
-      <x:c r="D155" s="5"/>
-      <x:c r="E155" s="5"/>
-      <x:c r="F155" s="39"/>
-      <x:c r="G155" s="5"/>
-      <x:c r="H155" s="5"/>
-      <x:c r="I155" s="5"/>
-      <x:c r="J155" s="5"/>
-      <x:c r="K155" s="5"/>
+      <x:c r="A155" s="5" t="str">
+        <x:v>TC_VIZI_147</x:v>
+      </x:c>
+      <x:c r="B155" s="39" t="str">
+        <x:v>Layer panel selection 56D</x:v>
+      </x:c>
+      <x:c r="C155" s="5" t="str">
+        <x:v>Xac minh click layer panel chon dung layer tren canvas va quick color ap dung vao layer dang chon</x:v>
+      </x:c>
+      <x:c r="D155" s="5" t="str">
+        <x:v>Frontend va backend local dang chay; tai khoan va draft QA tam</x:v>
+      </x:c>
+      <x:c r="E155" s="5" t="str">
+        <x:v>1. Chay npm run build
+2. Browser mo /editor/1 lay URL/title/console
+3. Playwright tao draft va mo /editor/:designId
+4. Kiem tra mac dinh layer 1 selected
+5. Click layer 2 va doi fill #A5382F
+6. Kiem tra Back/Front, mobile, save/API readback va cleanup QA</x:v>
+      </x:c>
+      <x:c r="F155" s="39" t="str">
+        <x:v>Click layer panel cap nhat active row, canvas selected outline va quick color target dung layer</x:v>
+      </x:c>
+      <x:c r="G155" s="5" t="str">
+        <x:v>Pass: build pass; Browser URL/title=Vizi console=0, DOM snapshot fallback do incrementalAriaSnapshot; Playwright /editor/22 co 3 layer buttons, mac dinh layer 1 selected, click layer 2 selected canvas layer 2 va color bar label 2. text, fill #A5382F ap dung vao layer 2/API readback dung, Back khong co layer va swatch disabled, Front giu selection, mobile chon layer 3 overflow=0, console error=0, DB cleanup users/designs=0</x:v>
+      </x:c>
+      <x:c r="H155" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I155" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="J155" s="5" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="K155" s="5" t="str">
+        <x:v>Build, Browser URL/title/console, Playwright layer selection desktop/mobile/API, DB readback</x:v>
+      </x:c>
       <x:c r="L155" s="5"/>
       <x:c r="M155" s="5"/>
       <x:c r="N155" s="5"/>
@@ -35595,8 +35622,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R388e131cd81449e9"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576d6af8c0e04b75"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae59ea05685f4942"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccbddcc12a9e4afa"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor layer visibility toggle
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R2ae696e19bbe48a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1c212736851943ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R413b3ea938d74619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1158963bc37648ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>145</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:f>COUNTIF(I9:I998,"Fail")</x:f>
@@ -4479,7 +4479,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>147</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -11914,17 +11914,44 @@
       <x:c r="Z155" s="5"/>
     </x:row>
     <x:row r="156">
-      <x:c r="A156" s="5"/>
-      <x:c r="B156" s="39"/>
-      <x:c r="C156" s="5"/>
-      <x:c r="D156" s="5"/>
-      <x:c r="E156" s="5"/>
-      <x:c r="F156" s="39"/>
-      <x:c r="G156" s="5"/>
-      <x:c r="H156" s="5"/>
-      <x:c r="I156" s="5"/>
-      <x:c r="J156" s="5"/>
-      <x:c r="K156" s="5"/>
+      <x:c r="A156" s="5" t="str">
+        <x:v>TC_VIZI_148</x:v>
+      </x:c>
+      <x:c r="B156" s="39" t="str">
+        <x:v>An hien layer tren editor</x:v>
+      </x:c>
+      <x:c r="C156" s="5" t="str">
+        <x:v>Xac nhan nut an/hien layer lam layer hidden khong render tren canvas nhung van con trong layer list/JSON va save reload giu trang thai.</x:v>
+      </x:c>
+      <x:c r="D156" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Dang nhap user test va mo /editor/23.
+B3: Dem canvas layer va layer row truoc khi an.
+B4: Bam nut Hide layer dau tien.
+B5: Save draft va reload editor.
+B6: Kiem tra canvas giam 1 layer, layer row van giu nguyen, bam Show de khoi phuc.</x:v>
+      </x:c>
+      <x:c r="E156" s="5" t="str">
+        <x:v>Local FE 127.0.0.1:5173; BE 127.0.0.1:8080; design #23; user step56e-20260706125353@example.test.</x:v>
+      </x:c>
+      <x:c r="F156" s="39" t="str">
+        <x:v>Layer hidden khong hien tren canvas; layer list van giu row; save/reload van giu trang thai hidden; show lai khoi phuc canvas; console khong co warning/error.</x:v>
+      </x:c>
+      <x:c r="G156" s="5" t="str">
+        <x:v>Pass: npm run build pass; Playwright Chrome smoke url=/editor/23, canvasBefore=3, layerRowsBefore=3, canvasAfterHide=2, layerRowsAfterHide=3, canvasAfterReloadHidden=2, layerRowsAfterReloadHidden=3, canvasAfterShow=3, consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H156" s="5" t="str">
+        <x:v>TC_VIZI_147; step 56D</x:v>
+      </x:c>
+      <x:c r="I156" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J156" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K156" s="5" t="str">
+        <x:v>Buoc 56E</x:v>
+      </x:c>
       <x:c r="L156" s="5"/>
       <x:c r="M156" s="5"/>
       <x:c r="N156" s="5"/>
@@ -35622,8 +35649,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae59ea05685f4942"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccbddcc12a9e4afa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f12d50640bd4afe"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1492657134e44a9"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor layer lock toggle
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R413b3ea938d74619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1158963bc37648ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R8e608cafee224772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R258c79bbd948483a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,24 +4462,21 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>146</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:f>COUNTIF(I9:I998,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="56" t="n">
-        <x:f>G5-E5-B5-A5</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="57"/>
       <x:c r="E5" s="56" t="n">
-        <x:f>COUNTIF(I$9:I$998,"N/A")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>148</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -11969,17 +11966,44 @@
       <x:c r="Z156" s="5"/>
     </x:row>
     <x:row r="157">
-      <x:c r="A157" s="5"/>
-      <x:c r="B157" s="39"/>
-      <x:c r="C157" s="5"/>
-      <x:c r="D157" s="5"/>
-      <x:c r="E157" s="5"/>
-      <x:c r="F157" s="39"/>
-      <x:c r="G157" s="5"/>
-      <x:c r="H157" s="5"/>
-      <x:c r="I157" s="5"/>
-      <x:c r="J157" s="5"/>
-      <x:c r="K157" s="5"/>
+      <x:c r="A157" s="5" t="str">
+        <x:v>TC_VIZI_149</x:v>
+      </x:c>
+      <x:c r="B157" s="39" t="str">
+        <x:v>Khoa mo khoa layer tren editor</x:v>
+      </x:c>
+      <x:c r="C157" s="5" t="str">
+        <x:v>Xac minh layer locked khong cho sua qua quick color/text input, trang thai locked duoc luu trong JSON va reload van giu.</x:v>
+      </x:c>
+      <x:c r="D157" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Dang nhap user test va mo /editor/24.
+B3: Khoa layer 1 va kiem tra swatch mau bi disabled.
+B4: Khoa layer text va kiem tra textarea bi disabled.
+B5: Save draft va reload editor.
+B6: Kiem tra locked van giu, sau do unlock de khoi phuc.</x:v>
+      </x:c>
+      <x:c r="E157" s="5" t="str">
+        <x:v>Local FE 127.0.0.1:5173; BE 127.0.0.1:8080; design #24; user step56f-20260706130857@example.test.</x:v>
+      </x:c>
+      <x:c r="F157" s="39" t="str">
+        <x:v>Layer locked khong cho sua quick color/text; save/reload giu locked; unlock tra ve editable; console khong co warning/error.</x:v>
+      </x:c>
+      <x:c r="G157" s="5" t="str">
+        <x:v>Pass: npm run build pass; Playwright Chrome smoke url=/editor/24, layerRows=3, firstLockPressed=true, disabledSwatchesAfterLock=6, lockedPropertyFirst=LockedYes, secondLockPressed=true, textDisabledAfterLock=true, locksAfterReload=[true,true,false], textDisabledAfterReload=true, locksAfterUnlock=[false,false,false], consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H157" s="5" t="str">
+        <x:v>TC_VIZI_148; step 56E</x:v>
+      </x:c>
+      <x:c r="I157" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J157" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K157" s="5" t="str">
+        <x:v>Buoc 56F</x:v>
+      </x:c>
       <x:c r="L157" s="5"/>
       <x:c r="M157" s="5"/>
       <x:c r="N157" s="5"/>
@@ -35649,8 +35673,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f12d50640bd4afe"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1492657134e44a9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0089bfa5c4c0461f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9b5038eca04e48"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor layer reorder controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R8e608cafee224772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R258c79bbd948483a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rdb67fedef8394e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5693222865184693"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>147</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4476,7 +4476,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -12021,17 +12021,44 @@
       <x:c r="Z157" s="5"/>
     </x:row>
     <x:row r="158">
-      <x:c r="A158" s="5"/>
-      <x:c r="B158" s="39"/>
-      <x:c r="C158" s="5"/>
-      <x:c r="D158" s="5"/>
-      <x:c r="E158" s="5"/>
-      <x:c r="F158" s="39"/>
-      <x:c r="G158" s="5"/>
-      <x:c r="H158" s="5"/>
-      <x:c r="I158" s="5"/>
-      <x:c r="J158" s="5"/>
-      <x:c r="K158" s="5"/>
+      <x:c r="A158" s="5" t="str">
+        <x:v>TC_VIZI_150</x:v>
+      </x:c>
+      <x:c r="B158" s="39" t="str">
+        <x:v>Sap xep layer len xuong tren editor</x:v>
+      </x:c>
+      <x:c r="C158" s="5" t="str">
+        <x:v>Xac minh nut move up/down doi thu tu layer, selected layer di theo vi tri moi, save/reload va API readback giu dung order.</x:v>
+      </x:c>
+      <x:c r="D158" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Tao user/draft test va mo /editor/26.
+B3: Kiem tra layer 1 khong move up va layer 3 khong move down.
+B4: Move layer 1 down, kiem tra order va selected label.
+B5: Move layer 2 up de khoi phuc, sau do move down lai va save.
+B6: Reload editor, kiem tra mobile 390x844 va doc API /api/designs/26 de xac minh order.</x:v>
+      </x:c>
+      <x:c r="E158" s="5" t="str">
+        <x:v>Local FE 127.0.0.1:5173; BE 127.0.0.1:8080; design #26; user step56g-20260706063323@example.test.</x:v>
+      </x:c>
+      <x:c r="F158" s="39" t="str">
+        <x:v>Layer order doi dung; nut bien disabled dung; selected layer theo vi tri moi; save/reload va API giu order; console khong co warning/error.</x:v>
+      </x:c>
+      <x:c r="G158" s="5" t="str">
+        <x:v>Pass: npm run build pass; Playwright Chrome smoke url=/editor/26, initialOrder=[1rect,2text,3text], boundary disabled=true/true, orderAfterMoveDown=[1text,2rect,3text], selectedAfterMoveDown=2. rect, orderAfterMoveUp=[1rect,2text,3text], selectedAfterMoveUp=1. rect, orderAfterReload=[1text,2rect,3text], mobileOverflow=0, mobileActionButtons=12, savedTypes=[text,rect,text], consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H158" s="5" t="str">
+        <x:v>TC_VIZI_149; step 56F</x:v>
+      </x:c>
+      <x:c r="I158" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J158" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K158" s="5" t="str">
+        <x:v>Buoc 56G</x:v>
+      </x:c>
       <x:c r="L158" s="5"/>
       <x:c r="M158" s="5"/>
       <x:c r="N158" s="5"/>
@@ -35673,8 +35700,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0089bfa5c4c0461f"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f9b5038eca04e48"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7801728d81a4ff3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49898d7dd39e43ee"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Organize backend code by domain packages
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rdb67fedef8394e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R5693222865184693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R0f5e34010cb44b04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Re0bf227ea2ed4331"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>148</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4476,7 +4476,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -12076,17 +12076,43 @@
       <x:c r="Z158" s="5"/>
     </x:row>
     <x:row r="159">
-      <x:c r="A159" s="5"/>
-      <x:c r="B159" s="39"/>
-      <x:c r="C159" s="5"/>
-      <x:c r="D159" s="5"/>
-      <x:c r="E159" s="5"/>
-      <x:c r="F159" s="39"/>
-      <x:c r="G159" s="5"/>
-      <x:c r="H159" s="5"/>
-      <x:c r="I159" s="5"/>
-      <x:c r="J159" s="5"/>
-      <x:c r="K159" s="5"/>
+      <x:c r="A159" s="5" t="str">
+        <x:v>TC_VIZI_151</x:v>
+      </x:c>
+      <x:c r="B159" s="39" t="str">
+        <x:v>Phan loai package backend theo domain</x:v>
+      </x:c>
+      <x:c r="C159" s="5" t="str">
+        <x:v>Xac minh source va test Spring Boot duoc chia vao auth, design, template, health, config va common/error ma khong thay doi API.</x:v>
+      </x:c>
+      <x:c r="D159" s="5" t="str">
+        <x:v>B1: Kiem tra package goc chi giu ViziApplication.
+B2: Compile 23 source files va 10 test files.
+B3: Chay toan bo Maven test.
+B4: Xac minh Spring tim thay ViziApplication va 4 JPA repositories.
+B5: Xac minh auth, design, template, health, error va Flyway migration van hoat dong.</x:v>
+      </x:c>
+      <x:c r="E159" s="5" t="str">
+        <x:v>Backend local; Java release 21; H2 test profile; PostgreSQL 17.10 tren localhost:55432 cho integration test.</x:v>
+      </x:c>
+      <x:c r="F159" s="39" t="str">
+        <x:v>Cau truc package ro rang; build thanh cong; 28 test pass; khong doi endpoint, schema hay response.</x:v>
+      </x:c>
+      <x:c r="G159" s="5" t="str">
+        <x:v>Pass: Maven compile 23 source + 10 test files; Tests run=28, Failures=0, Errors=0, Skipped=0; Spring Boot tim thay com.example.vizi.ViziApplication; 4 JPA repositories; PostgreSQL/Flyway integration pass.</x:v>
+      </x:c>
+      <x:c r="H159" s="5" t="str">
+        <x:v>TC_VIZI_150; step 56G</x:v>
+      </x:c>
+      <x:c r="I159" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J159" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K159" s="5" t="str">
+        <x:v>Buoc 57</x:v>
+      </x:c>
       <x:c r="L159" s="5"/>
       <x:c r="M159" s="5"/>
       <x:c r="N159" s="5"/>
@@ -35700,8 +35726,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7801728d81a4ff3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49898d7dd39e43ee"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b8f33f9a84740f1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1362bf6b232f47e9"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor multi-layer selection and group drag
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R0f5e34010cb44b04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Re0bf227ea2ed4331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R6bb1540559544d2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R067ec0c5130c4943"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4476,7 +4476,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -12130,17 +12130,45 @@
       <x:c r="Z159" s="5"/>
     </x:row>
     <x:row r="160">
-      <x:c r="A160" s="5"/>
-      <x:c r="B160" s="39"/>
-      <x:c r="C160" s="5"/>
-      <x:c r="D160" s="5"/>
-      <x:c r="E160" s="5"/>
-      <x:c r="F160" s="39"/>
-      <x:c r="G160" s="5"/>
-      <x:c r="H160" s="5"/>
-      <x:c r="I160" s="5"/>
-      <x:c r="J160" s="5"/>
-      <x:c r="K160" s="5"/>
+      <x:c r="A160" s="5" t="str">
+        <x:v>TC_VIZI_152</x:v>
+      </x:c>
+      <x:c r="B160" s="39" t="str">
+        <x:v>Chon nhieu layer va keo ca nhom 56H</x:v>
+      </x:c>
+      <x:c r="C160" s="5" t="str">
+        <x:v>Xac minh Shift/Ctrl/Cmd chon nhieu layer, keo nhom giu dung khoang cach, click workspace bo chon, save/reload va API giu vi tri.</x:v>
+      </x:c>
+      <x:c r="D160" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Tao user va draft test, mo editor.
+B3: Chon layer 2, Shift chon layer 3.
+B4: Keo nhom va so sanh delta x/y cua hai layer.
+B5: Xac minh layer khong chon khong di chuyen.
+B6: Click workspace de bo chon.
+B7: Save, reload, doc API va test mobile 390x844.</x:v>
+      </x:c>
+      <x:c r="E160" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #31; hai text layer va mot layer nen.</x:v>
+      </x:c>
+      <x:c r="F160" s="39" t="str">
+        <x:v>Hai layer duoc chon cung delta; layer nen khong doi; bo chon ve 0; vi tri duoc luu; mobile khong tran; console sach.</x:v>
+      </x:c>
+      <x:c r="G160" s="5" t="str">
+        <x:v>Pass: build pass; selection=2; delta ca hai layer x=7.5%, y=6.9444%; layer nen giu x=0,y=0; clear selection=0; save/reload/API giu vi tri; mobileOverflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H160" s="5" t="str">
+        <x:v>TC_VIZI_150; TC_VIZI_151; step 56G</x:v>
+      </x:c>
+      <x:c r="I160" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J160" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K160" s="5" t="str">
+        <x:v>Buoc 56H</x:v>
+      </x:c>
       <x:c r="L160" s="5"/>
       <x:c r="M160" s="5"/>
       <x:c r="N160" s="5"/>
@@ -35726,8 +35754,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b8f33f9a84740f1"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1362bf6b232f47e9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0ab8bf66b564141"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b28b71fd0d64610"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add canvas layer resize handle
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R6bb1540559544d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R067ec0c5130c4943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb43aae5f0832445f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rd0de25f8204c435a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4476,7 +4476,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -12186,17 +12186,45 @@
       <x:c r="Z160" s="5"/>
     </x:row>
     <x:row r="161">
-      <x:c r="A161" s="5"/>
-      <x:c r="B161" s="39"/>
-      <x:c r="C161" s="5"/>
-      <x:c r="D161" s="5"/>
-      <x:c r="E161" s="5"/>
-      <x:c r="F161" s="39"/>
-      <x:c r="G161" s="5"/>
-      <x:c r="H161" s="5"/>
-      <x:c r="I161" s="5"/>
-      <x:c r="J161" s="5"/>
-      <x:c r="K161" s="5"/>
+      <x:c r="A161" s="5" t="str">
+        <x:v>TC_VIZI_153</x:v>
+      </x:c>
+      <x:c r="B161" s="39" t="str">
+        <x:v>Resize layer bang handle 56I</x:v>
+      </x:c>
+      <x:c r="C161" s="5" t="str">
+        <x:v>Xac minh resize handle cap nhat width/height, giu x/y, khong anh huong layer khac, an khi lock/multi-select va luu duoc.</x:v>
+      </x:c>
+      <x:c r="D161" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Tao draft va mo editor.
+B3: Chon text layer 2 va keo resize handle.
+B4: So sanh x/y/width/height truoc sau.
+B5: Lock/unlock va multi-select de kiem tra handle.
+B6: Save, reload va doc API.
+B7: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E161" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #32; text layer width=45, height=16.</x:v>
+      </x:c>
+      <x:c r="F161" s="39" t="str">
+        <x:v>Width/height thay doi trong bien card; x/y va layer khac khong doi; handle dung trang thai; save/reload/API dung; mobile khong tran.</x:v>
+      </x:c>
+      <x:c r="G161" s="5" t="str">
+        <x:v>Pass: width 45-&gt;53.3333, height 16-&gt;22.9444; x=12,y=20 giu nguyen; handle lock=0, multi-select=0; API/reload dung; mobile handle=18x18, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H161" s="5" t="str">
+        <x:v>TC_VIZI_152; step 56H</x:v>
+      </x:c>
+      <x:c r="I161" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J161" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K161" s="5" t="str">
+        <x:v>Buoc 56I</x:v>
+      </x:c>
       <x:c r="L161" s="5"/>
       <x:c r="M161" s="5"/>
       <x:c r="N161" s="5"/>
@@ -35754,8 +35782,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0ab8bf66b564141"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b28b71fd0d64610"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3878305878ec4c15"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30d60ba8d38a4838"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add canvas layer rotate handle
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb43aae5f0832445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rd0de25f8204c435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R03e89a782a674010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4b02de3e3aa44b61"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4462,7 +4462,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4476,7 +4476,7 @@
       </x:c>
       <x:c r="F5" s="57"/>
       <x:c r="G5" s="50" t="n">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="H5" s="51"/>
       <x:c r="I5" s="52"/>
@@ -12242,17 +12242,45 @@
       <x:c r="Z161" s="5"/>
     </x:row>
     <x:row r="162">
-      <x:c r="A162" s="5"/>
-      <x:c r="B162" s="39"/>
-      <x:c r="C162" s="5"/>
-      <x:c r="D162" s="5"/>
-      <x:c r="E162" s="5"/>
-      <x:c r="F162" s="39"/>
-      <x:c r="G162" s="5"/>
-      <x:c r="H162" s="5"/>
-      <x:c r="I162" s="5"/>
-      <x:c r="J162" s="5"/>
-      <x:c r="K162" s="5"/>
+      <x:c r="A162" s="5" t="str">
+        <x:v>TC_VIZI_154</x:v>
+      </x:c>
+      <x:c r="B162" s="39" t="str">
+        <x:v>Rotate layer bang handle 56J</x:v>
+      </x:c>
+      <x:c r="C162" s="5" t="str">
+        <x:v>Xac minh rotate handle cap nhat rotation, giu x/y/width/height, an khi lock/multi-select va luu duoc.</x:v>
+      </x:c>
+      <x:c r="D162" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Tao draft va mo editor.
+B3: Chon text layer 2 va keo rotate handle.
+B4: So sanh x/y/width/height/rotation truoc sau.
+B5: Lock/unlock va multi-select de kiem tra handle.
+B6: Save, reload va doc API.
+B7: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E162" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #34; text layer rotation initial 0.</x:v>
+      </x:c>
+      <x:c r="F162" s="39" t="str">
+        <x:v>Rotation thay doi trong bien card; x/y/width/height va layer khac khong doi; handle dung trang thai; save/reload/API dung; mobile khong tran.</x:v>
+      </x:c>
+      <x:c r="G162" s="5" t="str">
+        <x:v>Pass: rotation 0-&gt;90; x=12,y=20,width=45,height=16 giu nguyen; handle lock=0, multi-select=0; API/reload dung; mobile handle=18x18, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H162" s="5" t="str">
+        <x:v>TC_VIZI_153; step 56I</x:v>
+      </x:c>
+      <x:c r="I162" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J162" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K162" s="5" t="str">
+        <x:v>Buoc 56J</x:v>
+      </x:c>
       <x:c r="L162" s="5"/>
       <x:c r="M162" s="5"/>
       <x:c r="N162" s="5"/>
@@ -35782,8 +35810,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3878305878ec4c15"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30d60ba8d38a4838"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc92d35be1f1f4d97"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3610c2ea5ea4357"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor text style controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf8082a2861de4589"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R7b5474a0f2654dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R7f8f66aeb0a24b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R6c9090f65f234f40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>155</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12637,17 +12637,46 @@
       <x:c r="Z163" s="5"/>
     </x:row>
     <x:row r="164">
-      <x:c r="A164" s="5"/>
-      <x:c r="B164" s="24"/>
-      <x:c r="C164" s="5"/>
-      <x:c r="D164" s="5"/>
-      <x:c r="E164" s="5"/>
-      <x:c r="F164" s="24"/>
-      <x:c r="G164" s="5"/>
-      <x:c r="H164" s="5"/>
-      <x:c r="I164" s="5"/>
-      <x:c r="J164" s="5"/>
-      <x:c r="K164" s="5"/>
+      <x:c r="A164" s="5" t="str">
+        <x:v>TC_VIZI_156</x:v>
+      </x:c>
+      <x:c r="B164" s="24" t="str">
+        <x:v>Chinh text style layer trong Properties 56L</x:v>
+      </x:c>
+      <x:c r="C164" s="5" t="str">
+        <x:v>Xac minh Properties panel cho sua font family/font size/font weight cua text layer, lock/multi-select/rect layer chan control va luu duoc.</x:v>
+      </x:c>
+      <x:c r="D164" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Tao draft va mo editor.
+B3: Chon text layer 2.
+B4: Doi Font=Georgia, Size=26, Weight=300 trong Properties.
+B5: Xac minh canvas computed style.
+B6: Lock/unlock, multi-select va rect layer de kiem tra control.
+B7: Save, reload va doc API.
+B8: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E164" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #38; layer 2 initial fontSize=18, fontWeight default 700.</x:v>
+      </x:c>
+      <x:c r="F164" s="24" t="str">
+        <x:v>Canvas cap nhat font/style; locked/multi-select/rect layer khong sua duoc; save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="G164" s="5" t="str">
+        <x:v>Pass: fontFamily=Georgia, fontSize=26, fontWeight=300; lock disabled control; multi-select/rect an control; API/reload dung; mobile controls=316px, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H164" s="5" t="str">
+        <x:v>TC_VIZI_155; step 56K</x:v>
+      </x:c>
+      <x:c r="I164" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J164" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K164" s="5" t="str">
+        <x:v>Buoc 56L</x:v>
+      </x:c>
       <x:c r="L164" s="5"/>
       <x:c r="M164" s="5"/>
       <x:c r="N164" s="5"/>
@@ -36121,8 +36150,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8dda094e5044ec2"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9704c794ffed41cf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11aa59d32b644fbe"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re24d7ada43294379"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor appearance controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R7f8f66aeb0a24b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R6c9090f65f234f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd4655d0bf07b40d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R55dd274cc5ab4f3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>154</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12694,17 +12694,46 @@
       <x:c r="Z164" s="5"/>
     </x:row>
     <x:row r="165">
-      <x:c r="A165" s="5"/>
-      <x:c r="B165" s="24"/>
-      <x:c r="C165" s="5"/>
-      <x:c r="D165" s="5"/>
-      <x:c r="E165" s="5"/>
-      <x:c r="F165" s="24"/>
-      <x:c r="G165" s="5"/>
-      <x:c r="H165" s="5"/>
-      <x:c r="I165" s="5"/>
-      <x:c r="J165" s="5"/>
-      <x:c r="K165" s="5"/>
+      <x:c r="A165" s="5" t="str">
+        <x:v>TC_VIZI_157</x:v>
+      </x:c>
+      <x:c r="B165" s="24" t="str">
+        <x:v>Chinh appearance layer trong Properties 56M</x:v>
+      </x:c>
+      <x:c r="C165" s="5" t="str">
+        <x:v>Xac minh Properties panel cho sua fill/stroke/opacity/stroke width cua layer, lock/multi-select chan control, text fill map thanh mau chu va luu duoc.</x:v>
+      </x:c>
+      <x:c r="D165" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Tao draft va mo editor.
+B3: Chon rect layer 1.
+B4: Doi Fill=#123456, Stroke=#654321, Opacity=0.42, Stroke W=8.
+B5: Xac minh computed style tren canvas.
+B6: Lock/unlock va multi-select de kiem tra control.
+B7: Chon text layer 2, doi Fill=#008877 va xac minh mau chu.
+B8: Save, reload, doc API, test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E165" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #40; rect layer 1, text layer 2.</x:v>
+      </x:c>
+      <x:c r="F165" s="24" t="str">
+        <x:v>Canvas cap nhat appearance; locked/multi-select khong sua duoc; text fill cap nhat color; save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="G165" s="5" t="str">
+        <x:v>Pass: rect fill/stroke/opacity/strokeWidth=#123456/#654321/0.42/8; text color=#008877; lock disabled control; multi-select an control; API/reload dung; mobile controls=154px, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H165" s="5" t="str">
+        <x:v>TC_VIZI_156; step 56L</x:v>
+      </x:c>
+      <x:c r="I165" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J165" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K165" s="5" t="str">
+        <x:v>Buoc 56M</x:v>
+      </x:c>
       <x:c r="L165" s="5"/>
       <x:c r="M165" s="5"/>
       <x:c r="N165" s="5"/>
@@ -36150,8 +36179,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11aa59d32b644fbe"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re24d7ada43294379"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d3d958c6b04eed"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62f9bf14605146a0"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor effect controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd4655d0bf07b40d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R55dd274cc5ab4f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf19ba98faa744150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Refa47bf74d40446d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>155</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12751,17 +12751,46 @@
       <x:c r="Z165" s="5"/>
     </x:row>
     <x:row r="166">
-      <x:c r="A166" s="5"/>
-      <x:c r="B166" s="24"/>
-      <x:c r="C166" s="5"/>
-      <x:c r="D166" s="5"/>
-      <x:c r="E166" s="5"/>
-      <x:c r="F166" s="24"/>
-      <x:c r="G166" s="5"/>
-      <x:c r="H166" s="5"/>
-      <x:c r="I166" s="5"/>
-      <x:c r="J166" s="5"/>
-      <x:c r="K166" s="5"/>
+      <x:c r="A166" s="5" t="str">
+        <x:v>TC_VIZI_158</x:v>
+      </x:c>
+      <x:c r="B166" s="24" t="str">
+        <x:v>Chinh shadow va blur layer trong Properties 56N</x:v>
+      </x:c>
+      <x:c r="C166" s="5" t="str">
+        <x:v>Xac minh Properties panel cho sua shadowX/shadowY/shadowBlur/shadowColor/blur cua layer, lock/multi-select chan control, clamp va luu duoc.</x:v>
+      </x:c>
+      <x:c r="D166" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Tao draft va mo editor.
+B3: Chon rect layer 1.
+B4: Doi Shadow X=6, Shadow Y=9, Shadow Blur=18, Shadow Color=#221100, Blur=1.5.
+B5: Xac minh computed style tren canvas.
+B6: Kiem tra lock/unlock va multi-select.
+B7: Nhap gia tri vuot gioi han de kiem tra clamp.
+B8: Save, reload, doc API, test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E166" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #41; rect layer 1.</x:v>
+      </x:c>
+      <x:c r="F166" s="24" t="str">
+        <x:v>Canvas cap nhat shadow/blur; locked/multi-select khong sua duoc; clamp dung; save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="G166" s="5" t="str">
+        <x:v>Pass: shadow=6px 9px 18px #221100; blur=1.5px; clamp ve 50/-50/50/50; API/reload dung; mobile controls=154px, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H166" s="5" t="str">
+        <x:v>TC_VIZI_157; step 56M</x:v>
+      </x:c>
+      <x:c r="I166" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J166" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K166" s="5" t="str">
+        <x:v>Buoc 56N</x:v>
+      </x:c>
       <x:c r="L166" s="5"/>
       <x:c r="M166" s="5"/>
       <x:c r="N166" s="5"/>
@@ -36179,8 +36208,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d3d958c6b04eed"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62f9bf14605146a0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f4d0c6470444fb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R759def00b1264d8a"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix editor fonts and shadow controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf19ba98faa744150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Refa47bf74d40446d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rc432c4a3a4434673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4d584ba614e94b8a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>158</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12808,17 +12808,46 @@
       <x:c r="Z166" s="5"/>
     </x:row>
     <x:row r="167">
-      <x:c r="A167" s="5"/>
-      <x:c r="B167" s="24"/>
-      <x:c r="C167" s="5"/>
-      <x:c r="D167" s="5"/>
-      <x:c r="E167" s="5"/>
-      <x:c r="F167" s="24"/>
-      <x:c r="G167" s="5"/>
-      <x:c r="H167" s="5"/>
-      <x:c r="I167" s="5"/>
-      <x:c r="J167" s="5"/>
-      <x:c r="K167" s="5"/>
+      <x:c r="A167" s="5" t="str">
+        <x:v>TC_VIZI_159</x:v>
+      </x:c>
+      <x:c r="B167" s="24" t="str">
+        <x:v>Sua bug shadow, font local va geometry label editor</x:v>
+      </x:c>
+      <x:c r="C167" s="5" t="str">
+        <x:v>Xac minh text shadow khong tao nen blob, shadow co spread/opacity, font local searchable, geometry hien don vi %, save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="D167" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Tao user/draft tam va mo /editor/{id}.
+B3: Chon text layer 2, tim font local SVN Adeline va doi font.
+B4: Doi Shadow X/Y/Blur/Spread/Color/Opacity va Blur cho text.
+B5: Xac minh text layer dung text-shadow, khong dung box-shadow.
+B6: Chon rect layer 1, doi shadow spread/opacity/blur va xac minh box-shadow.
+B7: Save, reload, doc API canvasJson.
+B8: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E167" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #43; localFonts 1479 file families.</x:v>
+      </x:c>
+      <x:c r="F167" s="24" t="str">
+        <x:v>Text layer khong con nen blob; font local searchable; shadow spread/opacity luu duoc; geometry label ro la %; mobile khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="G167" s="5" t="str">
+        <x:v>Pass: build OK; fontOptionCount=1484 co SVN Adeline; text boxShadow=none, textShadow rgba(0,0,0,.5) 4px 4px 4px; rect boxShadow co spread 6px; API/reload dung; mobile controls=7, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H167" s="5" t="str">
+        <x:v>TC_VIZI_158; bug editor polish</x:v>
+      </x:c>
+      <x:c r="I167" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J167" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K167" s="5" t="str">
+        <x:v>Bugfix editor</x:v>
+      </x:c>
       <x:c r="L167" s="5"/>
       <x:c r="M167" s="5"/>
       <x:c r="N167" s="5"/>
@@ -36208,8 +36237,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f4d0c6470444fb"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R759def00b1264d8a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9930a09f351a471b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb259020f8dbd40b4"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor layer history actions
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rc432c4a3a4434673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4d584ba614e94b8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb5d041108b82403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R44392fb14d8549fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>159</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12865,17 +12865,45 @@
       <x:c r="Z167" s="5"/>
     </x:row>
     <x:row r="168">
-      <x:c r="A168" s="5"/>
-      <x:c r="B168" s="24"/>
-      <x:c r="C168" s="5"/>
-      <x:c r="D168" s="5"/>
-      <x:c r="E168" s="5"/>
-      <x:c r="F168" s="24"/>
-      <x:c r="G168" s="5"/>
-      <x:c r="H168" s="5"/>
-      <x:c r="I168" s="5"/>
-      <x:c r="J168" s="5"/>
-      <x:c r="K168" s="5"/>
+      <x:c r="A168" s="5" t="str">
+        <x:v>TC_VIZI_160</x:v>
+      </x:c>
+      <x:c r="B168" s="24" t="str">
+        <x:v>Duplicate delete layer va undo redo editor 56O</x:v>
+      </x:c>
+      <x:c r="C168" s="5" t="str">
+        <x:v>Xac minh editor co the copy/xoa layer, undo/redo trong phien lam viec, save/reload va API giu dung layer JSON.</x:v>
+      </x:c>
+      <x:c r="D168" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Tao user/draft tam va mo /editor/{id}.
+B3: Chon text layer 2 va bam Copy.
+B4: Kiem tra layer tang 3-&gt;4, ban copy offset X/Y +4%.
+B5: Bam Undo, Redo, Delete, Undo va xac minh layer count.
+B6: Save, doc API /api/designs/{id}, reload editor.
+B7: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E168" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #44; layer 2 text.</x:v>
+      </x:c>
+      <x:c r="F168" s="24" t="str">
+        <x:v>Copy tao layer moi, delete xoa layer dang chon, undo/redo doi dung layer count, save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="G168" s="5" t="str">
+        <x:v>Pass: build OK; duplicate layer count 4; Undo ve 3; Redo ve 4; Delete ve 3; Undo ve 4; API layer count 4, duplicate x=16,y=24; mobile tools 155px, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H168" s="5" t="str">
+        <x:v>TC_VIZI_159; step 56O</x:v>
+      </x:c>
+      <x:c r="I168" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J168" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K168" s="5" t="str">
+        <x:v>Buoc 56O</x:v>
+      </x:c>
       <x:c r="L168" s="5"/>
       <x:c r="M168" s="5"/>
       <x:c r="N168" s="5"/>
@@ -36237,8 +36265,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9930a09f351a471b"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb259020f8dbd40b4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf463afc66655495b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b83a6bf1dd94366"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor keyboard shortcuts
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb5d041108b82403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R44392fb14d8549fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R7ca648faa8174f5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R23b2e9ce09ea4fda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>158</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>160</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12921,17 +12921,45 @@
       <x:c r="Z168" s="5"/>
     </x:row>
     <x:row r="169">
-      <x:c r="A169" s="5"/>
-      <x:c r="B169" s="24"/>
-      <x:c r="C169" s="5"/>
-      <x:c r="D169" s="5"/>
-      <x:c r="E169" s="5"/>
-      <x:c r="F169" s="24"/>
-      <x:c r="G169" s="5"/>
-      <x:c r="H169" s="5"/>
-      <x:c r="I169" s="5"/>
-      <x:c r="J169" s="5"/>
-      <x:c r="K169" s="5"/>
+      <x:c r="A169" s="5" t="str">
+        <x:v>TC_VIZI_161</x:v>
+      </x:c>
+      <x:c r="B169" s="24" t="str">
+        <x:v>Keyboard shortcut co ban editor 56P</x:v>
+      </x:c>
+      <x:c r="C169" s="5" t="str">
+        <x:v>Xac minh Delete, Ctrl+Z, Ctrl+Y, Ctrl+D hoat dong trong editor va khong kich hoat khi focus input.</x:v>
+      </x:c>
+      <x:c r="D169" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Tao user/draft tam va mo /editor/{id}.
+B3: Chon text layer 2.
+B4: Bam Ctrl+D, Ctrl+Z, Ctrl+Y, Delete, Ctrl+Z va kiem tra layer count.
+B5: Focus input Layer X, bam Ctrl+D va Delete de xac minh shortcut khong chay trong input.
+B6: Save, doc API /api/designs/{id}, reload editor.
+B7: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E169" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #45; layer 2 text.</x:v>
+      </x:c>
+      <x:c r="F169" s="24" t="str">
+        <x:v>Shortcut editor thay doi layer dung; input/textarea/select giu hanh vi native; save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="G169" s="5" t="str">
+        <x:v>Pass: build OK; Ctrl+D 3-&gt;4; Ctrl+Z 4-&gt;3; Ctrl+Y 3-&gt;4; Delete 4-&gt;3; Ctrl+Z 3-&gt;4; focus input khong duplicate/delete; API layer count 4; mobile overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H169" s="5" t="str">
+        <x:v>TC_VIZI_160; step 56P</x:v>
+      </x:c>
+      <x:c r="I169" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J169" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K169" s="5" t="str">
+        <x:v>Buoc 56P</x:v>
+      </x:c>
       <x:c r="L169" s="5"/>
       <x:c r="M169" s="5"/>
       <x:c r="N169" s="5"/>
@@ -36265,8 +36293,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf463afc66655495b"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b83a6bf1dd94366"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R917fbfe22b994a70"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6e20da85a9f450c"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor zoom and pan controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R7ca648faa8174f5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R23b2e9ce09ea4fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb8da2a3bfe994302"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rad05af2058b34bb9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>159</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -12977,17 +12977,46 @@
       <x:c r="Z169" s="5"/>
     </x:row>
     <x:row r="170">
-      <x:c r="A170" s="5"/>
-      <x:c r="B170" s="24"/>
-      <x:c r="C170" s="5"/>
-      <x:c r="D170" s="5"/>
-      <x:c r="E170" s="5"/>
-      <x:c r="F170" s="24"/>
-      <x:c r="G170" s="5"/>
-      <x:c r="H170" s="5"/>
-      <x:c r="I170" s="5"/>
-      <x:c r="J170" s="5"/>
-      <x:c r="K170" s="5"/>
+      <x:c r="A170" s="5" t="str">
+        <x:v>TC_VIZI_162</x:v>
+      </x:c>
+      <x:c r="B170" s="24" t="str">
+        <x:v>Zoom pan canvas editor 56Q</x:v>
+      </x:c>
+      <x:c r="C170" s="5" t="str">
+        <x:v>Xac minh zoom in/out/reset va pan canvas khong lam lech toa do layer, save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="D170" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Tao user/draft tam va mo /editor/{id}.
+B3: Chon text layer 2, dat X=20, Y=20.
+B4: Zoom in 2 lan len 120% va kiem tra frame lon hon.
+B5: Pan canvas sang phai/xuong duoi va kiem tra transform co translate.
+B6: Xac minh X/Y/W/H khong doi sau zoom/pan.
+B7: Reset ve 100%, save, doc API, reload.
+B8: Test mobile 390x844 va console.</x:v>
+      </x:c>
+      <x:c r="E170" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #54; layer 2 text.</x:v>
+      </x:c>
+      <x:c r="F170" s="24" t="str">
+        <x:v>Zoom/pan chi thay doi view state; layer geometry khong lech; save/reload/API/mobile dung.</x:v>
+      </x:c>
+      <x:c r="G170" s="5" t="str">
+        <x:v>Pass: build OK; zoom 100-&gt;120, frame lon hon; pan transform matrix(1.2,0,0,1.2,40,40); X/Y/W/H giu 20/20/45/16; API saved x=20,y=20; mobile overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H170" s="5" t="str">
+        <x:v>TC_VIZI_161; step 56Q</x:v>
+      </x:c>
+      <x:c r="I170" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J170" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K170" s="5" t="str">
+        <x:v>Buoc 56Q</x:v>
+      </x:c>
       <x:c r="L170" s="5"/>
       <x:c r="M170" s="5"/>
       <x:c r="N170" s="5"/>
@@ -36293,8 +36322,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R917fbfe22b994a70"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6e20da85a9f450c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b03e4a586c44c2d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R905b8fb77c324327"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Record editor JSON persistence testcase
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb8da2a3bfe994302"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rad05af2058b34bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd23a74b9c8d9436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4282bf349fbd4287"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>160</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13034,17 +13034,46 @@
       <x:c r="Z170" s="5"/>
     </x:row>
     <x:row r="171">
-      <x:c r="A171" s="5"/>
-      <x:c r="B171" s="24"/>
-      <x:c r="C171" s="5"/>
-      <x:c r="D171" s="5"/>
-      <x:c r="E171" s="5"/>
-      <x:c r="F171" s="24"/>
-      <x:c r="G171" s="5"/>
-      <x:c r="H171" s="5"/>
-      <x:c r="I171" s="5"/>
-      <x:c r="J171" s="5"/>
-      <x:c r="K171" s="5"/>
+      <x:c r="A171" s="5" t="str">
+        <x:v>TC_VIZI_163</x:v>
+      </x:c>
+      <x:c r="B171" s="24" t="str">
+        <x:v>Luu UI editor vao design JSON 56R</x:v>
+      </x:c>
+      <x:c r="C171" s="5" t="str">
+        <x:v>Xac minh layer order, lock, visible va style duoc luu chung vao canvasJson, refresh desktop/mobile van giu dung.</x:v>
+      </x:c>
+      <x:c r="D171" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Tao user/draft tam va mo /editor/{id}.
+B3: Move layer 1 down de doi order thanh text/rect/text.
+B4: Sua text layer fontFamily=Georgia, fontSize=28, fontWeight=700, color=#008877.
+B5: Sua rect fill/stroke/opacity/strokeWidth/shadow.
+B6: Lock rect layer va hide layer 3.
+B7: Save, doc API canvasJson va reload desktop.
+B8: Reload mobile 390x844 va kiem tra overflow/console.</x:v>
+      </x:c>
+      <x:c r="E171" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #55; 3 layer template.</x:v>
+      </x:c>
+      <x:c r="F171" s="24" t="str">
+        <x:v>CanvasJson luu dung order/lock/visible/style; reload desktop/mobile giu dung UI state va khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="G171" s="5" t="str">
+        <x:v>Pass: build OK; savedTypes=text/rect/text; text Georgia/28/700/#008877; rect fill #123456 stroke #654321 opacity .42 strokeWidth 8 shadow 6/9/18/6 #221100 .5 locked=true; layer3 visible=false; mobile overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H171" s="5" t="str">
+        <x:v>TC_VIZI_162; step 56R</x:v>
+      </x:c>
+      <x:c r="I171" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J171" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K171" s="5" t="str">
+        <x:v>Buoc 56R</x:v>
+      </x:c>
       <x:c r="L171" s="5"/>
       <x:c r="M171" s="5"/>
       <x:c r="N171" s="5"/>
@@ -36322,8 +36351,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b03e4a586c44c2d"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R905b8fb77c324327"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd80d8f4af58d4e43"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b14032c31814cfd"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor image preview
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd23a74b9c8d9436c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4282bf349fbd4287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R2c39daf3808240e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R33fe28d605a949bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>163</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13091,17 +13091,46 @@
       <x:c r="Z171" s="5"/>
     </x:row>
     <x:row r="172">
-      <x:c r="A172" s="5"/>
-      <x:c r="B172" s="24"/>
-      <x:c r="C172" s="5"/>
-      <x:c r="D172" s="5"/>
-      <x:c r="E172" s="5"/>
-      <x:c r="F172" s="24"/>
-      <x:c r="G172" s="5"/>
-      <x:c r="H172" s="5"/>
-      <x:c r="I172" s="5"/>
-      <x:c r="J172" s="5"/>
-      <x:c r="K172" s="5"/>
+      <x:c r="A172" s="5" t="str">
+        <x:v>TC_VIZI_164</x:v>
+      </x:c>
+      <x:c r="B172" s="24" t="str">
+        <x:v>Preview anh upload tren frontend 57</x:v>
+      </x:c>
+      <x:c r="C172" s="5" t="str">
+        <x:v>Xac minh Assets panel cho chon anh local de preview truoc upload, reject file khong an toan, clear duoc va mobile khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="D172" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Browser plugin check page identity/console; fallback Playwright do DOM snapshot runtime loi.
+B3: Tao user/draft tam va mo /editor/{id}.
+B4: Chon file PNG local trong Assets.
+B5: Xac minh preview image dung blob URL, alt/name/size hien dung.
+B6: Chon SVG co script va xac minh bi reject, preview bi xoa.
+B7: Chon PNG lai, bam Clear va xac minh empty state.
+B8: Reload mobile 390x844, chon PNG va kiem tra overflow/console.</x:v>
+      </x:c>
+      <x:c r="E172" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; draft tam #56; PNG 2x2; SVG test co script.</x:v>
+      </x:c>
+      <x:c r="F172" s="24" t="str">
+        <x:v>Anh PNG/JPG/WebP &lt;=5MB co preview truoc upload; SVG/unsupported bi reject; clear duoc; mobile khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="G172" s="5" t="str">
+        <x:v>Pass: build OK; Browser URL/title/logs OK, DOM snapshot loi runtime cu; Playwright desktop preview blob URL preview.png 2x2; SVG reject; Clear ve empty; mobile preview OK, overflow=0; consoleIssues=[].</x:v>
+      </x:c>
+      <x:c r="H172" s="5" t="str">
+        <x:v>TC_VIZI_163; step 57</x:v>
+      </x:c>
+      <x:c r="I172" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J172" s="5" t="n">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K172" s="5" t="str">
+        <x:v>Buoc 57</x:v>
+      </x:c>
       <x:c r="L172" s="5"/>
       <x:c r="M172" s="5"/>
       <x:c r="N172" s="5"/>
@@ -36351,8 +36380,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd80d8f4af58d4e43"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b14032c31814cfd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03412a46724e42a9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11c72116e5414f6c"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add backend image upload endpoint
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R2c39daf3808240e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R33fe28d605a949bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rc81fdc219a09482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R045e2f7372be499e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>164</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13148,17 +13148,46 @@
       <x:c r="Z172" s="5"/>
     </x:row>
     <x:row r="173">
-      <x:c r="A173" s="5"/>
-      <x:c r="B173" s="24"/>
-      <x:c r="C173" s="5"/>
-      <x:c r="D173" s="5"/>
-      <x:c r="E173" s="5"/>
-      <x:c r="F173" s="24"/>
-      <x:c r="G173" s="5"/>
-      <x:c r="H173" s="5"/>
-      <x:c r="I173" s="5"/>
-      <x:c r="J173" s="5"/>
-      <x:c r="K173" s="5"/>
+      <x:c r="A173" s="5" t="str">
+        <x:v>TC_VIZI_165</x:v>
+      </x:c>
+      <x:c r="B173" s="24" t="str">
+        <x:v>Backend upload image API 58</x:v>
+      </x:c>
+      <x:c r="C173" s="5" t="str">
+        <x:v>Xac minh POST /api/uploads/images nhan anh hop le, validate auth/CSRF/MIME/extension/magic bytes/size va tra URL doc duoc.</x:v>
+      </x:c>
+      <x:c r="D173" s="5" t="str">
+        <x:v>B1: Chay focused test ImageUploadApiTests.
+B2: Chay full backend mvnw test.
+B3: Upload PNG bang multipart voi user + CSRF.
+B4: Doc response JSON fileName/contentType/sizeBytes/storageKey/url.
+B5: GET url /uploads/images/{file} voi user.
+B6: Test unauthenticated va thieu CSRF.
+B7: Test reject SVG va fake PNG sai magic bytes.
+B8: Test reject file &gt;5MB.</x:v>
+      </x:c>
+      <x:c r="E173" s="5" t="str">
+        <x:v>Backend MockMvc; H2 test profile; temp upload dir; PNG test; SVG script test; fake PNG; oversized 5MB+1.</x:v>
+      </x:c>
+      <x:c r="F173" s="24" t="str">
+        <x:v>Endpoint luu file local theo config, tra URL /uploads/images/*, auth/CSRF bat buoc, validate upload an toan.</x:v>
+      </x:c>
+      <x:c r="G173" s="5" t="str">
+        <x:v>Pass: ImageUploadApiTests 4/4 pass; full backend test pass 32/32; PNG upload 201 + URL doc duoc; no auth=401, no CSRF=403; SVG/fake PNG/&gt;5MB deu 400; file luu trong temp dir.</x:v>
+      </x:c>
+      <x:c r="H173" s="5" t="str">
+        <x:v>TC_VIZI_164; step 58</x:v>
+      </x:c>
+      <x:c r="I173" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J173" s="5" t="str">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K173" s="5" t="str">
+        <x:v>Buoc 58</x:v>
+      </x:c>
       <x:c r="L173" s="5"/>
       <x:c r="M173" s="5"/>
       <x:c r="N173" s="5"/>
@@ -36380,8 +36409,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03412a46724e42a9"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11c72116e5414f6c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ac1758f884c4753"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R642f8966d9ea4471"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add uploaded images to editor canvas
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rc81fdc219a09482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R045e2f7372be499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re2b8ffc66f904ba1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R86474472824a4cc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>163</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>165</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13205,17 +13205,45 @@
       <x:c r="Z173" s="5"/>
     </x:row>
     <x:row r="174">
-      <x:c r="A174" s="5"/>
-      <x:c r="B174" s="24"/>
-      <x:c r="C174" s="5"/>
-      <x:c r="D174" s="5"/>
-      <x:c r="E174" s="5"/>
-      <x:c r="F174" s="24"/>
-      <x:c r="G174" s="5"/>
-      <x:c r="H174" s="5"/>
-      <x:c r="I174" s="5"/>
-      <x:c r="J174" s="5"/>
-      <x:c r="K174" s="5"/>
+      <x:c r="A174" s="5" t="str">
+        <x:v>TC_VIZI_166</x:v>
+      </x:c>
+      <x:c r="B174" s="24" t="str">
+        <x:v>Them asset anh vao canvas 60</x:v>
+      </x:c>
+      <x:c r="C174" s="5" t="str">
+        <x:v>Xac minh anh preview duoc upload len backend, them thanh image layer vao editor, save/reload va API readback van giu anh.</x:v>
+      </x:c>
+      <x:c r="D174" s="5" t="str">
+        <x:v>B1: Chay npm run build trong frontend.
+B2: Dam bao backend source moi dang chay va /api/uploads/images khong con 404.
+B3: Playwright tao user/draft tam va mo /editor/{designId}.
+B4: Chon PNG hop le trong Assets panel.
+B5: Bam Add to canvas va kiem tra canvas tang them 1 image layer.
+B6: Save draft va doc GET /api/designs/{designId}.
+B7: Reload desktop va mobile 390x844.</x:v>
+      </x:c>
+      <x:c r="E174" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; PNG 2x2; draft tam #59.</x:v>
+      </x:c>
+      <x:c r="F174" s="24" t="str">
+        <x:v>Image upload tra URL backend, image layer render duoc, canvas_json luu type=image/src/storageKey, reload va mobile khong mat anh.</x:v>
+      </x:c>
+      <x:c r="G174" s="5" t="str">
+        <x:v>Pass: build OK; smoke OK; layer count 3-&gt;4; image decoded naturalWidth=2; API readback co type=image va storageKey images/*; reload/mobile giu 1 image layer; console issues empty; mobile overflow 0.</x:v>
+      </x:c>
+      <x:c r="H174" s="5" t="str">
+        <x:v>TC_VIZI_165; step 60</x:v>
+      </x:c>
+      <x:c r="I174" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J174" s="5" t="str">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K174" s="5" t="str">
+        <x:v>Buoc 60</x:v>
+      </x:c>
       <x:c r="L174" s="5"/>
       <x:c r="M174" s="5"/>
       <x:c r="N174" s="5"/>
@@ -36409,8 +36437,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ac1758f884c4753"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R642f8966d9ea4471"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd14ca0366568431e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc18d605c2a464939"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add editor QR preview generation
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re2b8ffc66f904ba1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R86474472824a4cc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R9178889e4d92484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R24fe832f1c664804"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>164</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13261,17 +13261,45 @@
       <x:c r="Z174" s="5"/>
     </x:row>
     <x:row r="175">
-      <x:c r="A175" s="5"/>
-      <x:c r="B175" s="24"/>
-      <x:c r="C175" s="5"/>
-      <x:c r="D175" s="5"/>
-      <x:c r="E175" s="5"/>
-      <x:c r="F175" s="24"/>
-      <x:c r="G175" s="5"/>
-      <x:c r="H175" s="5"/>
-      <x:c r="I175" s="5"/>
-      <x:c r="J175" s="5"/>
-      <x:c r="K175" s="5"/>
+      <x:c r="A175" s="5" t="str">
+        <x:v>TC_VIZI_167</x:v>
+      </x:c>
+      <x:c r="B175" s="24" t="str">
+        <x:v>Tao QR code frontend 61</x:v>
+      </x:c>
+      <x:c r="C175" s="5" t="str">
+        <x:v>Xac minh editor tao QR preview tu text, QR la PNG data URL va co the scan ra dung noi dung.</x:v>
+      </x:c>
+      <x:c r="D175" s="5" t="str">
+        <x:v>B1: npm view qrcode va @types/qrcode de chon version hien tai.
+B2: npm install qrcode@1.5.4 @types/qrcode@1.5.6.
+B3: Chay npm run build.
+B4: Playwright tao user/draft tam va mo /editor/{designId}.
+B5: Nhap QR text va bam Generate QR.
+B6: Doc preview image, lay pixel bang canvas va decode bang jsQR.
+B7: Reload mobile 390x844 va tao QR lai.</x:v>
+      </x:c>
+      <x:c r="E175" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; QR text https://vizi.local/qr/{stamp}; jsQR test-only.</x:v>
+      </x:c>
+      <x:c r="F175" s="24" t="str">
+        <x:v>QR preview hien PNG data URL 256x256, decode scan ra dung QR text, UI khong tran mobile.</x:v>
+      </x:c>
+      <x:c r="G175" s="5" t="str">
+        <x:v>Pass: build OK; QR preview src data:image/png;base64; jsQR rawValue dung bang input; imageSize 256x256; mobile overflow 0; console issues empty.</x:v>
+      </x:c>
+      <x:c r="H175" s="5" t="str">
+        <x:v>TC_VIZI_166; step 61</x:v>
+      </x:c>
+      <x:c r="I175" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J175" s="5" t="str">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K175" s="5" t="str">
+        <x:v>Buoc 61</x:v>
+      </x:c>
       <x:c r="L175" s="5"/>
       <x:c r="M175" s="5"/>
       <x:c r="N175" s="5"/>
@@ -36437,8 +36465,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd14ca0366568431e"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc18d605c2a464939"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32fbdbffe0d44697"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf50a526244c42e0"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Persist QR layers in editor canvas
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R9178889e4d92484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R24fe832f1c664804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd24e62d5f0764ba1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Re5f267f05c30411d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>165</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13317,17 +13317,45 @@
       <x:c r="Z175" s="5"/>
     </x:row>
     <x:row r="176">
-      <x:c r="A176" s="5"/>
-      <x:c r="B176" s="24"/>
-      <x:c r="C176" s="5"/>
-      <x:c r="D176" s="5"/>
-      <x:c r="E176" s="5"/>
-      <x:c r="F176" s="24"/>
-      <x:c r="G176" s="5"/>
-      <x:c r="H176" s="5"/>
-      <x:c r="I176" s="5"/>
-      <x:c r="J176" s="5"/>
-      <x:c r="K176" s="5"/>
+      <x:c r="A176" s="5" t="str">
+        <x:v>TC_VIZI_168</x:v>
+      </x:c>
+      <x:c r="B176" s="24" t="str">
+        <x:v>Luu QR layer trong canvas_json 62</x:v>
+      </x:c>
+      <x:c r="C176" s="5" t="str">
+        <x:v>Xac minh QR preview duoc them thanh layer type=qr, scan duoc tren canvas, save/reload/API readback van giu QR.</x:v>
+      </x:c>
+      <x:c r="D176" s="5" t="str">
+        <x:v>B1: Chay npm run build.
+B2: Playwright tao user/draft tam va mo /editor/{designId}.
+B3: Nhap QR text, Generate QR, Add QR to canvas.
+B4: Decode QR layer tren canvas bang jsQR.
+B5: Save draft va doc GET /api/designs/{designId}.
+B6: Reload desktop va decode QR layer lai.
+B7: Reload mobile 390x844 va decode QR layer lai.</x:v>
+      </x:c>
+      <x:c r="E176" s="5" t="str">
+        <x:v>FE 127.0.0.1:5173; BE 127.0.0.1:8080; Chrome; QR text https://vizi.local/saved-qr/{stamp}; jsQR test-only.</x:v>
+      </x:c>
+      <x:c r="F176" s="24" t="str">
+        <x:v>Canvas co them QR layer, canvas_json luu type=qr/text/src data URL, reload desktop/mobile van scan ra dung QR text.</x:v>
+      </x:c>
+      <x:c r="G176" s="5" t="str">
+        <x:v>Pass: build OK; smoke OK; layer count 3-&gt;4; added/reload/mobile scan dung rawValue; API readback co type=qr, text, src data:image/png;base64; mobile overflow 0; console issues empty.</x:v>
+      </x:c>
+      <x:c r="H176" s="5" t="str">
+        <x:v>TC_VIZI_167; step 62</x:v>
+      </x:c>
+      <x:c r="I176" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J176" s="5" t="str">
+        <x:v>46210</x:v>
+      </x:c>
+      <x:c r="K176" s="5" t="str">
+        <x:v>Buoc 62</x:v>
+      </x:c>
       <x:c r="L176" s="5"/>
       <x:c r="M176" s="5"/>
       <x:c r="N176" s="5"/>
@@ -36465,8 +36493,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32fbdbffe0d44697"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf50a526244c42e0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae7fab4dea84c77"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08f838aacb164484"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add base preflight validation service
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd24e62d5f0764ba1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Re5f267f05c30411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R21dc3ac3999d41bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4d10d8854fab4f9c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13373,17 +13373,44 @@
       <x:c r="Z176" s="5"/>
     </x:row>
     <x:row r="177">
-      <x:c r="A177" s="5"/>
-      <x:c r="B177" s="24"/>
-      <x:c r="C177" s="5"/>
-      <x:c r="D177" s="5"/>
-      <x:c r="E177" s="5"/>
-      <x:c r="F177" s="24"/>
-      <x:c r="G177" s="5"/>
-      <x:c r="H177" s="5"/>
-      <x:c r="I177" s="5"/>
-      <x:c r="J177" s="5"/>
-      <x:c r="K177" s="5"/>
+      <x:c r="A177" s="5" t="str">
+        <x:v>TC_VIZI_169</x:v>
+      </x:c>
+      <x:c r="B177" s="24" t="str">
+        <x:v>Pre-flight service canvas rong 63</x:v>
+      </x:c>
+      <x:c r="C177" s="5" t="str">
+        <x:v>Xac minh PreflightService parse canvas va tra blocking error cho canvas rong hoac JSON khong hop le.</x:v>
+      </x:c>
+      <x:c r="D177" s="5" t="str">
+        <x:v>B1: Tao PreflightIssue, PreflightReport va PreflightService.
+B2: Chay focused PreflightServiceTests.
+B3: Test canvas layers rong tra EMPTY_CANVAS ERROR.
+B4: Test canvas co text layer tra valid=true.
+B5: Test JSON loi tra INVALID_CANVAS ERROR.
+B6: Chay full backend mvnw test.</x:v>
+      </x:c>
+      <x:c r="E177" s="5" t="str">
+        <x:v>Java 21 target; ObjectMapper; canvas 90x54 mm; JSON layers rong, co text layer va JSON bi hong.</x:v>
+      </x:c>
+      <x:c r="F177" s="24" t="str">
+        <x:v>Service tra report valid/issues on dinh; canvas rong va JSON loi bi chan, canvas co layer pass.</x:v>
+      </x:c>
+      <x:c r="G177" s="5" t="str">
+        <x:v>Pass: PreflightServiceTests 3/3; full backend 35/35; EMPTY_CANVAS va INVALID_CANVAS dung code/level; non-empty canvas valid; BUILD SUCCESS.</x:v>
+      </x:c>
+      <x:c r="H177" s="5" t="str">
+        <x:v>TC_VIZI_168; step 63</x:v>
+      </x:c>
+      <x:c r="I177" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J177" s="5" t="str">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K177" s="5" t="str">
+        <x:v>Buoc 63</x:v>
+      </x:c>
       <x:c r="L177" s="5"/>
       <x:c r="M177" s="5"/>
       <x:c r="N177" s="5"/>
@@ -36493,8 +36520,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae7fab4dea84c77"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08f838aacb164484"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra03cecbfb62f4b75"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf92c9bcbe2814798"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add safe zone preflight checks
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R21dc3ac3999d41bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R4d10d8854fab4f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Raad48d0c72714f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R10e94f44dadb4619"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13428,17 +13428,45 @@
       <x:c r="Z177" s="5"/>
     </x:row>
     <x:row r="178">
-      <x:c r="A178" s="5"/>
-      <x:c r="B178" s="24"/>
-      <x:c r="C178" s="5"/>
-      <x:c r="D178" s="5"/>
-      <x:c r="E178" s="5"/>
-      <x:c r="F178" s="24"/>
-      <x:c r="G178" s="5"/>
-      <x:c r="H178" s="5"/>
-      <x:c r="I178" s="5"/>
-      <x:c r="J178" s="5"/>
-      <x:c r="K178" s="5"/>
+      <x:c r="A178" s="5" t="str">
+        <x:v>TC_VIZI_170</x:v>
+      </x:c>
+      <x:c r="B178" s="24" t="str">
+        <x:v>Check layer ngoai safe zone 64</x:v>
+      </x:c>
+      <x:c r="C178" s="5" t="str">
+        <x:v>Xac minh PreflightService dung safe zone 3 mm, text/QR ngoai vung tra ERROR, image tra WARNING va background full-canvas duoc bo qua.</x:v>
+      </x:c>
+      <x:c r="D178" s="5" t="str">
+        <x:v>B1: Them safe-zone rule vao PreflightService.
+B2: Chay focused PreflightServiceTests.
+B3: Test text ngoai safe zone tra ERROR va valid=false.
+B4: Test image ngoai safe zone tra WARNING va valid=true.
+B5: Test rect full-canvas khong bi canh bao.
+B6: Test layer nam trong safe zone pass.
+B7: Chay full backend mvnw test.</x:v>
+      </x:c>
+      <x:c r="E178" s="5" t="str">
+        <x:v>Canvas 90x54 mm; safe zone 3 mm; text x=1/y=1; image x=0/y=0; rect 0/0/100/100; text trong zone.</x:v>
+      </x:c>
+      <x:c r="F178" s="24" t="str">
+        <x:v>Issue code LAYER_OUTSIDE_SAFE_ZONE dung level/layerIndex; blocking chi khi co ERROR; background khong bi false positive.</x:v>
+      </x:c>
+      <x:c r="G178" s="5" t="str">
+        <x:v>Pass: PreflightServiceTests 7/7; full backend 39/39; text outside=ERROR/invalid; image outside=WARNING/valid; full background va inside-zone pass; compiler khong con deprecated warning.</x:v>
+      </x:c>
+      <x:c r="H178" s="5" t="str">
+        <x:v>TC_VIZI_169; step 64</x:v>
+      </x:c>
+      <x:c r="I178" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J178" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K178" s="5" t="str">
+        <x:v>Buoc 64</x:v>
+      </x:c>
       <x:c r="L178" s="5"/>
       <x:c r="M178" s="5"/>
       <x:c r="N178" s="5"/>
@@ -36520,8 +36548,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra03cecbfb62f4b75"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf92c9bcbe2814798"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8c6606057f648bc"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40875894426544e2"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add image resolution preflight checks
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Raad48d0c72714f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R10e94f44dadb4619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R99b53c788add4cc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rf848742bcff0426c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13484,17 +13484,45 @@
       <x:c r="Z178" s="5"/>
     </x:row>
     <x:row r="179">
-      <x:c r="A179" s="5"/>
-      <x:c r="B179" s="24"/>
-      <x:c r="C179" s="5"/>
-      <x:c r="D179" s="5"/>
-      <x:c r="E179" s="5"/>
-      <x:c r="F179" s="24"/>
-      <x:c r="G179" s="5"/>
-      <x:c r="H179" s="5"/>
-      <x:c r="I179" s="5"/>
-      <x:c r="J179" s="5"/>
-      <x:c r="K179" s="5"/>
+      <x:c r="A179" s="5" t="str">
+        <x:v>TC_VIZI_171</x:v>
+      </x:c>
+      <x:c r="B179" s="24" t="str">
+        <x:v>Canh bao anh do phan giai thap 65</x:v>
+      </x:c>
+      <x:c r="C179" s="5" t="str">
+        <x:v>Xac minh image layer luu pixelWidth/pixelHeight va PreflightService tra WARNING LOW_IMAGE_RESOLUTION khi DPI in duoi nguong 150.</x:v>
+      </x:c>
+      <x:c r="D179" s="5" t="str">
+        <x:v>B1: Frontend lay naturalWidth/naturalHeight khi anh preview load.
+B2: Image layer them pixelWidth va pixelHeight khi Add to canvas.
+B3: Backend tinh DPI theo widthMm/heightMm va layer width/height.
+B4: Test anh 100x100 pixel bi WARNING LOW_IMAGE_RESOLUTION.
+B5: Test anh 1200x1200 pixel pass.
+B6: Test image cu thieu metadata khong bi false warning.
+B7: Chay frontend build, focused backend test va full backend test.</x:v>
+      </x:c>
+      <x:c r="E179" s="5" t="str">
+        <x:v>Canvas 90x54 mm; image 40%x40%; metadata 100x100 va 1200x1200; nguong 150 DPI.</x:v>
+      </x:c>
+      <x:c r="F179" s="24" t="str">
+        <x:v>Anh DPI thap tra WARNING nhung valid=true; anh du DPI pass; image cu khong co pixel metadata van tuong thich; frontend build khong loi type.</x:v>
+      </x:c>
+      <x:c r="G179" s="5" t="str">
+        <x:v>Pass: PreflightServiceTests 10/10; full backend 42/42; npm run build OK; LOW_IMAGE_RESOLUTION warning dung cho anh 100x100 va khong chan save.</x:v>
+      </x:c>
+      <x:c r="H179" s="5" t="str">
+        <x:v>TC_VIZI_170; step 65</x:v>
+      </x:c>
+      <x:c r="I179" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J179" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K179" s="5" t="str">
+        <x:v>Buoc 65</x:v>
+      </x:c>
       <x:c r="L179" s="5"/>
       <x:c r="M179" s="5"/>
       <x:c r="N179" s="5"/>
@@ -36548,8 +36576,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8c6606057f648bc"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40875894426544e2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19bce2a7e8b3481c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94118f4d266c4f8c"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add owned design preflight endpoint
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R99b53c788add4cc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rf848742bcff0426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re17e0afd2f254e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R8d6073d4b54b4543"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13540,17 +13540,45 @@
       <x:c r="Z179" s="5"/>
     </x:row>
     <x:row r="180">
-      <x:c r="A180" s="5"/>
-      <x:c r="B180" s="24"/>
-      <x:c r="C180" s="5"/>
-      <x:c r="D180" s="5"/>
-      <x:c r="E180" s="5"/>
-      <x:c r="F180" s="24"/>
-      <x:c r="G180" s="5"/>
-      <x:c r="H180" s="5"/>
-      <x:c r="I180" s="5"/>
-      <x:c r="J180" s="5"/>
-      <x:c r="K180" s="5"/>
+      <x:c r="A180" s="5" t="str">
+        <x:v>TC_VIZI_172</x:v>
+      </x:c>
+      <x:c r="B180" s="24" t="str">
+        <x:v>API pre-flight design 66</x:v>
+      </x:c>
+      <x:c r="C180" s="5" t="str">
+        <x:v>Xac minh POST /api/designs/{id}/preflight dung design cua current user, tra report issues tu PreflightService va chan user khac de tranh IDOR.</x:v>
+      </x:c>
+      <x:c r="D180" s="5" t="str">
+        <x:v>B1: Them endpoint POST /api/designs/{designId}/preflight trong DesignController.
+B2: DesignService lay design bang findByIdAndUser_Id.
+B3: Goi PreflightService voi canvasJson, widthMm va heightMm cua design.
+B4: Integration test owner tao design co text ngoai safe zone.
+B5: Owner POST preflight nhan valid=false va issue LAYER_OUTSIDE_SAFE_ZONE.
+B6: User khac POST cung design nhan 404.
+B7: Chay focused DesignApiIntegrationTests va full backend test.</x:v>
+      </x:c>
+      <x:c r="E180" s="5" t="str">
+        <x:v>User owner@example.test, other@example.test; card 90x54 mm; canvas co text x=1/y=1/w=30/h=10.</x:v>
+      </x:c>
+      <x:c r="F180" s="24" t="str">
+        <x:v>Endpoint tra JSON report valid/issues dung; non-owner/missing design khong lo du lieu; khong tao snapshot hay sua design.</x:v>
+      </x:c>
+      <x:c r="G180" s="5" t="str">
+        <x:v>Pass: DesignApiIntegrationTests 8/8; full backend 43/43; owner preflight OK; other user 404; response co valid=false va LAYER_OUTSIDE_SAFE_ZONE layerIndex=0.</x:v>
+      </x:c>
+      <x:c r="H180" s="5" t="str">
+        <x:v>TC_VIZI_171; step 66</x:v>
+      </x:c>
+      <x:c r="I180" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J180" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K180" s="5" t="str">
+        <x:v>Buoc 66</x:v>
+      </x:c>
       <x:c r="L180" s="5"/>
       <x:c r="M180" s="5"/>
       <x:c r="N180" s="5"/>
@@ -36576,8 +36604,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19bce2a7e8b3481c"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94118f4d266c4f8c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra07f68abf25f4904"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd3d7a22c6954d36"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add checkout print options page
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re17e0afd2f254e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R8d6073d4b54b4543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R02a1ca4f0d514363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Reb3242fab1ff4191"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13596,17 +13596,45 @@
       <x:c r="Z180" s="5"/>
     </x:row>
     <x:row r="181">
-      <x:c r="A181" s="5"/>
-      <x:c r="B181" s="24"/>
-      <x:c r="C181" s="5"/>
-      <x:c r="D181" s="5"/>
-      <x:c r="E181" s="5"/>
-      <x:c r="F181" s="24"/>
-      <x:c r="G181" s="5"/>
-      <x:c r="H181" s="5"/>
-      <x:c r="I181" s="5"/>
-      <x:c r="J181" s="5"/>
-      <x:c r="K181" s="5"/>
+      <x:c r="A181" s="5" t="str">
+        <x:v>TC_VIZI_173</x:v>
+      </x:c>
+      <x:c r="B181" s="24" t="str">
+        <x:v>Trang checkout tuy chon in 67</x:v>
+      </x:c>
+      <x:c r="C181" s="5" t="str">
+        <x:v>Xac minh route /checkout/{designId} load draft hien preview card va cho chon giay, so luong, bo goc; tong tam tinh cap nhat dung.</x:v>
+      </x:c>
+      <x:c r="D181" s="5" t="str">
+        <x:v>B1: Them CheckoutView va route /checkout/:designId.
+B2: Them link Checkout tu editor va draft detail.
+B3: Checkout goi getDesign va render CanvasPreview.
+B4: Chon Linen 300gsm, 500 cards va Rounded corners.
+B5: Kiem tra summary hien dung paper/quantity/rounded corners.
+B6: Kiem tra estimated total = 1.550.000 VND.
+B7: Chay npm run build va Playwright smoke voi API mock.</x:v>
+      </x:c>
+      <x:c r="E181" s="5" t="str">
+        <x:v>FE route /checkout/77; mock design 90x54 mm; paper Linen 300gsm; quantity 500; rounded corners on; mobile 390x844.</x:v>
+      </x:c>
+      <x:c r="F181" s="24" t="str">
+        <x:v>Checkout hien preview, select paper/quantity/rounded corners hoat dong, total tam tinh dung, mobile khong tran ngang, khong console error.</x:v>
+      </x:c>
+      <x:c r="G181" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright checkout smoke OK; totalText=1.550.000 ₫; mobile overflow=0; consoleIssues=[]; Create order disabled vi API order la buoc 68.</x:v>
+      </x:c>
+      <x:c r="H181" s="5" t="str">
+        <x:v>TC_VIZI_172; step 67</x:v>
+      </x:c>
+      <x:c r="I181" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J181" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K181" s="5" t="str">
+        <x:v>Buoc 67</x:v>
+      </x:c>
       <x:c r="L181" s="5"/>
       <x:c r="M181" s="5"/>
       <x:c r="N181" s="5"/>
@@ -36604,8 +36632,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra07f68abf25f4904"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd3d7a22c6954d36"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96ff41f4a25f4aa6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96c89316eede4ebe"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add order creation API
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R02a1ca4f0d514363"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Reb3242fab1ff4191"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R90ad5e06cc2a4268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R65549d8467584ec3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13652,17 +13652,46 @@
       <x:c r="Z181" s="5"/>
     </x:row>
     <x:row r="182">
-      <x:c r="A182" s="5"/>
-      <x:c r="B182" s="24"/>
-      <x:c r="C182" s="5"/>
-      <x:c r="D182" s="5"/>
-      <x:c r="E182" s="5"/>
-      <x:c r="F182" s="24"/>
-      <x:c r="G182" s="5"/>
-      <x:c r="H182" s="5"/>
-      <x:c r="I182" s="5"/>
-      <x:c r="J182" s="5"/>
-      <x:c r="K182" s="5"/>
+      <x:c r="A182" s="5" t="str">
+        <x:v>TC_VIZI_174</x:v>
+      </x:c>
+      <x:c r="B182" s="24" t="str">
+        <x:v>API tao order va order_items 68</x:v>
+      </x:c>
+      <x:c r="C182" s="5" t="str">
+        <x:v>Xac minh POST /api/orders tao order PENDING_PAYMENT va mot order_item tu design cua current user, luu print_config_json va design_snapshot_json.</x:v>
+      </x:c>
+      <x:c r="D182" s="5" t="str">
+        <x:v>B1: Tao package order voi OrderController, OrderService, ViziOrder va OrderItem.
+B2: Owner tao draft tu template.
+B3: POST /api/orders voi paper linen-300, quantity 500, roundedCorners=true.
+B4: Kiem tra response 201, status PENDING_PAYMENT, totalAmount 1550000 va 1 item.
+B5: DB readback order_items co 1 row, snapshot text Order, print_config paper linen-300.
+B6: User khac POST order tren design cua owner nhan 404.
+B7: Paper khong ho tro nhan 400.
+B8: Chay focused OrderApiIntegrationTests va full backend test.</x:v>
+      </x:c>
+      <x:c r="E182" s="5" t="str">
+        <x:v>PostgreSQL local 127.0.0.1:55432; owner@example.test; other@example.test; card 90x54 mm; linen-300; quantity 500; roundedCorners true.</x:v>
+      </x:c>
+      <x:c r="F182" s="24" t="str">
+        <x:v>Order va order_item duoc tao dung; non-owner khong dat hang duoc design cua owner; input paper sai bi chan; khong noi chuoi SQL.</x:v>
+      </x:c>
+      <x:c r="G182" s="5" t="str">
+        <x:v>Pass: OrderApiIntegrationTests 3/3; full backend 46/46; response 201 total=1550000; DB readback order_items=1, snapshot/print_config dung, co widthMm/heightMm; non-owner 404; unsupported paper 400.</x:v>
+      </x:c>
+      <x:c r="H182" s="5" t="str">
+        <x:v>TC_VIZI_173; step 68</x:v>
+      </x:c>
+      <x:c r="I182" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J182" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K182" s="5" t="str">
+        <x:v>Buoc 68</x:v>
+      </x:c>
       <x:c r="L182" s="5"/>
       <x:c r="M182" s="5"/>
       <x:c r="N182" s="5"/>
@@ -36632,8 +36661,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96ff41f4a25f4aa6"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96c89316eede4ebe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865c4e8dea8b469d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R641b91087a8145ab"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Verify order snapshots remain immutable
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R90ad5e06cc2a4268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R65549d8467584ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re5a60edeeb6c494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R86a875e1b70b4d6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13709,17 +13709,44 @@
       <x:c r="Z182" s="5"/>
     </x:row>
     <x:row r="183">
-      <x:c r="A183" s="5"/>
-      <x:c r="B183" s="24"/>
-      <x:c r="C183" s="5"/>
-      <x:c r="D183" s="5"/>
-      <x:c r="E183" s="5"/>
-      <x:c r="F183" s="24"/>
-      <x:c r="G183" s="5"/>
-      <x:c r="H183" s="5"/>
-      <x:c r="I183" s="5"/>
-      <x:c r="J183" s="5"/>
-      <x:c r="K183" s="5"/>
+      <x:c r="A183" s="5" t="str">
+        <x:v>TC_VIZI_175</x:v>
+      </x:c>
+      <x:c r="B183" s="24" t="str">
+        <x:v>Snapshot order khong doi sau khi sua design 69</x:v>
+      </x:c>
+      <x:c r="C183" s="5" t="str">
+        <x:v>Xac minh order_items.design_snapshot_json giu canvas tai thoi diem checkout, du design goc duoc sua sau do.</x:v>
+      </x:c>
+      <x:c r="D183" s="5" t="str">
+        <x:v>B1: Owner tao design tu template co text Original.
+B2: Owner POST /api/orders de tao order.
+B3: Owner PUT /api/designs/{id} doi canvas text thanh Changed.
+B4: DB readback designs.canvas_json da thanh Changed.
+B5: DB readback order_items.design_snapshot_json cua order cu van la Original.
+B6: Chay focused OrderApiIntegrationTests va full backend test.</x:v>
+      </x:c>
+      <x:c r="E183" s="5" t="str">
+        <x:v>PostgreSQL local 127.0.0.1:55432; owner@example.test; canvas Original -&gt; Changed; order tao truoc khi sua design.</x:v>
+      </x:c>
+      <x:c r="F183" s="24" t="str">
+        <x:v>Design hien tai doi duoc nhung snapshot trong order item khong doi; sua design sau checkout khong anh huong don da dat.</x:v>
+      </x:c>
+      <x:c r="G183" s="5" t="str">
+        <x:v>Pass: OrderApiIntegrationTests 4/4; full backend 47/47; designs.canvas_json=Changed; order_items.design_snapshot_json=Original.</x:v>
+      </x:c>
+      <x:c r="H183" s="5" t="str">
+        <x:v>TC_VIZI_174; step 69</x:v>
+      </x:c>
+      <x:c r="I183" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J183" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K183" s="5" t="str">
+        <x:v>Buoc 69</x:v>
+      </x:c>
       <x:c r="L183" s="5"/>
       <x:c r="M183" s="5"/>
       <x:c r="N183" s="5"/>
@@ -36661,8 +36688,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865c4e8dea8b469d"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R641b91087a8145ab"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcccaeea1cda0407e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd215d642d6034daf"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Connect checkout to order creation
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Re5a60edeeb6c494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R86a875e1b70b4d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rc0e3d82c7ad4497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rb893cf06d79a4cc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13764,17 +13764,45 @@
       <x:c r="Z183" s="5"/>
     </x:row>
     <x:row r="184">
-      <x:c r="A184" s="5"/>
-      <x:c r="B184" s="24"/>
-      <x:c r="C184" s="5"/>
-      <x:c r="D184" s="5"/>
-      <x:c r="E184" s="5"/>
-      <x:c r="F184" s="24"/>
-      <x:c r="G184" s="5"/>
-      <x:c r="H184" s="5"/>
-      <x:c r="I184" s="5"/>
-      <x:c r="J184" s="5"/>
-      <x:c r="K184" s="5"/>
+      <x:c r="A184" s="5" t="str">
+        <x:v>TC_VIZI_176</x:v>
+      </x:c>
+      <x:c r="B184" s="24" t="str">
+        <x:v>Checkout tao order va trang order detail 69A-69B</x:v>
+      </x:c>
+      <x:c r="C184" s="5" t="str">
+        <x:v>Xac minh FE checkout goi POST /api/orders bang CSRF, redirect sang /orders/{id}, va trang order detail load lai bang GET /api/orders/{id}.</x:v>
+      </x:c>
+      <x:c r="D184" s="5" t="str">
+        <x:v>B1: Them GET /api/orders/{id} co owner check.
+B2: Them FE createOrder va getOrder trong api client.
+B3: Checkout submit order that va redirect sang order detail.
+B4: Them route /orders/{orderId} va OrderDetailView.
+B5: Integration test owner doc duoc order, user khac nhan 404.
+B6: Chay npm run build, focused backend test, full backend test.
+B7: Playwright smoke mock API: /checkout/77 -&gt; Create order -&gt; /orders/910, desktop/mobile khong overflow.</x:v>
+      </x:c>
+      <x:c r="E184" s="5" t="str">
+        <x:v>Mock API design 77; order 910; total 180000; desktop 1280x900; mobile 390x844; PostgreSQL local cho backend tests.</x:v>
+      </x:c>
+      <x:c r="F184" s="24" t="str">
+        <x:v>Checkout tao order thanh cong; order detail hien status, quantity, total; GET order bi owner-filter; UI khong tran ngang mobile.</x:v>
+      </x:c>
+      <x:c r="G184" s="5" t="str">
+        <x:v>Pass: npm run build OK; OrderApiIntegrationTests 5/5; full backend 48/48; Playwright smoke OK; requests GET design, GET csrf, POST orders, GET order; consoleIssues=[]; desktop/mobile overflow=0.</x:v>
+      </x:c>
+      <x:c r="H184" s="5" t="str">
+        <x:v>TC_VIZI_175; step 69A-69B</x:v>
+      </x:c>
+      <x:c r="I184" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J184" s="5" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="K184" s="5" t="str">
+        <x:v>Buoc 69A-69B</x:v>
+      </x:c>
       <x:c r="L184" s="5"/>
       <x:c r="M184" s="5"/>
       <x:c r="N184" s="5"/>
@@ -36688,8 +36716,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcccaeea1cda0407e"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd215d642d6034daf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb74e125158e4a3c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70291c50b9674e8f"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add Gemini configuration status check
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rc0e3d82c7ad4497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rb893cf06d79a4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R22a82330c0414769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R6c958eaaa7014a7c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13820,17 +13820,45 @@
       <x:c r="Z184" s="5"/>
     </x:row>
     <x:row r="185">
-      <x:c r="A185" s="5"/>
-      <x:c r="B185" s="24"/>
-      <x:c r="C185" s="5"/>
-      <x:c r="D185" s="5"/>
-      <x:c r="E185" s="5"/>
-      <x:c r="F185" s="24"/>
-      <x:c r="G185" s="5"/>
-      <x:c r="H185" s="5"/>
-      <x:c r="I185" s="5"/>
-      <x:c r="J185" s="5"/>
-      <x:c r="K185" s="5"/>
+      <x:c r="A185" s="5" t="str">
+        <x:v>TC_VIZI_177</x:v>
+      </x:c>
+      <x:c r="B185" s="24" t="str">
+        <x:v>Gemini env backend va loi cau hinh buoc 70</x:v>
+      </x:c>
+      <x:c r="C185" s="5" t="str">
+        <x:v>Xac minh backend chi doc GEMINI_API_KEY tu env/property, thieu key tra loi ro, va response khong lo API key.</x:v>
+      </x:c>
+      <x:c r="D185" s="5" t="str">
+        <x:v>B1: Them app.ai.gemini.api-key map tu GEMINI_API_KEY.
+B2: Them text/image model env default cho Gemini Lite.
+B3: Them AiConfigService requireConfigured.
+B4: Them GET /api/ai/status goi config check.
+B5: Test thieu key tra 503 voi message ro.
+B6: Test configured status khong expose secret key.
+B7: Chay focused test va full backend regression.</x:v>
+      </x:c>
+      <x:c r="E185" s="5" t="str">
+        <x:v>Backend test profile; khong can key that; fake key test-secret-key chi dung trong unit test.</x:v>
+      </x:c>
+      <x:c r="F185" s="24" t="str">
+        <x:v>Thieu GEMINI_API_KEY bi chan bang SERVICE_UNAVAILABLE; co key thi status chi tra configured/model, khong tra secret.</x:v>
+      </x:c>
+      <x:c r="G185" s="5" t="str">
+        <x:v>Pass: AiConfigServiceTests 2/2; full backend 50/50; khong them dependency Gemini; secret khong hardcode.</x:v>
+      </x:c>
+      <x:c r="H185" s="5" t="str">
+        <x:v>TC_VIZI_176; step 70</x:v>
+      </x:c>
+      <x:c r="I185" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J185" s="5" t="n">
+        <x:v>46212</x:v>
+      </x:c>
+      <x:c r="K185" s="5" t="str">
+        <x:v>Buoc 70</x:v>
+      </x:c>
       <x:c r="L185" s="5"/>
       <x:c r="M185" s="5"/>
       <x:c r="N185" s="5"/>
@@ -36716,8 +36744,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb74e125158e4a3c"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70291c50b9674e8f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c7b7aa590f84245"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra00790281389410a"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Make editor route full screen
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R22a82330c0414769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R6c958eaaa7014a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rcc3f8b2c94834b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1f65d5cbd1194017"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13876,17 +13876,45 @@
       <x:c r="Z185" s="5"/>
     </x:row>
     <x:row r="186">
-      <x:c r="A186" s="5"/>
-      <x:c r="B186" s="24"/>
-      <x:c r="C186" s="5"/>
-      <x:c r="D186" s="5"/>
-      <x:c r="E186" s="5"/>
-      <x:c r="F186" s="24"/>
-      <x:c r="G186" s="5"/>
-      <x:c r="H186" s="5"/>
-      <x:c r="I186" s="5"/>
-      <x:c r="J186" s="5"/>
-      <x:c r="K186" s="5"/>
+      <x:c r="A186" s="5" t="str">
+        <x:v>TC_VIZI_178</x:v>
+      </x:c>
+      <x:c r="B186" s="24" t="str">
+        <x:v>Editor full-screen workspace 70A</x:v>
+      </x:c>
+      <x:c r="C186" s="5" t="str">
+        <x:v>Xac minh route /editor/:designId dung layout full-screen, an topbar chung, editor shell chiem viewport desktop va khong tran ngang desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="D186" s="5" t="str">
+        <x:v>B1: Them app-shell--editor theo route editor.
+B2: An topbar global tren editor route.
+B3: Ep editor-view full width/min-height 100vh.
+B4: Compact editor header 72px va editor-shell cao calc(100vh - 72px).
+B5: Sidebar scroll rieng, workspace khong tran.
+B6: Build frontend.
+B7: Playwright smoke mock /api/designs/15 desktop 1440x900 va mobile 390x844.</x:v>
+      </x:c>
+      <x:c r="E186" s="5" t="str">
+        <x:v>Mock design 15 co 4 layers; Browser plugin co ket noi nhung fallback Playwright vi can route mock API.</x:v>
+      </x:c>
+      <x:c r="F186" s="24" t="str">
+        <x:v>Desktop: topbarCount=0, app-shell--editor=1, editorShell=1440x828, page scrollHeight=clientHeight=900, overflow ngang 0. Mobile: overflow ngang 0, toolbar 6 nut, layer rows 4.</x:v>
+      </x:c>
+      <x:c r="G186" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke desktopPass=true, mobilePass=true, consoleIssues=[]; screenshots editor-fullscreen-desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="H186" s="5" t="str">
+        <x:v>TC_VIZI_177; step 70A</x:v>
+      </x:c>
+      <x:c r="I186" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J186" s="5" t="n">
+        <x:v>46212</x:v>
+      </x:c>
+      <x:c r="K186" s="5" t="str">
+        <x:v>Buoc 70A</x:v>
+      </x:c>
       <x:c r="L186" s="5"/>
       <x:c r="M186" s="5"/>
       <x:c r="N186" s="5"/>
@@ -36744,8 +36772,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c7b7aa590f84245"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra00790281389410a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R353d15ab25714ded"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2b82cefd4ff4c38"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Apply dark editor sidebars
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rcc3f8b2c94834b01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R1f65d5cbd1194017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R543bffbffc8049df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R01e7552cf33a4552"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13932,17 +13932,43 @@
       <x:c r="Z186" s="5"/>
     </x:row>
     <x:row r="187">
-      <x:c r="A187" s="5"/>
-      <x:c r="B187" s="24"/>
-      <x:c r="C187" s="5"/>
-      <x:c r="D187" s="5"/>
-      <x:c r="E187" s="5"/>
-      <x:c r="F187" s="24"/>
-      <x:c r="G187" s="5"/>
-      <x:c r="H187" s="5"/>
-      <x:c r="I187" s="5"/>
-      <x:c r="J187" s="5"/>
-      <x:c r="K187" s="5"/>
+      <x:c r="A187" s="5" t="str">
+        <x:v>TC_VIZI_179</x:v>
+      </x:c>
+      <x:c r="B187" s="24" t="str">
+        <x:v>Editor dark sidebars luxury 70B</x:v>
+      </x:c>
+      <x:c r="C187" s="5" t="str">
+        <x:v>Xac minh left/right sidebar trong editor route doi sang nen toi luxury, text/control du contrast, workspace giua van sang va khong tran ngang desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="D187" s="5" t="str">
+        <x:v>B1: Them scoped CSS .app-shell--editor cho editor sidebars.
+B2: Doi label, input, layer row, page switch, upload, QR va property controls sang nen toi.
+B3: Giu workspace va card giua mau sang.
+B4: Build frontend.
+B5: Playwright smoke mock /api/designs/15 desktop 1440x900 va mobile 390x844.</x:v>
+      </x:c>
+      <x:c r="E187" s="5" t="str">
+        <x:v>Mock design 15 co 4 layers; Browser plugin co ket noi nhung fallback Playwright vi can route mock API.</x:v>
+      </x:c>
+      <x:c r="F187" s="24" t="str">
+        <x:v>Desktop/mobile: left/right sidebar background rgb(21,22,21), workspace light, control dark, active Front readable, layer rows 4, overflow ngang 0.</x:v>
+      </x:c>
+      <x:c r="G187" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke desktopPass=true, mobilePass=true, consoleIssues=[]; screenshots editor-dark-sidebars-desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="H187" s="5" t="str">
+        <x:v>TC_VIZI_178; step 70B</x:v>
+      </x:c>
+      <x:c r="I187" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J187" s="5" t="n">
+        <x:v>46212</x:v>
+      </x:c>
+      <x:c r="K187" s="5" t="str">
+        <x:v>Buoc 70B</x:v>
+      </x:c>
       <x:c r="L187" s="5"/>
       <x:c r="M187" s="5"/>
       <x:c r="N187" s="5"/>
@@ -36772,8 +36798,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R353d15ab25714ded"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2b82cefd4ff4c38"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b82bc912a74064"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0bf059945974506"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Center editor card workspace
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R543bffbffc8049df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R01e7552cf33a4552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd9b5f35ec32d4d38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R2625a21f11bc4945"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>179</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -13986,17 +13986,43 @@
       <x:c r="Z187" s="5"/>
     </x:row>
     <x:row r="188">
-      <x:c r="A188" s="5"/>
-      <x:c r="B188" s="24"/>
-      <x:c r="C188" s="5"/>
-      <x:c r="D188" s="5"/>
-      <x:c r="E188" s="5"/>
-      <x:c r="F188" s="24"/>
-      <x:c r="G188" s="5"/>
-      <x:c r="H188" s="5"/>
-      <x:c r="I188" s="5"/>
-      <x:c r="J188" s="5"/>
-      <x:c r="K188" s="5"/>
+      <x:c r="A188" s="5" t="str">
+        <x:v>TC_VIZI_180</x:v>
+      </x:c>
+      <x:c r="B188" s="24" t="str">
+        <x:v>Editor center canvas workspace 70C</x:v>
+      </x:c>
+      <x:c r="C188" s="5" t="str">
+        <x:v>Xac minh center canvas cua editor toi uu cho card visit: card nam giua workspace, dung ti le 90/54, co khoang trong voi toolbar/color bar, zoom/pan khong tao tran ngang desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="D188" s="5" t="str">
+        <x:v>B1: Tinh gon nen grid workspace va card shadow.
+B2: Can lai padding editor-canvas-viewport desktop/mobile.
+B3: Thu nhe card mobile de khong sat toolbar/color bar.
+B4: Build frontend.
+B5: Playwright smoke mock /api/designs/15, do center/gap/ratio, zoom/pan desktop 150% va mobile 110%.</x:v>
+      </x:c>
+      <x:c r="E188" s="5" t="str">
+        <x:v>Mock design 15 co 4 layers; desktop 1440x900; mobile 390x844; Browser plugin co nhung dung Playwright fallback vi can route mock API.</x:v>
+      </x:c>
+      <x:c r="F188" s="24" t="str">
+        <x:v>Desktop: centerDeltaX=0, centerDeltaY=0, card ratio 1.6667, toolbar gap 138px, color bar gap 148px, zoom 150% van overflow ngang 0. Mobile: card ratio 1.6667, toolbar gap 21px, color gap 16.98px, zoom 110% van overflow ngang 0.</x:v>
+      </x:c>
+      <x:c r="G188" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke desktopPass=true, mobilePass=true, consoleIssues=[]; screenshots editor-center-canvas-desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="H188" s="5" t="str">
+        <x:v>TC_VIZI_179; step 70C</x:v>
+      </x:c>
+      <x:c r="I188" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J188" s="5" t="n">
+        <x:v>46212</x:v>
+      </x:c>
+      <x:c r="K188" s="5" t="str">
+        <x:v>Buoc 70C</x:v>
+      </x:c>
       <x:c r="L188" s="5"/>
       <x:c r="M188" s="5"/>
       <x:c r="N188" s="5"/>
@@ -36798,8 +36824,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b82bc912a74064"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0bf059945974506"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3199f768e54088"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ead63c862824a5d"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Apply dark editor floating controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rd9b5f35ec32d4d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R2625a21f11bc4945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R4f919ca8e6494e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R6e9b2edd41c04784"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4801,7 +4801,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -4815,7 +4815,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>180</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="H5" s="36"/>
       <x:c r="I5" s="37"/>
@@ -14040,17 +14040,42 @@
       <x:c r="Z188" s="5"/>
     </x:row>
     <x:row r="189">
-      <x:c r="A189" s="5"/>
-      <x:c r="B189" s="24"/>
-      <x:c r="C189" s="5"/>
-      <x:c r="D189" s="5"/>
-      <x:c r="E189" s="5"/>
-      <x:c r="F189" s="24"/>
-      <x:c r="G189" s="5"/>
-      <x:c r="H189" s="5"/>
-      <x:c r="I189" s="5"/>
-      <x:c r="J189" s="5"/>
-      <x:c r="K189" s="5"/>
+      <x:c r="A189" s="5" t="str">
+        <x:v>TC_VIZI_181</x:v>
+      </x:c>
+      <x:c r="B189" s="24" t="str">
+        <x:v>Editor dark floating controls 70D</x:v>
+      </x:c>
+      <x:c r="C189" s="5" t="str">
+        <x:v>Xac minh toolbar, zoom controls va quick color bar trong editor route chuyen sang dark floating UI, active state doc duoc va khong che card visit o trang thai mac dinh desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="D189" s="5" t="str">
+        <x:v>B1: Them scoped CSS .app-shell--editor cho editor-toolbar, editor-zoom-controls va editor-color-bar.
+B2: Doi active tool va active color target sang nen ivory de doc ro tren panel toi.
+B3: Build frontend.
+B4: Playwright smoke mock /api/designs/15, do mau nen, contrast co ban, khoang cach voi card va overflow desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="E189" s="5" t="str">
+        <x:v>Mock design 15 co 4 layers; desktop 1440x900; mobile 390x844; Browser plugin co nhung dung Playwright fallback vi can route mock API.</x:v>
+      </x:c>
+      <x:c r="F189" s="24" t="str">
+        <x:v>Desktop/mobile: toolbar/zoom/color bar background rgb(21,22,21), active tool/Fill nen rgb(248,243,231), toolbar buttons 6, overflow ngang 0. Desktop gap toolbar-card 138px, color-card 148px. Mobile gap toolbar-card 21px, color-card 16.98px.</x:v>
+      </x:c>
+      <x:c r="G189" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke desktopPass=true, mobilePass=true, consoleIssues=[]; screenshots editor-dark-floating-bars-desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="H189" s="5" t="str">
+        <x:v>TC_VIZI_180; step 70D</x:v>
+      </x:c>
+      <x:c r="I189" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J189" s="5" t="n">
+        <x:v>46212</x:v>
+      </x:c>
+      <x:c r="K189" s="5" t="str">
+        <x:v>Buoc 70D</x:v>
+      </x:c>
       <x:c r="L189" s="5"/>
       <x:c r="M189" s="5"/>
       <x:c r="N189" s="5"/>
@@ -36824,8 +36849,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3199f768e54088"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ead63c862824a5d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8116a341b1a46c4"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f73eab5d9684177"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add test-safe Gemini client
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -1049,7 +1049,7 @@
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>0</v>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F5" s="40" t="n"/>
       <c r="G5" s="35" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H5" s="36" t="n"/>
       <c r="I5" s="37" t="n"/>
@@ -14484,32 +14484,81 @@
       <c r="Z191" s="43" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="5" t="n"/>
-      <c r="B192" s="24" t="n"/>
-      <c r="C192" s="5" t="n"/>
-      <c r="D192" s="5" t="n"/>
-      <c r="E192" s="5" t="n"/>
-      <c r="F192" s="24" t="n"/>
-      <c r="G192" s="5" t="n"/>
-      <c r="H192" s="5" t="n"/>
-      <c r="I192" s="5" t="n"/>
-      <c r="J192" s="5" t="n"/>
-      <c r="K192" s="5" t="n"/>
-      <c r="L192" s="5" t="n"/>
-      <c r="M192" s="5" t="n"/>
-      <c r="N192" s="5" t="n"/>
-      <c r="O192" s="5" t="n"/>
-      <c r="P192" s="5" t="n"/>
-      <c r="Q192" s="5" t="n"/>
-      <c r="R192" s="5" t="n"/>
-      <c r="S192" s="5" t="n"/>
-      <c r="T192" s="5" t="n"/>
-      <c r="U192" s="5" t="n"/>
-      <c r="V192" s="5" t="n"/>
-      <c r="W192" s="5" t="n"/>
-      <c r="X192" s="5" t="n"/>
-      <c r="Y192" s="5" t="n"/>
-      <c r="Z192" s="5" t="n"/>
+      <c r="A192" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_184</t>
+        </is>
+      </c>
+      <c r="B192" s="67" t="inlineStr">
+        <is>
+          <t>GeminiClient backend test-safe 71</t>
+        </is>
+      </c>
+      <c r="C192" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh backend co GeminiClient goi generateContent qua JDK HttpClient, doc key tu env/config, unit test bang fake HTTP server va khong goi Gemini that.</t>
+        </is>
+      </c>
+      <c r="D192" s="43" t="inlineStr">
+        <is>
+          <t>B1: Them Spring Boot JSON starter cho Jackson 3 namespace tools.jackson.
+B2: Them GEMINI_BASE_URL de test/mock server local.
+B3: Them GeminiClient.generateText(prompt) dung AiConfigService.requireGeminiApiKey() va text model config.
+B4: Unit test fake Gemini server kiem tra path/query/body va parse candidates[].content.parts[].text.
+B5: Test missing key dung 503 va response rong dung 502.
+B6: Chay AI tests va full backend test.</t>
+        </is>
+      </c>
+      <c r="E192" s="43" t="inlineStr">
+        <is>
+          <t>Khong dung API key that; key test chi la chuoi gia lap. Local PostgreSQL test cluster kha dung.</t>
+        </is>
+      </c>
+      <c r="F192" s="67" t="inlineStr">
+        <is>
+          <t>AI tests pass 5/5; full backend test pass 53/53; GeminiClient khong hardcode secret va khong expose key qua status API.</t>
+        </is>
+      </c>
+      <c r="G192" s="43" t="inlineStr">
+        <is>
+          <t>Pass: .\mvnw.cmd "-Dtest=AiConfigServiceTests,GeminiClientTests" test OK; .\mvnw.cmd test OK.</t>
+        </is>
+      </c>
+      <c r="H192" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_183; step 71</t>
+        </is>
+      </c>
+      <c r="I192" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J192" s="43" t="inlineStr">
+        <is>
+          <t>46212</t>
+        </is>
+      </c>
+      <c r="K192" s="43" t="inlineStr">
+        <is>
+          <t>Buoc 71</t>
+        </is>
+      </c>
+      <c r="L192" s="43" t="n"/>
+      <c r="M192" s="43" t="n"/>
+      <c r="N192" s="43" t="n"/>
+      <c r="O192" s="43" t="n"/>
+      <c r="P192" s="43" t="n"/>
+      <c r="Q192" s="43" t="n"/>
+      <c r="R192" s="43" t="n"/>
+      <c r="S192" s="43" t="n"/>
+      <c r="T192" s="43" t="n"/>
+      <c r="U192" s="43" t="n"/>
+      <c r="V192" s="43" t="n"/>
+      <c r="W192" s="43" t="n"/>
+      <c r="X192" s="43" t="n"/>
+      <c r="Y192" s="43" t="n"/>
+      <c r="Z192" s="43" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>

</xml_diff>

<commit_message>
Add AI usage logging
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R33f819186ad7488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rcf68308a9cc94635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R73c612a644d44809"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R43b075871aa04b24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>183</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14621,21 +14621,48 @@
       <x:c r="Z193" s="5" t="n"/>
     </x:row>
     <x:row r="194">
-      <x:c r="A194" s="5" t="n"/>
-      <x:c r="B194" s="24" t="n"/>
-      <x:c r="C194" s="5" t="n"/>
-      <x:c r="D194" s="5" t="n"/>
-      <x:c r="E194" s="5" t="n"/>
-      <x:c r="F194" s="24" t="n"/>
-      <x:c r="G194" s="5" t="n"/>
-      <x:c r="H194" s="5" t="n"/>
-      <x:c r="I194" s="5" t="n"/>
-      <x:c r="J194" s="5" t="n"/>
-      <x:c r="K194" s="5" t="n"/>
-      <x:c r="L194" s="5" t="n"/>
-      <x:c r="M194" s="5" t="n"/>
-      <x:c r="N194" s="5" t="n"/>
-      <x:c r="O194" s="5" t="n"/>
+      <x:c r="A194" s="5" t="str">
+        <x:v>TC_VIZI_186</x:v>
+      </x:c>
+      <x:c r="B194" s="24" t="str">
+        <x:v>AI usage logs 72</x:v>
+      </x:c>
+      <x:c r="C194" s="5" t="str">
+        <x:v>Xac minh moi lan GeminiClient xu ly request hop le deu ghi feature/model/status/latency/error code vao ai_usage_logs ma khong luu prompt, response hoac API key.</x:v>
+      </x:c>
+      <x:c r="D194" s="5" t="str">
+        <x:v>B1: Tao Flyway V2 cho ai_usage_logs va index user/time.
+B2: Tao JPA entity/repository/service voi transaction rieng.
+B3: Ghi SUCCESS sau response hop le va FAILED cho loi config/upstream.
+B4: Unit test fake Gemini server va verify log success/failure.
+B5: Integration test H2 doc lai metadata, kiem tra khong co cot prompt/key.
+B6: Khoi dong PostgreSQL local, chay full backend test va Flyway migration V1-V2.</x:v>
+      </x:c>
+      <x:c r="E194" s="5" t="str">
+        <x:v>Khong goi Gemini that; fake HTTP server va key gia lap trong test; PostgreSQL 17 local chay port project 55432.</x:v>
+      </x:c>
+      <x:c r="F194" s="24" t="str">
+        <x:v>V2 tao bang/index dung; success va failure deu co status/latency; schema khong co prompt/response/api_key; Flyway ap dung sach tren PostgreSQL.</x:v>
+      </x:c>
+      <x:c r="G194" s="5" t="str">
+        <x:v>Pass: AI/migration tests 9 discovered, 8 pass va 1 skip truoc khi start PostgreSQL; sau khi start PostgreSQL, full backend 55/55 pass, 0 skip; Flyway applied V1-V2.</x:v>
+      </x:c>
+      <x:c r="H194" s="5" t="str">
+        <x:v>TC_VIZI_185; step 72</x:v>
+      </x:c>
+      <x:c r="I194" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J194" s="5" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K194" s="5" t="str">
+        <x:v>Buoc 72</x:v>
+      </x:c>
+      <x:c r="L194" s="5"/>
+      <x:c r="M194" s="5"/>
+      <x:c r="N194" s="5"/>
+      <x:c r="O194" s="5"/>
       <x:c r="P194" s="5" t="n"/>
       <x:c r="Q194" s="5" t="n"/>
       <x:c r="R194" s="5" t="n"/>
@@ -37265,7 +37292,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R009b024ede394e04"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1210bb44e96448d5"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add AI patch schema validation
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R73c612a644d44809"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R43b075871aa04b24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rac65b41d45d64c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc620303d84724194"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>186</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14676,21 +14676,47 @@
       <x:c r="Z194" s="5" t="n"/>
     </x:row>
     <x:row r="195">
-      <x:c r="A195" s="5" t="n"/>
-      <x:c r="B195" s="24" t="n"/>
-      <x:c r="C195" s="5" t="n"/>
-      <x:c r="D195" s="5" t="n"/>
-      <x:c r="E195" s="5" t="n"/>
-      <x:c r="F195" s="24" t="n"/>
-      <x:c r="G195" s="5" t="n"/>
-      <x:c r="H195" s="5" t="n"/>
-      <x:c r="I195" s="5" t="n"/>
-      <x:c r="J195" s="5" t="n"/>
-      <x:c r="K195" s="5" t="n"/>
-      <x:c r="L195" s="5" t="n"/>
-      <x:c r="M195" s="5" t="n"/>
-      <x:c r="N195" s="5" t="n"/>
-      <x:c r="O195" s="5" t="n"/>
+      <x:c r="A195" s="5" t="str">
+        <x:v>TC_VIZI_187</x:v>
+      </x:c>
+      <x:c r="B195" s="24" t="str">
+        <x:v>AI JSON patch schema 73</x:v>
+      </x:c>
+      <x:c r="C195" s="5" t="str">
+        <x:v>Xac minh parser DTO/schema JSON patch chi nhan root/action fields hop le, version va enum dung; JSON sai schema bi reject truoc khi den buoc whitelist action.</x:v>
+      </x:c>
+      <x:c r="D195" s="5" t="str">
+        <x:v>B1: Dinh nghia AiPatch, editStrength, targetSide va action fields cho text/style/geometry.
+B2: Parser kiem tra root fields, schemaVersion=1, action count va layerId format.
+B3: Reject field la, root thieu, version/enum sai, action khong co thay doi.
+B4: Cho phep op chua whitelist nhung co cau truc dung; whitelist de buoc 74 xu ly.
+B5: Chay unit tests va full backend regression tren PostgreSQL local.</x:v>
+      </x:c>
+      <x:c r="E195" s="5" t="str">
+        <x:v>JSON test gia lap; khong goi Gemini that; PostgreSQL 17 local project cluster dang chay.</x:v>
+      </x:c>
+      <x:c r="F195" s="24" t="str">
+        <x:v>Patch hop le parse thanh DTO; JSON sai schema tra IllegalArgumentException; field HTML/code la bi reject; action la chua bi whitelist o buoc nay.</x:v>
+      </x:c>
+      <x:c r="G195" s="5" t="str">
+        <x:v>Pass: AiPatchSchemaTests 3/3; full backend 58/58 pass, 0 skip; PostgreSQL Flyway V1-V2 van pass.</x:v>
+      </x:c>
+      <x:c r="H195" s="5" t="str">
+        <x:v>TC_VIZI_186; step 73</x:v>
+      </x:c>
+      <x:c r="I195" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J195" s="5" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K195" s="5" t="str">
+        <x:v>Buoc 73</x:v>
+      </x:c>
+      <x:c r="L195" s="5"/>
+      <x:c r="M195" s="5"/>
+      <x:c r="N195" s="5"/>
+      <x:c r="O195" s="5"/>
       <x:c r="P195" s="5" t="n"/>
       <x:c r="Q195" s="5" t="n"/>
       <x:c r="R195" s="5" t="n"/>
@@ -37292,7 +37318,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1210bb44e96448d5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdab3900d917343f6"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Validate AI patch actions
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rac65b41d45d64c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rc620303d84724194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb18e374a68bf4239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R273ffdc820834bdb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>187</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14730,21 +14730,47 @@
       <x:c r="Z195" s="5" t="n"/>
     </x:row>
     <x:row r="196">
-      <x:c r="A196" s="5" t="n"/>
-      <x:c r="B196" s="24" t="n"/>
-      <x:c r="C196" s="5" t="n"/>
-      <x:c r="D196" s="5" t="n"/>
-      <x:c r="E196" s="5" t="n"/>
-      <x:c r="F196" s="24" t="n"/>
-      <x:c r="G196" s="5" t="n"/>
-      <x:c r="H196" s="5" t="n"/>
-      <x:c r="I196" s="5" t="n"/>
-      <x:c r="J196" s="5" t="n"/>
-      <x:c r="K196" s="5" t="n"/>
-      <x:c r="L196" s="5" t="n"/>
-      <x:c r="M196" s="5" t="n"/>
-      <x:c r="N196" s="5" t="n"/>
-      <x:c r="O196" s="5" t="n"/>
+      <x:c r="A196" s="5" t="str">
+        <x:v>TC_VIZI_188</x:v>
+      </x:c>
+      <x:c r="B196" s="24" t="str">
+        <x:v>AI patch whitelist and layer target validation 74</x:v>
+      </x:c>
+      <x:c r="C196" s="5" t="str">
+        <x:v>Xac minh AI patch chi duoc phep dung action whitelist, chi sua layer ton tai, va add/remove layer chi khi endpoint da xac nhan co lenh ro rang cua nguoi dung.</x:v>
+      </x:c>
+      <x:c r="D196" s="5" t="str">
+        <x:v>B1: Parse canvas layers va uu tien id on dinh; layer cu khong co id dung layer-1, layer-2 theo vi tri.
+B2: Reject operation la, layerId khong ton tai, duplicate layer id va geometry vuot kho card.
+B3: Chi cho update_text/fill/stroke/font/geometry dung dung fields va range UI.
+B4: add_layer/remove_layer can explicit permission; add chi cho text/rect/shape, khong HTML/URL/image, va phai nam trong card.
+B5: Chay unit tests va full backend regression tren PostgreSQL local.</x:v>
+      </x:c>
+      <x:c r="E196" s="5" t="str">
+        <x:v>JSON test gia lap; khong goi Gemini that; PostgreSQL 17 local project cluster dang chay.</x:v>
+      </x:c>
+      <x:c r="F196" s="24" t="str">
+        <x:v>Patch hop le dung layer muc tieu; action hoac layer sai bi reject; them/xoa layer khong co explicit permission bi reject; layer moi khong the vuot kho card hoac chua HTML/field la.</x:v>
+      </x:c>
+      <x:c r="G196" s="5" t="str">
+        <x:v>Pass: AiPatchSchemaTests + AiPatchValidatorTests 8/8; full backend regression pass tren PostgreSQL local.</x:v>
+      </x:c>
+      <x:c r="H196" s="5" t="str">
+        <x:v>TC_VIZI_187; step 74</x:v>
+      </x:c>
+      <x:c r="I196" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J196" s="5" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K196" s="5" t="str">
+        <x:v>Buoc 74</x:v>
+      </x:c>
+      <x:c r="L196" s="5"/>
+      <x:c r="M196" s="5"/>
+      <x:c r="N196" s="5"/>
+      <x:c r="O196" s="5"/>
       <x:c r="P196" s="5" t="n"/>
       <x:c r="Q196" s="5" t="n"/>
       <x:c r="R196" s="5" t="n"/>
@@ -37318,7 +37344,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdab3900d917343f6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1497c665d724a7d"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add AI text rewrite preview API
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb18e374a68bf4239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R273ffdc820834bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb8aa2782686847d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Ra968ac4ab79743e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>186</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>188</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14784,21 +14784,48 @@
       <x:c r="Z196" s="5" t="n"/>
     </x:row>
     <x:row r="197">
-      <x:c r="A197" s="5" t="n"/>
-      <x:c r="B197" s="24" t="n"/>
-      <x:c r="C197" s="5" t="n"/>
-      <x:c r="D197" s="5" t="n"/>
-      <x:c r="E197" s="5" t="n"/>
-      <x:c r="F197" s="24" t="n"/>
-      <x:c r="G197" s="5" t="n"/>
-      <x:c r="H197" s="5" t="n"/>
-      <x:c r="I197" s="5" t="n"/>
-      <x:c r="J197" s="5" t="n"/>
-      <x:c r="K197" s="5" t="n"/>
-      <x:c r="L197" s="5" t="n"/>
-      <x:c r="M197" s="5" t="n"/>
-      <x:c r="N197" s="5" t="n"/>
-      <x:c r="O197" s="5" t="n"/>
+      <x:c r="A197" s="5" t="str">
+        <x:v>TC_VIZI_189</x:v>
+      </x:c>
+      <x:c r="B197" s="24" t="str">
+        <x:v>AI text rewrite API 75</x:v>
+      </x:c>
+      <x:c r="C197" s="5" t="str">
+        <x:v>Xac minh POST /api/ai/text/rewrite chi tao preview JSON patch update_text cho layer text thuoc design cua current user, khong ghi de canvas.</x:v>
+      </x:c>
+      <x:c r="D197" s="5" t="str">
+        <x:v>B1: Tao request designId/layerId/prompt/editStrength/targetSide co validation.
+B2: Doc current text tu owned canvas, khong tin currentText tu client.
+B3: Goi fake Gemini va parse schema JSON patch.
+B4: Chi chap nhan dung 1 update_text dung layer, strength va side; output sai tra 502.
+B5: Test auth/CSRF/IDOR, canvas khong doi, usage feature text.rewrite.
+B6: Chay focused va full backend regression tren H2/PostgreSQL local.</x:v>
+      </x:c>
+      <x:c r="E197" s="5" t="str">
+        <x:v>Fake Gemini HTTP server noi bo; khong goi Gemini that; H2 cho endpoint test; PostgreSQL 17 local cho full regression.</x:v>
+      </x:c>
+      <x:c r="F197" s="24" t="str">
+        <x:v>Owner + CSRF nhan patch preview; thieu CSRF bi 403; non-owner bi 404; model tra action sai bi 502; design canvas khong bi cap nhat.</x:v>
+      </x:c>
+      <x:c r="G197" s="5" t="str">
+        <x:v>Pass: AiTextRewriteApiIntegrationTests 4/4; focused AI tests 12/12; full backend 67/67 pass, 0 skip; PostgreSQL Flyway V1-V2 pass.</x:v>
+      </x:c>
+      <x:c r="H197" s="5" t="str">
+        <x:v>TC_VIZI_188; step 75</x:v>
+      </x:c>
+      <x:c r="I197" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J197" s="5" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K197" s="5" t="str">
+        <x:v>Buoc 75</x:v>
+      </x:c>
+      <x:c r="L197" s="5"/>
+      <x:c r="M197" s="5"/>
+      <x:c r="N197" s="5"/>
+      <x:c r="O197" s="5"/>
       <x:c r="P197" s="5" t="n"/>
       <x:c r="Q197" s="5" t="n"/>
       <x:c r="R197" s="5" t="n"/>
@@ -37344,7 +37371,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1497c665d724a7d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495c1967f8444a50"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add AI rewrite preview workflow
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb8aa2782686847d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Ra968ac4ab79743e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R75996d05313140ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R2216517029234a24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>187</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14839,21 +14839,49 @@
       <x:c r="Z197" s="5" t="n"/>
     </x:row>
     <x:row r="198">
-      <x:c r="A198" s="5" t="n"/>
-      <x:c r="B198" s="24" t="n"/>
-      <x:c r="C198" s="5" t="n"/>
-      <x:c r="D198" s="5" t="n"/>
-      <x:c r="E198" s="5" t="n"/>
-      <x:c r="F198" s="24" t="n"/>
-      <x:c r="G198" s="5" t="n"/>
-      <x:c r="H198" s="5" t="n"/>
-      <x:c r="I198" s="5" t="n"/>
-      <x:c r="J198" s="5" t="n"/>
-      <x:c r="K198" s="5" t="n"/>
-      <x:c r="L198" s="5" t="n"/>
-      <x:c r="M198" s="5" t="n"/>
-      <x:c r="N198" s="5" t="n"/>
-      <x:c r="O198" s="5" t="n"/>
+      <x:c r="A198" s="5" t="str">
+        <x:v>TC_VIZI_190</x:v>
+      </x:c>
+      <x:c r="B198" s="24" t="str">
+        <x:v>AI text rewrite preview 76</x:v>
+      </x:c>
+      <x:c r="C198" s="5" t="str">
+        <x:v>Xac minh Editor chi hien preview AI rewrite truoc, canvas khong doi cho den khi nguoi dung bam Apply; Reject giu nguyen va Apply co the Undo.</x:v>
+      </x:c>
+      <x:c r="D198" s="5" t="str">
+        <x:v>B1: Chon mot text layer trong Editor.
+B2: Nhap yeu cau rewrite va chon edit strength.
+B3: Mock CSRF + POST /api/ai/text/rewrite, kiem tra request payload.
+B4: Xac minh Current/Proposed hien ra nhung canvas van giu text cu.
+B5: Bam Reject va xac minh canvas khong doi.
+B6: Tao preview lai, bam Apply va xac minh canvas doi; bam Undo de khoi phuc.
+B7: Chay unit test helper, frontend build, desktop/mobile smoke va console check.</x:v>
+      </x:c>
+      <x:c r="E198" s="5" t="str">
+        <x:v>Mock design 76 co rect + text layer id company-name; API tra update_text tu Vizi Atelier thanh Vizi Maison; desktop va mobile 390x844.</x:v>
+      </x:c>
+      <x:c r="F198" s="24" t="str">
+        <x:v>Preview khong mutate canvas; Reject khong doi layer; Apply chi sua dung text layer, tao undo history; request co CSRF va khong co secret o FE.</x:v>
+      </x:c>
+      <x:c r="G198" s="5" t="str">
+        <x:v>Pass: helper unit tests 2/2; npm run build OK; Playwright Preview/Reject/Apply/Undo OK; payload va X-XSRF-TOKEN dung; mobile overflow=0; console errors=0.</x:v>
+      </x:c>
+      <x:c r="H198" s="5" t="str">
+        <x:v>TC_VIZI_189; step 76</x:v>
+      </x:c>
+      <x:c r="I198" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J198" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K198" s="5" t="str">
+        <x:v>Buoc 76</x:v>
+      </x:c>
+      <x:c r="L198" s="5"/>
+      <x:c r="M198" s="5"/>
+      <x:c r="N198" s="5"/>
+      <x:c r="O198" s="5"/>
       <x:c r="P198" s="5" t="n"/>
       <x:c r="Q198" s="5" t="n"/>
       <x:c r="R198" s="5" t="n"/>
@@ -37371,7 +37399,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495c1967f8444a50"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R307264f234464894"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Improve editor toolbar and layer panel
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R75996d05313140ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R2216517029234a24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R9f9bc85920104bc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rff6915f3729542c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>188</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1062,13 +1062,13 @@
       <x:c r="C5" s="39" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="40" t="n"/>
+      <x:c r="D5" s="40"/>
       <x:c r="E5" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F5" s="40" t="n"/>
+      <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14895,17 +14895,44 @@
       <x:c r="Z198" s="5" t="n"/>
     </x:row>
     <x:row r="199">
-      <x:c r="A199" s="5" t="n"/>
-      <x:c r="B199" s="24" t="n"/>
-      <x:c r="C199" s="5" t="n"/>
-      <x:c r="D199" s="5" t="n"/>
-      <x:c r="E199" s="5" t="n"/>
-      <x:c r="F199" s="24" t="n"/>
-      <x:c r="G199" s="5" t="n"/>
-      <x:c r="H199" s="5" t="n"/>
-      <x:c r="I199" s="5" t="n"/>
-      <x:c r="J199" s="5" t="n"/>
-      <x:c r="K199" s="5" t="n"/>
+      <x:c r="A199" s="5" t="str">
+        <x:v>TC_VIZI_191</x:v>
+      </x:c>
+      <x:c r="B199" s="24" t="str">
+        <x:v>Editor toolbar and layer panel 77</x:v>
+      </x:c>
+      <x:c r="C199" s="5" t="str">
+        <x:v>Xac minh toolbar tao layer khi click canvas, layer panel hien top-first, an/khoa nam tren row, sap xep bang drag/drop va menu chuot phai co hanh dong co ban.</x:v>
+      </x:c>
+      <x:c r="D199" s="5" t="str">
+        <x:v>B1: Build frontend.
+B2: Mock API design 15 co 4 layer.
+B3: Click Text tool roi click canvas.
+B4: Click Shape tool roi click canvas.
+B5: Kiem tra layer row, so thu tu tren cung, hide/lock inline, khong con nut up/down inline.
+B6: Right-click layer va kiem tra context menu Copy/Delete/Rename/Move up/Move down.</x:v>
+      </x:c>
+      <x:c r="E199" s="5" t="str">
+        <x:v>Mock design 15 co 4 layers; Playwright route API; frontend dev server 127.0.0.1:5174; backend API base 127.0.0.1:8080.</x:v>
+      </x:c>
+      <x:c r="F199" s="24" t="str">
+        <x:v>Text/Shape tool tao layer moi tai canvas; row tren cung danh so 1; moi row co hide/lock; khong hien up/down inline; right-click hien menu action co ban; drag/drop doi thu tu layer; khong co console error.</x:v>
+      </x:c>
+      <x:c r="G199" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke rows=6, firstNumber=1, firstHide=1, firstLock=1; context menu actions visible; drag/drop changed top order Accent -&gt; Role; no console errors in current run.</x:v>
+      </x:c>
+      <x:c r="H199" s="5" t="str">
+        <x:v>TC_VIZI_190; step 77</x:v>
+      </x:c>
+      <x:c r="I199" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J199" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K199" s="5" t="str">
+        <x:v>Buoc 77 bugfix</x:v>
+      </x:c>
       <x:c r="L199" s="5" t="n"/>
       <x:c r="M199" s="5" t="n"/>
       <x:c r="N199" s="5" t="n"/>
@@ -37399,7 +37426,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R307264f234464894"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942e30471e9e47f7"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Clean up editor layer menu markup
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R9f9bc85920104bc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rff6915f3729542c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R67939d236ad04f3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R53bcef50f4ec4855"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -14950,17 +14950,43 @@
       <x:c r="Z199" s="5" t="n"/>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" s="5" t="n"/>
-      <x:c r="B200" s="24" t="n"/>
-      <x:c r="C200" s="5" t="n"/>
-      <x:c r="D200" s="5" t="n"/>
-      <x:c r="E200" s="5" t="n"/>
-      <x:c r="F200" s="24" t="n"/>
-      <x:c r="G200" s="5" t="n"/>
-      <x:c r="H200" s="5" t="n"/>
-      <x:c r="I200" s="5" t="n"/>
-      <x:c r="J200" s="5" t="n"/>
-      <x:c r="K200" s="5" t="n"/>
+      <x:c r="A200" s="5" t="str">
+        <x:v>TC_VIZI_192</x:v>
+      </x:c>
+      <x:c r="B200" s="24" t="str">
+        <x:v>Editor context menu markup cleanup 78</x:v>
+      </x:c>
+      <x:c r="C200" s="5" t="str">
+        <x:v>Xac minh template Editor khong con hien literal newline marker sau context menu layer va menu chuot phai van hoat dong.</x:v>
+      </x:c>
+      <x:c r="D200" s="5" t="str">
+        <x:v>B1: Sua template context menu layer de tach dong that.
+B2: Build frontend.
+B3: Mock design /editor/15 bang Playwright.
+B4: Kiem tra body khong co literal marker.
+B5: Right-click layer va kiem tra menu Rename hien thi.</x:v>
+      </x:c>
+      <x:c r="E200" s="5" t="str">
+        <x:v>Mock design 15 co 3 layers; frontend dev server 127.0.0.1:5174; backend API base 127.0.0.1:8080.</x:v>
+      </x:c>
+      <x:c r="F200" s="24" t="str">
+        <x:v>DOM khong hien marker `r`n; context menu layer van hien va khong co console error.</x:v>
+      </x:c>
+      <x:c r="G200" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke noLiteralMarker=true, menuVisible=true; console errors=0.</x:v>
+      </x:c>
+      <x:c r="H200" s="5" t="str">
+        <x:v>TC_VIZI_191; step 78 bugfix</x:v>
+      </x:c>
+      <x:c r="I200" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J200" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K200" s="5" t="str">
+        <x:v>Buoc 78 bugfix</x:v>
+      </x:c>
       <x:c r="L200" s="5" t="n"/>
       <x:c r="M200" s="5" t="n"/>
       <x:c r="N200" s="5" t="n"/>
@@ -37426,7 +37452,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942e30471e9e47f7"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbf453faeed64d29"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Improve editor layer context menu behavior
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R67939d236ad04f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R53bcef50f4ec4855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Ree4712f0a1ea4e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R02889653bd354aa5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15004,17 +15004,44 @@
       <x:c r="Z200" s="5" t="n"/>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" s="5" t="n"/>
-      <x:c r="B201" s="24" t="n"/>
-      <x:c r="C201" s="5" t="n"/>
-      <x:c r="D201" s="5" t="n"/>
-      <x:c r="E201" s="5" t="n"/>
-      <x:c r="F201" s="24" t="n"/>
-      <x:c r="G201" s="5" t="n"/>
-      <x:c r="H201" s="5" t="n"/>
-      <x:c r="I201" s="5" t="n"/>
-      <x:c r="J201" s="5" t="n"/>
-      <x:c r="K201" s="5" t="n"/>
+      <x:c r="A201" s="5" t="str">
+        <x:v>TC_VIZI_193</x:v>
+      </x:c>
+      <x:c r="B201" s="24" t="str">
+        <x:v>Layer context menu dismissal 79</x:v>
+      </x:c>
+      <x:c r="C201" s="5" t="str">
+        <x:v>Xac minh context menu layer trong Editor dong dung bang Escape/click ngoai, khong dong khi hover ben trong, va khong tran viewport khi mo sat mep man hinh.</x:v>
+      </x:c>
+      <x:c r="D201" s="5" t="str">
+        <x:v>B1: Build frontend.
+B2: Mock design /editor/15 bang Playwright.
+B3: Right-click layer, kiem tra menu focus.
+B4: Bam Escape va kiem tra menu dong.
+B5: Mo lai menu, click ngoai va kiem tra menu dong.
+B6: Dispatch contextmenu sat mep phai/duoi va kiem tra bounding box trong viewport.</x:v>
+      </x:c>
+      <x:c r="E201" s="5" t="str">
+        <x:v>Mock design 15 co 3 layers; viewport 900x640; frontend dev server 127.0.0.1:5174; backend API base 127.0.0.1:8080.</x:v>
+      </x:c>
+      <x:c r="F201" s="24" t="str">
+        <x:v>Menu nhan focus khi mo; Escape va outside click dong menu; hover menu khong dong; menu sat mep duoc clamp trong viewport; khong co console error.</x:v>
+      </x:c>
+      <x:c r="G201" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke escapeCloses=true, outsideCloses=true, staysOnHover=true, box=716,372,176,250; console errors=0.</x:v>
+      </x:c>
+      <x:c r="H201" s="5" t="str">
+        <x:v>TC_VIZI_192; step 79</x:v>
+      </x:c>
+      <x:c r="I201" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J201" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K201" s="5" t="str">
+        <x:v>Buoc 79</x:v>
+      </x:c>
       <x:c r="L201" s="5" t="n"/>
       <x:c r="M201" s="5" t="n"/>
       <x:c r="N201" s="5" t="n"/>
@@ -37452,7 +37479,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbf453faeed64d29"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbe8c955bb814e61"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add rect and ellipse editor tools
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Ree4712f0a1ea4e0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R02889653bd354aa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rbf4ee17f89394c89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3c722252ef354bd2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>193</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15059,17 +15059,43 @@
       <x:c r="Z201" s="5" t="n"/>
     </x:row>
     <x:row r="202">
-      <x:c r="A202" s="5" t="n"/>
-      <x:c r="B202" s="24" t="n"/>
-      <x:c r="C202" s="5" t="n"/>
-      <x:c r="D202" s="5" t="n"/>
-      <x:c r="E202" s="5" t="n"/>
-      <x:c r="F202" s="24" t="n"/>
-      <x:c r="G202" s="5" t="n"/>
-      <x:c r="H202" s="5" t="n"/>
-      <x:c r="I202" s="5" t="n"/>
-      <x:c r="J202" s="5" t="n"/>
-      <x:c r="K202" s="5" t="n"/>
+      <x:c r="A202" s="5" t="str">
+        <x:v>TC_VIZI_194</x:v>
+      </x:c>
+      <x:c r="B202" s="24" t="str">
+        <x:v>Editor rect and ellipse toolbar 80</x:v>
+      </x:c>
+      <x:c r="C202" s="5" t="str">
+        <x:v>Xac minh toolbar co Rect/Ellipse rieng, tao layer dung loai va renderer hien ellipse tron.</x:v>
+      </x:c>
+      <x:c r="D202" s="5" t="str">
+        <x:v>B1: Build frontend.
+B2: Mock design /editor/15 co san 3 layer.
+B3: Click Rect tool roi click canvas.
+B4: Click Ellipse tool roi click canvas.
+B5: Kiem tra layer rows, top layer, class renderer, border radius, old Shape tool va console error.</x:v>
+      </x:c>
+      <x:c r="E202" s="5" t="str">
+        <x:v>Mock design 15 co 3 layers; frontend dev server 127.0.0.1:5174; backend API base 127.0.0.1:8080; Chrome channel Playwright.</x:v>
+      </x:c>
+      <x:c r="F202" s="24" t="str">
+        <x:v>Rect tool tao rect layer; Ellipse tool tao ellipse layer; top layer label Ellipse; CanvasPreview render .canvas-layer--ellipse voi radius tron; old Shape tool khong con hien; khong co console error.</x:v>
+      </x:c>
+      <x:c r="G202" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke rows=5, topLayer=Ellipse, ellipseCount=1, rectCount=3, radius=9999px; console errors=0.</x:v>
+      </x:c>
+      <x:c r="H202" s="5" t="str">
+        <x:v>TC_VIZI_193; step 80</x:v>
+      </x:c>
+      <x:c r="I202" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J202" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K202" s="5" t="str">
+        <x:v>Buoc 80</x:v>
+      </x:c>
       <x:c r="L202" s="5" t="n"/>
       <x:c r="M202" s="5" t="n"/>
       <x:c r="N202" s="5" t="n"/>
@@ -37479,7 +37505,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbe8c955bb814e61"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3c162101094232"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Guard QR toolbar placement
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rbf4ee17f89394c89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3c722252ef354bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R31b4d628fcee4511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rae753166ef014104"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15113,17 +15113,44 @@
       <x:c r="Z202" s="5" t="n"/>
     </x:row>
     <x:row r="203">
-      <x:c r="A203" s="5" t="n"/>
-      <x:c r="B203" s="24" t="n"/>
-      <x:c r="C203" s="5" t="n"/>
-      <x:c r="D203" s="5" t="n"/>
-      <x:c r="E203" s="5" t="n"/>
-      <x:c r="F203" s="24" t="n"/>
-      <x:c r="G203" s="5" t="n"/>
-      <x:c r="H203" s="5" t="n"/>
-      <x:c r="I203" s="5" t="n"/>
-      <x:c r="J203" s="5" t="n"/>
-      <x:c r="K203" s="5" t="n"/>
+      <x:c r="A203" s="5" t="str">
+        <x:v>TC_VIZI_195</x:v>
+      </x:c>
+      <x:c r="B203" s="24" t="str">
+        <x:v>Editor QR toolbar placement guard 81</x:v>
+      </x:c>
+      <x:c r="C203" s="5" t="str">
+        <x:v>Xac minh QR tool tren toolbar khong tao layer rong khi thieu QR text va tao QR layer co anh PNG khi text hop le.</x:v>
+      </x:c>
+      <x:c r="D203" s="5" t="str">
+        <x:v>B1: Build frontend.
+B2: Mock design /editor/15 co san 3 layer.
+B3: Xoa QR text, chon QR tool va click canvas.
+B4: Kiem tra error va layer count khong doi.
+B5: Nhap QR text hop le, click canvas.
+B6: Kiem tra layer QR nam tren cung, co class .canvas-layer--qr va img data PNG.</x:v>
+      </x:c>
+      <x:c r="E203" s="5" t="str">
+        <x:v>Mock design 15 co 3 layers; QR text https://vizi.local/step81-smoke; frontend dev server 127.0.0.1:5174; Chrome channel Playwright.</x:v>
+      </x:c>
+      <x:c r="F203" s="24" t="str">
+        <x:v>QR text rong hien loi va khong them layer; QR text hop le them dung 1 layer QR tai canvas; top layer la QR code; src bat dau bang data:image/png;base64; khong co console error.</x:v>
+      </x:c>
+      <x:c r="G203" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke rows=4, topLayer=QR code, hasQrImage=true, srcPrefix=data:image/png;base64, console errors=0.</x:v>
+      </x:c>
+      <x:c r="H203" s="5" t="str">
+        <x:v>TC_VIZI_194; step 81</x:v>
+      </x:c>
+      <x:c r="I203" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J203" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K203" s="5" t="str">
+        <x:v>Buoc 81</x:v>
+      </x:c>
       <x:c r="L203" s="5" t="n"/>
       <x:c r="M203" s="5" t="n"/>
       <x:c r="N203" s="5" t="n"/>
@@ -37505,7 +37532,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3c162101094232"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re88fdbb81f404131"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Open image picker from editor toolbar
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R31b4d628fcee4511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rae753166ef014104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rccd9bcbab3eb4bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R462d3da92c784f68"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>193</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15168,17 +15168,44 @@
       <x:c r="Z203" s="5" t="n"/>
     </x:row>
     <x:row r="204">
-      <x:c r="A204" s="5" t="n"/>
-      <x:c r="B204" s="24" t="n"/>
-      <x:c r="C204" s="5" t="n"/>
-      <x:c r="D204" s="5" t="n"/>
-      <x:c r="E204" s="5" t="n"/>
-      <x:c r="F204" s="24" t="n"/>
-      <x:c r="G204" s="5" t="n"/>
-      <x:c r="H204" s="5" t="n"/>
-      <x:c r="I204" s="5" t="n"/>
-      <x:c r="J204" s="5" t="n"/>
-      <x:c r="K204" s="5" t="n"/>
+      <x:c r="A204" s="5" t="str">
+        <x:v>TC_VIZI_196</x:v>
+      </x:c>
+      <x:c r="B204" s="24" t="str">
+        <x:v>Editor image toolbar file picker 82</x:v>
+      </x:c>
+      <x:c r="C204" s="5" t="str">
+        <x:v>Xac minh Image tool tren toolbar mo file picker khi chua co preview va khong mo lai file picker khi da co preview san sang de dat len canvas.</x:v>
+      </x:c>
+      <x:c r="D204" s="5" t="str">
+        <x:v>B1: Build frontend.
+B2: Mock design /editor/15 co san 3 layer.
+B3: Click Image tool va bat su kien file chooser.
+B4: Chon PNG mau.
+B5: Kiem tra asset preview hien ten file va Image tool active.
+B6: Click Image tool lan nua khi da co preview va xac minh file chooser khong mo lai.</x:v>
+      </x:c>
+      <x:c r="E204" s="5" t="str">
+        <x:v>Mock design 15 co 3 layers; sample.png 1x1 PNG; frontend dev server 127.0.0.1:5174; Chrome channel Playwright.</x:v>
+      </x:c>
+      <x:c r="F204" s="24" t="str">
+        <x:v>Lan dau click Image tool mo file picker; sau khi chon PNG, preview hien sample.png va toolbar active; click Image tool khi da co preview khong mo file picker lai; khong co console error.</x:v>
+      </x:c>
+      <x:c r="G204" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke preview=sample.png, imageToolActive=true, reopenedWithPreview=false, console errors=0.</x:v>
+      </x:c>
+      <x:c r="H204" s="5" t="str">
+        <x:v>TC_VIZI_195; step 82</x:v>
+      </x:c>
+      <x:c r="I204" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J204" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K204" s="5" t="str">
+        <x:v>Buoc 82</x:v>
+      </x:c>
       <x:c r="L204" s="5" t="n"/>
       <x:c r="M204" s="5" t="n"/>
       <x:c r="N204" s="5" t="n"/>
@@ -37532,7 +37559,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re88fdbb81f404131"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a2033f4fd184b96"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Render toolbar icons as icon layers
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rccd9bcbab3eb4bc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R462d3da92c784f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf1e8463ec5a74aa1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3c15babcf5de4316"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15223,17 +15223,43 @@
       <x:c r="Z204" s="5" t="n"/>
     </x:row>
     <x:row r="205">
-      <x:c r="A205" s="5" t="n"/>
-      <x:c r="B205" s="24" t="n"/>
-      <x:c r="C205" s="5" t="n"/>
-      <x:c r="D205" s="5" t="n"/>
-      <x:c r="E205" s="5" t="n"/>
-      <x:c r="F205" s="24" t="n"/>
-      <x:c r="G205" s="5" t="n"/>
-      <x:c r="H205" s="5" t="n"/>
-      <x:c r="I205" s="5" t="n"/>
-      <x:c r="J205" s="5" t="n"/>
-      <x:c r="K205" s="5" t="n"/>
+      <x:c r="A205" s="5" t="str">
+        <x:v>TC_VIZI_197</x:v>
+      </x:c>
+      <x:c r="B205" s="24" t="str">
+        <x:v>Editor icon toolbar visible layer 83</x:v>
+      </x:c>
+      <x:c r="C205" s="5" t="str">
+        <x:v>Xac minh Icon tool tren toolbar tao layer icon rieng, hien ky tu icon dung va renderer khong con coi icon la shape co nen hop.</x:v>
+      </x:c>
+      <x:c r="D205" s="5" t="str">
+        <x:v>B1: Build frontend.
+B2: Mock design /editor/15 co san 3 layer.
+B3: Click Icon tool roi click canvas.
+B4: Kiem tra layer count va top layer.
+B5: Kiem tra renderer co .canvas-layer--icon, khong co .canvas-layer--shape moi, text la ky tu ◆, background transparent, border 0 va khong co console error.</x:v>
+      </x:c>
+      <x:c r="E205" s="5" t="str">
+        <x:v>Mock design 15 co 3 layers; frontend dev server 127.0.0.1:5174; Chrome channel Playwright.</x:v>
+      </x:c>
+      <x:c r="F205" s="24" t="str">
+        <x:v>Icon tool them dung 1 layer type icon; top layer la Icon; icon text hien ◆; nen transparent, border 0, khong tao shape box; khong co console error.</x:v>
+      </x:c>
+      <x:c r="G205" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke rows=4, topLayer=Icon, iconText=◆, background=rgba(0, 0, 0, 0), border=0px, console errors=0.</x:v>
+      </x:c>
+      <x:c r="H205" s="5" t="str">
+        <x:v>TC_VIZI_196; step 83</x:v>
+      </x:c>
+      <x:c r="I205" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J205" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K205" s="5" t="str">
+        <x:v>Buoc 83</x:v>
+      </x:c>
       <x:c r="L205" s="5" t="n"/>
       <x:c r="M205" s="5" t="n"/>
       <x:c r="N205" s="5" t="n"/>
@@ -37559,7 +37585,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a2033f4fd184b96"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb05f19db0b654877"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Remove QR editor tooling
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rf1e8463ec5a74aa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3c15babcf5de4316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rcc0d82ae15e14add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rf2b1718dd5ca4050"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15277,17 +15277,44 @@
       <x:c r="Z205" s="5" t="n"/>
     </x:row>
     <x:row r="206">
-      <x:c r="A206" s="5" t="n"/>
-      <x:c r="B206" s="24" t="n"/>
-      <x:c r="C206" s="5" t="n"/>
-      <x:c r="D206" s="5" t="n"/>
-      <x:c r="E206" s="5" t="n"/>
-      <x:c r="F206" s="24" t="n"/>
-      <x:c r="G206" s="5" t="n"/>
-      <x:c r="H206" s="5" t="n"/>
-      <x:c r="I206" s="5" t="n"/>
-      <x:c r="J206" s="5" t="n"/>
-      <x:c r="K206" s="5" t="n"/>
+      <x:c r="A206" s="5" t="str">
+        <x:v>TC_VIZI_198</x:v>
+      </x:c>
+      <x:c r="B206" s="24" t="str">
+        <x:v>Editor remove QR feature 84</x:v>
+      </x:c>
+      <x:c r="C206" s="5" t="str">
+        <x:v>Xac minh editor khong con QR tool/generator va cac tool con lai van tao layer.</x:v>
+      </x:c>
+      <x:c r="D206" s="5" t="str">
+        <x:v>B1: Go qrcode/@types/qrcode khoi frontend package.
+B2: Build frontend.
+B3: Mo /editor/15 bang Playwright voi mock design.
+B4: Xac minh toolbar khong co QR tool va Assets khong co QR generator.
+B5: Click Text/Rect/Ellipse/Icon va dispatch pointerdown tren canvas de tao layer.
+B6: Kiem tra console khong co error.</x:v>
+      </x:c>
+      <x:c r="E206" s="5" t="str">
+        <x:v>Mock design 15 rong; frontend dev server 127.0.0.1:5174; Chrome channel Playwright; npm run build.</x:v>
+      </x:c>
+      <x:c r="F206" s="24" t="str">
+        <x:v>Khong con QR UI/dependency; toolbar chi con Select/Text/Rect/Ellipse/Image/Icon; Text/Rect/Ellipse/Icon van tao layer dung loai.</x:v>
+      </x:c>
+      <x:c r="G206" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke PASS step84 remove QR smoke; rg khong con QR/qrcode trong frontend source/package.</x:v>
+      </x:c>
+      <x:c r="H206" s="5" t="str">
+        <x:v>TC_VIZI_197; step 84</x:v>
+      </x:c>
+      <x:c r="I206" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J206" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K206" s="5" t="str">
+        <x:v>Buoc 84</x:v>
+      </x:c>
       <x:c r="L206" s="5" t="n"/>
       <x:c r="M206" s="5" t="n"/>
       <x:c r="N206" s="5" t="n"/>
@@ -37585,7 +37612,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb05f19db0b654877"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03b828f9bd5d4876"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add basic editor icon search
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rcc0d82ae15e14add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rf2b1718dd5ca4050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rdc22a489fe634ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3c2bea342ea24b12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15332,17 +15332,45 @@
       <x:c r="Z206" s="5" t="n"/>
     </x:row>
     <x:row r="207">
-      <x:c r="A207" s="5" t="n"/>
-      <x:c r="B207" s="24" t="n"/>
-      <x:c r="C207" s="5" t="n"/>
-      <x:c r="D207" s="5" t="n"/>
-      <x:c r="E207" s="5" t="n"/>
-      <x:c r="F207" s="24" t="n"/>
-      <x:c r="G207" s="5" t="n"/>
-      <x:c r="H207" s="5" t="n"/>
-      <x:c r="I207" s="5" t="n"/>
-      <x:c r="J207" s="5" t="n"/>
-      <x:c r="K207" s="5" t="n"/>
+      <x:c r="A207" s="5" t="str">
+        <x:v>TC_VIZI_199</x:v>
+      </x:c>
+      <x:c r="B207" s="24" t="str">
+        <x:v>Editor icon search library 85</x:v>
+      </x:c>
+      <x:c r="C207" s="5" t="str">
+        <x:v>Xac minh Assets panel co tim kiem icon basic va Icon tool tao dung icon dang chon.</x:v>
+      </x:c>
+      <x:c r="D207" s="5" t="str">
+        <x:v>B1: Them icon library local nho trong editor.
+B2: Build frontend.
+B3: Mo /editor/15 bang Playwright voi mock design.
+B4: Tim tu khoa star trong Icon search.
+B5: Chon Star icon va xac minh Icon tool active.
+B6: Tao layer tren canvas va kiem tra glyph/name.
+B7: Kiem tra QR tool van khong hien va console khong co error.</x:v>
+      </x:c>
+      <x:c r="E207" s="5" t="str">
+        <x:v>Mock design 15 rong; frontend dev server 127.0.0.1:5174; Chrome channel Playwright; query icon star.</x:v>
+      </x:c>
+      <x:c r="F207" s="24" t="str">
+        <x:v>Search star chi hien Star phu hop; chon icon kich hoat Icon tool; canvas tao layer icon ★ va layer list hien 1. Star.</x:v>
+      </x:c>
+      <x:c r="G207" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke PASS step85 icon search smoke; QR tool count=0.</x:v>
+      </x:c>
+      <x:c r="H207" s="5" t="str">
+        <x:v>TC_VIZI_198; step 85</x:v>
+      </x:c>
+      <x:c r="I207" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J207" s="5" t="n">
+        <x:v>46213</x:v>
+      </x:c>
+      <x:c r="K207" s="5" t="str">
+        <x:v>Buoc 85</x:v>
+      </x:c>
       <x:c r="L207" s="5" t="n"/>
       <x:c r="M207" s="5" t="n"/>
       <x:c r="N207" s="5" t="n"/>
@@ -37612,7 +37640,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03b828f9bd5d4876"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd810d6cac124c26"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Align QR removal with preflight spec
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rdc22a489fe634ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3c2bea342ea24b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R05406ce05d42467f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rf2b2151fe1464bb9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>199</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15388,17 +15388,43 @@
       <x:c r="Z207" s="5" t="n"/>
     </x:row>
     <x:row r="208">
-      <x:c r="A208" s="5" t="n"/>
-      <x:c r="B208" s="24" t="n"/>
-      <x:c r="C208" s="5" t="n"/>
-      <x:c r="D208" s="5" t="n"/>
-      <x:c r="E208" s="5" t="n"/>
-      <x:c r="F208" s="24" t="n"/>
-      <x:c r="G208" s="5" t="n"/>
-      <x:c r="H208" s="5" t="n"/>
-      <x:c r="I208" s="5" t="n"/>
-      <x:c r="J208" s="5" t="n"/>
-      <x:c r="K208" s="5" t="n"/>
+      <x:c r="A208" s="5" t="str">
+        <x:v>TC_VIZI_200</x:v>
+      </x:c>
+      <x:c r="B208" s="24" t="str">
+        <x:v>QR removal preflight spec sync 86</x:v>
+      </x:c>
+      <x:c r="C208" s="5" t="str">
+        <x:v>Xac minh backend preflight va Vizi.md khong con coi QR la tinh nang MVP/current.</x:v>
+      </x:c>
+      <x:c r="D208" s="5" t="str">
+        <x:v>B1: Doi preflight de chi text la critical khi ngoai safe zone.
+B2: Them test QR legacy ngoai safe zone chi tra WARNING.
+B3: Cap nhat Vizi.md: QR tam hoan sau MVP, toolbar/roadmap dung icon asset search.
+B4: Chay backend test scoped va full backend test.
+B5: Grep cac cum QR current-scope da bi loai bo.</x:v>
+      </x:c>
+      <x:c r="E208" s="5" t="str">
+        <x:v>PreflightServiceTests; Vizi.md; canvas qr layer ngoai safe zone; Maven backend test local.</x:v>
+      </x:c>
+      <x:c r="F208" s="24" t="str">
+        <x:v>Text ngoai safe zone van ERROR; QR legacy ngoai safe zone la WARNING; tai lieu chi ghi QR tam hoan sau MVP.</x:v>
+      </x:c>
+      <x:c r="G208" s="5" t="str">
+        <x:v>Pass: PreflightServiceTests 11/11; backend full test 68/68; grep current QR phrases khong con ket qua.</x:v>
+      </x:c>
+      <x:c r="H208" s="5" t="str">
+        <x:v>TC_VIZI_199; step 86</x:v>
+      </x:c>
+      <x:c r="I208" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J208" s="5" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="K208" s="5" t="str">
+        <x:v>Buoc 86</x:v>
+      </x:c>
       <x:c r="L208" s="5" t="n"/>
       <x:c r="M208" s="5" t="n"/>
       <x:c r="N208" s="5" t="n"/>
@@ -37640,7 +37666,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd810d6cac124c26"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf76a8baf0d9448fa"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add icon asset metadata search
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R05406ce05d42467f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rf2b2151fe1464bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R5458767ad0804128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R0af9300e54fc45f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>200</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15442,17 +15442,45 @@
       <x:c r="Z208" s="5" t="n"/>
     </x:row>
     <x:row r="209">
-      <x:c r="A209" s="5" t="n"/>
-      <x:c r="B209" s="24" t="n"/>
-      <x:c r="C209" s="5" t="n"/>
-      <x:c r="D209" s="5" t="n"/>
-      <x:c r="E209" s="5" t="n"/>
-      <x:c r="F209" s="24" t="n"/>
-      <x:c r="G209" s="5" t="n"/>
-      <x:c r="H209" s="5" t="n"/>
-      <x:c r="I209" s="5" t="n"/>
-      <x:c r="J209" s="5" t="n"/>
-      <x:c r="K209" s="5" t="n"/>
+      <x:c r="A209" s="5" t="str">
+        <x:v>TC_VIZI_201</x:v>
+      </x:c>
+      <x:c r="B209" s="24" t="str">
+        <x:v>Icon asset metadata search 88</x:v>
+      </x:c>
+      <x:c r="C209" s="5" t="str">
+        <x:v>Xac minh icon library co tags/description/keywords va search duoc theo tu khoa Viet/Russian/English co ban.</x:v>
+      </x:c>
+      <x:c r="D209" s="5" t="str">
+        <x:v>B1: Them description va keywords cho icon asset local.
+B2: Search haystack gom label, description, tags va keywords.
+B3: Build frontend.
+B4: Mo /editor/15 bang Playwright voi mock design.
+B5: Search spa vang phai ra Flower.
+B6: Search telefoon/telefon Russian phai ra Phone.
+B7: Chon Flower va tao icon layer tren canvas.</x:v>
+      </x:c>
+      <x:c r="E209" s="5" t="str">
+        <x:v>Frontend dev server 127.0.0.1:5175; mock design 15 rong; Chrome channel Playwright; query spa vang va telefoon Russian.</x:v>
+      </x:c>
+      <x:c r="F209" s="24" t="str">
+        <x:v>Search spa vang chi hien Flower; search Russian phone chi hien Phone; tao layer Flower thanh cong; console khong co error.</x:v>
+      </x:c>
+      <x:c r="G209" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke PASS step88 icon metadata smoke.</x:v>
+      </x:c>
+      <x:c r="H209" s="5" t="str">
+        <x:v>TC_VIZI_200; step 88</x:v>
+      </x:c>
+      <x:c r="I209" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J209" s="5" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="K209" s="5" t="str">
+        <x:v>Buoc 88</x:v>
+      </x:c>
       <x:c r="L209" s="5" t="n"/>
       <x:c r="M209" s="5" t="n"/>
       <x:c r="N209" s="5" t="n"/>
@@ -37666,7 +37694,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf76a8baf0d9448fa"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73698762f55549c4"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Improve icon asset text search
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R5458767ad0804128"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R0af9300e54fc45f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R4158168695ca4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R73d3e59587ff4991"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>199</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1068,7 +1068,7 @@
       </x:c>
       <x:c r="F5" s="40"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -15498,17 +15498,45 @@
       <x:c r="Z209" s="5" t="n"/>
     </x:row>
     <x:row r="210">
-      <x:c r="A210" s="5" t="n"/>
-      <x:c r="B210" s="24" t="n"/>
-      <x:c r="C210" s="5" t="n"/>
-      <x:c r="D210" s="5" t="n"/>
-      <x:c r="E210" s="5" t="n"/>
-      <x:c r="F210" s="24" t="n"/>
-      <x:c r="G210" s="5" t="n"/>
-      <x:c r="H210" s="5" t="n"/>
-      <x:c r="I210" s="5" t="n"/>
-      <x:c r="J210" s="5" t="n"/>
-      <x:c r="K210" s="5" t="n"/>
+      <x:c r="A210" s="5" t="str">
+        <x:v>TC_VIZI_202</x:v>
+      </x:c>
+      <x:c r="B210" s="24" t="str">
+        <x:v>Icon asset text search 89</x:v>
+      </x:c>
+      <x:c r="C210" s="5" t="str">
+        <x:v>Xac minh search asset/icon basic ho tro bo dau tieng Viet va token nhieu tu.</x:v>
+      </x:c>
+      <x:c r="D210" s="5" t="str">
+        <x:v>B1: Them normalize bo dau cho icon search.
+B2: Tach query thanh token va yeu cau moi token co trong metadata.
+B3: Build frontend.
+B4: Mo /editor/15 bang Playwright voi mock design.
+B5: Search dien thoai co dau ra Phone.
+B6: Search kim cuong co dau ra Diamond.
+B7: Search spa vang co dau ra Flower va tao layer icon.</x:v>
+      </x:c>
+      <x:c r="E210" s="5" t="str">
+        <x:v>Frontend dev server 127.0.0.1:5175; mock design 15 rong; Chrome channel Playwright; query dien thoai, kim cuong, spa vang co dau.</x:v>
+      </x:c>
+      <x:c r="F210" s="24" t="str">
+        <x:v>Search bo dau/tach token tra dung icon; Flower tao duoc icon layer; console khong co error.</x:v>
+      </x:c>
+      <x:c r="G210" s="5" t="str">
+        <x:v>Pass: npm run build OK; Playwright smoke PASS step89 icon text search smoke.</x:v>
+      </x:c>
+      <x:c r="H210" s="5" t="str">
+        <x:v>TC_VIZI_201; step 89</x:v>
+      </x:c>
+      <x:c r="I210" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J210" s="5" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="K210" s="5" t="str">
+        <x:v>Buoc 89</x:v>
+      </x:c>
       <x:c r="L210" s="5" t="n"/>
       <x:c r="M210" s="5" t="n"/>
       <x:c r="N210" s="5" t="n"/>
@@ -37694,7 +37722,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73698762f55549c4"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd129b00f063a4cd0"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Record frontend production build test
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -15987,32 +15987,78 @@
       <c r="Z211" s="43" t="n"/>
     </row>
     <row r="212">
-      <c r="A212" s="5" t="n"/>
-      <c r="B212" s="24" t="n"/>
-      <c r="C212" s="5" t="n"/>
-      <c r="D212" s="5" t="n"/>
-      <c r="E212" s="5" t="n"/>
-      <c r="F212" s="24" t="n"/>
-      <c r="G212" s="5" t="n"/>
-      <c r="H212" s="5" t="n"/>
-      <c r="I212" s="5" t="n"/>
-      <c r="J212" s="5" t="n"/>
-      <c r="K212" s="5" t="n"/>
-      <c r="L212" s="5" t="n"/>
-      <c r="M212" s="5" t="n"/>
-      <c r="N212" s="5" t="n"/>
-      <c r="O212" s="5" t="n"/>
-      <c r="P212" s="5" t="n"/>
-      <c r="Q212" s="5" t="n"/>
-      <c r="R212" s="5" t="n"/>
-      <c r="S212" s="5" t="n"/>
-      <c r="T212" s="5" t="n"/>
-      <c r="U212" s="5" t="n"/>
-      <c r="V212" s="5" t="n"/>
-      <c r="W212" s="5" t="n"/>
-      <c r="X212" s="5" t="n"/>
-      <c r="Y212" s="5" t="n"/>
-      <c r="Z212" s="5" t="n"/>
+      <c r="A212" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_204</t>
+        </is>
+      </c>
+      <c r="B212" s="67" t="inlineStr">
+        <is>
+          <t>Frontend production build 101</t>
+        </is>
+      </c>
+      <c r="C212" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh frontend Vue/Vite build production thanh cong va dist artifact khong bi dua vao Git.</t>
+        </is>
+      </c>
+      <c r="D212" s="43" t="inlineStr">
+        <is>
+          <t>B1: Chay npm run build trong frontend.
+B2: Xac minh vue-tsc --noEmit pass.
+B3: Xac minh vite build tao dist/index.html va assets hash.
+B4: Kiem tra git status de dam bao frontend/dist dang ignored, khong stage artifact build.
+B5: Ghi testcase vao workbook va chi stage workbook.</t>
+        </is>
+      </c>
+      <c r="E212" s="43" t="inlineStr">
+        <is>
+          <t>Frontend Vue/Vite; package.json build script; frontend/.env.example chi co VITE_API_BASE_URL; dist ignored trong Git.</t>
+        </is>
+      </c>
+      <c r="F212" s="67" t="inlineStr">
+        <is>
+          <t>npm run build pass; dist co index/assets; khong co file dist staged; khong co secret frontend env.</t>
+        </is>
+      </c>
+      <c r="G212" s="43" t="inlineStr">
+        <is>
+          <t>Pass: npm run build OK; output dist/index.html, CSS 32.88 kB, JS 287.19 kB; git status khong hien frontend/dist; .env.example chi co VITE_API_BASE_URL.</t>
+        </is>
+      </c>
+      <c r="H212" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_203; step 101; step 100 blocked by missing cloud deploy target</t>
+        </is>
+      </c>
+      <c r="I212" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J212" s="68" t="n">
+        <v>46214</v>
+      </c>
+      <c r="K212" s="43" t="inlineStr">
+        <is>
+          <t>Buoc 101</t>
+        </is>
+      </c>
+      <c r="L212" s="43" t="n"/>
+      <c r="M212" s="43" t="n"/>
+      <c r="N212" s="43" t="n"/>
+      <c r="O212" s="43" t="n"/>
+      <c r="P212" s="43" t="n"/>
+      <c r="Q212" s="43" t="n"/>
+      <c r="R212" s="43" t="n"/>
+      <c r="S212" s="43" t="n"/>
+      <c r="T212" s="43" t="n"/>
+      <c r="U212" s="43" t="n"/>
+      <c r="V212" s="43" t="n"/>
+      <c r="W212" s="43" t="n"/>
+      <c r="X212" s="43" t="n"/>
+      <c r="Y212" s="43" t="n"/>
+      <c r="Z212" s="43" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="5" t="n"/>

</xml_diff>

<commit_message>
Add frontend SPA fallback for static hosting
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -16061,32 +16061,77 @@
       <c r="Z212" s="43" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" s="5" t="n"/>
-      <c r="B213" s="24" t="n"/>
-      <c r="C213" s="5" t="n"/>
-      <c r="D213" s="5" t="n"/>
-      <c r="E213" s="5" t="n"/>
-      <c r="F213" s="24" t="n"/>
-      <c r="G213" s="5" t="n"/>
-      <c r="H213" s="5" t="n"/>
-      <c r="I213" s="5" t="n"/>
-      <c r="J213" s="5" t="n"/>
-      <c r="K213" s="5" t="n"/>
-      <c r="L213" s="5" t="n"/>
-      <c r="M213" s="5" t="n"/>
-      <c r="N213" s="5" t="n"/>
-      <c r="O213" s="5" t="n"/>
-      <c r="P213" s="5" t="n"/>
-      <c r="Q213" s="5" t="n"/>
-      <c r="R213" s="5" t="n"/>
-      <c r="S213" s="5" t="n"/>
-      <c r="T213" s="5" t="n"/>
-      <c r="U213" s="5" t="n"/>
-      <c r="V213" s="5" t="n"/>
-      <c r="W213" s="5" t="n"/>
-      <c r="X213" s="5" t="n"/>
-      <c r="Y213" s="5" t="n"/>
-      <c r="Z213" s="5" t="n"/>
+      <c r="A213" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_205</t>
+        </is>
+      </c>
+      <c r="B213" s="67" t="inlineStr">
+        <is>
+          <t>Frontend static host SPA fallback 102-prep</t>
+        </is>
+      </c>
+      <c r="C213" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh Cloudflare Pages/static host co fallback cho Vue history routing de refresh route con khong bi 404.</t>
+        </is>
+      </c>
+      <c r="D213" s="43" t="inlineStr">
+        <is>
+          <t>B1: Them frontend/public/_redirects voi rule /* /index.html 200.
+B2: Chay npm run build trong frontend.
+B3: Doc frontend/dist/_redirects sau build.
+B4: Kiem tra git status dam bao chi stage _redirects va testcase, khong stage dist artifact.</t>
+        </is>
+      </c>
+      <c r="E213" s="43" t="inlineStr">
+        <is>
+          <t>Frontend Vue Router createWebHistory; Cloudflare Pages static hosting; Vite public asset copy.</t>
+        </is>
+      </c>
+      <c r="F213" s="67" t="inlineStr">
+        <is>
+          <t>Production build pass; dist/_redirects ton tai va co rule /* /index.html 200; dist khong staged.</t>
+        </is>
+      </c>
+      <c r="G213" s="43" t="inlineStr">
+        <is>
+          <t>Pass: npm run build OK; frontend/dist/_redirects = /* /index.html 200; git status khong hien frontend/dist.</t>
+        </is>
+      </c>
+      <c r="H213" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_204; step 102 prep; full step 102 still needs Cloudflare deployment URL</t>
+        </is>
+      </c>
+      <c r="I213" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J213" s="68" t="n">
+        <v>46214</v>
+      </c>
+      <c r="K213" s="43" t="inlineStr">
+        <is>
+          <t>Buoc 102 prep</t>
+        </is>
+      </c>
+      <c r="L213" s="43" t="n"/>
+      <c r="M213" s="43" t="n"/>
+      <c r="N213" s="43" t="n"/>
+      <c r="O213" s="43" t="n"/>
+      <c r="P213" s="43" t="n"/>
+      <c r="Q213" s="43" t="n"/>
+      <c r="R213" s="43" t="n"/>
+      <c r="S213" s="43" t="n"/>
+      <c r="T213" s="43" t="n"/>
+      <c r="U213" s="43" t="n"/>
+      <c r="V213" s="43" t="n"/>
+      <c r="W213" s="43" t="n"/>
+      <c r="X213" s="43" t="n"/>
+      <c r="Y213" s="43" t="n"/>
+      <c r="Z213" s="43" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="5" t="n"/>

</xml_diff>

<commit_message>
Add backend SQL injection guard test
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -16134,32 +16134,78 @@
       <c r="Z213" s="43" t="n"/>
     </row>
     <row r="214">
-      <c r="A214" s="5" t="n"/>
-      <c r="B214" s="24" t="n"/>
-      <c r="C214" s="5" t="n"/>
-      <c r="D214" s="5" t="n"/>
-      <c r="E214" s="5" t="n"/>
-      <c r="F214" s="24" t="n"/>
-      <c r="G214" s="5" t="n"/>
-      <c r="H214" s="5" t="n"/>
-      <c r="I214" s="5" t="n"/>
-      <c r="J214" s="5" t="n"/>
-      <c r="K214" s="5" t="n"/>
-      <c r="L214" s="5" t="n"/>
-      <c r="M214" s="5" t="n"/>
-      <c r="N214" s="5" t="n"/>
-      <c r="O214" s="5" t="n"/>
-      <c r="P214" s="5" t="n"/>
-      <c r="Q214" s="5" t="n"/>
-      <c r="R214" s="5" t="n"/>
-      <c r="S214" s="5" t="n"/>
-      <c r="T214" s="5" t="n"/>
-      <c r="U214" s="5" t="n"/>
-      <c r="V214" s="5" t="n"/>
-      <c r="W214" s="5" t="n"/>
-      <c r="X214" s="5" t="n"/>
-      <c r="Y214" s="5" t="n"/>
-      <c r="Z214" s="5" t="n"/>
+      <c r="A214" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_206</t>
+        </is>
+      </c>
+      <c r="B214" s="67" t="inlineStr">
+        <is>
+          <t>Backend SQL injection guard 105</t>
+        </is>
+      </c>
+      <c r="C214" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh production backend khong dung raw SQL API de tranh SQL Injection va khoa bang unit test tu dong.</t>
+        </is>
+      </c>
+      <c r="D214" s="43" t="inlineStr">
+        <is>
+          <t>B1: Rg production source voi cac marker raw SQL/JDBC.
+B2: Them ProductionSqlInjectionGuardTests scan src/main/java.
+B3: Guard fail neu production code dung Statement, prepareStatement, createNativeQuery, JdbcTemplate, EntityManager hoac @Query.
+B4: Chay full backend test.
+B5: Kiem tra staged files khong gom file local/secret.</t>
+        </is>
+      </c>
+      <c r="E214" s="43" t="inlineStr">
+        <is>
+          <t>Backend Spring Boot; production source src/main/java; Spring Data repository pattern; Maven test suite.</t>
+        </is>
+      </c>
+      <c r="F214" s="67" t="inlineStr">
+        <is>
+          <t>Production code chi dung Spring Data/JPA repository pattern, khong co marker raw SQL; full backend test pass.</t>
+        </is>
+      </c>
+      <c r="G214" s="43" t="inlineStr">
+        <is>
+          <t>Pass: mvnw test OK; Tests run 69, Failures 0, Errors 0; ProductionSqlInjectionGuardTests 1/1 pass.</t>
+        </is>
+      </c>
+      <c r="H214" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_205; step 105</t>
+        </is>
+      </c>
+      <c r="I214" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J214" s="68" t="n">
+        <v>46214</v>
+      </c>
+      <c r="K214" s="43" t="inlineStr">
+        <is>
+          <t>Buoc 105</t>
+        </is>
+      </c>
+      <c r="L214" s="43" t="n"/>
+      <c r="M214" s="43" t="n"/>
+      <c r="N214" s="43" t="n"/>
+      <c r="O214" s="43" t="n"/>
+      <c r="P214" s="43" t="n"/>
+      <c r="Q214" s="43" t="n"/>
+      <c r="R214" s="43" t="n"/>
+      <c r="S214" s="43" t="n"/>
+      <c r="T214" s="43" t="n"/>
+      <c r="U214" s="43" t="n"/>
+      <c r="V214" s="43" t="n"/>
+      <c r="W214" s="43" t="n"/>
+      <c r="X214" s="43" t="n"/>
+      <c r="Y214" s="43" t="n"/>
+      <c r="Z214" s="43" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="5" t="n"/>

</xml_diff>

<commit_message>
Add frontend XSS guard test
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -16208,32 +16208,78 @@
       <c r="Z214" s="43" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" s="5" t="n"/>
-      <c r="B215" s="24" t="n"/>
-      <c r="C215" s="5" t="n"/>
-      <c r="D215" s="5" t="n"/>
-      <c r="E215" s="5" t="n"/>
-      <c r="F215" s="24" t="n"/>
-      <c r="G215" s="5" t="n"/>
-      <c r="H215" s="5" t="n"/>
-      <c r="I215" s="5" t="n"/>
-      <c r="J215" s="5" t="n"/>
-      <c r="K215" s="5" t="n"/>
-      <c r="L215" s="5" t="n"/>
-      <c r="M215" s="5" t="n"/>
-      <c r="N215" s="5" t="n"/>
-      <c r="O215" s="5" t="n"/>
-      <c r="P215" s="5" t="n"/>
-      <c r="Q215" s="5" t="n"/>
-      <c r="R215" s="5" t="n"/>
-      <c r="S215" s="5" t="n"/>
-      <c r="T215" s="5" t="n"/>
-      <c r="U215" s="5" t="n"/>
-      <c r="V215" s="5" t="n"/>
-      <c r="W215" s="5" t="n"/>
-      <c r="X215" s="5" t="n"/>
-      <c r="Y215" s="5" t="n"/>
-      <c r="Z215" s="5" t="n"/>
+      <c r="A215" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_207</t>
+        </is>
+      </c>
+      <c r="B215" s="67" t="inlineStr">
+        <is>
+          <t>Frontend XSS guard 106</t>
+        </is>
+      </c>
+      <c r="C215" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh frontend khong dung raw HTML sink de render text user/AI va backend upload van chan SVG script.</t>
+        </is>
+      </c>
+      <c r="D215" s="43" t="inlineStr">
+        <is>
+          <t>B1: Ra soat frontend render text/layer khong dung v-html/innerHTML.
+B2: Them xssStaticGuard.test.mjs scan src cho HTML sinks.
+B3: Them npm script test:xss.
+B4: Chay npm run test:xss va npm run build.
+B5: Chay backend test de xac minh upload SVG/script van bi reject.</t>
+        </is>
+      </c>
+      <c r="E215" s="43" t="inlineStr">
+        <is>
+          <t>Frontend Vue/Vite; CanvasPreview render text bang mustache; backend ImageUploadApiTests co case SVG script bi reject.</t>
+        </is>
+      </c>
+      <c r="F215" s="67" t="inlineStr">
+        <is>
+          <t>Khong co v-html/innerHTML/DOMParser/insertAdjacentHTML trong frontend src; frontend build pass; backend upload SVG test nam trong suite pass.</t>
+        </is>
+      </c>
+      <c r="G215" s="43" t="inlineStr">
+        <is>
+          <t>Pass: npm run test:xss OK; npm run build OK; backend mvnw test OK 69/69 trong cung turn.</t>
+        </is>
+      </c>
+      <c r="H215" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_206; step 106</t>
+        </is>
+      </c>
+      <c r="I215" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J215" s="68" t="n">
+        <v>46214</v>
+      </c>
+      <c r="K215" s="43" t="inlineStr">
+        <is>
+          <t>Buoc 106</t>
+        </is>
+      </c>
+      <c r="L215" s="43" t="n"/>
+      <c r="M215" s="43" t="n"/>
+      <c r="N215" s="43" t="n"/>
+      <c r="O215" s="43" t="n"/>
+      <c r="P215" s="43" t="n"/>
+      <c r="Q215" s="43" t="n"/>
+      <c r="R215" s="43" t="n"/>
+      <c r="S215" s="43" t="n"/>
+      <c r="T215" s="43" t="n"/>
+      <c r="U215" s="43" t="n"/>
+      <c r="V215" s="43" t="n"/>
+      <c r="W215" s="43" t="n"/>
+      <c r="X215" s="43" t="n"/>
+      <c r="Y215" s="43" t="n"/>
+      <c r="Z215" s="43" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="5" t="n"/>

</xml_diff>

<commit_message>
Add CSRF write protection test
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -16282,32 +16282,73 @@
       <c r="Z215" s="43" t="n"/>
     </row>
     <row r="216">
-      <c r="A216" s="5" t="n"/>
-      <c r="B216" s="24" t="n"/>
-      <c r="C216" s="5" t="n"/>
-      <c r="D216" s="5" t="n"/>
-      <c r="E216" s="5" t="n"/>
-      <c r="F216" s="24" t="n"/>
-      <c r="G216" s="5" t="n"/>
-      <c r="H216" s="5" t="n"/>
-      <c r="I216" s="5" t="n"/>
-      <c r="J216" s="5" t="n"/>
-      <c r="K216" s="5" t="n"/>
-      <c r="L216" s="5" t="n"/>
-      <c r="M216" s="5" t="n"/>
-      <c r="N216" s="5" t="n"/>
-      <c r="O216" s="5" t="n"/>
-      <c r="P216" s="5" t="n"/>
-      <c r="Q216" s="5" t="n"/>
-      <c r="R216" s="5" t="n"/>
-      <c r="S216" s="5" t="n"/>
-      <c r="T216" s="5" t="n"/>
-      <c r="U216" s="5" t="n"/>
-      <c r="V216" s="5" t="n"/>
-      <c r="W216" s="5" t="n"/>
-      <c r="X216" s="5" t="n"/>
-      <c r="Y216" s="5" t="n"/>
-      <c r="Z216" s="5" t="n"/>
+      <c r="A216" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_208</t>
+        </is>
+      </c>
+      <c r="B216" s="67" t="inlineStr">
+        <is>
+          <t>Backend CSRF write guard 107</t>
+        </is>
+      </c>
+      <c r="C216" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh cac request ghi du lieu quan trong cua backend bi chan khi thieu CSRF token, ke ca khi da authenticated.</t>
+        </is>
+      </c>
+      <c r="D216" s="43" t="inlineStr">
+        <is>
+          <t>B1: Them CsrfWriteProtectionTests cho create/update/delete design va create order khong kem CSRF.
+B2: Chay backend test scoped.
+B3: Chay full backend test.
+B4: Kiem tra git status/staged files khong gom file local/secret/runtime upload.</t>
+        </is>
+      </c>
+      <c r="E216" s="43" t="inlineStr">
+        <is>
+          <t>Backend Spring Security HttpSessionCsrfTokenRepository; MockMvc authenticated request khong with(csrf()).</t>
+        </is>
+      </c>
+      <c r="F216" s="67" t="inlineStr">
+        <is>
+          <t>Tat ca POST/PUT/DELETE write endpoint trong test tra 403 Forbidden khi thieu CSRF; full backend suite pass.</t>
+        </is>
+      </c>
+      <c r="G216" s="43" t="inlineStr">
+        <is>
+          <t>Pass: scoped CsrfWriteProtectionTests 1/1; backend mvnw test OK 70/70; write endpoints without CSRF return 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="H216" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_207; step 107</t>
+        </is>
+      </c>
+      <c r="I216" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J216" s="68" t="n">
+        <v>46214</v>
+      </c>
+      <c r="K216" s="43" t="n"/>
+      <c r="L216" s="43" t="n"/>
+      <c r="M216" s="43" t="n"/>
+      <c r="N216" s="43" t="n"/>
+      <c r="O216" s="43" t="n"/>
+      <c r="P216" s="43" t="n"/>
+      <c r="Q216" s="43" t="n"/>
+      <c r="R216" s="43" t="n"/>
+      <c r="S216" s="43" t="n"/>
+      <c r="T216" s="43" t="n"/>
+      <c r="U216" s="43" t="n"/>
+      <c r="V216" s="43" t="n"/>
+      <c r="W216" s="43" t="n"/>
+      <c r="X216" s="43" t="n"/>
+      <c r="Y216" s="43" t="n"/>
+      <c r="Z216" s="43" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="5" t="n"/>

</xml_diff>

<commit_message>
Protect uploaded images by owner
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -16351,32 +16351,74 @@
       <c r="Z216" s="43" t="n"/>
     </row>
     <row r="217">
-      <c r="A217" s="5" t="n"/>
-      <c r="B217" s="24" t="n"/>
-      <c r="C217" s="5" t="n"/>
-      <c r="D217" s="5" t="n"/>
-      <c r="E217" s="5" t="n"/>
-      <c r="F217" s="24" t="n"/>
-      <c r="G217" s="5" t="n"/>
-      <c r="H217" s="5" t="n"/>
-      <c r="I217" s="5" t="n"/>
-      <c r="J217" s="5" t="n"/>
-      <c r="K217" s="5" t="n"/>
-      <c r="L217" s="5" t="n"/>
-      <c r="M217" s="5" t="n"/>
-      <c r="N217" s="5" t="n"/>
-      <c r="O217" s="5" t="n"/>
-      <c r="P217" s="5" t="n"/>
-      <c r="Q217" s="5" t="n"/>
-      <c r="R217" s="5" t="n"/>
-      <c r="S217" s="5" t="n"/>
-      <c r="T217" s="5" t="n"/>
-      <c r="U217" s="5" t="n"/>
-      <c r="V217" s="5" t="n"/>
-      <c r="W217" s="5" t="n"/>
-      <c r="X217" s="5" t="n"/>
-      <c r="Y217" s="5" t="n"/>
-      <c r="Z217" s="5" t="n"/>
+      <c r="A217" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_209</t>
+        </is>
+      </c>
+      <c r="B217" s="67" t="inlineStr">
+        <is>
+          <t>Upload asset owner guard 108</t>
+        </is>
+      </c>
+      <c r="C217" s="43" t="inlineStr">
+        <is>
+          <t>Xac minh URL anh upload chi doc duoc boi owner, user khac co URL cung khong doc duoc file.</t>
+        </is>
+      </c>
+      <c r="D217" s="43" t="inlineStr">
+        <is>
+          <t>B1: Bo static resource handler cho /uploads/images/**.
+B2: Them endpoint readImage qua controller va service loadOwnedImage.
+B3: Query asset theo fileName + owner email.
+B4: Them test other user GET cung URL bi 404, owner van 200.
+B5: Chay upload scoped test va full backend regression.</t>
+        </is>
+      </c>
+      <c r="E217" s="43" t="inlineStr">
+        <is>
+          <t>Backend upload asset; Spring Security authenticated session; assets.user_id ownership; MockMvc owner vs other user.</t>
+        </is>
+      </c>
+      <c r="F217" s="67" t="inlineStr">
+        <is>
+          <t>Owner upload/read duoc anh; other user co URL nhung nhan 404; full backend suite pass.</t>
+        </is>
+      </c>
+      <c r="G217" s="43" t="inlineStr">
+        <is>
+          <t>Pass: ImageUploadApiTests 5/5; backend mvnw test OK 71/71; khong con static resource bypass cho upload image URL.</t>
+        </is>
+      </c>
+      <c r="H217" s="43" t="inlineStr">
+        <is>
+          <t>TC_VIZI_208; step 108</t>
+        </is>
+      </c>
+      <c r="I217" s="43" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J217" s="68" t="n">
+        <v>46214</v>
+      </c>
+      <c r="K217" s="43" t="n"/>
+      <c r="L217" s="43" t="n"/>
+      <c r="M217" s="43" t="n"/>
+      <c r="N217" s="43" t="n"/>
+      <c r="O217" s="43" t="n"/>
+      <c r="P217" s="43" t="n"/>
+      <c r="Q217" s="43" t="n"/>
+      <c r="R217" s="43" t="n"/>
+      <c r="S217" s="43" t="n"/>
+      <c r="T217" s="43" t="n"/>
+      <c r="U217" s="43" t="n"/>
+      <c r="V217" s="43" t="n"/>
+      <c r="W217" s="43" t="n"/>
+      <c r="X217" s="43" t="n"/>
+      <c r="Y217" s="43" t="n"/>
+      <c r="Z217" s="43" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="5" t="n"/>

</xml_diff>

<commit_message>
Rate limit image uploads
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R85607f0444e4454e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R3dea91a0c8244ade"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb4c06a0a22be452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R8a4f3c6e09d940f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1072,7 +1072,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>203</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -16474,16 +16474,36 @@
       <x:c r="Z218" s="5" t="n"/>
     </x:row>
     <x:row r="219">
-      <x:c r="A219" s="5" t="n"/>
-      <x:c r="B219" s="24" t="n"/>
-      <x:c r="C219" s="5" t="n"/>
-      <x:c r="D219" s="5" t="n"/>
-      <x:c r="E219" s="5" t="n"/>
-      <x:c r="F219" s="24" t="n"/>
-      <x:c r="G219" s="5" t="n"/>
-      <x:c r="H219" s="5" t="n"/>
-      <x:c r="I219" s="5" t="n"/>
-      <x:c r="J219" s="5" t="n"/>
+      <x:c r="A219" s="5" t="str">
+        <x:v>TC_VIZI_211</x:v>
+      </x:c>
+      <x:c r="B219" s="24" t="str">
+        <x:v>Backend upload rate limit guard 110</x:v>
+      </x:c>
+      <x:c r="C219" s="5" t="str">
+        <x:v>Verify authenticated image upload is rate-limited to reduce upload spam and storage abuse risk.</x:v>
+      </x:c>
+      <x:c r="D219" s="5" t="str">
+        <x:v>Add /api/uploads/images to RateLimitFilter; test direct filter limit; test MockMvc multipart upload succeeds 10 times and returns 429 on request 11 from the same IP; run scoped and full backend suites.</x:v>
+      </x:c>
+      <x:c r="E219" s="5" t="str">
+        <x:v>Spring Security; OncePerRequestFilter; POST /api/uploads/images; multipart PNG; MockMvc; owner@example.test.</x:v>
+      </x:c>
+      <x:c r="F219" s="24" t="str">
+        <x:v>Requests under upload threshold return 201; the next request from the same IP returns HTTP 429 with JSON message; existing upload validation and owner checks still pass.</x:v>
+      </x:c>
+      <x:c r="G219" s="5" t="str">
+        <x:v>PASS: scoped backend tests 10/10; full backend test suite 77/77.</x:v>
+      </x:c>
+      <x:c r="H219" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I219" s="5" t="str">
+        <x:v>2026-07-11</x:v>
+      </x:c>
+      <x:c r="J219" s="5" t="str">
+        <x:v>TC_VIZI_210; step 110</x:v>
+      </x:c>
       <x:c r="K219" s="5" t="n"/>
       <x:c r="L219" s="5" t="n"/>
       <x:c r="M219" s="5" t="n"/>
@@ -38418,7 +38438,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e76a0066a7e4e8c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a93b11a936f4586"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add production secret scan guard
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="Rb4c06a0a22be452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="R8a4f3c6e09d940f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="&lt;Tên&gt;_&lt;MSV&gt;" sheetId="1" r:id="R4832714cfee0445d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng Quyết định (nếu có)" sheetId="2" r:id="Rd08606e181164245"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1058,7 +1058,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="n">
-        <x:v>200</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
         <x:v>0</x:v>
@@ -1072,7 +1072,7 @@
       </x:c>
       <x:c r="F5" s="40" t="n"/>
       <x:c r="G5" s="35" t="n">
-        <x:v>204</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="H5" s="36" t="n"/>
       <x:c r="I5" s="37" t="n"/>
@@ -16522,21 +16522,41 @@
       <x:c r="Z219" s="5" t="n"/>
     </x:row>
     <x:row r="220">
-      <x:c r="A220" s="5" t="n"/>
-      <x:c r="B220" s="24" t="n"/>
-      <x:c r="C220" s="5" t="n"/>
-      <x:c r="D220" s="5" t="n"/>
-      <x:c r="E220" s="5" t="n"/>
-      <x:c r="F220" s="24" t="n"/>
-      <x:c r="G220" s="5" t="n"/>
-      <x:c r="H220" s="5" t="n"/>
-      <x:c r="I220" s="5" t="n"/>
-      <x:c r="J220" s="5" t="n"/>
-      <x:c r="K220" s="5" t="n"/>
-      <x:c r="L220" s="5" t="n"/>
-      <x:c r="M220" s="5" t="n"/>
-      <x:c r="N220" s="5" t="n"/>
-      <x:c r="O220" s="5" t="n"/>
+      <x:c r="A220" s="5" t="str">
+        <x:v>TC_VIZI_212</x:v>
+      </x:c>
+      <x:c r="B220" s="24" t="str">
+        <x:v>Backend secret scan guard 111</x:v>
+      </x:c>
+      <x:c r="C220" s="5" t="str">
+        <x:v>Verify production source and config do not contain hardcoded API keys, tokens, passwords, or provider secrets before commit.</x:v>
+      </x:c>
+      <x:c r="D220" s="5" t="str">
+        <x:v>Add ProductionSecretScanTests; scan backend production Java/resources, env production example, and frontend src; reject provider key formats and secret-like literal assignments; run scoped secret scan and full backend regression.</x:v>
+      </x:c>
+      <x:c r="E220" s="5" t="str">
+        <x:v>Spring Boot production source/config; provider patterns AIza, AQ., gh token prefixes, sk-; env placeholders allowed.</x:v>
+      </x:c>
+      <x:c r="F220" s="24" t="str">
+        <x:v>Hardcoded secrets fail the automated test; environment placeholders and example placeholders are allowed; full backend suite remains green.</x:v>
+      </x:c>
+      <x:c r="G220" s="5" t="str">
+        <x:v>PASS: ProductionSecretScanTests 1/1; full backend test suite 78/78.</x:v>
+      </x:c>
+      <x:c r="H220" s="5" t="str">
+        <x:v>TC_VIZI_211; step 111</x:v>
+      </x:c>
+      <x:c r="I220" s="5" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J220" s="5" t="str">
+        <x:v>2026-07-11</x:v>
+      </x:c>
+      <x:c r="K220" s="5"/>
+      <x:c r="L220" s="5"/>
+      <x:c r="M220" s="5"/>
+      <x:c r="N220" s="5"/>
+      <x:c r="O220" s="5"/>
       <x:c r="P220" s="5" t="n"/>
       <x:c r="Q220" s="5" t="n"/>
       <x:c r="R220" s="5" t="n"/>
@@ -38438,7 +38458,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a93b11a936f4586"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbd378e54f8647e4"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix transparent image rendering and editor chrome
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R4ed8f35d973746de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R3fcc641d45a84944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R22103a7a3e6b474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R2799097851f34e95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4550,6 +4550,44 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>E2E-094</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>Editor/Assets/Transparency UI</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Transparent image layer and quick color bar removal</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>Open editor with an image layer; inspect computed image CSS at desktop/mobile; verify the bottom quick color bar is absent; rerun background removal upload smoke.</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Processed PNG shows the card behind transparent pixels without a white rectangle; quick color bar is not rendered; mobile editor has no horizontal overflow.</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>PASS: frontend build; focused Playwright desktop/mobile smoke confirmed background rgba(0,0,0,0), no quick color bar, no console errors; real background-removal end-to-end smoke PASS.</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>Image layers no longer receive the generic white fill/border; mobile header padding is constrained for narrow editor viewports.</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>localhost FE5173 BE8080 rembg7000 Chrome</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4584,7 +4622,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Background removal upload flow + responsive editor smoke</x:v>
+        <x:v>Background removal + transparent image layer + editor chrome regression smoke</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4636,7 +4674,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-001,003,004,006-010,018,082-084,093</x:v>
+        <x:v>E2E-001,003,004,006-010,018,082-084,093-094</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4680,7 +4718,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local editor background-removal smoke evidence</x:v>
+        <x:v>Local background-removal and editor transparency smoke evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Build editor V2 foundation
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R22103a7a3e6b474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R2799097851f34e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra9a8053b951c4592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rda2b9a1f2e764e92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4588,6 +4588,258 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>E2E-095</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Independent V2 route and shell</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>Open /editor/phase1</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>V2 shell replaces editor route without loading V1</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>data-editor-version=2; two sidebars, center workspace, floating toolbar and V2 canvas rendered</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H75"/>
+      <x:c r="I75" t="str">
+        <x:v>V1 remains recoverable from local tag editor-v1-backup-20260716</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L75" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>E2E-096</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Fixed Front and Back sides</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Switch Front then Back from Pages panel</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>Exactly two sides; canvas, layer list and properties follow selected side</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Front 3 layers and Back 1 layer rendered; no add-page action</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H76"/>
+      <x:c r="I76" t="str">
+        <x:v>Playwright semantic snapshot</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>E2E-097</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Canvas zoom control</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Click Zoom in from 100%</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>Zoom changes without changing document geometry</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Zoom displayed 110%; canvas remained inside workspace</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H77"/>
+      <x:c r="I77" t="str">
+        <x:v>View-only UI state</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K77" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>E2E-098</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Local V2 save</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Click Save and read localStorage</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>Serializable schemaVersion 2 document is stored under the route design id</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>vizi.editor.v2.phase1 stored schemaVersion=2 with front/back pages and card metadata</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H78"/>
+      <x:c r="I78" t="str">
+        <x:v>Backend persistence intentionally deferred</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K78" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L78" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>E2E-099</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Invalid local document fallback</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Store malformed JSON then reload /editor/invalid-storage</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>Editor ignores malformed local data and creates a valid starter document</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Starter document rendered after reload; console remained clear</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H79"/>
+      <x:c r="I79" t="str">
+        <x:v>Parser returned safe fallback</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>E2E-100</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Mobile responsive containment</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Resize browser to 390x844 and inspect layout</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>No horizontal overflow; controls and card remain readable</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>scrollWidth=390 clientWidth=390; canvas width=377.5px</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H80"/>
+      <x:c r="I80" t="str">
+        <x:v>Screenshot output/playwright/editor-v2-mobile.png</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>localhost FE5175 390x844</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>E2E-101</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Editor console and auth request guard</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Reload V2 route and inspect browser console/network</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>No console errors and editor route does not request account API</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>0 console errors, 0 warnings after App editor-route guard</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H81"/>
+      <x:c r="I81" t="str">
+        <x:v>Frontend build also passed</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4622,7 +4874,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Background removal + transparent image layer + editor chrome regression smoke</x:v>
+        <x:v>Editor V2 Phase 1 shell, schema V2, local persistence and responsive regression</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4631,10 +4883,8 @@
           <x:t xml:space="preserve">FE</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">http://127.0.0.1:5173</x:t>
-        </x:is>
+      <x:c r="B4" t="str">
+        <x:v>http://127.0.0.1:5175</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4643,10 +4893,8 @@
           <x:t xml:space="preserve">BE</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">http://127.0.0.1:8080</x:t>
-        </x:is>
+      <x:c r="B5" t="str">
+        <x:v>Baseline backend suite 87/87 PASS; no backend required by V2 Phase 1</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4654,7 +4902,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>UP vizi-backend + rembg u2netp</x:v>
+        <x:v>Frontend build PASS; browser console 0 errors and 0 warnings</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4663,10 +4911,8 @@
           <x:t xml:space="preserve">Template seed</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">id=12 Vizi Luxury Demo Card 90x54 business</x:t>
-        </x:is>
+      <x:c r="B7" t="str">
+        <x:v>Editor V2 local starter document 90x54 with fixed Front and Back</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4674,7 +4920,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-001,003,004,006-010,018,082-084,093-094</x:v>
+        <x:v>E2E-095 through E2E-101</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4683,10 +4929,8 @@
           <x:t xml:space="preserve">Retest FAIL</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">E2E-025 grammar split, E2E-026 back link to /</x:t>
-        </x:is>
+      <x:c r="B9" t="str">
+        <x:v>None in Editor V2 Phase 1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4695,10 +4939,8 @@
           <x:t xml:space="preserve">Prior P0 open</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">E2E-031 Back place, E2E-037 text binding, E2E-046/075 preflight UI</x:t>
-        </x:is>
+      <x:c r="B10" t="str">
+        <x:v>E2E-031 Back place, E2E-037 text binding, E2E-046/075 preflight UI</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4707,10 +4949,8 @@
           <x:t xml:space="preserve">Shell</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">terminal/create not implemented   browser-only</x:t>
-        </x:is>
+      <x:c r="B11" t="str">
+        <x:v>Editor V2 route active; V1 recovery tag kept locally</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4718,7 +4958,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local background-removal and editor transparency smoke evidence</x:v>
+        <x:v>output/playwright/editor-v2-desktop.png; output/playwright/editor-v2-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Redesign editor V2 workspace UI
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra9a8053b951c4592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rda2b9a1f2e764e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R06e7a3161ba84dce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R88e94a6497d94973"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4840,6 +4840,258 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>E2E-102</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>Visual editor shell redesign</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>Open /editor/phase1 at 1440x900</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>UI follows the reference structure with a light header, vertical rail, Elements panel, center workspace and right Inspector</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Desktop screenshot shows the new five-region product editor surface; old dark shell is absent</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H82"/>
+      <x:c r="I82" t="str">
+        <x:v>Playwright screenshot .codex-work/editor-v2-redesign-desktop.png</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K82" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>E2E-103</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>Fixed card sides and format dock</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>Inspect bottom card sides and switch Front/Back</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>Only Front and Back are available; no Add page action; card format remains 90 x 54 mm</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>Front and Back dock rendered; both sides switch canvas and inspector metadata; fixed card format visible</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H83"/>
+      <x:c r="I83" t="str">
+        <x:v>Playwright semantic snapshot</x:v>
+      </x:c>
+      <x:c r="J83" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K83" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L83" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>E2E-104</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>Text layer inspector</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>Open editor with starter document</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>Inspector opens with text content, font, weight, size, alignment, fill and geometry controls</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>TEXT inspector rendered with Vizi Studio, font controls, fill swatches and X/Y/W/H inputs</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H84"/>
+      <x:c r="I84" t="str">
+        <x:v>Selected starter text layer</x:v>
+      </x:c>
+      <x:c r="J84" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K84" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L84" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>E2E-105</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>Layer panel controls</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>Open Layers rail and inspect Front</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>Layers panel lists the current side and exposes visibility and lock buttons</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>Front layers=3; Tagline, Brand name and Accent each expose visibility and lock controls</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H85"/>
+      <x:c r="I85" t="str">
+        <x:v>Playwright semantic snapshot</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K85" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L85" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>E2E-106</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>Responsive editor containment</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>Resize browser to 390x844</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>No horizontal overflow and card remains inside viewport</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>scrollWidth=390 clientWidth=390; canvas width=304.2px; canvasRight=377.7px</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H86"/>
+      <x:c r="I86" t="str">
+        <x:v>Mobile screenshot .codex-work/editor-v2-redesign-mobile.png</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K86" t="str">
+        <x:v>localhost FE5175 390x844</x:v>
+      </x:c>
+      <x:c r="L86" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>E2E-107</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>Browser console regression</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Reload redesigned editor and read console</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>No errors or warnings from the new shell</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Playwright console reported Errors=0 and Warnings=0</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H87"/>
+      <x:c r="I87" t="str">
+        <x:v>Playwright console command</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K87" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L87" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>E2E-108</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>Frontend source guards</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Run production build and XSS guard</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>Vue typecheck/build and static XSS guard remain green after UI redesign</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>npm run build PASS; npm run test:xss PASS</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H88"/>
+      <x:c r="I88" t="str">
+        <x:v>Vite chunk warning remains non-blocking</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K88" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L88" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4874,7 +5126,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 Phase 1 shell, schema V2, local persistence and responsive regression</x:v>
+        <x:v>Editor V2 visual shell redesign, fixed card dock, layer inspector and responsive containment</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4894,7 +5146,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Baseline backend suite 87/87 PASS; no backend required by V2 Phase 1</x:v>
+        <x:v>Backend unchanged; previous 87/87 suite remains green</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4902,7 +5154,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Frontend build PASS; browser console 0 errors and 0 warnings</x:v>
+        <x:v>Frontend build PASS; XSS guard PASS; browser console 0 errors and 0 warnings</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4912,7 +5164,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor V2 local starter document 90x54 with fixed Front and Back</x:v>
+        <x:v>Editor V2 visual shell with fixed 90x54 card and Front/Back only</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4920,7 +5172,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-095 through E2E-101</x:v>
+        <x:v>E2E-095 through E2E-108</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4930,7 +5182,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None in Editor V2 Phase 1</x:v>
+        <x:v>None in Editor V2 visual shell phase</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4950,7 +5202,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Editor V2 route active; V1 recovery tag kept locally</x:v>
+        <x:v>Editor V2 visual shell active; V1 recovery tag kept locally</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4958,7 +5210,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>output/playwright/editor-v2-desktop.png; output/playwright/editor-v2-mobile.png</x:v>
+        <x:v>.codex-work/editor-v2-redesign-desktop.png; .codex-work/editor-v2-redesign-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Implement bounded layer dragging
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R06e7a3161ba84dce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R88e94a6497d94973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R6d6a445e2b81493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rc1bc894d0d9c48ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5092,6 +5092,222 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>E2E-109</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>Bounded layer drag</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Open /editor/phase1 at 1440x900 and select an unlocked text layer</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>Dragging a layer updates its X/Y position while retaining selection</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Real Playwright mouse drag moved Business card editor V2 from its starter position to X=31.9, Y=67.2</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H89"/>
+      <x:c r="I89" t="str">
+        <x:v>Playwright mouse drag and geometry readback</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K89" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L89" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>E2E-110</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>Canvas boundary clamp</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>Select an unlocked layer and drag beyond the canvas edges</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>Layer position is clamped so the full layer remains inside the fixed card</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>Top-left clamp returned X=0, Y=0; bottom-right clamp returned X=34, Y=88 for W=66, H=12</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H90"/>
+      <x:c r="I90" t="str">
+        <x:v>Playwright boundary drags and geometry readback</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K90" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>E2E-111</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>Locked layer drag protection</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Lock Vizi Studio and drag across the canvas</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>Locked layer cannot move and remains selected after the pointer gesture</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Geometry stayed X=0, Y=0 and Vizi Studio remained selected after a long drag</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H91"/>
+      <x:c r="I91" t="str">
+        <x:v>Playwright lock, drag and geometry readback</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K91" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L91" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>E2E-112</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>Unsaved drag state</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Drag an unlocked layer</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>A position change is visible as an unsaved local edit</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Header changed to Unsaved changes immediately after the drag</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H92"/>
+      <x:c r="I92" t="str">
+        <x:v>Playwright status readback</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K92" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L92" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>E2E-113</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>Drag preserves card invariants</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Switch Back and return Front after drag</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>The editor keeps exactly two sides and the selected 90 x 54 mm card format</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Back card canvas and Front card canvas switched successfully; 2 sides and 90 x 54 mm remained visible; no Add page action</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H93"/>
+      <x:c r="I93" t="str">
+        <x:v>Playwright side-switch and semantic readback</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K93" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L93" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>E2E-114</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Drag regression checks</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>Run mobile browser check, console check, build and XSS guard</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>The drag implementation does not introduce overflow, console regressions or source guard failures</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>390x844 scrollWidth=390/clientWidth=390; console Errors=0 Warnings=0; npm run build PASS; npm run test:xss PASS</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H94"/>
+      <x:c r="I94" t="str">
+        <x:v>Playwright mobile/console plus npm checks; existing Vite chunk warning is non-blocking</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="K94" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L94" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5126,7 +5342,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 visual shell redesign, fixed card dock, layer inspector and responsive containment</x:v>
+        <x:v>Editor V2 Canvas Core 2A: bounded layer dragging, lock protection and dirty state</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5154,7 +5370,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Frontend build PASS; XSS guard PASS; browser console 0 errors and 0 warnings</x:v>
+        <x:v>Browser drag PASS; boundary clamp PASS; locked layer PASS; mobile containment PASS; console 0 errors and 0 warnings; build PASS; XSS guard PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5164,7 +5380,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor V2 visual shell with fixed 90x54 card and Front/Back only</x:v>
+        <x:v>Editor V2 visual shell with fixed 90x54 card, Front/Back only and bounded layer movement</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5172,7 +5388,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-095 through E2E-108</x:v>
+        <x:v>E2E-095 through E2E-114</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5182,7 +5398,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None in Editor V2 visual shell phase</x:v>
+        <x:v>None in Canvas Core 2A</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5192,7 +5408,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-031 Back place, E2E-037 text binding, E2E-046/075 preflight UI</x:v>
+        <x:v>E2E-102 shell, E2E-103 fixed sides/format, E2E-105 layer controls, E2E-108 source guards</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5202,7 +5418,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Editor V2 visual shell active; V1 recovery tag kept locally</x:v>
+        <x:v>Editor V2 Canvas Core 2A active; V1 recovery tag kept locally</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5210,7 +5426,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>.codex-work/editor-v2-redesign-desktop.png; .codex-work/editor-v2-redesign-mobile.png</x:v>
+        <x:v>.codex-work/editor-v2-drag-desktop.png; .codex-work/editor-v2-drag-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add bounded layer resizing
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R6d6a445e2b81493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rc1bc894d0d9c48ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rd98d8493fb7a4c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R44dc36bac57f4af4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5308,6 +5308,258 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>E2E-115</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>Selected layer resize handle</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Open /editor/resize-step-2b with the starter Brand name selected</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Exactly one accessible resize handle is visible for the selected unlocked layer</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Semantic snapshot exposed button Resize Brand name; handleCount=1 and no handle appeared on unselected layers</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H95"/>
+      <x:c r="I95" t="str">
+        <x:v>Playwright semantic snapshot and DOM readback</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K95" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L95" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>E2E-116</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>Pointer resize and dirty state</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Drag the selected Brand name bottom-right resize handle</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>W/H update from pointer movement, selection remains, and the editor becomes dirty</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Real mouse drag changed W/H from 66/20 to 77.1/29.3; Vizi Studio remained selected; status became Unsaved changes</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H96"/>
+      <x:c r="I96" t="str">
+        <x:v>Playwright real mouse resize and geometry readback</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K96" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L96" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>E2E-117</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Resize min and card boundary clamp</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Drag the resize handle far inward, then beyond the card bottom-right</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Layer dimensions stay above the minimum and the full layer remains inside the fixed card</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Minimum clamp returned W=2, H=2; maximum clamp returned W=82, H=76 at X=18, Y=24; rendered bounds stayed inside canvas</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H97"/>
+      <x:c r="I97" t="str">
+        <x:v>Playwright min/max pointer drags and DOM bounds</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>E2E-118</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Locked layer resize protection</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Lock the selected Brand name and attempt a pointer gesture at its bottom-right</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Resize handle is hidden and locked geometry cannot change</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>handleCount=0; geometry stayed X=18, Y=24, W=82, H=76; Vizi Studio remained selected</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H98"/>
+      <x:c r="I98" t="str">
+        <x:v>Playwright lock and pointer regression</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K98" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L98" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>E2E-119</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>Mobile resize containment</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Resize viewport to 390x844 and resize the selected unlocked layer</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>Handle remains usable inside the card and the editor does not overflow horizontally</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>Mobile resize changed W/H to 69.8/54.1; handleRight=337.8 within canvasRight=377.7; scrollWidth=390 clientWidth=390</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H99"/>
+      <x:c r="I99" t="str">
+        <x:v>Playwright mobile pointer resize and screenshot</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K99" t="str">
+        <x:v>localhost FE5175 390x844</x:v>
+      </x:c>
+      <x:c r="L99" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>E2E-120</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>Resize local save and reload</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>Save the resized document locally and reopen the same editor URL</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>Resized W/H serialize in V2 JSON and restore after reload</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Stored front-title width=69.8 and height=54.1; reload restored geometry, selection and one resize handle</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H100"/>
+      <x:c r="I100" t="str">
+        <x:v>localStorage JSON readback and Playwright reload</x:v>
+      </x:c>
+      <x:c r="J100" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K100" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L100" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>E2E-121</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>Resize regression checks</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Run frontend production build, XSS guard, browser console and visual screenshots</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>Resize introduces no type, build, XSS, console or responsive regression</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>npm run build PASS; npm run test:xss PASS; console Errors=0 Warnings=0; desktop/mobile screenshots visually inspected</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H101"/>
+      <x:c r="I101" t="str">
+        <x:v>Vite chunk warning remains non-blocking</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K101" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L101" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5334,7 +5586,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>2026-07-16</x:v>
+        <x:v>2026-07-17</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5342,7 +5594,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 Canvas Core 2A: bounded layer dragging, lock protection and dirty state</x:v>
+        <x:v>Editor V2 Canvas Core 2B: selected-layer resize, min/max clamp, lock protection and persistence</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5362,7 +5614,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Backend unchanged; previous 87/87 suite remains green</x:v>
+        <x:v>Backend unchanged and not rerun in this frontend-only step; last baseline 87/87 PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5370,7 +5622,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Browser drag PASS; boundary clamp PASS; locked layer PASS; mobile containment PASS; console 0 errors and 0 warnings; build PASS; XSS guard PASS</x:v>
+        <x:v>Pointer resize PASS; min/max clamp PASS; locked layer PASS; mobile containment PASS; save/reload PASS; console 0 errors and 0 warnings; build PASS; XSS guard PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5380,7 +5632,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor V2 visual shell with fixed 90x54 card, Front/Back only and bounded layer movement</x:v>
+        <x:v>Editor V2 fixed 90x54 card with Front/Back only, bounded layer movement and bounded selected-layer resize</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5388,7 +5640,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-095 through E2E-114</x:v>
+        <x:v>E2E-095 through E2E-121</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5398,7 +5650,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None in Canvas Core 2A</x:v>
+        <x:v>None in Canvas Core 2B</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5408,7 +5660,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-102 shell, E2E-103 fixed sides/format, E2E-105 layer controls, E2E-108 source guards</x:v>
+        <x:v>E2E-109 drag, E2E-110 movement clamp, E2E-111 lock protection, E2E-114 source guards</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5418,7 +5670,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Editor V2 Canvas Core 2A active; V1 recovery tag kept locally</x:v>
+        <x:v>Editor V2 Canvas Core 2B active; V1 recovery tag kept locally</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5426,7 +5678,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>.codex-work/editor-v2-drag-desktop.png; .codex-work/editor-v2-drag-mobile.png</x:v>
+        <x:v>.codex-work/editor-v2-resize-desktop.png; .codex-work/editor-v2-resize-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add layer rotation controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rd98d8493fb7a4c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R44dc36bac57f4af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R464bedd8000a4778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R0fea4e61dbfd4faa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5560,6 +5560,294 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>E2E-122</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>Selected layer rotate handle</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>Open /editor/rotate-step-2c with the starter Brand name selected</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>Exactly one accessible rotate handle is visible for the selected unlocked layer</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Semantic snapshot exposed button Rotate Brand name; handleCount=1 and the selected layer retained its resize handle</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H102"/>
+      <x:c r="I102" t="str">
+        <x:v>Playwright semantic snapshot and DOM readback</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K102" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L102" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>E2E-123</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>Pointer rotation and dirty state</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>Drag the rotate handle around the selected layer center</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>Rotation follows the pointer, selection remains, and the editor becomes dirty</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>Real mouse rotation changed the rendered transform to rotate(90.5deg); Vizi Studio remained selected; status became Unsaved changes</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H103"/>
+      <x:c r="I103" t="str">
+        <x:v>Playwright real mouse rotation and DOM transform readback</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K103" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L103" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>E2E-124</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>Rotation normalization</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>Continue rotating through the opposite side of the layer center</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>Rotation remains normalized to a stable 0..360 degree value</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>Second pointer rotation produced rotate(270.4deg), preserving one-decimal precision and normalized range</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H104"/>
+      <x:c r="I104" t="str">
+        <x:v>Playwright multi-angle rotation</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K104" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L104" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>E2E-125</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>Locked layer rotate protection</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Lock the selected Brand name and attempt a pointer gesture</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>Rotate handle is hidden and locked rotation cannot change</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>handleCount=0; transform stayed rotate(270.4deg); Vizi Studio remained selected</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H105"/>
+      <x:c r="I105" t="str">
+        <x:v>Playwright lock and pointer regression</x:v>
+      </x:c>
+      <x:c r="J105" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K105" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L105" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>E2E-126</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>Mobile rotate containment</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Resize viewport to 390x844 and rotate the selected unlocked layer</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>Rotate handle remains usable and rotation does not create horizontal overflow</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>Mobile rotation produced rotate(176.1deg); scrollWidth=390 clientWidth=390; handle stayed inside the card viewport</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H106"/>
+      <x:c r="I106" t="str">
+        <x:v>Playwright mobile pointer rotation and screenshot</x:v>
+      </x:c>
+      <x:c r="J106" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K106" t="str">
+        <x:v>localhost FE5175 390x844</x:v>
+      </x:c>
+      <x:c r="L106" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>E2E-127</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>Rotate local save and reload</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>Save the rotated document locally and reopen the same editor URL</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>Rotation serializes in V2 JSON and restores after reload</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Stored front-title rotation=176.1; reload restored transform rotate(176.1deg) and one rotate handle</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H107"/>
+      <x:c r="I107" t="str">
+        <x:v>localStorage JSON readback and Playwright reload</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K107" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L107" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>E2E-128</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>Rotate preserves card invariants</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>Switch Back and return Front after rotating a layer</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>The editor keeps exactly two sides and the fixed 90 x 54 mm card format</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Back card canvas and Front card canvas switched successfully; 2 sides and 90 x 54 mm remained visible</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H108"/>
+      <x:c r="I108" t="str">
+        <x:v>Playwright side-switch and semantic readback</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K108" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L108" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>E2E-129</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>Rotate regression checks</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Run frontend production build, XSS guard, browser console and visual screenshots</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>Rotate introduces no type, build, XSS, console or responsive regression</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>npm run build PASS; npm run test:xss PASS; console Errors=0 Warnings=0; desktop/mobile screenshots visually inspected</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H109"/>
+      <x:c r="I109" t="str">
+        <x:v>Vite chunk warning remains non-blocking</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K109" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L109" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5594,7 +5882,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 Canvas Core 2B: selected-layer resize, min/max clamp, lock protection and persistence</x:v>
+        <x:v>Editor V2 Canvas Core 2C: selected-layer rotation, normalized angles, lock protection and persistence</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5622,7 +5910,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Pointer resize PASS; min/max clamp PASS; locked layer PASS; mobile containment PASS; save/reload PASS; console 0 errors and 0 warnings; build PASS; XSS guard PASS</x:v>
+        <x:v>Pointer rotation PASS; normalized angle PASS; locked layer PASS; mobile containment PASS; save/reload PASS; Front/Back invariant PASS; console 0 errors and 0 warnings; build PASS; XSS guard PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5632,7 +5920,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor V2 fixed 90x54 card with Front/Back only, bounded layer movement and bounded selected-layer resize</x:v>
+        <x:v>Editor V2 fixed 90x54 card with Front/Back only, bounded movement/resize and selected-layer rotation</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5640,7 +5928,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-095 through E2E-121</x:v>
+        <x:v>E2E-095 through E2E-129</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5650,7 +5938,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None in Canvas Core 2B</x:v>
+        <x:v>None in Canvas Core 2C</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5660,7 +5948,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-109 drag, E2E-110 movement clamp, E2E-111 lock protection, E2E-114 source guards</x:v>
+        <x:v>E2E-115 resize handle, E2E-117 resize clamp, E2E-118 lock protection, E2E-121 source guards</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5670,7 +5958,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Editor V2 Canvas Core 2B active; V1 recovery tag kept locally</x:v>
+        <x:v>Editor V2 Canvas Core 2C active; V1 recovery tag kept locally</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5678,7 +5966,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>.codex-work/editor-v2-resize-desktop.png; .codex-work/editor-v2-resize-mobile.png</x:v>
+        <x:v>.codex-work/editor-v2-rotate-desktop.png; .codex-work/editor-v2-rotate-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Implement editor selection chrome toolbar
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R464bedd8000a4778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R0fea4e61dbfd4faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R49cb67fc4c2c4f6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R83e50c82db274a40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5848,6 +5848,366 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>E2E-130</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>Eight-handle selection chrome</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Select Brand name on Front canvas</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>Blue border, 8 resize handles, top rotate stem and 5-button floating toolbar render</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>8 resize handles, rotate handle and Duplicate/Lock/Bring/Send/Delete toolbar rendered</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H110"/>
+      <x:c r="I110" t="str">
+        <x:v>Visual comparison against supplied selection reference</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K110" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L110" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>E2E-131</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>Directional pointer resize</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>Drag NW handle down/right, then drag E handle left</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>NW updates X/Y/W/H; E updates only W; geometry remains inside card</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>NW 18/24/66/20 -&gt; 23/28.2/61/15.8; E -&gt; 23/28.2/55.7/15.8</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H111"/>
+      <x:c r="I111" t="str">
+        <x:v>Real Playwright mouse events on two independent directions</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K111" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L111" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>E2E-132</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>Rotation chrome and live badge</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Drag top rotate handle about 15 degrees and inspect toolbar/badge</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>Selection rotates; toolbar stays horizontal above bounding box; live size/angle badge appears below</x:v>
+      </x:c>
+      <x:c r="F112" t="str">
+        <x:v>Badge 66 x 20 - 14.8 degrees; toolbar gap above rotated bounds 45.87px</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H112"/>
+      <x:c r="I112" t="str">
+        <x:v>Screenshot editor-v2-selection-chrome-rotating.png</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K112" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L112" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>E2E-133</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>Duplicate toolbar action</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Click Duplicate layer</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>One offset copy is created and selected without console error</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>Layer count 3 -&gt; 4; copy at X20 Y26; reactive proxy clone error fixed; console 0 errors</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H113"/>
+      <x:c r="I113" t="str">
+        <x:v>Retested after replacing structuredClone with flat layer copy</x:v>
+      </x:c>
+      <x:c r="J113" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K113" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L113" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>E2E-134</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>Toolbar lock guard</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Lock selected copy, inspect handles, then attempt drag</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>Resize/rotate controls disappear and locked geometry cannot move; Unlock remains available</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>Handles 8 -&gt; 0; rotate 1 -&gt; 0; geometry stayed 20/26/66/20 after drag</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H114"/>
+      <x:c r="I114" t="str">
+        <x:v>Toolbar remains available for unlock</x:v>
+      </x:c>
+      <x:c r="J114" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K114" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L114" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>E2E-135</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>Layer z-order toolbar actions</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>Click Bring forward then Send backward on selected copy</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>Selected layer moves one index in each direction and returns to original order</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>DOM order changed accent/title/copy/subtitle -&gt; accent/title/subtitle/copy -&gt; original</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H115"/>
+      <x:c r="I115" t="str">
+        <x:v>Canvas render order and Layers panel follow array order</x:v>
+      </x:c>
+      <x:c r="J115" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K115" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L115" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>E2E-136</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>Delete toolbar action</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>Delete selected copy</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>Layer is removed and selection falls back to a visible text layer</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>Layer count 4 -&gt; 3; selected Vizi Studio fallback retained 8 handles</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H116"/>
+      <x:c r="I116" t="str">
+        <x:v>No stale selection or console error</x:v>
+      </x:c>
+      <x:c r="J116" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K116" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L116" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>E2E-137</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>Toolbar action persistence</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>Duplicate, Save, reload same editor route, then switch Back</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>Copy persists; exactly Front/Back remain; both sides keep 90 x 54 mm</x:v>
+      </x:c>
+      <x:c r="F117" t="str">
+        <x:v>Reload retained 4 Front layers with 1 copy; Back had 1 layer; side buttons=2; size=90 x 54 mm</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H117"/>
+      <x:c r="I117" t="str">
+        <x:v>Schema V2 unchanged</x:v>
+      </x:c>
+      <x:c r="J117" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K117" t="str">
+        <x:v>localhost FE5175 localStorage</x:v>
+      </x:c>
+      <x:c r="L117" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>E2E-138</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>Mobile selection containment</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Resize browser to 390x844 on Back side and inspect layout</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>No horizontal overflow; card, toolbar, sides and Inspector remain contained</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>innerWidth=390; body/root scrollWidth=390; toolbar left=132.59 right=318.59</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H118"/>
+      <x:c r="I118" t="str">
+        <x:v>Screenshot editor-v2-selection-chrome-mobile.png</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K118" t="str">
+        <x:v>localhost FE5175 390x844</x:v>
+      </x:c>
+      <x:c r="L118" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>E2E-139</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>Final build, XSS and console guard</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Run frontend build, XSS static guard and browser console scan</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>Typecheck/build and XSS pass; browser has no errors or warnings</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>vue-tsc plus Vite build PASS; XSS static guard PASS; console 0 errors and 0 warnings</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H119"/>
+      <x:c r="I119" t="str">
+        <x:v>Chunk-size warning unchanged and non-blocking</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K119" t="str">
+        <x:v>frontend and localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L119" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5882,7 +6242,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 Canvas Core 2C: selected-layer rotation, normalized angles, lock protection and persistence</x:v>
+        <x:v>Editor V2 selection chrome correction and floating toolbar actions</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5902,7 +6262,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Backend unchanged and not rerun in this frontend-only step; last baseline 87/87 PASS</x:v>
+        <x:v>Backend unchanged; not rerun for frontend-only selection chrome work</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5910,7 +6270,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Pointer rotation PASS; normalized angle PASS; locked layer PASS; mobile containment PASS; save/reload PASS; Front/Back invariant PASS; console 0 errors and 0 warnings; build PASS; XSS guard PASS</x:v>
+        <x:v>Frontend build and XSS guard PASS; browser console 0 errors and 0 warnings</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5920,7 +6280,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor V2 fixed 90x54 card with Front/Back only, bounded movement/resize and selected-layer rotation</x:v>
+        <x:v>Schema V2 unchanged; fixed 90 x 54 mm Front and Back document</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5928,7 +6288,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-095 through E2E-129</x:v>
+        <x:v>E2E-130 through E2E-139</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5938,7 +6298,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None in Canvas Core 2C</x:v>
+        <x:v>None after DataCloneError fix and full retest</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5948,7 +6308,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-115 resize handle, E2E-117 resize clamp, E2E-118 lock protection, E2E-121 source guards</x:v>
+        <x:v>E2E-115 through E2E-129 resize, rotate and persistence regression</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5958,7 +6318,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Editor V2 Canvas Core 2C active; V1 recovery tag kept locally</x:v>
+        <x:v>Eight-handle selection chrome and toolbar actions verified end to end</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5966,7 +6326,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>.codex-work/editor-v2-rotate-desktop.png; .codex-work/editor-v2-rotate-mobile.png</x:v>
+        <x:v>output/playwright/editor-v2-selection-chrome-desktop.png; output/playwright/editor-v2-selection-chrome-rotating.png; output/playwright/editor-v2-selection-chrome-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add V2 editor layer creation tools
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R49cb67fc4c2c4f6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R83e50c82db274a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Re8944ed615524dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R16b951abdfca4626"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6208,6 +6208,330 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>E2E-140</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>Text tool layer creation</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Click the Canvas tools Text button on Front</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>A new text layer is added, selected, editable in Inspector and geometry stays within the card</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>Front layers 3 -&gt; 4; New text selected; TEXT inspector and 90 x 54 mm card remained visible; status Unsaved changes</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H120"/>
+      <x:c r="I120" t="str">
+        <x:v>Real Playwright click and semantic snapshot</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L120" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>E2E-141</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>Rectangle tool layer creation</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Click the Rectangle shape/tool button</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>A rectangle layer is added with visible fill, selection chrome and geometry inside the card</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>Front layers 4 -&gt; 5; Rectangle selected; fill #d9b979; W/H 28/28; 8 handles and rotate control rendered</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H121"/>
+      <x:c r="I121" t="str">
+        <x:v>Canvas tool and Elements shape path</x:v>
+      </x:c>
+      <x:c r="J121" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K121" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L121" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>E2E-142</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>Ellipse tool layer creation</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Click the Ellipse shape/tool button</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>An ellipse layer is added with ellipse rendering and independent selection</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>Front layers 5 -&gt; 6; Ellipse selected; fill #0d766d; ellipse selection chrome rendered</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H122"/>
+      <x:c r="I122" t="str">
+        <x:v>Real Playwright click and inspector readback</x:v>
+      </x:c>
+      <x:c r="J122" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K122" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L122" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>E2E-143</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>Image file picker layer creation</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Open Image tool and upload a valid PNG</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>A rendered image layer is added from a serializable data URL and selected</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>Front layers 6 -&gt; 7; data:image/png;base64 source; img complete=true; naturalWidth=1440; image selected</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H123"/>
+      <x:c r="I123" t="str">
+        <x:v>Playwright file chooser upload using a real local PNG</x:v>
+      </x:c>
+      <x:c r="J123" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K123" t="str">
+        <x:v>localhost FE5175 1440x900</x:v>
+      </x:c>
+      <x:c r="L123" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>E2E-144</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>Image MIME guard</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Open Image tool and provide a non-image text file</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>Invalid MIME is rejected without adding a layer or unsafe source</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>Vizi.md upload left Front layer count at 7; no image layer was created</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H124"/>
+      <x:c r="I124" t="str">
+        <x:v>Upload trust-boundary negative test</x:v>
+      </x:c>
+      <x:c r="J124" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K124" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L124" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>E2E-145</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>Created layer persistence</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Save the created layers and reload the same editor route</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>Text, rectangle, ellipse and image layers persist with image data URL</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>Reload retained 7 Front layers and 1 rendered image; all created layer ids remained in V2 JSON</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H125"/>
+      <x:c r="I125" t="str">
+        <x:v>LocalStorage save/reload and DOM readback</x:v>
+      </x:c>
+      <x:c r="J125" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K125" t="str">
+        <x:v>localhost FE5175 localStorage</x:v>
+      </x:c>
+      <x:c r="L125" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>E2E-146</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>Fixed card page invariants</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Switch to Back after creating Front layers</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>Only Front/Back are available, Back data is isolated, and card format remains fixed</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>Back card canvas; Back has 1 layer; page buttons=2; 90 x 54 mm remained visible</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H126"/>
+      <x:c r="I126" t="str">
+        <x:v>Playwright side switch and semantic readback</x:v>
+      </x:c>
+      <x:c r="J126" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K126" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L126" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>E2E-147</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>Mobile layer creation containment</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>Resize browser to 390x844 and inspect the selected layer toolbar</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>No horizontal overflow and floating chrome remains inside the viewport</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>body/root scrollWidth=375 &lt;= viewport 390; toolbar left=132.59 right=318.59; mobile screenshot captured</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H127"/>
+      <x:c r="I127" t="str">
+        <x:v>Screenshot editor-v2-layer-creation-mobile.png</x:v>
+      </x:c>
+      <x:c r="J127" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K127" t="str">
+        <x:v>localhost FE5175 390x844</x:v>
+      </x:c>
+      <x:c r="L127" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>E2E-148</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>Layer creation regression guards</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Run frontend build, XSS guard and browser console scan</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>Typecheck/build, XSS and console checks pass after tool and upload changes</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>vue-tsc plus Vite build PASS; XSS static guard PASS; console 0 errors and 0 warnings</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H128"/>
+      <x:c r="I128" t="str">
+        <x:v>Chunk-size warning unchanged and non-blocking</x:v>
+      </x:c>
+      <x:c r="J128" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K128" t="str">
+        <x:v>frontend and localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L128" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6242,7 +6566,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 selection chrome correction and floating toolbar actions</x:v>
+        <x:v>Editor V2 real layer creation from Text, Rectangle, Ellipse and Image</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -6262,7 +6586,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Backend unchanged; not rerun for frontend-only selection chrome work</x:v>
+        <x:v>Backend unchanged; not rerun for frontend-only layer creation work</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6288,7 +6612,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-130 through E2E-139</x:v>
+        <x:v>E2E-140 through E2E-148</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6298,7 +6622,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after DataCloneError fix and full retest</x:v>
+        <x:v>None after valid/invalid image upload and save-reload retest</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6308,7 +6632,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-115 through E2E-129 resize, rotate and persistence regression</x:v>
+        <x:v>E2E-130 through E2E-139 selection chrome and toolbar actions</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6318,7 +6642,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Eight-handle selection chrome and toolbar actions verified end to end</x:v>
+        <x:v>Text, shape and image layer creation verified end to end with serializable image data</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6326,7 +6650,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>output/playwright/editor-v2-selection-chrome-desktop.png; output/playwright/editor-v2-selection-chrome-rotating.png; output/playwright/editor-v2-selection-chrome-mobile.png</x:v>
+        <x:v>output/playwright/editor-v2-layer-creation-desktop.png; output/playwright/editor-v2-layer-creation-mobile.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Build contextual Editor V2 toolbars
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Re8944ed615524dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R16b951abdfca4626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ree539fb619c4490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rd37ecc48dcf0498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6532,6 +6532,386 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>E2E-149</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>Editor V2/Toolbars</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>Desktop two-sidebar layout</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Open /editor/toolbars-smoke at 1440x1000 and measure rail, left panel, workspace, inspector and canvas bounds.</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>Both side toolbars remain separate from the central workspace and do not clip the card canvas.</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>Rail 68px; left 288px; workspace 754px; right 330px; 660px canvas stayed inside workspace bounds.</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H129" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I129" t="str">
+        <x:v>Automated bounding-box assertions.</x:v>
+      </x:c>
+      <x:c r="J129" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K129" t="str">
+        <x:v>localhost FE5173 Chrome 1440x1000</x:v>
+      </x:c>
+      <x:c r="L129" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="str">
+        <x:v>E2E-150</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>Editor V2/Left toolbar</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>Working editor sections only</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Inspect and use Elements, Text, Uploads, Brand and Layers panels.</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>Visible sections expose working controls; unsupported AI, Stock and Apps placeholders are not shown.</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>Five functional sections rendered; text presets, three supported shapes, image upload, colors and layer controls operated.</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H130" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I130" t="str">
+        <x:v>No fake unsupported controls in the rail.</x:v>
+      </x:c>
+      <x:c r="J130" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K130" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L130" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" t="str">
+        <x:v>E2E-151</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>Editor V2/Right toolbar</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>Page inspector and fixed card constraints</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Clear selection, switch Front/Back and inspect Page settings.</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>Page inspector shows fixed 90 x 54 mm card, exactly Front/Back, and editable background.</x:v>
+      </x:c>
+      <x:c r="F131" t="str">
+        <x:v>Page inspector displayed 90 x 54 mm; two side buttons only; side/background actions updated the active page.</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H131" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I131" t="str">
+        <x:v>Business-card page count remains fixed.</x:v>
+      </x:c>
+      <x:c r="J131" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K131" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L131" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="str">
+        <x:v>E2E-152</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>Editor V2/Right toolbar</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>Text contextual inspector</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>Add Title; edit content, font size, alignment, bold, fill and X position in millimeters.</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>Text controls update serializable text-layer fields and content is rendered as text, not HTML.</x:v>
+      </x:c>
+      <x:c r="F132" t="str">
+        <x:v>Content, size 24, center alignment, bold and X=10mm serialized; injected img/onerror text created no DOM image and no marker.</x:v>
+      </x:c>
+      <x:c r="G132" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H132" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I132" t="str">
+        <x:v>Includes XSS negative check.</x:v>
+      </x:c>
+      <x:c r="J132" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K132" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L132" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>E2E-153</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>Editor V2/Right toolbar</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>Shape contextual inspector</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>Add Rounded shape; set stroke width and opacity; inspect radius and geometry.</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>Rounded preset and shape controls update fill/stroke/radius/geometry/opacity without leaving card bounds.</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>cornerRadius=16, strokeWidth=2 and opacity=0.65 serialized for Rounded rectangle.</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H133" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I133" t="str">
+        <x:v>Shape state persisted in V2 JSON.</x:v>
+      </x:c>
+      <x:c r="J133" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K133" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L133" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>E2E-154</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>Editor V2/Right toolbar</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>Image contextual inspector and media list</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>Upload a valid PNG, inspect Image panel, media thumbnail and Replace image action.</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>Valid image is selected, previewed, listed under Your media and can be replaced.</x:v>
+      </x:c>
+      <x:c r="F134" t="str">
+        <x:v>Image inspector and Replace image rendered; one safe data:image/png;base64 source listed and serialized.</x:v>
+      </x:c>
+      <x:c r="G134" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H134" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I134" t="str">
+        <x:v>PNG trust boundary retained.</x:v>
+      </x:c>
+      <x:c r="J134" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K134" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L134" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>E2E-155</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>Editor V2/Layers</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>Layer drag reorder</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>Open Layers and drag the top Image layer before the bottom layer.</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>Displayed layer order and backing render order change, selection remains valid and document becomes dirty.</x:v>
+      </x:c>
+      <x:c r="F135" t="str">
+        <x:v>Order changed from Image|Rounded rectangle|Title|Tagline|Brand name|Accent to Rounded rectangle|Title|Tagline|Brand name|Image|Accent.</x:v>
+      </x:c>
+      <x:c r="G135" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H135" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I135" t="str">
+        <x:v>Native HTML drag-and-drop with JSON order readback.</x:v>
+      </x:c>
+      <x:c r="J135" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K135" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L135" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>E2E-156</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>Editor V2/Persistence</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>Toolbar edits save and reload</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>Save the edited document, reload the route and inspect localStorage/document layers.</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>Text, shape, image and reordered layers persist while card size and two-side invariant remain unchanged.</x:v>
+      </x:c>
+      <x:c r="F136" t="str">
+        <x:v>Six Front layers reloaded; fixed 90 x 54 mm retained; text, shape and image fields matched saved values.</x:v>
+      </x:c>
+      <x:c r="G136" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H136" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I136" t="str">
+        <x:v>LocalStorage V2 persistence regression.</x:v>
+      </x:c>
+      <x:c r="J136" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K136" t="str">
+        <x:v>localhost FE5173 localStorage</x:v>
+      </x:c>
+      <x:c r="L136" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>E2E-157</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>Editor V2/Responsive</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>Mobile two-toolbar containment</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Resize to 390x844 and measure editor, rail, workspace, inspector and document scroll width.</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>Each major editor region uses full mobile width and no horizontal overflow is introduced.</x:v>
+      </x:c>
+      <x:c r="F137" t="str">
+        <x:v>Editor, rail, workspace and inspector each measured 390px; document scrollWidth=390px.</x:v>
+      </x:c>
+      <x:c r="G137" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H137" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I137" t="str">
+        <x:v>Fixed app-shell mobile padding regression.</x:v>
+      </x:c>
+      <x:c r="J137" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K137" t="str">
+        <x:v>localhost FE5173 Chrome 390x844</x:v>
+      </x:c>
+      <x:c r="L137" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" t="str">
+        <x:v>E2E-158</x:v>
+      </x:c>
+      <x:c r="B138" t="str">
+        <x:v>Editor V2/Regression</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>Build, runtime console and server-error scan</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>Run vue-tsc/Vite build and full toolbar browser smoke with console, pageerror and HTTP 5xx listeners.</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>Build passes and browser run has zero console errors, page errors and server 5xx responses.</x:v>
+      </x:c>
+      <x:c r="F138" t="str">
+        <x:v>vue-tsc and Vite build PASS; consoleErrors=0; pageErrors=0; serverErrors=0.</x:v>
+      </x:c>
+      <x:c r="G138" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H138" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I138" t="str">
+        <x:v>Vite chunk-size warning remains non-blocking and unchanged.</x:v>
+      </x:c>
+      <x:c r="J138" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K138" t="str">
+        <x:v>frontend build + localhost FE5173</x:v>
+      </x:c>
+      <x:c r="L138" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6566,27 +6946,23 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 real layer creation from Text, Rectangle, Ellipse and Image</x:v>
+        <x:v>Editor V2 two-sided toolbars: functional left library/layers and contextual right inspector</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FE</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>FE</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>http://127.0.0.1:5175</x:v>
+        <x:v>http://127.0.0.1:5173</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BE</x:t>
-        </x:is>
+      <x:c r="A5" t="str">
+        <x:v>BE</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Backend unchanged; not rerun for frontend-only layer creation work</x:v>
+        <x:v>Backend unchanged; frontend-only editor toolbar work</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6594,14 +6970,12 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Frontend build and XSS guard PASS; browser console 0 errors and 0 warnings</x:v>
+        <x:v>Frontend build PASS; browser console/page errors/HTTP 5xx all zero</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Template seed</x:t>
-        </x:is>
+      <x:c r="A7" t="str">
+        <x:v>Template seed</x:v>
       </x:c>
       <x:c r="B7" t="str">
         <x:v>Schema V2 unchanged; fixed 90 x 54 mm Front and Back document</x:v>
@@ -6612,37 +6986,31 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-140 through E2E-148</x:v>
+        <x:v>E2E-149 through E2E-158</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Retest FAIL</x:t>
-        </x:is>
+      <x:c r="A9" t="str">
+        <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after valid/invalid image upload and save-reload retest</x:v>
+        <x:v>None after mobile app-shell padding fix and full rerun</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prior P0 open</x:t>
-        </x:is>
+      <x:c r="A10" t="str">
+        <x:v>Prior P0 open</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-130 through E2E-139 selection chrome and toolbar actions</x:v>
+        <x:v>E2E-140 through E2E-148 layer creation coverage retained</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shell</x:t>
-        </x:is>
+      <x:c r="A11" t="str">
+        <x:v>Shell</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Text, shape and image layer creation verified end to end with serializable image data</x:v>
+        <x:v>Left tools, contextual inspector, drag reorder, mm geometry and persistence verified</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -6650,7 +7018,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>output/playwright/editor-v2-layer-creation-desktop.png; output/playwright/editor-v2-layer-creation-mobile.png</x:v>
+        <x:v>Local-only editor-v2-toolbars desktop and mobile browser evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Connect V2 background removal assets
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ree539fb619c4490b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rd37ecc48dcf0498a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rd8a285cd9ae54c42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Re673d3aea20c4b85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6912,6 +6912,196 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>E2E-159</x:v>
+      </x:c>
+      <x:c r="B139" t="str">
+        <x:v>Editor V2/Image inspector</x:v>
+      </x:c>
+      <x:c r="C139" t="str">
+        <x:v>Remove background API action</x:v>
+      </x:c>
+      <x:c r="D139" t="str">
+        <x:v>Upload a valid PNG and press Remove background in the contextual Image inspector.</x:v>
+      </x:c>
+      <x:c r="E139" t="str">
+        <x:v>The existing authenticated remove-background contract is called once with POST multipart/form-data and the processed response is accepted.</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>Mocked browser request method=POST and contentType=multipart/form-data; processed assetId=701 returned and UI status became Background removed.</x:v>
+      </x:c>
+      <x:c r="G139" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H139" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I139" t="str">
+        <x:v>Frontend contract test with API mock; backend unchanged.</x:v>
+      </x:c>
+      <x:c r="J139" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K139" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L139" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>E2E-160</x:v>
+      </x:c>
+      <x:c r="B140" t="str">
+        <x:v>Editor V2/Image assets</x:v>
+      </x:c>
+      <x:c r="C140" t="str">
+        <x:v>Original and processed metadata</x:v>
+      </x:c>
+      <x:c r="D140" t="str">
+        <x:v>After background removal, save the document, reload it, then use Use original.</x:v>
+      </x:c>
+      <x:c r="E140" t="str">
+        <x:v>Original source remains available; processed URL, assetId and storageKey persist; restore switches the live image back without deleting processed metadata.</x:v>
+      </x:c>
+      <x:c r="F140" t="str">
+        <x:v>originalSrc stayed data:image/png; processedSrc, processedAssetId=701 and processedStorageKey persisted; live and saved source restored to original.</x:v>
+      </x:c>
+      <x:c r="G140" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H140" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I140" t="str">
+        <x:v>V2 document schema now carries separate asset metadata.</x:v>
+      </x:c>
+      <x:c r="J140" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K140" t="str">
+        <x:v>localhost FE5173 localStorage</x:v>
+      </x:c>
+      <x:c r="L140" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>E2E-161</x:v>
+      </x:c>
+      <x:c r="B141" t="str">
+        <x:v>Editor V2/Image lifecycle</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>Reload without File object</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>Reload a saved processed image and press Remove background before re-uploading its source file.</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>The UI blocks the request and explains that the image must be re-uploaded because a browser File object is not persisted in localStorage.</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>Message Re-upload this image before removing its background rendered; removal request count remained one.</x:v>
+      </x:c>
+      <x:c r="G141" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H141" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I141" t="str">
+        <x:v>Intentional boundary for local-only V2 persistence.</x:v>
+      </x:c>
+      <x:c r="J141" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K141" t="str">
+        <x:v>localhost FE5173 Chrome reload</x:v>
+      </x:c>
+      <x:c r="L141" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
+        <x:v>E2E-162</x:v>
+      </x:c>
+      <x:c r="B142" t="str">
+        <x:v>Backend/Uploads</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>Image upload and background removal contract regression</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>Run ImageUploadApiTests and BackgroundRemovalClientTests after the V2 integration.</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>Authentication, multipart validation, protected output handling and background-removal client behavior remain green.</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>Maven tests: 10 run, 0 failures, 0 errors, 0 skipped; BUILD SUCCESS.</x:v>
+      </x:c>
+      <x:c r="G142" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H142" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I142" t="str">
+        <x:v>No backend source changes in this step.</x:v>
+      </x:c>
+      <x:c r="J142" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K142" t="str">
+        <x:v>Spring Boot test profile + H2</x:v>
+      </x:c>
+      <x:c r="L142" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>E2E-163</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>Editor V2/Regression</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>Desktop, mobile and runtime scan</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>Run the complete background-removal browser smoke at 1440x1000 and 390x844.</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>Desktop and mobile screenshots are produced; no horizontal overflow, page errors, console errors or HTTP 5xx responses occur.</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>Desktop/mobile screenshots produced; mobile documentWidth=390px; consoleErrors=0; pageErrors=0; serverErrors=0.</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H143" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I143" t="str">
+        <x:v>Chrome headless smoke with mocked API and processed PNG delivery.</x:v>
+      </x:c>
+      <x:c r="J143" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K143" t="str">
+        <x:v>localhost FE5173 Chrome desktop/mobile</x:v>
+      </x:c>
+      <x:c r="L143" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6946,7 +7136,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 two-sided toolbars: functional left library/layers and contextual right inspector</x:v>
+        <x:v>Editor V2 image inspector background removal with original/processed asset metadata</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -6962,7 +7152,7 @@
         <x:v>BE</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Backend unchanged; frontend-only editor toolbar work</x:v>
+        <x:v>Existing authenticated multipart endpoint verified; backend source unchanged</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6970,15 +7160,15 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Frontend build PASS; browser console/page errors/HTTP 5xx all zero</x:v>
+        <x:v>FE build/XSS PASS; browser mock PASS; backend upload/removal tests 10/10 PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Template seed</x:v>
+        <x:v>Schema</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Schema V2 unchanged; fixed 90 x 54 mm Front and Back document</x:v>
+        <x:v>V2 image layers preserve originalSrc and processedSrc/assetId/storageKey separately</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6986,7 +7176,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-149 through E2E-158</x:v>
+        <x:v>E2E-159 through E2E-163</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6994,7 +7184,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after mobile app-shell padding fix and full rerun</x:v>
+        <x:v>None after API mock route and localStorage assertion corrections</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -7002,15 +7192,15 @@
         <x:v>Prior P0 open</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-140 through E2E-148 layer creation coverage retained</x:v>
+        <x:v>E2E-149 through E2E-158 toolbar foundation retained</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Shell</x:v>
+        <x:v>Boundary</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Left tools, contextual inspector, drag reorder, mm geometry and persistence verified</x:v>
+        <x:v>After reload, re-upload is required before a new removal request because File is in-memory only</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7018,7 +7208,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local-only editor-v2-toolbars desktop and mobile browser evidence</x:v>
+        <x:v>Local-only Editor V2 background-removal desktop and mobile browser evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Persist Editor V2 drafts through backend
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rd8a285cd9ae54c42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Re673d3aea20c4b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rccaaeda1523f4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R235732c3dfbe4297"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7102,6 +7102,272 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>E2E-164</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>Backend/Design validation</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>V2 canvas validator accepts exactly front and back</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>Run DesignServiceV2Tests with a schemaVersion 2 document containing front/back pages, an extra page, and no pages object.</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>The valid two-page document is accepted; extra-page and missing-pages payloads are rejected as controlled validation errors.</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>Focused service tests: 3 run, 0 failures, 0 errors; V2 validator guard includes pages != null and exact front/back ids.</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I144" t="str">
+        <x:v>Unit coverage protects the two-page contract and malformed JSON boundary.</x:v>
+      </x:c>
+      <x:c r="J144" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K144" t="str">
+        <x:v>Spring Boot Maven test</x:v>
+      </x:c>
+      <x:c r="L144" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>E2E-165</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>Backend/API</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>Save and read V2 front/back canvas through API</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>Run DesignApiIntegrationTests against the PostgreSQL test profile and PUT then GET a schemaVersion 2 canvas.</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>Owner-scoped PUT accepts the V2 canvas and GET returns both front and back layer content.</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>DesignApiIntegrationTests: 9 run, 0 failures, 0 errors; PostgreSQL 17.10; PUT/GET readback preserved Front API and Back API.</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H145" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I145" t="str">
+        <x:v>CSRF and ownership filters remained active in the integration path.</x:v>
+      </x:c>
+      <x:c r="J145" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K145" t="str">
+        <x:v>PostgreSQL 17.10 + MockMvc</x:v>
+      </x:c>
+      <x:c r="L145" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>E2E-166</x:v>
+      </x:c>
+      <x:c r="B146" t="str">
+        <x:v>Editor V2/Draft load</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>Numeric draft loads backend document and card size</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>Open numeric route 4242 with mocked GET /api/designs/4242 returning V2 front/back and widthMm=85, heightMm=55.</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>The editor loads both pages and applies the backend card dimensions as the selected document size.</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>Browser smoke observed GET count=3 for 4242; front/back loaded; widthMm=85 and heightMm=55 applied to the editor document.</x:v>
+      </x:c>
+      <x:c r="G146" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H146" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I146" t="str">
+        <x:v>Non-numeric demo routes retain local-only behavior.</x:v>
+      </x:c>
+      <x:c r="J146" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K146" t="str">
+        <x:v>localhost FE5173 Chrome mock API</x:v>
+      </x:c>
+      <x:c r="L146" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>E2E-167</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>Editor V2/Draft save</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>Save through CSRF-protected backend and reload</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>Edit front text, click Save, clear localStorage, reload the numeric route, then inspect the saved payload and visible text.</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>The client requests the CSRF token, sends PUT with X-XSRF-TOKEN, persists schemaVersion 2, and reloads the saved text from backend.</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>Payload schemaVersion=2, documentId=4242, front text=Saved through backend; PUT carried X-XSRF-TOKEN; reload after localStorage clear restored the text.</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I147" t="str">
+        <x:v>Save status distinguishes loading, saving, saved, dirty and error states.</x:v>
+      </x:c>
+      <x:c r="J147" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K147" t="str">
+        <x:v>localhost FE5173 Chrome mock API</x:v>
+      </x:c>
+      <x:c r="L147" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>E2E-168</x:v>
+      </x:c>
+      <x:c r="B148" t="str">
+        <x:v>Editor V2/Migration</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>Legacy V1 draft becomes explicit V2 dirty state</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>Open numeric route 4343 with a legacy layers-only canvas, confirm unsaved state, save, then inspect the outgoing canvas.</x:v>
+      </x:c>
+      <x:c r="E148" t="str">
+        <x:v>Legacy content is not silently reported as saved; first save converts it to schemaVersion 2 with exactly front/back pages.</x:v>
+      </x:c>
+      <x:c r="F148" t="str">
+        <x:v>V1 route marked Unsaved changes; save sent schemaVersion=2; migrated document contained exactly front and back; savedDesignIds included 4343.</x:v>
+      </x:c>
+      <x:c r="G148" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H148" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I148" t="str">
+        <x:v>Migration is explicit on first save and avoids silently overwriting an unverified legacy shape.</x:v>
+      </x:c>
+      <x:c r="J148" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K148" t="str">
+        <x:v>localhost FE5173 Chrome mock API</x:v>
+      </x:c>
+      <x:c r="L148" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>E2E-169</x:v>
+      </x:c>
+      <x:c r="B149" t="str">
+        <x:v>Editor V2/Regression</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>UI, responsive and background removal regressions</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>Run draft-persistence, toolbar, and background-removal browser smokes at desktop and 390x844 mobile viewports.</x:v>
+      </x:c>
+      <x:c r="E149" t="str">
+        <x:v>Two toolbars, layer reorder, image background removal, mobile layout and reload behavior remain functional without runtime errors.</x:v>
+      </x:c>
+      <x:c r="F149" t="str">
+        <x:v>All three browser smokes PASS; mobile documentWidth=390; toolbar reorder and multipart POST verified; consoleErrors=0, pageErrors=0, serverErrors=0.</x:v>
+      </x:c>
+      <x:c r="G149" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H149" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I149" t="str">
+        <x:v>Screenshots remain local under .codex-work and are not staged.</x:v>
+      </x:c>
+      <x:c r="J149" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K149" t="str">
+        <x:v>localhost FE5173 Chrome desktop/mobile</x:v>
+      </x:c>
+      <x:c r="L149" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>E2E-170</x:v>
+      </x:c>
+      <x:c r="B150" t="str">
+        <x:v>Full verification</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>Backend, frontend build, XSS guard and workbook evidence</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>Run full Maven suite, frontend production build, frontend XSS static guard, then read back and render this workbook.</x:v>
+      </x:c>
+      <x:c r="E150" t="str">
+        <x:v>All automated checks pass and the workbook contains the new PASS rows with no formula errors.</x:v>
+      </x:c>
+      <x:c r="F150" t="str">
+        <x:v>Backend 91/91 PASS; npm run build PASS; npm run test:xss PASS; workbook readback/formula scan/render completed for E2E-164..170.</x:v>
+      </x:c>
+      <x:c r="G150" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H150" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I150" t="str">
+        <x:v>Only intended source/test/workbook files are candidates for staging; private agent artifacts excluded.</x:v>
+      </x:c>
+      <x:c r="J150" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K150" t="str">
+        <x:v>Maven + Vite + artifact-tool</x:v>
+      </x:c>
+      <x:c r="L150" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7136,7 +7402,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 image inspector background removal with original/processed asset metadata</x:v>
+        <x:v>Editor V2 backend draft persistence with exact front/back pages and selected card size</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7152,7 +7418,7 @@
         <x:v>BE</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Existing authenticated multipart endpoint verified; backend source unchanged</x:v>
+        <x:v>Owner-scoped design GET/PUT and CSRF-protected update path verified</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -7160,7 +7426,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>FE build/XSS PASS; browser mock PASS; backend upload/removal tests 10/10 PASS</x:v>
+        <x:v>Backend 91/91; FE build/XSS PASS; browser persistence/toolbar/background removal smokes PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -7168,7 +7434,7 @@
         <x:v>Schema</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>V2 image layers preserve originalSrc and processedSrc/assetId/storageKey separately</x:v>
+        <x:v>Numeric routes load/save schemaVersion 2; V1 routes require explicit first-save migration</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7176,7 +7442,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-159 through E2E-163</x:v>
+        <x:v>E2E-164 through E2E-170</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7184,7 +7450,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after API mock route and localStorage assertion corrections</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -7192,7 +7458,7 @@
         <x:v>Prior P0 open</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-149 through E2E-158 toolbar foundation retained</x:v>
+        <x:v>E2E-159 through E2E-163 background removal and toolbar foundation retained</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7200,7 +7466,7 @@
         <x:v>Boundary</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>After reload, re-upload is required before a new removal request because File is in-memory only</x:v>
+        <x:v>Non-numeric demo routes remain local-only; backend V1 documents migrate on first save</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7208,7 +7474,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local-only Editor V2 background-removal desktop and mobile browser evidence</x:v>
+        <x:v>Local-only draft persistence, toolbar and background-removal desktop/mobile browser evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add Editor V2 print guides
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rccaaeda1523f4184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R235732c3dfbe4297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R6ea2e24e9be2427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Re8fea96ebea8422a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7368,6 +7368,196 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
+        <x:v>E2E-171</x:v>
+      </x:c>
+      <x:c r="B151" t="str">
+        <x:v>Editor V2/Print guides</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>Print guide toggle defaults on and controls both overlays</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>Open the Page inspector, verify Show print guides is checked, uncheck it, then check it again.</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>Bleed and safe-zone guides are visible by default; the toggle hides and restores both without changing card content.</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>RED timed out before implementation; GREEN found two guide overlays, then 0 after uncheck and 2 after recheck.</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I151" t="str">
+        <x:v>View-only state; toggling guides does not mark the design dirty.</x:v>
+      </x:c>
+      <x:c r="J151" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K151" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L151" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>E2E-172</x:v>
+      </x:c>
+      <x:c r="B152" t="str">
+        <x:v>Editor V2/Safe zone</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>Safe-zone geometry follows the fixed 3 mm print rule</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>Measure the safe guide against a 90 x 54 mm card rendered at 660 x 396 px.</x:v>
+      </x:c>
+      <x:c r="E152" t="str">
+        <x:v>Horizontal inset equals 3/90 of canvas width and vertical inset equals 3/54 of canvas height within border tolerance.</x:v>
+      </x:c>
+      <x:c r="F152" t="str">
+        <x:v>Measured safe inset approximately 22.9 px horizontal and 22.9 px vertical; geometry assertions passed within 2 px tolerance.</x:v>
+      </x:c>
+      <x:c r="G152" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H152" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I152" t="str">
+        <x:v>Matches the existing backend PreflightService 3 mm safe-zone rule.</x:v>
+      </x:c>
+      <x:c r="J152" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K152" t="str">
+        <x:v>Chrome geometry + backend contract</x:v>
+      </x:c>
+      <x:c r="L152" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>E2E-173</x:v>
+      </x:c>
+      <x:c r="B153" t="str">
+        <x:v>Editor V2/Bleed</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>Bleed guide extends 2 mm beyond card edges on both sides</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>Measure the bleed overlay outside the card, switch Front to Back, and count guide overlays again.</x:v>
+      </x:c>
+      <x:c r="E153" t="str">
+        <x:v>Bleed extends by 2/90 horizontally and 2/54 vertically; both bleed and safe guides remain on Front and Back.</x:v>
+      </x:c>
+      <x:c r="F153" t="str">
+        <x:v>Bleed geometry assertions passed; guide count remained 2 after switching to Back.</x:v>
+      </x:c>
+      <x:c r="G153" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H153" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I153" t="str">
+        <x:v>Guide is visual only and does not alter saved canvas dimensions.</x:v>
+      </x:c>
+      <x:c r="J153" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K153" t="str">
+        <x:v>localhost FE5173 Chrome</x:v>
+      </x:c>
+      <x:c r="L153" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>E2E-174</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>Editor V2/Responsive</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>Print guides remain visible and contained on mobile</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>Render the guide state at desktop and 390 x 844 mobile, capture screenshots, and scan runtime errors.</x:v>
+      </x:c>
+      <x:c r="E154" t="str">
+        <x:v>Guides stay legible; workspace and inspector remain full width; no horizontal overflow or runtime/server errors occur.</x:v>
+      </x:c>
+      <x:c r="F154" t="str">
+        <x:v>Desktop/mobile screenshots inspected; mobile documentWidth=390, guideCount=2, workspaceWidth=390, inspectorWidth=390; all error arrays empty.</x:v>
+      </x:c>
+      <x:c r="G154" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H154" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I154" t="str">
+        <x:v>Bleed line stays outside the card without expanding the page width.</x:v>
+      </x:c>
+      <x:c r="J154" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K154" t="str">
+        <x:v>Chrome desktop/mobile</x:v>
+      </x:c>
+      <x:c r="L154" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>E2E-175</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>Full verification</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>Guide change preserves editor, security and preflight behavior</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>Run frontend build, XSS guard, persistence/toolbar/background-removal smokes, print-guide smoke, and backend PreflightServiceTests.</x:v>
+      </x:c>
+      <x:c r="E155" t="str">
+        <x:v>All checks pass and existing draft, toolbar, upload/background-removal and 3 mm preflight behavior remain green.</x:v>
+      </x:c>
+      <x:c r="F155" t="str">
+        <x:v>Vite build PASS; XSS PASS; 4 browser smokes PASS; PreflightServiceTests 11/11 PASS; console/page/server errors=0.</x:v>
+      </x:c>
+      <x:c r="G155" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H155" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I155" t="str">
+        <x:v>No backend production source changed in this step.</x:v>
+      </x:c>
+      <x:c r="J155" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K155" t="str">
+        <x:v>Vite + Chrome + Maven</x:v>
+      </x:c>
+      <x:c r="L155" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7402,7 +7592,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 backend draft persistence with exact front/back pages and selected card size</x:v>
+        <x:v>Editor V2 fixed 2 mm bleed and 3 mm safe-zone print guides</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7418,7 +7608,7 @@
         <x:v>BE</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Owner-scoped design GET/PUT and CSRF-protected update path verified</x:v>
+        <x:v>PreflightService 3 mm safe-zone contract verified; backend source unchanged</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -7426,15 +7616,15 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Backend 91/91; FE build/XSS PASS; browser persistence/toolbar/background removal smokes PASS</x:v>
+        <x:v>FE build/XSS PASS; four browser smokes PASS; PreflightServiceTests 11/11 PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Schema</x:v>
+        <x:v>Geometry</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Numeric routes load/save schemaVersion 2; V1 routes require explicit first-save migration</x:v>
+        <x:v>90 x 54 mm card maps bleed and safe-zone insets proportionally at every rendered size</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7442,7 +7632,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-164 through E2E-170</x:v>
+        <x:v>E2E-171 through E2E-175</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7450,7 +7640,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None</x:v>
+        <x:v>None after the expected RED timeout before implementation</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -7458,7 +7648,7 @@
         <x:v>Prior P0 open</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-159 through E2E-163 background removal and toolbar foundation retained</x:v>
+        <x:v>E2E-164 through E2E-170 backend draft persistence retained</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7466,7 +7656,7 @@
         <x:v>Boundary</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Non-numeric demo routes remain local-only; backend V1 documents migrate on first save</x:v>
+        <x:v>Guides are view-only and intentionally excluded from saved canvas JSON</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7474,7 +7664,7 @@
         <x:v>Screenshots</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local-only draft persistence, toolbar and background-removal desktop/mobile browser evidence</x:v>
+        <x:v>Local-only print-guide desktop and mobile browser evidence inspected</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Support Editor V2 preflight reports
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R6ea2e24e9be2427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Re8fea96ebea8422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R5e058ec4f7b748b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R476648eb5db5488d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7558,6 +7558,234 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>E2E-176</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>Editor V2/Backend preflight</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>Schema V2 checks both Front and Back layer groups</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>Run PreflightService against a schemaVersion 2 document with an unsafe Front text layer and a low-DPI Back image layer.</x:v>
+      </x:c>
+      <x:c r="E156" t="str">
+        <x:v>Report contains both safe-zone and DPI issues instead of INVALID_CANVAS; report is blocking because the text issue is an error.</x:v>
+      </x:c>
+      <x:c r="F156" t="str">
+        <x:v>TDD RED returned INVALID_CANVAS; GREEN returned LAYER_OUTSIDE_SAFE_ZONE then LOW_IMAGE_RESOLUTION with valid=false.</x:v>
+      </x:c>
+      <x:c r="G156" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H156" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I156" t="str">
+        <x:v>Legacy root layers remain supported.</x:v>
+      </x:c>
+      <x:c r="J156" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K156" t="str">
+        <x:v>Maven unit test</x:v>
+      </x:c>
+      <x:c r="L156" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>E2E-177</x:v>
+      </x:c>
+      <x:c r="B157" t="str">
+        <x:v>Editor V2/API security</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>Owned V2 preflight response identifies the affected side</x:v>
+      </x:c>
+      <x:c r="D157" t="str">
+        <x:v>Create a V2 draft through the design API, run POST /api/designs/{id}/preflight as owner, then retry as another user.</x:v>
+      </x:c>
+      <x:c r="E157" t="str">
+        <x:v>Owner receives side=front and layerIndex=0; non-owner receives 404; CSRF remains required.</x:v>
+      </x:c>
+      <x:c r="F157" t="str">
+        <x:v>PostgreSQL integration suite passed; owner response included side=front and another user received 404.</x:v>
+      </x:c>
+      <x:c r="G157" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H157" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I157" t="str">
+        <x:v>Covers API serialization and IDOR boundary.</x:v>
+      </x:c>
+      <x:c r="J157" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K157" t="str">
+        <x:v>Spring MockMvc + PostgreSQL 17</x:v>
+      </x:c>
+      <x:c r="L157" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>E2E-178</x:v>
+      </x:c>
+      <x:c r="B158" t="str">
+        <x:v>Editor V2/Preflight flow</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>Preflight saves the latest V2 document before checking</x:v>
+      </x:c>
+      <x:c r="D158" t="str">
+        <x:v>Edit a numeric-route draft and click the Preflight header button while intercepting PUT and POST requests.</x:v>
+      </x:c>
+      <x:c r="E158" t="str">
+        <x:v>PUT /api/designs/{id} occurs before POST /preflight and sends schemaVersion 2 with Front and Back pages.</x:v>
+      </x:c>
+      <x:c r="F158" t="str">
+        <x:v>Browser request order was save,preflight for every run; saved payload retained schemaVersion=2.</x:v>
+      </x:c>
+      <x:c r="G158" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H158" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I158" t="str">
+        <x:v>Prevents server checks from using stale canvas data.</x:v>
+      </x:c>
+      <x:c r="J158" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K158" t="str">
+        <x:v>Chrome desktop/mobile</x:v>
+      </x:c>
+      <x:c r="L158" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>E2E-179</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
+        <x:v>Editor V2/Issue navigation</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>Issue rows focus the correct card side and layer</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>Return one Front error and one Back warning, click the Back issue, then edit layer opacity.</x:v>
+      </x:c>
+      <x:c r="E159" t="str">
+        <x:v>Back becomes active, Image inspector selects the matching layer, and any subsequent edit removes the stale report.</x:v>
+      </x:c>
+      <x:c r="F159" t="str">
+        <x:v>Two issue rows rendered with side labels; Back issue selected the Back image; opacity edit cleared the report.</x:v>
+      </x:c>
+      <x:c r="G159" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H159" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I159" t="str">
+        <x:v>Global issues without side/layer remain visible but non-clickable.</x:v>
+      </x:c>
+      <x:c r="J159" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K159" t="str">
+        <x:v>Chrome interaction smoke</x:v>
+      </x:c>
+      <x:c r="L159" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>E2E-180</x:v>
+      </x:c>
+      <x:c r="B160" t="str">
+        <x:v>Editor V2/Preflight states</x:v>
+      </x:c>
+      <x:c r="C160" t="str">
+        <x:v>Inspector renders failed and passed preflight states</x:v>
+      </x:c>
+      <x:c r="D160" t="str">
+        <x:v>Run preflight once with error/warning issues and again with valid=true and no issues.</x:v>
+      </x:c>
+      <x:c r="E160" t="str">
+        <x:v>Failed state shows counts and messages; passed state shows Preflight passed and no issue rows.</x:v>
+      </x:c>
+      <x:c r="F160" t="str">
+        <x:v>Failed report showed 1 error / 1 warning; valid report showed Preflight passed with zero issue rows.</x:v>
+      </x:c>
+      <x:c r="G160" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H160" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I160" t="str">
+        <x:v>Report uses aria-live and error text remains escaped by Vue.</x:v>
+      </x:c>
+      <x:c r="J160" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K160" t="str">
+        <x:v>Chrome + XSS guard</x:v>
+      </x:c>
+      <x:c r="L160" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>E2E-181</x:v>
+      </x:c>
+      <x:c r="B161" t="str">
+        <x:v>Editor V2/Image DPI and regression</x:v>
+      </x:c>
+      <x:c r="C161" t="str">
+        <x:v>Uploaded image dimensions persist for DPI checks without layout regressions</x:v>
+      </x:c>
+      <x:c r="D161" t="str">
+        <x:v>Replace an image with a 1 x 1 PNG, save through preflight, then run build, XSS and all V2 regression smokes at desktop and 390 x 844.</x:v>
+      </x:c>
+      <x:c r="E161" t="str">
+        <x:v>Saved image layer includes pixelWidth/pixelHeight; all editor flows pass with no horizontal overflow, console errors, page errors or HTTP 5xx.</x:v>
+      </x:c>
+      <x:c r="F161" t="str">
+        <x:v>Saved metadata was 1 x 1; build/XSS, preflight, draft, toolbar, background-removal and guide smokes passed; mobile documentWidth=390.</x:v>
+      </x:c>
+      <x:c r="G161" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H161" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I161" t="str">
+        <x:v>No new dependency; natural image dimensions are read in-browser.</x:v>
+      </x:c>
+      <x:c r="J161" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K161" t="str">
+        <x:v>Vite + Chrome + Maven</x:v>
+      </x:c>
+      <x:c r="L161" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7592,7 +7820,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 fixed 2 mm bleed and 3 mm safe-zone print guides</x:v>
+        <x:v>Editor V2 schema V2 preflight report and issue navigation</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7600,7 +7828,7 @@
         <x:v>FE</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>http://127.0.0.1:5173</x:v>
+        <x:v>http://127.0.0.1:5173/editor/15</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -7608,7 +7836,7 @@
         <x:v>BE</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>PreflightService 3 mm safe-zone contract verified; backend source unchanged</x:v>
+        <x:v>V2 Front/Back preflight, side-aware issues, owner-scoped API</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -7616,15 +7844,15 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>FE build/XSS PASS; four browser smokes PASS; PreflightServiceTests 11/11 PASS</x:v>
+        <x:v>Frontend build/XSS and five browser smokes PASS; backend targeted suites 24/24 PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Geometry</x:v>
+        <x:v>Contract</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>90 x 54 mm card maps bleed and safe-zone insets proportionally at every rendered size</x:v>
+        <x:v>Editor saves current schema V2 before POST /preflight; response carries side plus layerIndex</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7632,7 +7860,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-171 through E2E-175</x:v>
+        <x:v>E2E-176 through E2E-181</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7640,31 +7868,31 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after the expected RED timeout before implementation</x:v>
+        <x:v>None after expected TDD RED failures</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Prior P0 open</x:v>
+        <x:v>Security</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>E2E-164 through E2E-170 backend draft persistence retained</x:v>
+        <x:v>CSRF retained; non-owner preflight returns 404; no v-html rendering</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Boundary</x:v>
+        <x:v>Responsive</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Guides are view-only and intentionally excluded from saved canvas JSON</x:v>
+        <x:v>Desktop and 390 x 844 mobile contained; no console/page/server errors</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>Screenshots</x:v>
+        <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local-only print-guide desktop and mobile browser evidence inspected</x:v>
+        <x:v>Local-only preflight screenshots and smoke scripts inspected</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Complete Editor V2 checkout preflight flow
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R5e058ec4f7b748b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R476648eb5db5488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R74525e35b3ef4e42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R016c576721ca45eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7786,6 +7786,196 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>E2E-182</x:v>
+      </x:c>
+      <x:c r="B162" t="str">
+        <x:v>Editor V2/Checkout preview</x:v>
+      </x:c>
+      <x:c r="C162" t="str">
+        <x:v>Checkout renders schema V2 Front and Back pages</x:v>
+      </x:c>
+      <x:c r="D162" t="str">
+        <x:v>Open an owned schemaVersion 2 design in checkout, inspect Front, then switch to Back.</x:v>
+      </x:c>
+      <x:c r="E162" t="str">
+        <x:v>Each side shows only its own layers, page background and V2 content; exactly two fixed side buttons are available.</x:v>
+      </x:c>
+      <x:c r="F162" t="str">
+        <x:v>Front and Back content/background checks passed; no layers were mixed between sides.</x:v>
+      </x:c>
+      <x:c r="G162" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H162" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I162" t="str">
+        <x:v>Legacy root-layer drafts remain supported by the same parser.</x:v>
+      </x:c>
+      <x:c r="J162" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K162" t="str">
+        <x:v>Chrome desktop browser smoke</x:v>
+      </x:c>
+      <x:c r="L162" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" t="str">
+        <x:v>E2E-183</x:v>
+      </x:c>
+      <x:c r="B163" t="str">
+        <x:v>Editor V2/Checkout navigation</x:v>
+      </x:c>
+      <x:c r="C163" t="str">
+        <x:v>Editor saves the latest draft before checkout navigation</x:v>
+      </x:c>
+      <x:c r="D163" t="str">
+        <x:v>Change a selected Front text layer and click the Checkout header command while intercepting API requests.</x:v>
+      </x:c>
+      <x:c r="E163" t="str">
+        <x:v>PUT /api/designs/{id} completes before routing to /checkout/{id}; checkout preview shows the new text.</x:v>
+      </x:c>
+      <x:c r="F163" t="str">
+        <x:v>Request order was save-rejected,save; the intentional 409 stayed in Editor and only the successful save navigated to checkout with the latest V2 text.</x:v>
+      </x:c>
+      <x:c r="G163" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H163" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I163" t="str">
+        <x:v>A failed save keeps the user in Editor through the existing save error state.</x:v>
+      </x:c>
+      <x:c r="J163" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K163" t="str">
+        <x:v>Chrome interaction and API interception</x:v>
+      </x:c>
+      <x:c r="L163" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>E2E-184</x:v>
+      </x:c>
+      <x:c r="B164" t="str">
+        <x:v>Checkout/Preflight UX</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>Errors block checkout while warnings remain allowed</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>Run checkout preflight with one Front error and one Back warning, then rerun with warning only.</x:v>
+      </x:c>
+      <x:c r="E164" t="str">
+        <x:v>Issues show Front/Back labels; error report removes override and disables Create order; warning-only report enables it.</x:v>
+      </x:c>
+      <x:c r="F164" t="str">
+        <x:v>Error state blocked order creation and showed both sides; warning-only state passed without unsafe override.</x:v>
+      </x:c>
+      <x:c r="G164" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H164" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I164" t="str">
+        <x:v>Preflight API failure also blocks order creation.</x:v>
+      </x:c>
+      <x:c r="J164" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K164" t="str">
+        <x:v>Chrome accessibility and state smoke</x:v>
+      </x:c>
+      <x:c r="L164" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>E2E-185</x:v>
+      </x:c>
+      <x:c r="B165" t="str">
+        <x:v>Backend/Order guard</x:v>
+      </x:c>
+      <x:c r="C165" t="str">
+        <x:v>Direct order API cannot bypass preflight errors</x:v>
+      </x:c>
+      <x:c r="D165" t="str">
+        <x:v>Create an owned design with text outside the 3 mm safe-zone and call POST /api/orders directly with CSRF.</x:v>
+      </x:c>
+      <x:c r="E165" t="str">
+        <x:v>API returns 400 and persists zero orders; ownership, paper and quantity validation remain enforced.</x:v>
+      </x:c>
+      <x:c r="F165" t="str">
+        <x:v>TDD RED returned 201; GREEN returned 400 and OrderApiIntegrationTests passed 6/6 on PostgreSQL 17.</x:v>
+      </x:c>
+      <x:c r="G165" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H165" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I165" t="str">
+        <x:v>Enforces the print rule server-side instead of trusting frontend state.</x:v>
+      </x:c>
+      <x:c r="J165" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K165" t="str">
+        <x:v>Spring MockMvc + PostgreSQL 17</x:v>
+      </x:c>
+      <x:c r="L165" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>E2E-186</x:v>
+      </x:c>
+      <x:c r="B166" t="str">
+        <x:v>Checkout/Regression</x:v>
+      </x:c>
+      <x:c r="C166" t="str">
+        <x:v>Checkout options, order redirect and responsive layout remain correct</x:v>
+      </x:c>
+      <x:c r="D166" t="str">
+        <x:v>Select Linen 300gsm, quantity 500 and rounded corners after warning-only preflight; submit, then run build/XSS, V2 smokes and full backend tests.</x:v>
+      </x:c>
+      <x:c r="E166" t="str">
+        <x:v>Order payload remains exact and redirects to order detail; desktop/mobile have no overlap or overflow; all regression suites pass.</x:v>
+      </x:c>
+      <x:c r="F166" t="str">
+        <x:v>Payload was designId 6262, linen-300, 500, rounded=true; mobile width 390/390; six browser smokes, build/XSS and backend 93/93 passed.</x:v>
+      </x:c>
+      <x:c r="G166" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H166" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I166" t="str">
+        <x:v>Desktop/mobile screenshots were inspected; the intentional 409 was observed and unexpected console/page/server errors were zero.</x:v>
+      </x:c>
+      <x:c r="J166" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K166" t="str">
+        <x:v>Vite + Chrome + Maven</x:v>
+      </x:c>
+      <x:c r="L166" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7820,7 +8010,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 schema V2 preflight report and issue navigation</x:v>
+        <x:v>Editor V2 checkout preview, side switch and preflight order guard</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7828,7 +8018,7 @@
         <x:v>FE</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>http://127.0.0.1:5173/editor/15</x:v>
+        <x:v>http://127.0.0.1:5173/editor/15 -&gt; /checkout/{designId}</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -7836,7 +8026,7 @@
         <x:v>BE</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>V2 Front/Back preflight, side-aware issues, owner-scoped API</x:v>
+        <x:v>POST /api/orders enforces PreflightService before persistence</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -7844,7 +8034,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Frontend build/XSS and five browser smokes PASS; backend targeted suites 24/24 PASS</x:v>
+        <x:v>Frontend build/XSS and six browser smokes PASS; full backend 93/93 PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -7852,7 +8042,7 @@
         <x:v>Contract</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor saves current schema V2 before POST /preflight; response carries side plus layerIndex</x:v>
+        <x:v>Editor saves schema V2 before checkout; errors block orders; warnings remain allowed</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7860,7 +8050,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-176 through E2E-181</x:v>
+        <x:v>E2E-182 through E2E-186</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7876,7 +8066,7 @@
         <x:v>Security</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>CSRF retained; non-owner preflight returns 404; no v-html rendering</x:v>
+        <x:v>CSRF and owner filtering retained; direct API cannot bypass preflight errors</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7884,7 +8074,7 @@
         <x:v>Responsive</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Desktop and 390 x 844 mobile contained; no console/page/server errors</x:v>
+        <x:v>Desktop and 390 x 844 mobile contained; side switch width 147 px</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7892,7 +8082,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local-only preflight screenshots and smoke scripts inspected</x:v>
+        <x:v>Checkout screenshots, exact order payload and rejected-save then successful-save sequence were inspected</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Complete Editor V2 print export and acceptance
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R74525e35b3ef4e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R016c576721ca45eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rb38704dca53745eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R1b1b53e85ffc47a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7976,6 +7976,234 @@
         <x:v>YES</x:v>
       </x:c>
     </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>E2E-187</x:v>
+      </x:c>
+      <x:c r="B167" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C167" t="str">
+        <x:v>Print export guard</x:v>
+      </x:c>
+      <x:c r="D167" t="str">
+        <x:v>Draft co the luu va backend preflight hoat dong</x:v>
+      </x:c>
+      <x:c r="E167" t="str">
+        <x:v>1. Bam Export khi preflight tra ERROR. 2. Bam lai khi preflight chi tra WARNING.</x:v>
+      </x:c>
+      <x:c r="F167" t="str">
+        <x:v>Lan ERROR khong tai file; lan WARNING tai dung mot file sau thu tu save -&gt; preflight.</x:v>
+      </x:c>
+      <x:c r="G167" t="str">
+        <x:v>ERROR: no download. WARNING: one PDF. Unsafe image source: no second PDF. Request order: save, preflight-errors, save, preflight-warnings, save, preflight-warnings.</x:v>
+      </x:c>
+      <x:c r="H167" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I167" t="str">
+        <x:v>Browser smoke + network interception</x:v>
+      </x:c>
+      <x:c r="J167" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K167" t="str">
+        <x:v>Phase 6E</x:v>
+      </x:c>
+      <x:c r="L167" t="str">
+        <x:v>No backend-preflight bypass; unsafe or missing image source blocks export with a clear error.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" t="str">
+        <x:v>E2E-188</x:v>
+      </x:c>
+      <x:c r="B168" t="str">
+        <x:v>Print PDF</x:v>
+      </x:c>
+      <x:c r="C168" t="str">
+        <x:v>Two-sided document</x:v>
+      </x:c>
+      <x:c r="D168" t="str">
+        <x:v>Card 90 x 54 mm co Front va Back</x:v>
+      </x:c>
+      <x:c r="E168" t="str">
+        <x:v>Xuat PDF va kiem tra cau truc binary/media box.</x:v>
+      </x:c>
+      <x:c r="F168" t="str">
+        <x:v>Dung 2 trang Front/Back, khong co trang thu ba; kich thuoc moi trang 94 x 58 mm.</x:v>
+      </x:c>
+      <x:c r="G168" t="str">
+        <x:v>2 pages; media box moi trang 266.4567 x 164.4094 pt; ten file Print-Export-Card-6263-print.pdf.</x:v>
+      </x:c>
+      <x:c r="H168" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I168" t="str">
+        <x:v>PDF parser + browser download</x:v>
+      </x:c>
+      <x:c r="J168" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K168" t="str">
+        <x:v>Phase 6E</x:v>
+      </x:c>
+      <x:c r="L168" t="str">
+        <x:v>Bleed nam trong kich thuoc trang.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" t="str">
+        <x:v>E2E-189</x:v>
+      </x:c>
+      <x:c r="B169" t="str">
+        <x:v>Print PDF</x:v>
+      </x:c>
+      <x:c r="C169" t="str">
+        <x:v>Bleed and resolution</x:v>
+      </x:c>
+      <x:c r="D169" t="str">
+        <x:v>Card trim 90 x 54 mm</x:v>
+      </x:c>
+      <x:c r="E169" t="str">
+        <x:v>Tinh spec va kiem tra canvas xuat o 300 DPI.</x:v>
+      </x:c>
+      <x:c r="F169" t="str">
+        <x:v>Bleed 2 mm moi canh; tong 94 x 58 mm; output 1110 x 685 px; trim dung ti le chinh xac.</x:v>
+      </x:c>
+      <x:c r="G169" t="str">
+        <x:v>PRINT_DPI=300; bleed=2 mm; 94 x 58 mm; 1110 x 685 px; toa do trim tinh theo ti le canvas.</x:v>
+      </x:c>
+      <x:c r="H169" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I169" t="str">
+        <x:v>Unit-level spec + browser smoke</x:v>
+      </x:c>
+      <x:c r="J169" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K169" t="str">
+        <x:v>Phase 6E</x:v>
+      </x:c>
+      <x:c r="L169" t="str">
+        <x:v>Giua bleed va trim khong bi lech do lam tron pixel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" t="str">
+        <x:v>E2E-190</x:v>
+      </x:c>
+      <x:c r="B170" t="str">
+        <x:v>Print PDF</x:v>
+      </x:c>
+      <x:c r="C170" t="str">
+        <x:v>Visual render</x:v>
+      </x:c>
+      <x:c r="D170" t="str">
+        <x:v>Tai lieu co text, rect, ellipse, image, rotation, opacity va background</x:v>
+      </x:c>
+      <x:c r="E170" t="str">
+        <x:v>Xuat PDF, render ca hai trang bang PDFium va kiem tra anh.</x:v>
+      </x:c>
+      <x:c r="F170" t="str">
+        <x:v>Hai mat hien dung noi dung; khong blank, glyph loi, guide, selection handle hoac editor controls.</x:v>
+      </x:c>
+      <x:c r="G170" t="str">
+        <x:v>Front/Back render da inspect; layer va background khac nhau; khong co control/guide trong output.</x:v>
+      </x:c>
+      <x:c r="H170" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I170" t="str">
+        <x:v>PDFium render + visual inspection</x:v>
+      </x:c>
+      <x:c r="J170" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K170" t="str">
+        <x:v>Phase 6E</x:v>
+      </x:c>
+      <x:c r="L170" t="str">
+        <x:v>Image loi/khong doc duoc se block export voi thong bao ro.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>E2E-191</x:v>
+      </x:c>
+      <x:c r="B171" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>Responsive export UI</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>Desktop va mobile 390 x 844</x:v>
+      </x:c>
+      <x:c r="E171" t="str">
+        <x:v>Mo editor, kiem tra nut Export tren header/inspector va tran ngang.</x:v>
+      </x:c>
+      <x:c r="F171" t="str">
+        <x:v>Export dung duoc tren desktop/mobile; documentWidth bang viewport; khong console/page/server error.</x:v>
+      </x:c>
+      <x:c r="G171" t="str">
+        <x:v>Mobile viewport 390, documentWidth 390, inspector export width 366; 0 unexpected errors.</x:v>
+      </x:c>
+      <x:c r="H171" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I171" t="str">
+        <x:v>Playwright desktop/mobile</x:v>
+      </x:c>
+      <x:c r="J171" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K171" t="str">
+        <x:v>Phase 7</x:v>
+      </x:c>
+      <x:c r="L171" t="str">
+        <x:v>Nut Export tren header duoc giu khi mobile.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>E2E-192</x:v>
+      </x:c>
+      <x:c r="B172" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C172" t="str">
+        <x:v>Final acceptance</x:v>
+      </x:c>
+      <x:c r="D172" t="str">
+        <x:v>Frontend, backend va cac luong hoi quy san sang</x:v>
+      </x:c>
+      <x:c r="E172" t="str">
+        <x:v>Chay build, XSS, audit, 7 browser smoke suites, full backend test va kiem tra PDF.</x:v>
+      </x:c>
+      <x:c r="F172" t="str">
+        <x:v>Tat ca check xanh; khong regression chuc nang Editor V2; backend test 93/93.</x:v>
+      </x:c>
+      <x:c r="G172" t="str">
+        <x:v>FE build PASS; XSS PASS; npm audit 0; 7 browser suites PASS; BE 93/93; PDF binary + visual PASS.</x:v>
+      </x:c>
+      <x:c r="H172" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I172" t="str">
+        <x:v>Multi-layer acceptance suite</x:v>
+      </x:c>
+      <x:c r="J172" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K172" t="str">
+        <x:v>Phase 7</x:v>
+      </x:c>
+      <x:c r="L172" t="str">
+        <x:v>PDF MVP dung RGB raster-backed; PDF/X va CMYK profile de hardening sau.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8010,23 +8238,23 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Editor V2 checkout preview, side switch and preflight order guard</x:v>
+        <x:v>Phase 6E print PDF and Phase 7 Editor V2 acceptance</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>FE</x:v>
+        <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>http://127.0.0.1:5173/editor/15 -&gt; /checkout/{designId}</x:v>
+        <x:v>http://127.0.0.1:5173</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>BE</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>POST /api/orders enforces PreflightService before persistence</x:v>
+        <x:v>Full suite PASS 93/93</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -8034,15 +8262,15 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Frontend build/XSS and six browser smokes PASS; full backend 93/93 PASS</x:v>
+        <x:v>Build, XSS, npm audit, 7 browser suites and backend suite PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Contract</x:v>
+        <x:v>Export</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Editor saves schema V2 before checkout; errors block orders; warnings remain allowed</x:v>
+        <x:v>2 pages Front/Back, 94 x 58 mm, 300 DPI, 2 mm bleed</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -8050,7 +8278,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-182 through E2E-186</x:v>
+        <x:v>E2E-187 through E2E-192</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -8058,23 +8286,23 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after expected TDD RED failures</x:v>
+        <x:v>None after locator and backend record-name fixes were retested</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Security</x:v>
+        <x:v>Phase</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>CSRF and owner filtering retained; direct API cannot bypass preflight errors</x:v>
+        <x:v>Editor V2 MVP accepted end-to-end</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Responsive</x:v>
+        <x:v>Boundary</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Desktop and 390 x 844 mobile contained; side switch width 147 px</x:v>
+        <x:v>RGB raster-backed PDF MVP; PDF/X and CMYK printer profiles remain production hardening</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -8082,7 +8310,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Checkout screenshots, exact order payload and rejected-save then successful-save sequence were inspected</x:v>
+        <x:v>Local browser screenshots and PDF renders inspected; no personal paths recorded</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Cut over draft previews to Editor V2
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rb38704dca53745eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R1b1b53e85ffc47a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R53a2338afbe9498b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R293ee7b669864084"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8204,6 +8204,196 @@
         <x:v>PDF MVP dung RGB raster-backed; PDF/X va CMYK profile de hardening sau.</x:v>
       </x:c>
     </x:row>
+    <x:row r="173">
+      <x:c r="A173" t="str">
+        <x:v>E2E-193</x:v>
+      </x:c>
+      <x:c r="B173" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C173" t="str">
+        <x:v>Source cutover</x:v>
+      </x:c>
+      <x:c r="D173" t="str">
+        <x:v>Route editor da tro den EditorV2View va V1 con nam trong trang detail</x:v>
+      </x:c>
+      <x:c r="E173" t="str">
+        <x:v>Kiem tra router, xoa nhanh V1 khong con duoc goi va quet cac dau vet editor-shell/isEditorRoute.</x:v>
+      </x:c>
+      <x:c r="F173" t="str">
+        <x:v>DesignDetail chi con trang xem draft; khong con toolbar, save inline, AI/upload/background-removal V1.</x:v>
+      </x:c>
+      <x:c r="G173" t="str">
+        <x:v>Editor route van tro EditorV2View; DesignDetail giam tu 3225 xuong 151 dong; static scan khong con dau vet V1.</x:v>
+      </x:c>
+      <x:c r="H173" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I173" t="str">
+        <x:v>Static route and source scan</x:v>
+      </x:c>
+      <x:c r="J173" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K173" t="str">
+        <x:v>Cutover</x:v>
+      </x:c>
+      <x:c r="L173" t="str">
+        <x:v>Tag editor-v1-backup-20260716 van giu kha nang khoi phuc; khong reset du lieu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>E2E-194</x:v>
+      </x:c>
+      <x:c r="B174" t="str">
+        <x:v>Draft detail</x:v>
+      </x:c>
+      <x:c r="C174" t="str">
+        <x:v>V2 Front and Back preview</x:v>
+      </x:c>
+      <x:c r="D174" t="str">
+        <x:v>Draft schemaVersion 2 co background va text khac nhau o hai mat</x:v>
+      </x:c>
+      <x:c r="E174" t="str">
+        <x:v>Mo /designs/7272, kiem tra Front, chuyen Back va doi chieu background/noi dung.</x:v>
+      </x:c>
+      <x:c r="F174" t="str">
+        <x:v>Chi dung 2 mat; moi mat hien dung layer/background; link Open editor va Checkout dung design id.</x:v>
+      </x:c>
+      <x:c r="G174" t="str">
+        <x:v>Front/Back deu dung; khong tron layer; href /editor/7272 va /checkout/7272.</x:v>
+      </x:c>
+      <x:c r="H174" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I174" t="str">
+        <x:v>Playwright API mock</x:v>
+      </x:c>
+      <x:c r="J174" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K174" t="str">
+        <x:v>Cutover</x:v>
+      </x:c>
+      <x:c r="L174" t="str">
+        <x:v>Trang detail chi doc; moi thay doi duoc chuyen sang Editor V2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" t="str">
+        <x:v>E2E-195</x:v>
+      </x:c>
+      <x:c r="B175" t="str">
+        <x:v>Draft preview</x:v>
+      </x:c>
+      <x:c r="C175" t="str">
+        <x:v>V2 and legacy compatibility</x:v>
+      </x:c>
+      <x:c r="D175" t="str">
+        <x:v>Danh sach co mot draft V2 va mot draft schema cu</x:v>
+      </x:c>
+      <x:c r="E175" t="str">
+        <x:v>Mo My drafts va detail cua tung draft; kiem tra thumbnail Front va chuyen Front/Back cua schema cu.</x:v>
+      </x:c>
+      <x:c r="F175" t="str">
+        <x:v>V2 khong con thumbnail trong; draft cu van doc duoc ma khong migration/reset.</x:v>
+      </x:c>
+      <x:c r="G175" t="str">
+        <x:v>V2 FRONT CONTENT va LEGACY FRONT/BACK CONTENT deu render dung.</x:v>
+      </x:c>
+      <x:c r="H175" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I175" t="str">
+        <x:v>Shared parser + browser smoke</x:v>
+      </x:c>
+      <x:c r="J175" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K175" t="str">
+        <x:v>Cutover</x:v>
+      </x:c>
+      <x:c r="L175" t="str">
+        <x:v>Khong sua canvasJson khi chi xem preview.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" t="str">
+        <x:v>E2E-196</x:v>
+      </x:c>
+      <x:c r="B176" t="str">
+        <x:v>Draft detail</x:v>
+      </x:c>
+      <x:c r="C176" t="str">
+        <x:v>Delete confirmation and responsive</x:v>
+      </x:c>
+      <x:c r="D176" t="str">
+        <x:v>Draft thuoc user hien tai; viewport desktop va 390 x 844</x:v>
+      </x:c>
+      <x:c r="E176" t="str">
+        <x:v>Bam Delete draft mot lan, xac nhan lan hai, kiem tra request/redirect va tran ngang mobile.</x:v>
+      </x:c>
+      <x:c r="F176" t="str">
+        <x:v>Lan dau khong gui DELETE; lan hai gui dung 1 request va ve /designs; mobile khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="G176" t="str">
+        <x:v>DELETE calls 1 sau confirm; viewport/document 390; shell 358 px; 0 console/page/server errors.</x:v>
+      </x:c>
+      <x:c r="H176" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I176" t="str">
+        <x:v>Playwright interaction + network</x:v>
+      </x:c>
+      <x:c r="J176" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K176" t="str">
+        <x:v>Cutover</x:v>
+      </x:c>
+      <x:c r="L176" t="str">
+        <x:v>API backend van chiu trach nhiem kiem tra ownership va CSRF.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" t="str">
+        <x:v>E2E-197</x:v>
+      </x:c>
+      <x:c r="B177" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C177" t="str">
+        <x:v>Cutover regression acceptance</x:v>
+      </x:c>
+      <x:c r="D177" t="str">
+        <x:v>Source cutover va preview parser chung da hoan thanh</x:v>
+      </x:c>
+      <x:c r="E177" t="str">
+        <x:v>Chay build, XSS, npm audit, smoke cutover, 7 regression browser suites va full backend test.</x:v>
+      </x:c>
+      <x:c r="F177" t="str">
+        <x:v>Tat ca check xanh; checkout/editor/export/xoa nen/preflight/guide khong regression.</x:v>
+      </x:c>
+      <x:c r="G177" t="str">
+        <x:v>FE build PASS; XSS PASS; audit 0; 8 browser suites PASS; BE 93/93; main JS 1951.69 -&gt; 334.69 kB.</x:v>
+      </x:c>
+      <x:c r="H177" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I177" t="str">
+        <x:v>Multi-layer acceptance suite</x:v>
+      </x:c>
+      <x:c r="J177" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K177" t="str">
+        <x:v>Cutover</x:v>
+      </x:c>
+      <x:c r="L177" t="str">
+        <x:v>Giam khoang 82.9% main JS; PDF/X/CMYK van la production hardening rieng.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8238,7 +8428,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Phase 6E print PDF and Phase 7 Editor V2 acceptance</x:v>
+        <x:v>Editor V2 source cutover and V2/legacy draft preview compatibility</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -8262,15 +8452,15 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Build, XSS, npm audit, 7 browser suites and backend suite PASS</x:v>
+        <x:v>Build, XSS, npm audit, 8 browser suites and backend suite PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Export</x:v>
+        <x:v>Cutover</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>2 pages Front/Back, 94 x 58 mm, 300 DPI, 2 mm bleed</x:v>
+        <x:v>Dead Editor V1 branch removed; edit route remains EditorV2View</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -8278,7 +8468,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>E2E-187 through E2E-192</x:v>
+        <x:v>E2E-193 through E2E-197</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -8286,15 +8476,15 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>None after locator and backend record-name fixes were retested</x:v>
+        <x:v>None after full browser and backend retest</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Phase</x:v>
+        <x:v>Performance</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>Editor V2 MVP accepted end-to-end</x:v>
+        <x:v>Main JS reduced from 1951.69 kB to 334.69 kB</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -8302,7 +8492,7 @@
         <x:v>Boundary</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>RGB raster-backed PDF MVP; PDF/X and CMYK printer profiles remain production hardening</x:v>
+        <x:v>Existing V1 draft data preserved; reset requires separate explicit approval</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -8310,7 +8500,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Local browser screenshots and PDF renders inspected; no personal paths recorded</x:v>
+        <x:v>Local browser screenshots inspected; no personal paths recorded</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Replace Brand panel with Icons8 library
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R53a2338afbe9498b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R293ee7b669864084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R299aae82f5024f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R9edd24c9904e40e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,12 +32,22 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -70,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
@@ -86,6 +96,25 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -357,6 +386,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="44" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="inlineStr">
@@ -8392,6 +8435,766 @@
       </x:c>
       <x:c r="L177" t="str">
         <x:v>Giam khoang 82.9% main JS; PDF/X/CMYK van la production hardening rieng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="84" customHeight="1">
+      <x:c r="A178" s="7" t="str">
+        <x:v>E2E-198</x:v>
+      </x:c>
+      <x:c r="B178" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C178" s="7" t="str">
+        <x:v>Zoom min, max and presets</x:v>
+      </x:c>
+      <x:c r="D178" s="7" t="str">
+        <x:v>Draft co card 90 x 54 mm; zoom control dang hoat dong</x:v>
+      </x:c>
+      <x:c r="E178" s="7" t="str">
+        <x:v>Mo menu zoom, chon lan luot 5% va 800%, sau do bam tru/cong o hai bien.</x:v>
+      </x:c>
+      <x:c r="F178" s="7" t="str">
+        <x:v>Co 7 preset 5/25/50/100/200/400/800; canvas scale dung; khong vuot duoi 5% hoac tren 800%.</x:v>
+      </x:c>
+      <x:c r="G178" s="7" t="str">
+        <x:v>5% render matrix 0.05; 800% render matrix 8; nut tru/cong deu clamp dung bien.</x:v>
+      </x:c>
+      <x:c r="H178" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I178" s="7" t="str">
+        <x:v>Playwright interaction + computed transform</x:v>
+      </x:c>
+      <x:c r="J178" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K178" s="7" t="str">
+        <x:v>Zoom and image</x:v>
+      </x:c>
+      <x:c r="L178" s="7" t="str">
+        <x:v>Menu dong bang Escape; khong co console/page/server error.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="84" customHeight="1">
+      <x:c r="A179" s="7" t="str">
+        <x:v>E2E-199</x:v>
+      </x:c>
+      <x:c r="B179" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C179" s="7" t="str">
+        <x:v>Fit card and Zoom to selection</x:v>
+      </x:c>
+      <x:c r="D179" s="7" t="str">
+        <x:v>Card 90 x 54 mm co mot layer nam lech tam; viewport desktop va 390 x 844</x:v>
+      </x:c>
+      <x:c r="E179" s="7" t="str">
+        <x:v>Chon Fit card, chon layer, chay Zoom to selection va doi chieu kich thuoc/transform/responsive.</x:v>
+      </x:c>
+      <x:c r="F179" s="7" t="str">
+        <x:v>Fit card nam tron workspace; selection duoc phong to va dua vao tam; menu mobile khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="G179" s="7" t="str">
+        <x:v>Fit 102%; selection 278%; canvas matrix co pan X/Y; viewport/document 390/390.</x:v>
+      </x:c>
+      <x:c r="H179" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I179" s="7" t="str">
+        <x:v>Playwright geometry + responsive</x:v>
+      </x:c>
+      <x:c r="J179" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K179" s="7" t="str">
+        <x:v>Zoom and image</x:v>
+      </x:c>
+      <x:c r="L179" s="7" t="str">
+        <x:v>Pan chi la trang thai hien thi, khong thay doi toa do layer trong draft.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="84" customHeight="1">
+      <x:c r="A180" s="7" t="str">
+        <x:v>E2E-200</x:v>
+      </x:c>
+      <x:c r="B180" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C180" s="7" t="str">
+        <x:v>Extract and re-extract image palette</x:v>
+      </x:c>
+      <x:c r="D180" s="7" t="str">
+        <x:v>Anh mau mau co 6 dai mau ro rang</x:v>
+      </x:c>
+      <x:c r="E180" s="7" t="str">
+        <x:v>Chon anh, bam Extract palette, doi chieu 6 swatch, sau do bam Re-extract palette.</x:v>
+      </x:c>
+      <x:c r="F180" s="7" t="str">
+        <x:v>Tra ve toi da 6 mau hop le va khac nhau; re-extract doc lai anh; UI hien swatch dung.</x:v>
+      </x:c>
+      <x:c r="G180" s="7" t="str">
+        <x:v>Lay dung #ef4444, #f59e0b, #10b981, #3b82f6, #8b5cf6, #111827; image request tang khi re-extract.</x:v>
+      </x:c>
+      <x:c r="H180" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I180" s="7" t="str">
+        <x:v>Playwright image analysis + visual screenshot</x:v>
+      </x:c>
+      <x:c r="J180" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K180" s="7" t="str">
+        <x:v>Zoom and image</x:v>
+      </x:c>
+      <x:c r="L180" s="7" t="str">
+        <x:v>Xu ly trong browser; bo qua pixel trong suot va tu choi response khong phai image/qua 15 MB.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="84" customHeight="1">
+      <x:c r="A181" s="7" t="str">
+        <x:v>E2E-201</x:v>
+      </x:c>
+      <x:c r="B181" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C181" s="7" t="str">
+        <x:v>Palette document colors and persistence</x:v>
+      </x:c>
+      <x:c r="D181" s="7" t="str">
+        <x:v>Draft V2 co image va shape; API save co CSRF mock</x:v>
+      </x:c>
+      <x:c r="E181" s="7" t="str">
+        <x:v>Extract palette, ap mau dau tien cho shape, Save draft, xoa local cache va reload tu backend.</x:v>
+      </x:c>
+      <x:c r="F181" s="7" t="str">
+        <x:v>Mau da extract xuat hien trong document colors; shape nhan mau; palette con nguyen sau backend reload.</x:v>
+      </x:c>
+      <x:c r="G181" s="7" t="str">
+        <x:v>Shape fill #ef4444; 6 mau luu trong extractedPalette; CSRF header dung; reload van co Re-extract palette.</x:v>
+      </x:c>
+      <x:c r="H181" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I181" s="7" t="str">
+        <x:v>Playwright save/reload + JSON readback</x:v>
+      </x:c>
+      <x:c r="J181" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K181" s="7" t="str">
+        <x:v>Zoom and image</x:v>
+      </x:c>
+      <x:c r="L181" s="7" t="str">
+        <x:v>Schema chi chap nhan toi da 8 gia tri hex; thay anh/xoa nen se xoa palette cu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="84" customHeight="1">
+      <x:c r="A182" s="7" t="str">
+        <x:v>E2E-202</x:v>
+      </x:c>
+      <x:c r="B182" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C182" s="7" t="str">
+        <x:v>Zoom and palette regression acceptance</x:v>
+      </x:c>
+      <x:c r="D182" s="7" t="str">
+        <x:v>Zoom va palette da hoan thanh tren Editor V2</x:v>
+      </x:c>
+      <x:c r="E182" s="7" t="str">
+        <x:v>Chay FE build, XSS guard, npm audit, 6 browser suites va full backend test.</x:v>
+      </x:c>
+      <x:c r="F182" s="7" t="str">
+        <x:v>Tat ca check xanh; draft, xoa nen, toolbar va PDF khong regression.</x:v>
+      </x:c>
+      <x:c r="G182" s="7" t="str">
+        <x:v>FE build PASS; XSS PASS; audit 0; palette/zoom/draft/background/toolbars/PDF PASS; BE 93/93.</x:v>
+      </x:c>
+      <x:c r="H182" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I182" s="7" t="str">
+        <x:v>Multi-layer acceptance suite</x:v>
+      </x:c>
+      <x:c r="J182" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K182" s="7" t="str">
+        <x:v>Zoom and image</x:v>
+      </x:c>
+      <x:c r="L182" s="7" t="str">
+        <x:v>Thay doi chi o frontend/schema JSON; khong them dependency, secret hoac endpoint public.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="88" customHeight="1">
+      <x:c r="A183" s="7" t="str">
+        <x:v>E2E-203</x:v>
+      </x:c>
+      <x:c r="B183" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C183" s="7" t="str">
+        <x:v>Swap rectangle, rounded and ellipse</x:v>
+      </x:c>
+      <x:c r="D183" s="7" t="str">
+        <x:v>Shape co x/y/width/height/rotation/opacity co dinh</x:v>
+      </x:c>
+      <x:c r="E183" s="7" t="str">
+        <x:v>Doi Rectangle sang Ellipse, save/reload, doi Rounded roi Rectangle; kiem tra mobile.</x:v>
+      </x:c>
+      <x:c r="F183" s="7" t="str">
+        <x:v>Loai shape va corner radius doi dung; id va geometry khong doi; save/reload va mobile hop le.</x:v>
+      </x:c>
+      <x:c r="G183" s="7" t="str">
+        <x:v>Geometry truoc/sau giong het; ellipse radius 50%; rounded 16 px; payload ellipse/rect; viewport/document/inspector 390/390/390.</x:v>
+      </x:c>
+      <x:c r="H183" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I183" s="7" t="str">
+        <x:v>Playwright computed style + API payload</x:v>
+      </x:c>
+      <x:c r="J183" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K183" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L183" s="7" t="str">
+        <x:v>Khong thay doi layer id, toa do, kich thuoc, rotation hoac opacity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="88" customHeight="1">
+      <x:c r="A184" s="7" t="str">
+        <x:v>E2E-204</x:v>
+      </x:c>
+      <x:c r="B184" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C184" s="7" t="str">
+        <x:v>Linear and radial gradient</x:v>
+      </x:c>
+      <x:c r="D184" s="7" t="str">
+        <x:v>Shape V2 co solid fill</x:v>
+      </x:c>
+      <x:c r="E184" s="7" t="str">
+        <x:v>Bat Gradient; chinh angle, 3 color stops; chuyen Radial, chinh center/radius; save/reload va mo draft preview.</x:v>
+      </x:c>
+      <x:c r="F184" s="7" t="str">
+        <x:v>Editor va shared preview render cung gradient; JSON giu stops, opacity, center/radius; mobile khong tran.</x:v>
+      </x:c>
+      <x:c r="G184" s="7" t="str">
+        <x:v>Radial 74% tai 35%/62%; stops #6138db, #f97316@48%, #00aaff; save/reload PASS; mobile 390 px.</x:v>
+      </x:c>
+      <x:c r="H184" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I184" s="7" t="str">
+        <x:v>Playwright editor + shared preview + JSON</x:v>
+      </x:c>
+      <x:c r="J184" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K184" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L184" s="7" t="str">
+        <x:v>Toi da 4 stops; schema chi chap nhan hex, offset/opacity hop le.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="88" customHeight="1">
+      <x:c r="A185" s="7" t="str">
+        <x:v>E2E-205</x:v>
+      </x:c>
+      <x:c r="B185" s="7" t="str">
+        <x:v>Print PDF</x:v>
+      </x:c>
+      <x:c r="C185" s="7" t="str">
+        <x:v>Gradient print rendering</x:v>
+      </x:c>
+      <x:c r="D185" s="7" t="str">
+        <x:v>Tai lieu 2 mat co Linear va Radial gradient 3 stops</x:v>
+      </x:c>
+      <x:c r="E185" s="7" t="str">
+        <x:v>Xuat PDF va theo doi CanvasGradient/addColorStop tren canvas 300 DPI.</x:v>
+      </x:c>
+      <x:c r="F185" s="7" t="str">
+        <x:v>Linear/Radial duoc tao trong print canvas; offset va alpha khong mat; PDF hop le.</x:v>
+      </x:c>
+      <x:c r="G185" s="7" t="str">
+        <x:v>2 gradient calls; moi call 3 stops; stop 0.48 co alpha 0.65; radial radius 0.74; PDF 284470 bytes.</x:v>
+      </x:c>
+      <x:c r="H185" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I185" s="7" t="str">
+        <x:v>Canvas instrumentation + PDF binary</x:v>
+      </x:c>
+      <x:c r="J185" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K185" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L185" s="7" t="str">
+        <x:v>PDF van 2 mat, 94 x 58 mm va 1110 x 685 px theo smoke tong quat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="88" customHeight="1">
+      <x:c r="A186" s="7" t="str">
+        <x:v>E2E-206</x:v>
+      </x:c>
+      <x:c r="B186" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C186" s="7" t="str">
+        <x:v>Shadow, Hollow and Glow</x:v>
+      </x:c>
+      <x:c r="D186" s="7" t="str">
+        <x:v>Shape solid khong effect</x:v>
+      </x:c>
+      <x:c r="E186" s="7" t="str">
+        <x:v>Bat Shadow va chinh X/Y/blur/color/opacity; chuyen Hollow; chuyen Glow; save/reload va shared preview.</x:v>
+      </x:c>
+      <x:c r="F186" s="7" t="str">
+        <x:v>Shadow va Glow render dung; Hollow bo fill va tu bat stroke &gt;=2 px; persistence va preview khop editor.</x:v>
+      </x:c>
+      <x:c r="G186" s="7" t="str">
+        <x:v>Shadow rgba(18,52,86,.55) 6/9/24; Hollow transparent + stroke 2; Glow rgba(0,204,255,.75) 0/0/28; mobile 390 px.</x:v>
+      </x:c>
+      <x:c r="H186" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I186" s="7" t="str">
+        <x:v>Playwright computed style + save/reload</x:v>
+      </x:c>
+      <x:c r="J186" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K186" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L186" s="7" t="str">
+        <x:v>Hollow giu fill goc de co the quay lai effect khac ma khong mat mau.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="88" customHeight="1">
+      <x:c r="A187" s="7" t="str">
+        <x:v>E2E-207</x:v>
+      </x:c>
+      <x:c r="B187" s="7" t="str">
+        <x:v>Print PDF</x:v>
+      </x:c>
+      <x:c r="C187" s="7" t="str">
+        <x:v>Shape effects print rendering</x:v>
+      </x:c>
+      <x:c r="D187" s="7" t="str">
+        <x:v>Front Shadow; Back Glow va Hollow</x:v>
+      </x:c>
+      <x:c r="E187" s="7" t="str">
+        <x:v>Xuat PDF, theo doi fill/stroke/clip va shadow state cua print canvas.</x:v>
+      </x:c>
+      <x:c r="F187" s="7" t="str">
+        <x:v>Shadow/Glow duoc scale theo print; Hollow khong fill; stroke khong nhan shadow lan hai; bong khong bi clip.</x:v>
+      </x:c>
+      <x:c r="G187" s="7" t="str">
+        <x:v>2 fill calls; 3 stroke calls; clip=0; shadow/glow offsets dung; PDF 87686 bytes.</x:v>
+      </x:c>
+      <x:c r="H187" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I187" s="7" t="str">
+        <x:v>Canvas paint instrumentation + PDF binary</x:v>
+      </x:c>
+      <x:c r="J187" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K187" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L187" s="7" t="str">
+        <x:v>Shadow spread chua mo trong UI; X/Y/blur/color/opacity duoc dong bo print.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="88" customHeight="1">
+      <x:c r="A188" s="7" t="str">
+        <x:v>E2E-208</x:v>
+      </x:c>
+      <x:c r="B188" s="7" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C188" s="7" t="str">
+        <x:v>Editor and preview regression</x:v>
+      </x:c>
+      <x:c r="D188" s="7" t="str">
+        <x:v>Shape Core hoan thanh</x:v>
+      </x:c>
+      <x:c r="E188" s="7" t="str">
+        <x:v>Chay draft persistence, toolbar/layer reorder, background removal, zoom, print export, template legacy preview, image palette va visual desktop/mobile.</x:v>
+      </x:c>
+      <x:c r="F188" s="7" t="str">
+        <x:v>Tat ca luong cu xanh; preview legacy background khong bi trong suot; UI Shape Core khong overlap/tran ngang.</x:v>
+      </x:c>
+      <x:c r="G188" s="7" t="str">
+        <x:v>8 browser/visual suites PASS; legacy template preview text dung; viewport/document/inspector mobile 390/390/390; runtime errors=0.</x:v>
+      </x:c>
+      <x:c r="H188" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I188" s="7" t="str">
+        <x:v>Browser regression + visual QA</x:v>
+      </x:c>
+      <x:c r="J188" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K188" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L188" s="7" t="str">
+        <x:v>Runbook zoom cu tro toi file stale da duoc thay bang editor-v2-zoom-smoke.cjs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="88" customHeight="1">
+      <x:c r="A189" s="7" t="str">
+        <x:v>E2E-209</x:v>
+      </x:c>
+      <x:c r="B189" s="7" t="str">
+        <x:v>Acceptance</x:v>
+      </x:c>
+      <x:c r="C189" s="7" t="str">
+        <x:v>Shape Core full acceptance</x:v>
+      </x:c>
+      <x:c r="D189" s="7" t="str">
+        <x:v>Code Shape Core va regression fixes</x:v>
+      </x:c>
+      <x:c r="E189" s="7" t="str">
+        <x:v>Chay FE build/typecheck, XSS guard, npm audit, 5 Shape Core suites, regression browser va full backend suite.</x:v>
+      </x:c>
+      <x:c r="F189" s="7" t="str">
+        <x:v>Tat ca check xanh; khong them dependency, endpoint public, secret hay thay doi backend production.</x:v>
+      </x:c>
+      <x:c r="G189" s="7" t="str">
+        <x:v>FE build PASS; XSS PASS; npm audit 0; Shape Core + regression PASS; backend 93/93.</x:v>
+      </x:c>
+      <x:c r="H189" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I189" s="7" t="str">
+        <x:v>Multi-layer acceptance suite</x:v>
+      </x:c>
+      <x:c r="J189" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K189" s="7" t="str">
+        <x:v>Shape Core</x:v>
+      </x:c>
+      <x:c r="L189" s="7" t="str">
+        <x:v>Chi sua frontend schema/render/UI va workbook kiem thu local; chua push GitHub.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="88" customHeight="1">
+      <x:c r="A190" s="7" t="str">
+        <x:v>E2E-210</x:v>
+      </x:c>
+      <x:c r="B190" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C190" s="7" t="str">
+        <x:v>Extended shape presets</x:v>
+      </x:c>
+      <x:c r="D190" s="7" t="str">
+        <x:v>Elements panel mo va card trong</x:v>
+      </x:c>
+      <x:c r="E190" s="7" t="str">
+        <x:v>Them lan luot 11 shape; kiem tra loai shape, renderer, schema va save/reload.</x:v>
+      </x:c>
+      <x:c r="F190" s="7" t="str">
+        <x:v>Rectangle, Rounded, Ellipse, Triangle, Pentagon, Hexagon, Star, Diamond, Octagon, Burst va Pill tao dung shapeKind; UI va payload hop le.</x:v>
+      </x:c>
+      <x:c r="G190" s="7" t="str">
+        <x:v>11/11 shape PASS; shapeCount 11; id rieng; editor/shared preview va schema persistence dong bo.</x:v>
+      </x:c>
+      <x:c r="H190" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I190" s="7" t="str">
+        <x:v>Playwright UI + computed render + API payload</x:v>
+      </x:c>
+      <x:c r="J190" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K190" s="7" t="str">
+        <x:v>Shapes &amp; Frames</x:v>
+      </x:c>
+      <x:c r="L190" s="7" t="str">
+        <x:v>Khong them dependency hay schema group rieng; shapeKind la metadata tuy chon tren layer V2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="88" customHeight="1">
+      <x:c r="A191" s="7" t="str">
+        <x:v>E2E-211</x:v>
+      </x:c>
+      <x:c r="B191" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C191" s="7" t="str">
+        <x:v>Frames and grid presets</x:v>
+      </x:c>
+      <x:c r="D191" s="7" t="str">
+        <x:v>Elements panel mo va card trong</x:v>
+      </x:c>
+      <x:c r="E191" s="7" t="str">
+        <x:v>Them 12 frame/grid preset; dem placeholder va kiem tra frameId, geometry, chon/keo/resize tung o.</x:v>
+      </x:c>
+      <x:c r="F191" s="7" t="str">
+        <x:v>Frame, Circle, Rounded, 2/3/4/6/9 photos, Feature left/right/top va Hero mosaic tao dung bo cuc; moi nhom co frameId rieng.</x:v>
+      </x:c>
+      <x:c r="G191" s="7" t="str">
+        <x:v>12/12 preset PASS; tong 40 image placeholder; group sizes va frameId doc nhat dung; layer thao tac doc lap.</x:v>
+      </x:c>
+      <x:c r="H191" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I191" s="7" t="str">
+        <x:v>Playwright layer count + group/schema assertions</x:v>
+      </x:c>
+      <x:c r="J191" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K191" s="7" t="str">
+        <x:v>Shapes &amp; Frames</x:v>
+      </x:c>
+      <x:c r="L191" s="7" t="str">
+        <x:v>Frame dung image layer chuan de giu luong select, drag, resize, lock va save/reload hien co.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="88" customHeight="1">
+      <x:c r="A192" s="7" t="str">
+        <x:v>E2E-212</x:v>
+      </x:c>
+      <x:c r="B192" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C192" s="7" t="str">
+        <x:v>Replace selected frame image</x:v>
+      </x:c>
+      <x:c r="D192" s="7" t="str">
+        <x:v>Da chon mot image placeholder</x:v>
+      </x:c>
+      <x:c r="E192" s="7" t="str">
+        <x:v>Mo Uploads, upload anh vao frame dang chon, save draft, reload va kiem tra responsive mobile.</x:v>
+      </x:c>
+      <x:c r="F192" s="7" t="str">
+        <x:v>Anh thay placeholder nhung giu geometry, shapeKind va frameId; CSRF/save/reload hop le; mobile khong tran ngang.</x:v>
+      </x:c>
+      <x:c r="G192" s="7" t="str">
+        <x:v>Upload selected frame PASS; payload reload PASS; viewport/document/inspector 390/390/390; runtime errors=0.</x:v>
+      </x:c>
+      <x:c r="H192" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I192" s="7" t="str">
+        <x:v>Playwright upload + save/reload + mobile</x:v>
+      </x:c>
+      <x:c r="J192" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K192" s="7" t="str">
+        <x:v>Shapes &amp; Frames</x:v>
+      </x:c>
+      <x:c r="L192" s="7" t="str">
+        <x:v>Empty frame hien placeholder tren editor/preview; frame co anh render cover theo hinh dang.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="88" customHeight="1">
+      <x:c r="A193" s="7" t="str">
+        <x:v>E2E-213</x:v>
+      </x:c>
+      <x:c r="B193" s="7" t="str">
+        <x:v>Print PDF</x:v>
+      </x:c>
+      <x:c r="C193" s="7" t="str">
+        <x:v>Extended shapes and empty frames</x:v>
+      </x:c>
+      <x:c r="D193" s="7" t="str">
+        <x:v>Tai lieu co polygon, pill, ellipse, frame rong va frame co anh</x:v>
+      </x:c>
+      <x:c r="E193" s="7" t="str">
+        <x:v>Xuat PDF, theo doi Canvas path/fill/clip va kiem tra binary PDF.</x:v>
+      </x:c>
+      <x:c r="F193" s="7" t="str">
+        <x:v>Polygon/pill/ellipse dung path; frame co anh clip theo shape; empty frame khong in; ordinary image thieu source van bi chan.</x:v>
+      </x:c>
+      <x:c r="G193" s="7" t="str">
+        <x:v>lineTo 11; roundRect radius &gt;0; ellipse 1; fill 4; clip 1; empty frame skipped; PDF 36925 bytes hop le.</x:v>
+      </x:c>
+      <x:c r="H193" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I193" s="7" t="str">
+        <x:v>Canvas instrumentation + PDF binary</x:v>
+      </x:c>
+      <x:c r="J193" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K193" s="7" t="str">
+        <x:v>Shapes &amp; Frames</x:v>
+      </x:c>
+      <x:c r="L193" s="7" t="str">
+        <x:v>Placeholder chi la huong dan UI, khong phai noi dung in.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="88" customHeight="1">
+      <x:c r="A194" s="7" t="str">
+        <x:v>E2E-214</x:v>
+      </x:c>
+      <x:c r="B194" s="7" t="str">
+        <x:v>Acceptance</x:v>
+      </x:c>
+      <x:c r="C194" s="7" t="str">
+        <x:v>Shapes and Frames full regression</x:v>
+      </x:c>
+      <x:c r="D194" s="7" t="str">
+        <x:v>Code va workbook cua batch da hoan tat</x:v>
+      </x:c>
+      <x:c r="E194" s="7" t="str">
+        <x:v>Chay FE build/typecheck, XSS guard, npm audit, browser smoke moi/cu, print smoke, persistence va full backend suite.</x:v>
+      </x:c>
+      <x:c r="F194" s="7" t="str">
+        <x:v>Tat ca check xanh; khong co regression FE/BE, dependency moi, endpoint public hay secret.</x:v>
+      </x:c>
+      <x:c r="G194" s="7" t="str">
+        <x:v>FE build PASS; XSS PASS; npm audit 0; browser/print/persistence PASS; backend 93/93; visual desktop/mobile PASS.</x:v>
+      </x:c>
+      <x:c r="H194" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I194" s="7" t="str">
+        <x:v>Multi-layer acceptance suite</x:v>
+      </x:c>
+      <x:c r="J194" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K194" s="7" t="str">
+        <x:v>Shapes &amp; Frames</x:v>
+      </x:c>
+      <x:c r="L194" s="7" t="str">
+        <x:v>Chua commit/push; cho local UAT truoc khi dua len GitHub.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="88" customHeight="1">
+      <x:c r="A195" s="7" t="str">
+        <x:v>E2E-215</x:v>
+      </x:c>
+      <x:c r="B195" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C195" s="7" t="str">
+        <x:v>Bundled local font library</x:v>
+      </x:c>
+      <x:c r="D195" s="7" t="str">
+        <x:v>Text panel mo va co font search</x:v>
+      </x:c>
+      <x:c r="E195" s="7" t="str">
+        <x:v>Mo Text, kiem tra manifest font, Show more, tim SVN Adeline, chon font, save/reload va mobile.</x:v>
+      </x:c>
+      <x:c r="F195" s="7" t="str">
+        <x:v>Hien thi font pack da co san; font local tai dung file, ap dung vao text layer, Canvas 2D nhan font va persistence khong mat.</x:v>
+      </x:c>
+      <x:c r="G195" s="7" t="str">
+        <x:v>1481 fonts; batch 40 -&gt; 80; SVN Adeline response 200; rendered/canvas/reload dung; viewport/document/panel 390/390/390; runtime errors=0.</x:v>
+      </x:c>
+      <x:c r="H195" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I195" s="7" t="str">
+        <x:v>Playwright browser + HTTP font response + Canvas 2D + API payload</x:v>
+      </x:c>
+      <x:c r="J195" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K195" s="7" t="str">
+        <x:v>Typography</x:v>
+      </x:c>
+      <x:c r="L195" s="7" t="str">
+        <x:v>Chi dung font files da bundle trong frontend; khong them upload endpoint hay secret.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="88" customHeight="1">
+      <x:c r="A196" s="7" t="str">
+        <x:v>E2E-216</x:v>
+      </x:c>
+      <x:c r="B196" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C196" s="7" t="str">
+        <x:v>Keyboard shortcuts and laptop viewport</x:v>
+      </x:c>
+      <x:c r="D196" s="7" t="str">
+        <x:v>Editor mo va co layer dang duoc chon</x:v>
+      </x:c>
+      <x:c r="E196" s="7" t="str">
+        <x:v>Kiem tra Ctrl/Cmd+C, V, D, Z, Shift+Z, Y, S; Delete, Backspace guard, mui ten, zoom; textarea; viewport 1366x700 va 390x844.</x:v>
+      </x:c>
+      <x:c r="F196" s="7" t="str">
+        <x:v>Shortcut thao tac dung layer; undo/redo va nut header dong bo; input khong bi hijack; day editor khong bi taskbar che.</x:v>
+      </x:c>
+      <x:c r="G196" s="7" t="str">
+        <x:v>Copy/paste 2-&gt;3; undo/redo/delete/duplicate/nudge PASS; zoom 100-&gt;110-&gt;100; save 1 request; laptop root/layout/pages bottom=700; mobile width=390; runtime errors=0.</x:v>
+      </x:c>
+      <x:c r="H196" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I196" s="7" t="str">
+        <x:v>Playwright keyboard interaction + API save mock + responsive geometry + regression suites</x:v>
+      </x:c>
+      <x:c r="J196" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K196" s="7" t="str">
+        <x:v>Keyboard and viewport</x:v>
+      </x:c>
+      <x:c r="L196" s="7" t="str">
+        <x:v>Clipboard chi nam trong editor; web app khong dieu khien OS taskbar, layout bam theo dynamic viewport; khong them secret.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="9" t="str">
+        <x:v>E2E-217</x:v>
+      </x:c>
+      <x:c r="B197" s="9" t="str">
+        <x:v>Editor V2/Icons8</x:v>
+      </x:c>
+      <x:c r="C197" s="9" t="str">
+        <x:v>Replace Brand panel with Icons8 asset library</x:v>
+      </x:c>
+      <x:c r="D197" s="9" t="str">
+        <x:v>Open editor, choose Icons8, search phone with Material style, click Add, check desktop and 390px mobile layout</x:v>
+      </x:c>
+      <x:c r="E197" s="9" t="str">
+        <x:v>Brand is replaced by Icons8; search results use upstream preview, attribution remains visible, Add creates an image layer, and the panel has no horizontal overflow</x:v>
+      </x:c>
+      <x:c r="F197" s="9" t="str">
+        <x:v>Icons8 panel smoke PASS; query term=phone platform=material amount=24; preview https://img.icons8.com/96/material/phone.png rendered; image layer added; desktop/mobile runtime errors=0</x:v>
+      </x:c>
+      <x:c r="G197" s="11" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H197" s="13" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I197" s="9" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="J197" s="9" t="str">
+        <x:v>Playwright browser smoke + FE build + Icons8ServiceTests</x:v>
+      </x:c>
+      <x:c r="K197" s="9" t="str">
+        <x:v>Backend reads ICONS8_API_KEY from environment; no key stored in frontend; upstream preview URL restricted to Icons8 hosts</x:v>
+      </x:c>
+      <x:c r="L197" s="9" t="str">
+        <x:v>Free use keeps Icons by Icons8 attribution link visible</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8402,105 +9205,109 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="92" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="inlineStr">
+      <x:c r="A1" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Field</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" t="inlineStr">
+      <x:c r="B1" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Value</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="7" t="str">
         <x:v>Date</x:v>
       </x:c>
-      <x:c r="B2" t="str">
-        <x:v>2026-07-17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
+      <x:c r="B2" s="7" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="7" t="str">
         <x:v>Focus</x:v>
       </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Editor V2 source cutover and V2/legacy draft preview compatibility</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
+      <x:c r="B3" s="7" t="str">
+        <x:v>Editor V2 keyboard shortcuts, history and laptop-safe viewport</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="7" t="str">
         <x:v>Frontend</x:v>
       </x:c>
-      <x:c r="B4" t="str">
-        <x:v>http://127.0.0.1:5173</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="B4" s="7" t="str">
+        <x:v>http://127.0.0.1:5173/editor/15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="7" t="str">
         <x:v>Backend</x:v>
       </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Full suite PASS 93/93</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="B5" s="7" t="str">
+        <x:v>No backend change; save API and existing draft persistence browser regression PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="7" t="str">
         <x:v>Health</x:v>
       </x:c>
-      <x:c r="B6" t="str">
-        <x:v>Build, XSS, npm audit, 8 browser suites and backend suite PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Cutover</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Dead Editor V1 branch removed; edit route remains EditorV2View</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="B6" s="7" t="str">
+        <x:v>Build, XSS, npm audit, keyboard, zoom, draft and toolbar browser suites PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="7" t="str">
+        <x:v>Shortcuts</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="str">
+        <x:v>Copy, paste, duplicate, delete, undo, redo, save, nudge and zoom verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="7" t="str">
+        <x:v>History</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="str">
+        <x:v>Header Undo/Redo state verified; save clears session history</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="7" t="str">
+        <x:v>Input safety</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="str">
+        <x:v>Textarea keeps native Delete behavior; editor shortcut does not remove layer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="7" t="str">
+        <x:v>Laptop viewport</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="str">
+        <x:v>1366x700 root/layout/pages bottom=700; zoom bottom=608; mobile width=390</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="7" t="str">
         <x:v>Retest PASS</x:v>
       </x:c>
-      <x:c r="B8" t="str">
-        <x:v>E2E-193 through E2E-197</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="B11" s="7" t="str">
+        <x:v>E2E-216</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="7" t="str">
         <x:v>Retest FAIL</x:v>
       </x:c>
-      <x:c r="B9" t="str">
-        <x:v>None after full browser and backend retest</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Performance</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Main JS reduced from 1951.69 kB to 334.69 kB</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>Boundary</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Existing V1 draft data preserved; reset requires separate explicit approval</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>Evidence</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>Local browser screenshots inspected; no personal paths recorded</x:v>
+      <x:c r="B12" s="7" t="str">
+        <x:v>None after final regression retest</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(editor): add drag drop placement and shortcut reference
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R299aae82f5024f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R9edd24c9904e40e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra967aeb2f6e54771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R2ea79c0c1ba844c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9197,6 +9197,44 @@
         <x:v>Free use keeps Icons by Icons8 attribution link visible</x:v>
       </x:c>
     </x:row>
+    <x:row r="198" ht="96" customHeight="1">
+      <x:c r="A198" s="7" t="str">
+        <x:v>E2E-218</x:v>
+      </x:c>
+      <x:c r="B198" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C198" s="7" t="str">
+        <x:v>Drag and drop media and editor assets</x:v>
+      </x:c>
+      <x:c r="D198" s="7" t="str">
+        <x:v>Open /editor/15 at 1440x900</x:v>
+      </x:c>
+      <x:c r="E198" s="7" t="str">
+        <x:v>Drop a file on either sidebar stores it in Your Media only; drop on the card stores it and places a new layer at the pointer; internal icon, shape and text cards can be dragged onto the card.</x:v>
+      </x:c>
+      <x:c r="F198" s="7" t="str">
+        <x:v>Each accepted image is validated as PNG, JPEG, WebP or GIF up to 5 MB; media-only drops do not change layers; canvas drops and internal assets create layers at the drop point; duplicate media is reused.</x:v>
+      </x:c>
+      <x:c r="G198" s="7" t="str">
+        <x:v>Playwright PASS: icon, rectangle and text placement; library and inspector media-only drops; canvas media plus layer; duplicate reuse; drop overlays cleared; console errors 0; build and XSS guard PASS.</x:v>
+      </x:c>
+      <x:c r="H198" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I198" s="7" t="str">
+        <x:v>Browser drag/drop smoke + DOM media/layer readback + build + XSS + keyboard and toolbar regressions</x:v>
+      </x:c>
+      <x:c r="J198" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K198" s="7" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L198" s="7" t="str">
+        <x:v>No secret or personal data; uploaded media is session-only until a backend asset library is added.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9222,92 +9260,92 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2" ht="34" customHeight="1">
+    <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="7" t="str">
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>2026-07-17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="38" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Editor V2 keyboard shortcuts, history and laptop-safe viewport</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="34" customHeight="1">
+        <x:v>Editor V2 drag and drop for external files and internal assets; searchable shortcut reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
       <x:c r="A4" s="7" t="str">
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5173/editor/15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
+        <x:v>http://127.0.0.1:5175/editor/15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>No backend change; save API and existing draft persistence browser regression PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="34" customHeight="1">
+        <x:v>No backend change; media library remains session-only and upload validation stays client-side</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Build, XSS, npm audit, keyboard, zoom, draft and toolbar browser suites PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="34" customHeight="1">
+        <x:v>Build, XSS guard, drag/drop smoke, shortcut regression and toolbar regression PASS; browser console errors 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="7" t="str">
+        <x:v>Drag and drop</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="str">
+        <x:v>Sidebar and inspector file drops add Your Media only; canvas file drop adds media and layer; internal icon, shape and text placement PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="38" customHeight="1">
+      <x:c r="A8" s="7" t="str">
         <x:v>Shortcuts</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
-        <x:v>Copy, paste, duplicate, delete, undo, redo, save, nudge and zoom verified</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="7" t="str">
-        <x:v>History</x:v>
-      </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Header Undo/Redo state verified; save clears session history</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="34" customHeight="1">
+        <x:v>Button below Layers, searchable dialog, ? opens, Esc closes, Zoom search PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>Input safety</x:v>
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>Textarea keeps native Delete behavior; editor shortcut does not remove layer</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="34" customHeight="1">
+        <x:v>PNG/JPEG/WebP/GIF only, maximum 5 MB; duplicate media source is reused</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="7" t="str">
-        <x:v>Laptop viewport</x:v>
+        <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>1366x700 root/layout/pages bottom=700; zoom bottom=608; mobile width=390</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="34" customHeight="1">
+        <x:v>E2E-218</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" s="7" t="str">
-        <x:v>Retest PASS</x:v>
+        <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>E2E-216</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="34" customHeight="1">
+        <x:v>None after final browser retest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="7" t="str">
-        <x:v>Retest FAIL</x:v>
+        <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>None after final regression retest</x:v>
+        <x:v>.codex-work/editor-v2-drag-drop-shortcuts-smoke.cjs; build; XSS guard; keyboard and toolbar regression output</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(editor): streamline header and add card preview
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra967aeb2f6e54771"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R2ea79c0c1ba844c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra4e9605f48434b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R3e4ac036c5264a82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9235,6 +9235,44 @@
         <x:v>No secret or personal data; uploaded media is session-only until a backend asset library is added.</x:v>
       </x:c>
     </x:row>
+    <x:row r="199" ht="96" customHeight="1">
+      <x:c r="A199" s="7" t="str">
+        <x:v>E2E-219</x:v>
+      </x:c>
+      <x:c r="B199" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C199" s="7" t="str">
+        <x:v>Header tool consolidation and Front/Back preview</x:v>
+      </x:c>
+      <x:c r="D199" s="7" t="str">
+        <x:v>Open /editor/15 at 1440x900, 1366x700 and 390x844; inspect the header, open Preview, switch Front/Back and press Esc.</x:v>
+      </x:c>
+      <x:c r="E199" s="7" t="str">
+        <x:v>Header keeps Preview, Preflight, Export PDF, Checkout and Save; Presentation, Comments, Notifications, More actions and Share are absent; Preview renders both fixed card sides without changing the design.</x:v>
+      </x:c>
+      <x:c r="F199" s="7" t="str">
+        <x:v>Required tools remain visible on desktop/mobile; Preview opens the shared canvas renderer, defaults to Front, switches to Back and closes with Esc; responsive header and modal stay inside the viewport.</x:v>
+      </x:c>
+      <x:c r="G199" s="7" t="str">
+        <x:v>Playwright PASS: 5 required tools, 5 redundant tools removed, 2 preview sides, desktop/mobile screenshots, document width equals viewport width, console errors 0; keyboard and toolbar regressions PASS; build and XSS guard PASS.</x:v>
+      </x:c>
+      <x:c r="H199" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I199" s="7" t="str">
+        <x:v>Browser preview smoke + visual screenshots + responsive geometry + keyboard/toolbar regressions + build + XSS guard</x:v>
+      </x:c>
+      <x:c r="J199" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K199" s="7" t="str">
+        <x:v>localhost FE5175</x:v>
+      </x:c>
+      <x:c r="L199" s="7" t="str">
+        <x:v>No backend or collaboration feature added; Preview reuses CanvasPreview and no secret or personal data is stored.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9273,7 +9311,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Editor V2 drag and drop for external files and internal assets; searchable shortcut reference</x:v>
+        <x:v>Editor V2 compact header and functional Front/Back preview</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
@@ -9289,7 +9327,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>No backend change; media library remains session-only and upload validation stays client-side</x:v>
+        <x:v>No backend change; collaboration-only controls intentionally removed</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -9297,31 +9335,31 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Build, XSS guard, drag/drop smoke, shortcut regression and toolbar regression PASS; browser console errors 0</x:v>
+        <x:v>Build, XSS guard, header preview smoke, keyboard regression and toolbar regression PASS; console errors 0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Drag and drop</x:v>
+        <x:v>Required tools</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Sidebar and inspector file drops add Your Media only; canvas file drop adds media and layer; internal icon, shape and text placement PASS</x:v>
+        <x:v>Preview, Preflight, Export PDF, Checkout and Save remain available</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Shortcuts</x:v>
+        <x:v>Removed tools</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Button below Layers, searchable dialog, ? opens, Esc closes, Zoom search PASS</x:v>
+        <x:v>Presentation view, Comments, Notifications, More actions and Share</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>Scope</x:v>
+        <x:v>Preview</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>PNG/JPEG/WebP/GIF only, maximum 5 MB; duplicate media source is reused</x:v>
+        <x:v>Shared CanvasPreview renderer, Front/Back tabs, Esc close, desktop/mobile containment PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -9329,7 +9367,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>E2E-218</x:v>
+        <x:v>E2E-219</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -9345,7 +9383,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>.codex-work/editor-v2-drag-drop-shortcuts-smoke.cjs; build; XSS guard; keyboard and toolbar regression output</x:v>
+        <x:v>output/playwright/header-preview-desktop.png; output/playwright/header-preview-mobile.png; browser/build/XSS regression outputs</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(editor): align card rulers and add grid controls
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra4e9605f48434b3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R3e4ac036c5264a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rbfbd33e4ae2542e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R6972359b211f4526"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9273,6 +9273,44 @@
         <x:v>No backend or collaboration feature added; Preview reuses CanvasPreview and no secret or personal data is stored.</x:v>
       </x:c>
     </x:row>
+    <x:row r="200" ht="112" customHeight="1">
+      <x:c r="A200" s="7" t="str">
+        <x:v>E2E-220</x:v>
+      </x:c>
+      <x:c r="B200" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C200" s="7" t="str">
+        <x:v>Card-aligned rulers, grid toggle and offline status</x:v>
+      </x:c>
+      <x:c r="D200" s="7" t="str">
+        <x:v>Open /editor/15 at 1440x900, zoom 100% and 200%, pan via Zoom to selection, toggle grid and rulers, then retest at 390x844 and with Vizi backend on port 18080.</x:v>
+      </x:c>
+      <x:c r="E200" s="7" t="str">
+        <x:v>Header center stays centered; rulers align to the transformed card at each zoom/pan state; 5 mm grid is clipped to the card; ruler toggle hides rulers; narrow viewport remains within document width; network failure does not expose raw fetch error.</x:v>
+      </x:c>
+      <x:c r="F200" s="7" t="str">
+        <x:v>PASS: dynamic top/left card rulers align at 100% and 200% after zoom/pan; grid appears and is card-clipped; ruler visibility toggles; desktop/mobile geometry and console checks pass; backend health HTTP 200 on 18080; real localhost smoke PASS.</x:v>
+      </x:c>
+      <x:c r="G200" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H200" s="7" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I200" s="7" t="str">
+        <x:v>Playwright ruler-grid smoke, backend health check, frontend HTTP check, build, XSS guard, keyboard/header/toolbar regressions</x:v>
+      </x:c>
+      <x:c r="J200" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K200" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L200" s="7" t="str">
+        <x:v>8080 was occupied by an unrelated Express service; no service was stopped and no secret or personal data was recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9311,7 +9349,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Editor V2 compact header and functional Front/Back preview</x:v>
+        <x:v>Editor V2 card-aligned rulers, grid toggle and runtime alignment</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
@@ -9319,7 +9357,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5175/editor/15</x:v>
+        <x:v>http://127.0.0.1:5176/editor/15</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
@@ -9327,7 +9365,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>No backend change; collaboration-only controls intentionally removed</x:v>
+        <x:v>http://127.0.0.1:18080/api/health returned HTTP 200</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -9335,31 +9373,31 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Build, XSS guard, header preview smoke, keyboard regression and toolbar regression PASS; console errors 0</x:v>
+        <x:v>Build, XSS guard, ruler/grid smoke, backend health and real localhost smoke PASS; console errors 0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Required tools</x:v>
+        <x:v>Rulers</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Preview, Preflight, Export PDF, Checkout and Save remain available</x:v>
+        <x:v>Top/left rulers follow card bounds through zoom and pan; 5 mm ticks; hidden below narrow mobile breakpoint</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Removed tools</x:v>
+        <x:v>Grid</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Presentation view, Comments, Notifications, More actions and Share</x:v>
+        <x:v>Optional 5 mm card-clipped grid with major/minor lines; toggle in centered header</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>Preview</x:v>
+        <x:v>Runtime</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>Shared CanvasPreview renderer, Front/Back tabs, Esc close, desktop/mobile containment PASS</x:v>
+        <x:v>8080 Express conflict isolated; Vizi runs FE5176 to BE18080 without changing tracked env files</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -9367,7 +9405,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>E2E-219</x:v>
+        <x:v>E2E-220</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -9375,7 +9413,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>None after final browser retest</x:v>
+        <x:v>None after final browser and runtime retest</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -9383,7 +9421,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>output/playwright/header-preview-desktop.png; output/playwright/header-preview-mobile.png; browser/build/XSS regression outputs</x:v>
+        <x:v>output/playwright/ruler-grid-desktop.png; output/playwright/ruler-grid-mobile.png; backend health; frontend HTTP; build/XSS/regression outputs</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(editor): center floating canvas toolbar
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rbfbd33e4ae2542e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R6972359b211f4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Re55942b42f6a4201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R83fdc87d85034f23"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9311,6 +9311,44 @@
         <x:v>8080 was occupied by an unrelated Express service; no service was stopped and no secret or personal data was recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="201" ht="104" customHeight="1">
+      <x:c r="A201" s="7" t="str">
+        <x:v>E2E-221</x:v>
+      </x:c>
+      <x:c r="B201" s="7" t="str">
+        <x:v>Editor V2</x:v>
+      </x:c>
+      <x:c r="C201" s="7" t="str">
+        <x:v>Floating canvas toolbar sizing and icon alignment</x:v>
+      </x:c>
+      <x:c r="D201" s="7" t="str">
+        <x:v>Open /editor/canvas-toolbar-size at 1440x900; measure the toolbar and all seven tool buttons; run toolbar and ruler/grid regressions, then retest at 390x844.</x:v>
+      </x:c>
+      <x:c r="E201" s="7" t="str">
+        <x:v>Every tool button is square and shares the toolbar center line; no button overflows the 34 px rail; the toolbar is compact without changing tool behavior or responsive containment.</x:v>
+      </x:c>
+      <x:c r="F201" s="7" t="str">
+        <x:v>PASS: all button center offsets are 0 px; seven buttons are 28 x 28 px; rail is 34 x 225 px with 2 px gap and 4 px/2 px padding; desktop/mobile regressions and browser error checks pass.</x:v>
+      </x:c>
+      <x:c r="G201" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H201" s="7" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I201" s="7" t="str">
+        <x:v>Geometry smoke + visual screenshot + toolbar regression + ruler/grid regression + build + XSS guard</x:v>
+      </x:c>
+      <x:c r="J201" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K201" s="7" t="str">
+        <x:v>localhost FE5176</x:v>
+      </x:c>
+      <x:c r="L201" s="7" t="str">
+        <x:v>CSS-only sizing correction; no backend, data contract, secret, or personal information change.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9349,7 +9387,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Editor V2 card-aligned rulers, grid toggle and runtime alignment</x:v>
+        <x:v>Editor V2 floating canvas toolbar sizing and icon alignment</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
@@ -9357,7 +9395,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/editor/15</x:v>
+        <x:v>http://127.0.0.1:5176/editor/canvas-toolbar-size</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
@@ -9365,7 +9403,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>http://127.0.0.1:18080/api/health returned HTTP 200</x:v>
+        <x:v>No backend change</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -9373,31 +9411,31 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Build, XSS guard, ruler/grid smoke, backend health and real localhost smoke PASS; console errors 0</x:v>
+        <x:v>Build, XSS guard, geometry smoke, toolbar regression and ruler/grid regression PASS; console/page/server errors 0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Rulers</x:v>
+        <x:v>Geometry</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Top/left rulers follow card bounds through zoom and pan; 5 mm ticks; hidden below narrow mobile breakpoint</x:v>
+        <x:v>Rail 34 x 225 px; buttons 28 x 28 px; center offset 0 px</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Grid</x:v>
+        <x:v>Spacing</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Optional 5 mm card-clipped grid with major/minor lines; toggle in centered header</x:v>
+        <x:v>2 px row gap; 4 px vertical and 2 px horizontal rail padding</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>Runtime</x:v>
+        <x:v>Responsive</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>8080 Express conflict isolated; Vizi runs FE5176 to BE18080 without changing tracked env files</x:v>
+        <x:v>Desktop and 390 x 844 mobile containment PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -9405,7 +9443,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>E2E-220</x:v>
+        <x:v>E2E-221</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -9413,7 +9451,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>None after final browser and runtime retest</x:v>
+        <x:v>None after final browser retest</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -9421,7 +9459,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>output/playwright/ruler-grid-desktop.png; output/playwright/ruler-grid-mobile.png; backend health; frontend HTTP; build/XSS/regression outputs</x:v>
+        <x:v>.codex-work/editor-v2-canvas-toolbar-size-before.png; geometry/browser/build/XSS regression outputs</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(designs): add card size creation dialog
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Re55942b42f6a4201"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R83fdc87d85034f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R3deda908e42d4b87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rde50e4c61ff14160"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9349,6 +9349,44 @@
         <x:v>CSS-only sizing correction; no backend, data contract, secret, or personal information change.</x:v>
       </x:c>
     </x:row>
+    <x:row r="202" ht="112" customHeight="1">
+      <x:c r="A202" s="7" t="str">
+        <x:v>E2E-222</x:v>
+      </x:c>
+      <x:c r="B202" s="7" t="str">
+        <x:v>Templates / My drafts</x:v>
+      </x:c>
+      <x:c r="C202" s="7" t="str">
+        <x:v>Start a design with standard or custom card size</x:v>
+      </x:c>
+      <x:c r="D202" s="7" t="str">
+        <x:v>Open /templates and /designs; click Start a design; inspect nine presets and Custom; enter invalid 5 mm then valid 87.5 x 52.5 mm; close with Escape; repeat at 390 x 844.</x:v>
+      </x:c>
+      <x:c r="E202" s="7" t="str">
+        <x:v>Both pages expose Start a design; modal uses millimetres, supports Vietnam/US/Europe/Asia/ISO/square/mini/folded presets and Custom; invalid size blocks creation; valid size enables it; desktop/mobile remain contained.</x:v>
+      </x:c>
+      <x:c r="F202" s="7" t="str">
+        <x:v>PASS: frontend production build passed; browser smoke found ten size choices, invalid custom width disabled Create, valid custom dimensions enabled Create, Escape closed the modal, and desktop/mobile geometry passed.</x:v>
+      </x:c>
+      <x:c r="G202" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H202" s="7" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I202" s="7" t="str">
+        <x:v>Frontend build + Playwright behavior smoke + desktop/mobile screenshots + git diff check</x:v>
+      </x:c>
+      <x:c r="J202" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K202" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L202" s="7" t="str">
+        <x:v>Uses existing authenticated blank-design API and its 10-200 mm validation; no backend, secret, or personal-data change.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9387,7 +9425,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Editor V2 floating canvas toolbar sizing and icon alignment</x:v>
+        <x:v>Start a design from Templates and My drafts</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
@@ -9395,7 +9433,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/editor/canvas-toolbar-size</x:v>
+        <x:v>http://127.0.0.1:5176/templates and /designs</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
@@ -9403,7 +9441,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>No backend change</x:v>
+        <x:v>Existing POST /api/designs contract; no backend change</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -9411,23 +9449,23 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Build, XSS guard, geometry smoke, toolbar regression and ruler/grid regression PASS; console/page/server errors 0</x:v>
+        <x:v>Production build and browser behavior/geometry smoke PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Geometry</x:v>
+        <x:v>Presets</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Rail 34 x 225 px; buttons 28 x 28 px; center offset 0 px</x:v>
+        <x:v>Vietnam 90 x 54, Vietnam 90 x 50, US, Europe, Asia, ISO ID-1, square, mini and folded card</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Spacing</x:v>
+        <x:v>Custom</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>2 px row gap; 4 px vertical and 2 px horizontal rail padding</x:v>
+        <x:v>10-200 mm per side; invalid values disable Create</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -9435,7 +9473,7 @@
         <x:v>Responsive</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>Desktop and 390 x 844 mobile containment PASS</x:v>
+        <x:v>Desktop 1440 x 1000 and mobile 390 x 844 containment PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -9443,7 +9481,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>E2E-221</x:v>
+        <x:v>E2E-222</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -9451,7 +9489,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>None after final browser retest</x:v>
+        <x:v>None after final build and browser retest</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -9459,7 +9497,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>.codex-work/editor-v2-canvas-toolbar-size-before.png; geometry/browser/build/XSS regression outputs</x:v>
+        <x:v>output/start-design-desktop.png; output/start-design-mobile.png; frontend production build</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(order): add paper catalog and exact quantities
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R3deda908e42d4b87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rde50e4c61ff14160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R791ad533ed124487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Ra5475a0201e54761"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9387,6 +9387,44 @@
         <x:v>Uses existing authenticated blank-design API and its 10-200 mm validation; no backend, secret, or personal-data change.</x:v>
       </x:c>
     </x:row>
+    <x:row r="203" ht="96" customHeight="1">
+      <x:c r="A203" s="7" t="str">
+        <x:v>E2E-223</x:v>
+      </x:c>
+      <x:c r="B203" s="7" t="str">
+        <x:v>Checkout / Admin</x:v>
+      </x:c>
+      <x:c r="C203" s="7" t="str">
+        <x:v>Paper catalog, stock status and exact quantity</x:v>
+      </x:c>
+      <x:c r="D203" s="7" t="str">
+        <x:v>Open admin paper stock and checkout with mocked authenticated API data</x:v>
+      </x:c>
+      <x:c r="E203" s="7" t="str">
+        <x:v>Admin can create/edit/delete paper types and mark them in or out of stock; checkout accepts any whole quantity and disables unavailable paper.</x:v>
+      </x:c>
+      <x:c r="F203" s="7" t="str">
+        <x:v>Paper catalog is server-backed with seven seeded types; admin update sends the selected status; checkout accepts 137 cards and calculates the exact prorated estimate.</x:v>
+      </x:c>
+      <x:c r="G203" s="7" t="str">
+        <x:v>Targeted backend tests 12/12 PASS; frontend build PASS; Playwright admin/checkout smoke PASS; migration schema/index/seed assertions PASS; no browser console errors.</x:v>
+      </x:c>
+      <x:c r="H203" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I203" s="7" t="str">
+        <x:v>Spring Boot integration tests + Flyway migration test + Playwright browser smoke + responsive screenshots</x:v>
+      </x:c>
+      <x:c r="J203" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K203" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L203" s="7" t="str">
+        <x:v>Prices and availability are read from the backend; no secret, token or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9425,7 +9463,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Start a design from Templates and My drafts</x:v>
+        <x:v>Paper catalog CRUD, stock availability and arbitrary checkout quantity</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
@@ -9433,7 +9471,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/templates and /designs</x:v>
+        <x:v>http://127.0.0.1:5176/admin and /checkout/15</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
@@ -9441,7 +9479,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Existing POST /api/designs contract; no backend change</x:v>
+        <x:v>Spring Boot http://127.0.0.1:18080; Flyway V5 paper_stocks</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -9449,55 +9487,55 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Production build and browser behavior/geometry smoke PASS</x:v>
+        <x:v>Frontend build, targeted backend tests, migration assertions and browser smoke PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Presets</x:v>
+        <x:v>Paper catalog</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Vietnam 90 x 54, Vietnam 90 x 50, US, Europe, Asia, ISO ID-1, square, mini and folded card</x:v>
+        <x:v>Seven seeded types; admin edit changed IN_STOCK to OUT_OF_STOCK; checkout disabled unavailable option</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Custom</x:v>
+        <x:v>Quantity</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>10-200 mm per side; invalid values disable Create</x:v>
+        <x:v>Numeric input accepts exact whole quantity 137; estimate prorated from price per 100</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>Responsive</x:v>
+        <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>Desktop 1440 x 1000 and mobile 390 x 844 containment PASS</x:v>
+        <x:v>E2E-223</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="7" t="str">
-        <x:v>Retest PASS</x:v>
+        <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>E2E-222</x:v>
+        <x:v>None after final build and browser retest</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" s="7" t="str">
-        <x:v>Retest FAIL</x:v>
+        <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>None after final build and browser retest</x:v>
+        <x:v>output/paper-admin.png; output/paper-checkout.png; backend test output; browser smoke</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="7" t="str">
-        <x:v>Evidence</x:v>
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>output/start-design-desktop.png; output/start-design-mobile.png; frontend production build</x:v>
+        <x:v>No secrets or personal data recorded; native print workflow is phase 3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(admin): add print imposition workflow
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R791ad533ed124487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Ra5475a0201e54761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Reeeb405d3c0444f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R4b862793237e4c7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9425,6 +9425,44 @@
         <x:v>Prices and availability are read from the backend; no secret, token or personal data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="204" ht="108" customHeight="1">
+      <x:c r="A204" s="7" t="str">
+        <x:v>E2E-224</x:v>
+      </x:c>
+      <x:c r="B204" s="7" t="str">
+        <x:v>Admin / Print</x:v>
+      </x:c>
+      <x:c r="C204" s="7" t="str">
+        <x:v>Order and template card imposition</x:v>
+      </x:c>
+      <x:c r="D204" s="7" t="str">
+        <x:v>Open Admin Print, choose an order snapshot or saved template, select side and A-series paper, then print.</x:v>
+      </x:c>
+      <x:c r="E204" s="7" t="str">
+        <x:v>Admin can use the frozen order snapshot or a saved template, choose Front/Back and A0-A4, enter an exact template quantity, and get a non-clipped imposed layout.</x:v>
+      </x:c>
+      <x:c r="F204" s="7" t="str">
+        <x:v>Order quantity 137 at 90 x 54 mm calculates A4 as 6 cards per sheet and 23 sheets; A3 recalculates to 16 cards per sheet and 9 sheets; template quantity 137 and browser print action also pass.</x:v>
+      </x:c>
+      <x:c r="G204" s="7" t="str">
+        <x:v>OrderApiIntegrationTests 7/7 PASS; full backend 103/103; frontend build PASS; Playwright order/template print smoke PASS; A4/A3 placement and responsive assertions PASS.</x:v>
+      </x:c>
+      <x:c r="H204" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I204" s="7" t="str">
+        <x:v>Backend JSON response + pure imposition calculation + Playwright browser smoke + responsive screenshots</x:v>
+      </x:c>
+      <x:c r="J204" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K204" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L204" s="7" t="str">
+        <x:v>Order snapshot is used for production; native print dialog remains controlled by the browser/printer; no secret or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9450,7 +9488,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2" ht="38" customHeight="1">
+    <x:row r="2" ht="40" customHeight="1">
       <x:c r="A2" s="7" t="str">
         <x:v>Date</x:v>
       </x:c>
@@ -9458,84 +9496,84 @@
         <x:v>2026-07-18</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="38" customHeight="1">
+    <x:row r="3" ht="40" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Paper catalog CRUD, stock availability and arbitrary checkout quantity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="38" customHeight="1">
+        <x:v>Admin printing from order snapshot or saved template with A0-A4 imposition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="40" customHeight="1">
       <x:c r="A4" s="7" t="str">
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/admin and /checkout/15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="38" customHeight="1">
+        <x:v>http://127.0.0.1:5176/admin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="40" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Spring Boot http://127.0.0.1:18080; Flyway V5 paper_stocks</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="38" customHeight="1">
+        <x:v>Spring Boot http://127.0.0.1:18080; order items expose snapshot and card geometry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="40" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Frontend build, targeted backend tests, migration assertions and browser smoke PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="38" customHeight="1">
+        <x:v>Frontend build, full backend tests and browser print smoke PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="40" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Paper catalog</x:v>
+        <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Seven seeded types; admin edit changed IN_STOCK to OUT_OF_STOCK; checkout disabled unavailable option</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="38" customHeight="1">
+        <x:v>Order snapshot is immutable for production; saved template is available for reusable samples</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="40" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Quantity</x:v>
+        <x:v>Imposition</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Numeric input accepts exact whole quantity 137; estimate prorated from price per 100</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="38" customHeight="1">
+        <x:v>2mm bleed, 4mm gutter, 10mm margin; A4 90x54 = 6 cards/sheet; 137 = 23 sheets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="40" customHeight="1">
       <x:c r="A9" s="7" t="str">
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-223</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="38" customHeight="1">
+        <x:v>E2E-224</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="40" customHeight="1">
       <x:c r="A10" s="7" t="str">
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>None after final build and browser retest</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="38" customHeight="1">
+        <x:v>None after final build, backend and browser retest</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
       <x:c r="A11" s="7" t="str">
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>output/paper-admin.png; output/paper-checkout.png; backend test output; browser smoke</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="38" customHeight="1">
+        <x:v>output/admin-print.png; output/admin-print-mobile.png; backend test output; browser smoke</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
       <x:c r="A12" s="7" t="str">
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>No secrets or personal data recorded; native print workflow is phase 3</x:v>
+        <x:v>No secrets or personal data recorded; OS printer selection remains browser-controlled</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(admin): add duplex print registration
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Reeeb405d3c0444f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R4b862793237e4c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra0d3cc4fda864751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R1c4619170db443ea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9463,6 +9463,44 @@
         <x:v>Order snapshot is used for production; native print dialog remains controlled by the browser/printer; no secret or personal data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="205" ht="108" customHeight="1">
+      <x:c r="A205" s="7" t="str">
+        <x:v>E2E-225</x:v>
+      </x:c>
+      <x:c r="B205" s="7" t="str">
+        <x:v>Admin / Print</x:v>
+      </x:c>
+      <x:c r="C205" s="7" t="str">
+        <x:v>Duplex imposition with crop marks</x:v>
+      </x:c>
+      <x:c r="D205" s="7" t="str">
+        <x:v>Open Admin Print, choose an order snapshot or saved template, select Front + Back, test each back-alignment mode and crop marks, then print.</x:v>
+      </x:c>
+      <x:c r="E205" s="7" t="str">
+        <x:v>Admin can prepare Front, Back or paired duplex sheets; mirror the back for long-edge or short-edge feed; keep the exact quantity; and optionally include four crop-mark corners per card.</x:v>
+      </x:c>
+      <x:c r="F205" s="7" t="str">
+        <x:v>Order quantity 137 at 90 x 54 mm calculates A4 as 6 cards per sheet, 23 physical sheets and 46 printed sides. Front and Back are paired, X/Y/same alignment passes, crop marks toggle passes, and print output contains no site navigation.</x:v>
+      </x:c>
+      <x:c r="G205" s="7" t="str">
+        <x:v>Frontend build and XSS guard PASS; full backend 103/103 PASS; Playwright duplex print smoke PASS across A0-A4, long/short/same alignment, crop marks, print media, laptop and mobile.</x:v>
+      </x:c>
+      <x:c r="H205" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I205" s="7" t="str">
+        <x:v>Typecheck/build + XSS guard + full backend suite + Playwright duplex/print-media assertions + visual screenshots</x:v>
+      </x:c>
+      <x:c r="J205" s="7" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K205" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L205" s="7" t="str">
+        <x:v>Duplex alignment controls sheet placement only; printer driver settings still need to match the selected feed edge. Native print dialog remains browser/printer controlled; no secret or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9501,7 +9539,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Admin printing from order snapshot or saved template with A0-A4 imposition</x:v>
+        <x:v>Admin duplex printing with paired Front/Back sheets, back reflection and crop marks</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9525,7 +9563,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Frontend build, full backend tests and browser print smoke PASS</x:v>
+        <x:v>Frontend build, XSS guard, full backend 103/103 and duplex browser print smoke PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9541,7 +9579,7 @@
         <x:v>Imposition</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>2mm bleed, 4mm gutter, 10mm margin; A4 90x54 = 6 cards/sheet; 137 = 23 sheets</x:v>
+        <x:v>2mm bleed, 4mm gutter, 10mm margin; A4 90x54 = 6 cards/sheet; 137 = 23 physical sheets / 46 printed sides</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9549,7 +9587,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-224</x:v>
+        <x:v>E2E-225</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9565,7 +9603,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>output/admin-print.png; output/admin-print-mobile.png; backend test output; browser smoke</x:v>
+        <x:v>output/admin-print-duplex.png; output/admin-print-duplex-sheet.png; output/admin-print-duplex-mobile.png; browser and backend test output</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9573,7 +9611,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>No secrets or personal data recorded; OS printer selection remains browser-controlled</x:v>
+        <x:v>No secrets or personal data recorded; printer feed edge and OS print dialog remain operator-controlled</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(auth): record local login transport verification
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Ra0d3cc4fda864751"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R1c4619170db443ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rcd981e2092d84223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rdf094ab75b844b3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9501,6 +9501,42 @@
         <x:v>Duplex alignment controls sheet placement only; printer driver settings still need to match the selected feed edge. Native print dialog remains browser/printer controlled; no secret or personal data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="206">
+      <x:c r="A206" t="str">
+        <x:v>E2E-226</x:v>
+      </x:c>
+      <x:c r="B206" t="str">
+        <x:v>Account / Auth</x:v>
+      </x:c>
+      <x:c r="C206" t="str">
+        <x:v>Local login transport and CORS</x:v>
+      </x:c>
+      <x:c r="D206" t="str">
+        <x:v>Open /account at FE 5176 and submit synthetic invalid credentials; inspect auth request URLs, CORS preflight and CSRF response.</x:v>
+      </x:c>
+      <x:c r="E206" t="str">
+        <x:v>Frontend calls the Vizi backend at 18080; localhost and 127.0.0.1 origins pass CORS; CSRF is available; invalid credentials return a normal 401 message rather than Failed to fetch.</x:v>
+      </x:c>
+      <x:c r="F206" t="str">
+        <x:v>Auth requests use 18080; preflight returns 200 with the requesting origin and credentials enabled; CSRF returns 200; synthetic login returns 401; UI shows Email or password is incorrect and not Failed to fetch.</x:v>
+      </x:c>
+      <x:c r="G206" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H206"/>
+      <x:c r="I206" t="str">
+        <x:v>Browser network smoke + direct CORS preflight/CSRF checks + frontend production build</x:v>
+      </x:c>
+      <x:c r="J206" t="str">
+        <x:v>2026-07-18</x:v>
+      </x:c>
+      <x:c r="K206" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L206" t="str">
+        <x:v>No real credentials logged; local-only .env and startup settings remain ignored; no secret or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9539,7 +9575,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Admin duplex printing with paired Front/Back sheets, back reflection and crop marks</x:v>
+        <x:v>Local account login transport and CORS</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9547,7 +9583,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/admin</x:v>
+        <x:v>http://127.0.0.1:5176/account</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -9555,7 +9591,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Spring Boot http://127.0.0.1:18080; order items expose snapshot and card geometry</x:v>
+        <x:v>Spring Boot http://127.0.0.1:18080; CSRF and CORS verified</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9563,7 +9599,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Frontend build, XSS guard, full backend 103/103 and duplex browser print smoke PASS</x:v>
+        <x:v>Frontend build, CORS preflight, CSRF and synthetic invalid-login smoke PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9571,7 +9607,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Order snapshot is immutable for production; saved template is available for reusable samples</x:v>
+        <x:v>No production data changed; local runtime points to the existing Vizi backend</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
@@ -9579,7 +9615,7 @@
         <x:v>Imposition</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>2mm bleed, 4mm gutter, 10mm margin; A4 90x54 = 6 cards/sheet; 137 = 23 physical sheets / 46 printed sides</x:v>
+        <x:v>E2E-226</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9587,7 +9623,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-225</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9595,7 +9631,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>None after final build, backend and browser retest</x:v>
+        <x:v>Browser auth network smoke + direct preflight/CSRF checks + npm build</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" customHeight="1">
@@ -9603,7 +9639,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>output/admin-print-duplex.png; output/admin-print-duplex-sheet.png; output/admin-print-duplex-mobile.png; browser and backend test output</x:v>
+        <x:v>No real credentials logged; local-only settings are ignored; no secret or personal data recorded</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9611,7 +9647,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>No secrets or personal data recorded; printer feed edge and OS print dialog remain operator-controlled</x:v>
+        <x:v>Local transport fix only; real account verification remains manual because credentials are not handled by the test harness</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(data): record local dataset reset verification
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="Rcd981e2092d84223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rdf094ab75b844b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R8eb25675128c4039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R481c30af195f4634"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9537,6 +9537,42 @@
         <x:v>No real credentials logged; local-only .env and startup settings remain ignored; no secret or personal data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="207">
+      <x:c r="A207" t="str">
+        <x:v>E2E-227</x:v>
+      </x:c>
+      <x:c r="B207" t="str">
+        <x:v>Local data reset</x:v>
+      </x:c>
+      <x:c r="C207" t="str">
+        <x:v>Local reset and sample admin access</x:v>
+      </x:c>
+      <x:c r="D207" t="str">
+        <x:v>Run the local reset flow, open the local account page, and sign in with each of the three local sample fixtures.</x:v>
+      </x:c>
+      <x:c r="E207" t="str">
+        <x:v>Only the local PostgreSQL dataset is reset; card data is empty, paper stock catalog remains available, and each sample fixture is ADMIN.</x:v>
+      </x:c>
+      <x:c r="F207" t="str">
+        <x:v>Database readback: users=3, templates/designs/snapshots/assets/orders/order_items/AI logs=0, paper_stocks=7. Browser login smoke returned HTTP 200 and ADMIN for all three local fixtures. FE /account=200 and BE /api/health=200.</x:v>
+      </x:c>
+      <x:c r="G207" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H207"/>
+      <x:c r="I207" t="str">
+        <x:v>PostgreSQL readback + Playwright login/API smoke + frontend/backend HTTP health</x:v>
+      </x:c>
+      <x:c r="J207" t="str">
+        <x:v>2026-07-19</x:v>
+      </x:c>
+      <x:c r="K207" t="str">
+        <x:v>localhost FE5176 / BE18080 / PostgreSQL55432</x:v>
+      </x:c>
+      <x:c r="L207" t="str">
+        <x:v>No passwords, tokens, or personal account identifiers recorded; cloud datasource untouched.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9575,7 +9611,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Local account login transport and CORS</x:v>
+        <x:v>Local data reset and sample admin access</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9591,7 +9627,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Spring Boot http://127.0.0.1:18080; CSRF and CORS verified</x:v>
+        <x:v>Local PostgreSQL 127.0.0.1:55432/vizi; backend 18080</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9599,7 +9635,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Frontend build, CORS preflight, CSRF and synthetic invalid-login smoke PASS</x:v>
+        <x:v>Database reset, 3 admin login smoke, FE/BE health checks PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9607,7 +9643,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>No production data changed; local runtime points to the existing Vizi backend</x:v>
+        <x:v>Card data tables cleared; paper_stocks preserved (7 rows)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
@@ -9615,7 +9651,7 @@
         <x:v>Imposition</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>E2E-226</x:v>
+        <x:v>E2E-227</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9631,7 +9667,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>Browser auth network smoke + direct preflight/CSRF checks + npm build</x:v>
+        <x:v>PostgreSQL readback + browser login/API smoke + FE/BE HTTP health</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" customHeight="1">
@@ -9639,7 +9675,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>No real credentials logged; local-only settings are ignored; no secret or personal data recorded</x:v>
+        <x:v>No passwords, tokens, or personal account identifiers recorded</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9647,7 +9683,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Local transport fix only; real account verification remains manual because credentials are not handled by the test harness</x:v>
+        <x:v>Local-only reset; cloud datasource untouched</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Persist authentication sessions and revoke on password change
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R8eb25675128c4039"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R481c30af195f4634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R415fb79850af4df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Redf8945c3e34442e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -80,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
@@ -116,6 +116,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -9573,6 +9576,44 @@
         <x:v>No passwords, tokens, or personal account identifiers recorded; cloud datasource untouched.</x:v>
       </x:c>
     </x:row>
+    <x:row r="208" ht="96" customHeight="1">
+      <x:c r="A208" s="14" t="str">
+        <x:v>E2E-228</x:v>
+      </x:c>
+      <x:c r="B208" s="14" t="str">
+        <x:v>Account / Auth</x:v>
+      </x:c>
+      <x:c r="C208" s="14" t="str">
+        <x:v>Persistent login session and password-change revocation</x:v>
+      </x:c>
+      <x:c r="D208" s="14" t="str">
+        <x:v>Run focused auth/migration/security tests and the full backend suite; build the frontend; start the packaged backend, log in, record the SESSION cookie attributes, restart the backend, then call /api/auth/me with the existing cookie.</x:v>
+      </x:c>
+      <x:c r="E208" s="14" t="str">
+        <x:v>Login rotates the session ID; SESSION lasts 30 days with HttpOnly and SameSite=Lax; JDBC session survives backend restart; changing a password revokes every session and requires sign-in with the new password.</x:v>
+      </x:c>
+      <x:c r="F208" s="14" t="str">
+        <x:v>Focused tests 19/19 PASS; full backend 108/108 PASS; frontend production build PASS; packaged runtime smoke completed in 16.5 s with login 204, rotated session, 30-day cookie attributes and /api/auth/me 200 after restart.</x:v>
+      </x:c>
+      <x:c r="G208" s="14" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H208" s="14" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I208" s="14" t="str">
+        <x:v>Spring MockMvc + Flyway migration + frontend production build + packaged runtime HTTP restart smoke</x:v>
+      </x:c>
+      <x:c r="J208" s="14" t="str">
+        <x:v>2026-07-19</x:v>
+      </x:c>
+      <x:c r="K208" s="14" t="str">
+        <x:v>localhost FE5176 / BE18080 / smoke18082 / PostgreSQL55432</x:v>
+      </x:c>
+      <x:c r="L208" s="14" t="str">
+        <x:v>Password-change tests revoked all sessions and rejected the old password. No passwords, session IDs, cookie values or personal account identifiers recorded; runtime smoke defaults to read-only.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9603,7 +9644,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>2026-07-18</x:v>
+        <x:v>2026-07-19</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="40" customHeight="1">
@@ -9611,7 +9652,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Local data reset and sample admin access</x:v>
+        <x:v>Persistent login session and password-change revocation</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9627,7 +9668,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Local PostgreSQL 127.0.0.1:55432/vizi; backend 18080</x:v>
+        <x:v>Local PostgreSQL 127.0.0.1:55432/vizi; backend 18080; packaged smoke 18082</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9635,7 +9676,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Database reset, 3 admin login smoke, FE/BE health checks PASS</x:v>
+        <x:v>Focused backend 19/19, full backend 108/108, frontend build and packaged restart smoke PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9643,15 +9684,15 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Card data tables cleared; paper_stocks preserved (7 rows)</x:v>
+        <x:v>Spring Session JDBC migration V6; 30-day SESSION cookie; session fixation rotation</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Imposition</x:v>
+        <x:v>Test case</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>E2E-227</x:v>
+        <x:v>E2E-228</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9659,7 +9700,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>None</x:v>
+        <x:v>E2E-228</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9667,7 +9708,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>PostgreSQL readback + browser login/API smoke + FE/BE HTTP health</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" customHeight="1">
@@ -9675,7 +9716,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>No passwords, tokens, or personal account identifiers recorded</x:v>
+        <x:v>No passwords, tokens, session IDs, cookie values or personal account identifiers recorded</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9683,7 +9724,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Local-only reset; cloud datasource untouched</x:v>
+        <x:v>Local auth/session verification; cloud datasource untouched</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(editor): migrate legacy templates into editor v2
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R415fb79850af4df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Redf8945c3e34442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R37a7f0970e254679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R281788bf47cd4979"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9614,6 +9614,44 @@
         <x:v>Password-change tests revoked all sessions and rejected the old password. No passwords, session IDs, cookie values or personal account identifiers recorded; runtime smoke defaults to read-only.</x:v>
       </x:c>
     </x:row>
+    <x:row r="209" ht="108" customHeight="1">
+      <x:c r="A209" s="7" t="str">
+        <x:v>E2E-229</x:v>
+      </x:c>
+      <x:c r="B209" s="7" t="str">
+        <x:v>Templates / Editor V2</x:v>
+      </x:c>
+      <x:c r="C209" s="7" t="str">
+        <x:v>Legacy template canvas migration</x:v>
+      </x:c>
+      <x:c r="D209" s="7" t="str">
+        <x:v>Open each template from /templates, choose Save draft -&gt; Open editor; inspect Front and Back, then reload once with a cached local edit while the remote JSON remains legacy.</x:v>
+      </x:c>
+      <x:c r="E209" s="7" t="str">
+        <x:v>Every legacy layers[] template opens with its own content in Editor V2 schemaVersion 2, fixed Front/Back pages, correct card dimensions, and no starter V2 content; a cached local edit is preserved.</x:v>
+      </x:c>
+      <x:c r="F209" s="7" t="str">
+        <x:v>Frontend build PASS; mock template-to-editor regression PASS; all 7 live templates PASS (0-12 Front layers, 0-2 Back layers); draft persistence, cutover and live backend E2E PASS; no console/page/server errors; temporary live draft cleaned.</x:v>
+      </x:c>
+      <x:c r="G209" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H209" s="7" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I209" s="7" t="str">
+        <x:v>Browser migration smoke + all-template matrix + frontend build + draft persistence/cutover + live backend E2E</x:v>
+      </x:c>
+      <x:c r="J209" s="7" t="str">
+        <x:v>2026-07-20</x:v>
+      </x:c>
+      <x:c r="K209" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080 / local PostgreSQL</x:v>
+      </x:c>
+      <x:c r="L209" s="7" t="str">
+        <x:v>Backend legacy JSON remains unchanged; migration is client-side and persisted as V2 on save. Existing user drafts are not overwritten automatically; no secret or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9644,7 +9682,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>2026-07-19</x:v>
+        <x:v>2026-07-20</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="40" customHeight="1">
@@ -9652,7 +9690,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Persistent login session and password-change revocation</x:v>
+        <x:v>Legacy template canvas migration into Editor V2 with cached local edit protection</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9660,7 +9698,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/account</x:v>
+        <x:v>http://127.0.0.1:5176/templates</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -9668,7 +9706,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>Local PostgreSQL 127.0.0.1:55432/vizi; backend 18080; packaged smoke 18082</x:v>
+        <x:v>http://127.0.0.1:18080; local PostgreSQL used for live template E2E</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9676,7 +9714,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Focused backend 19/19, full backend 108/108, frontend build and packaged restart smoke PASS</x:v>
+        <x:v>Frontend build, mock migration, all 7 templates, draft persistence, cutover and live E2E PASS; runtime errors=0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9684,7 +9722,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Spring Session JDBC migration V6; 30-day SESSION cookie; session fixation rotation</x:v>
+        <x:v>Legacy layers[] -&gt; Editor V2 schemaVersion 2; fixed Front/Back pages; local cache precedence</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
@@ -9692,7 +9730,7 @@
         <x:v>Test case</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>E2E-228</x:v>
+        <x:v>E2E-229</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9700,7 +9738,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-228</x:v>
+        <x:v>E2E-229</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9716,7 +9754,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>No passwords, tokens, session IDs, cookie values or personal account identifiers recorded</x:v>
+        <x:v>Template migration browser smoke, all-template matrix, persistence/cutover smoke, live backend E2E; temporary draft deleted</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9724,7 +9762,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Local auth/session verification; cloud datasource untouched</x:v>
+        <x:v>Legacy backend JSON is preserved; client migration is saved as V2; no secrets or personal data recorded</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(preview): scale thumbnail canvas content proportionally
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R37a7f0970e254679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R281788bf47cd4979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R40ab84e98e0540a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rc36dd50699f04711"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9652,6 +9652,44 @@
         <x:v>Backend legacy JSON remains unchanged; migration is client-side and persisted as V2 on save. Existing user drafts are not overwritten automatically; no secret or personal data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="210" ht="108" customHeight="1">
+      <x:c r="A210" s="7" t="str">
+        <x:v>E2E-230</x:v>
+      </x:c>
+      <x:c r="B210" s="7" t="str">
+        <x:v>Templates / Drafts</x:v>
+      </x:c>
+      <x:c r="C210" s="7" t="str">
+        <x:v>Thumbnail canvas content scaling</x:v>
+      </x:c>
+      <x:c r="D210" s="7" t="str">
+        <x:v>Open /templates, inspect template IDs 3-7, open a template detail page, and inspect a saved draft thumbnail.</x:v>
+      </x:c>
+      <x:c r="E210" s="7" t="str">
+        <x:v>Thumbnail keeps the 90 x 54 ratio; text and icon layers scale from the canonical preview without clipping; detail preview remains unchanged.</x:v>
+      </x:c>
+      <x:c r="F210" s="7" t="str">
+        <x:v>Thumbnail smoke PASS for all 5 live templates, draft thumbnail and detail preview; frame=260x156; no clipped text layers; no console/page/server errors. Frontend build, editor cutover and checkout preview regression also PASS.</x:v>
+      </x:c>
+      <x:c r="G210" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H210" s="7" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I210" s="7" t="str">
+        <x:v>Browser regression with red-before-fix and green-after-fix evidence + frontend build + related editor/checkout smoke</x:v>
+      </x:c>
+      <x:c r="J210" s="7" t="str">
+        <x:v>2026-07-20</x:v>
+      </x:c>
+      <x:c r="K210" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L210" s="7" t="str">
+        <x:v>CanvasPreview now scales text and icons against the canonical 520 px preview instead of applying a thumbnail-breaking minimum; no secret or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9690,7 +9728,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Legacy template canvas migration into Editor V2 with cached local edit protection</x:v>
+        <x:v>Template and draft thumbnail rendering after canonical canvas scaling fix</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9706,7 +9744,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>http://127.0.0.1:18080; local PostgreSQL used for live template E2E</x:v>
+        <x:v>http://127.0.0.1:18080; live template and draft preview data</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9714,7 +9752,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Frontend build, mock migration, all 7 templates, draft persistence, cutover and live E2E PASS; runtime errors=0</x:v>
+        <x:v>Thumbnail matrix 5/5, draft, detail, editor cutover, checkout preview and frontend build PASS; runtime errors=0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9722,7 +9760,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Legacy layers[] -&gt; Editor V2 schemaVersion 2; fixed Front/Back pages; local cache precedence</x:v>
+        <x:v>Shared CanvasPreview; canonical 520 px reference; proportional text/icon sizing in list thumbnails</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
@@ -9730,7 +9768,7 @@
         <x:v>Test case</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>E2E-229</x:v>
+        <x:v>E2E-230</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9738,7 +9776,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-229</x:v>
+        <x:v>E2E-230</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9746,7 +9784,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>None</x:v>
+        <x:v>None after fix</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" customHeight="1">
@@ -9754,7 +9792,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>Template migration browser smoke, all-template matrix, persistence/cutover smoke, live backend E2E; temporary draft deleted</x:v>
+        <x:v>template-thumbnail-scaling-smoke.cjs; frontend build; editor cutover and checkout preview smoke; rendered workbook readback</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9762,7 +9800,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Legacy backend JSON is preserved; client migration is saved as V2; no secrets or personal data recorded</x:v>
+        <x:v>No secrets or personal data recorded; unrelated pre-existing worktree files were not included</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(auth): allow local frontend CORS on port 5176
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R40ab84e98e0540a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="Rc36dd50699f04711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R1bb0725aeb5449ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R359a25e81ed842ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9690,6 +9690,44 @@
         <x:v>CanvasPreview now scales text and icons against the canonical 520 px preview instead of applying a thumbnail-breaking minimum; no secret or personal data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="211" ht="108" customHeight="1">
+      <x:c r="A211" s="7" t="str">
+        <x:v>E2E-231</x:v>
+      </x:c>
+      <x:c r="B211" s="7" t="str">
+        <x:v>Account / Auth</x:v>
+      </x:c>
+      <x:c r="C211" s="7" t="str">
+        <x:v>Local 5176 CORS and clean-session login</x:v>
+      </x:c>
+      <x:c r="D211" s="7" t="str">
+        <x:v>Open /account from FE 5176 in a clean browser context; request CSRF and login through BE 18080; repeat with the local fixture accounts.</x:v>
+      </x:c>
+      <x:c r="E211" s="7" t="str">
+        <x:v>CORS allows localhost and 127.0.0.1 on port 5176; invalid credentials return a normal 401 instead of Failed to fetch; valid fixture login creates a session without relying on an old cookie.</x:v>
+      </x:c>
+      <x:c r="F211" s="7" t="str">
+        <x:v>Before fix: browser net::ERR_FAILED and direct CSRF returned 403 Invalid CORS request. After fix: CSRF CORS response 200, invalid login 401, all 3 local fixture logins 200 with ADMIN role; no browser network failure. Frontend build and full backend suite also pass.</x:v>
+      </x:c>
+      <x:c r="G211" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="H211" s="7" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="I211" s="7" t="str">
+        <x:v>Playwright network smoke + direct CORS/API check + fixture login smoke + frontend build + full backend test suite</x:v>
+      </x:c>
+      <x:c r="J211" s="7" t="str">
+        <x:v>2026-07-21</x:v>
+      </x:c>
+      <x:c r="K211" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080 / PostgreSQL55432</x:v>
+      </x:c>
+      <x:c r="L211" s="7" t="str">
+        <x:v>Added 5176 localhost origins to the safe CORS default; no password, token, cookie value or personal account data recorded.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9720,7 +9758,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>2026-07-20</x:v>
+        <x:v>2026-07-21</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="40" customHeight="1">
@@ -9728,7 +9766,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Template and draft thumbnail rendering after canonical canvas scaling fix</x:v>
+        <x:v>Local login Failed to fetch caused by missing CORS origins for FE port 5176</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9736,7 +9774,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/templates</x:v>
+        <x:v>http://127.0.0.1:5176/account</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -9744,7 +9782,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>http://127.0.0.1:18080; live template and draft preview data</x:v>
+        <x:v>http://127.0.0.1:18080; local PostgreSQL 127.0.0.1:55432</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9752,7 +9790,7 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Thumbnail matrix 5/5, draft, detail, editor cutover, checkout preview and frontend build PASS; runtime errors=0</x:v>
+        <x:v>CORS/API PASS; invalid login returns normal 401; 3 fixture ADMIN logins PASS; frontend build and backend 108/108 PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
@@ -9760,7 +9798,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>Shared CanvasPreview; canonical 520 px reference; proportional text/icon sizing in list thumbnails</x:v>
+        <x:v>application.properties app.cors.allowed-origins default now includes localhost:5176 and 127.0.0.1:5176</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
@@ -9768,7 +9806,7 @@
         <x:v>Test case</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>E2E-230</x:v>
+        <x:v>E2E-231</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9776,7 +9814,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-230</x:v>
+        <x:v>E2E-231</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9792,7 +9830,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>template-thumbnail-scaling-smoke.cjs; frontend build; editor cutover and checkout preview smoke; rendered workbook readback</x:v>
+        <x:v>login-network-smoke.cjs; direct CSRF/CORS check; local-admin-login-smoke.cjs; npm run build; mvnw test</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9800,7 +9838,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>No secrets or personal data recorded; unrelated pre-existing worktree files were not included</x:v>
+        <x:v>Clean browser context used for login verification; no credentials, tokens or personal data recorded</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: complete commerce and editor workflow updates
</commit_message>
<xml_diff>
--- a/Template_TestCase.xlsx
+++ b/Template_TestCase.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R1bb0725aeb5449ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R359a25e81ed842ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E_Results" sheetId="1" r:id="R60e2a25fe5bf4f41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retest_Summary" sheetId="2" r:id="R6b723fed2d034e21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9728,6 +9728,234 @@
         <x:v>Added 5176 localhost origins to the safe CORS default; no password, token, cookie value or personal account data recorded.</x:v>
       </x:c>
     </x:row>
+    <x:row r="212">
+      <x:c r="A212" t="str">
+        <x:v>E2E-232</x:v>
+      </x:c>
+      <x:c r="B212" t="str">
+        <x:v>Checkout / Preflight</x:v>
+      </x:c>
+      <x:c r="C212" t="str">
+        <x:v>Safe-zone correction for Noir Nocturne</x:v>
+      </x:c>
+      <x:c r="D212" t="str">
+        <x:v>Open draft #7 at 90 x 54 mm; the nn-contact text layer is at Y 48.6 mm with H 3.2 mm.</x:v>
+      </x:c>
+      <x:c r="E212" t="str">
+        <x:v>Move only nn-contact upward so the text remains inside the fixed 3 mm safe zone; save, run preflight in editor and checkout, and verify ordering is enabled.</x:v>
+      </x:c>
+      <x:c r="F212" t="str">
+        <x:v>Y changed from 48.6 mm to 47.5 mm; the draft was saved; the template source was updated to the same normalized coordinate; visual layout was preserved.</x:v>
+      </x:c>
+      <x:c r="G212" t="str">
+        <x:v>Editor and checkout preflight PASS with 0 errors / 3 non-blocking full-bleed warnings; Create order enabled; DB readback passed; browser console had 0 errors; focused backend suite 20/20 PASS.</x:v>
+      </x:c>
+      <x:c r="H212" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I212" t="str">
+        <x:v>P1 - browser UI + PostgreSQL readback + Spring tests</x:v>
+      </x:c>
+      <x:c r="J212" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+      <x:c r="K212" t="str">
+        <x:v>localhost FE5176 / BE18080 / PostgreSQL55432</x:v>
+      </x:c>
+      <x:c r="L212" t="str">
+        <x:v>No order was created. Only draft #7 and template source #3 were adjusted; no credentials, cookies, or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="108" customHeight="1">
+      <x:c r="A213" s="7" t="str">
+        <x:v>E2E-233</x:v>
+      </x:c>
+      <x:c r="B213" s="7" t="str">
+        <x:v>Admin / Print</x:v>
+      </x:c>
+      <x:c r="C213" s="7" t="str">
+        <x:v>Configurable print layout and print modes</x:v>
+      </x:c>
+      <x:c r="D213" s="7" t="str">
+        <x:v>Open Admin Print; choose an order snapshot or saved template; test Front only, Back only and Front + Back; adjust card width/height, bleed, horizontal/vertical gap, sheet margin, paper size and orientation; then print.</x:v>
+      </x:c>
+      <x:c r="E213" s="7" t="str">
+        <x:v>Single-sided modes render only the chosen side. Duplex renders paired Front/Back sheets and exposes back alignment. Every layout value recalculates placement while preserving the exact requested quantity.</x:v>
+      </x:c>
+      <x:c r="F213" s="7" t="str">
+        <x:v>Order quantity 137: default A4 portrait at 90 x 54 mm remains 6 cards/sheet and 23 physical sheets. Custom A4 landscape at 85 x 55 mm, 3 mm bleed, 8 x 12 mm gaps and 15 mm margin recalculates to 4 cards/sheet with 297 x 210 mm sheet geometry. Reset restores design size.</x:v>
+      </x:c>
+      <x:c r="G213" s="7" t="str">
+        <x:v>Frontend build/typecheck PASS; XSS guard PASS; full backend 128/128 PASS; Playwright print smoke PASS for print modes, A0-A4, custom size/spacing/orientation, crop marks, print media, laptop/mobile and zero runtime errors.</x:v>
+      </x:c>
+      <x:c r="H213" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I213" s="7" t="str">
+        <x:v>P1 - Vue build + XSS guard + Spring tests + Playwright DOM geometry/runtime/responsive assertions</x:v>
+      </x:c>
+      <x:c r="J213" s="7" t="str">
+        <x:v>2026-07-22</x:v>
+      </x:c>
+      <x:c r="K213" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L213" s="7" t="str">
+        <x:v>Order and template data were not changed; print settings are local to the admin session. The browser cannot force a printer's hardware duplex mode, so the native print dialog must match the selected feed edge. No secrets or personal data recorded.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="108" customHeight="1">
+      <x:c r="A214" s="7" t="str">
+        <x:v>E2E-234</x:v>
+      </x:c>
+      <x:c r="B214" s="7" t="str">
+        <x:v>Orders / API</x:v>
+      </x:c>
+      <x:c r="C214" s="7" t="str">
+        <x:v>Customer order history is owner-scoped</x:v>
+      </x:c>
+      <x:c r="D214" s="7" t="str">
+        <x:v>Create orders for two users, authenticate as one customer, request GET /api/orders, and compare the returned IDs and order.</x:v>
+      </x:c>
+      <x:c r="E214" s="7" t="str">
+        <x:v>The response contains only the authenticated customer's orders, sorted newest first. Anonymous requests are rejected.</x:v>
+      </x:c>
+      <x:c r="F214" s="7" t="str">
+        <x:v>The authenticated customer received exactly their two orders newest first; another user's order was excluded. A live unauthenticated request returned HTTP 401.</x:v>
+      </x:c>
+      <x:c r="G214" s="7" t="str">
+        <x:v>Focused order API suite 9/9 PASS; full backend suite 129/129 PASS; live HTTP authorization check PASS.</x:v>
+      </x:c>
+      <x:c r="H214" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I214" s="7" t="str">
+        <x:v>P0 - Spring integration tests + live HTTP ownership/authorization check</x:v>
+      </x:c>
+      <x:c r="J214" s="7" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="K214" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L214" s="7" t="str">
+        <x:v>Order lookup is filtered by current user ID. No customer may request another customer's order list.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="108" customHeight="1">
+      <x:c r="A215" s="7" t="str">
+        <x:v>E2E-235</x:v>
+      </x:c>
+      <x:c r="B215" s="7" t="str">
+        <x:v>Orders / UI</x:v>
+      </x:c>
+      <x:c r="C215" s="7" t="str">
+        <x:v>Customer order status and detail navigation</x:v>
+      </x:c>
+      <x:c r="D215" s="7" t="str">
+        <x:v>Open Orders as an authenticated customer on desktop and mobile; verify status badges, quantity, total, timestamps and the link to each order detail.</x:v>
+      </x:c>
+      <x:c r="E215" s="7" t="str">
+        <x:v>The page shows the customer's newest orders with readable statuses and detail links, without overlap or horizontal overflow.</x:v>
+      </x:c>
+      <x:c r="F215" s="7" t="str">
+        <x:v>Two orders rendered with PRINTING and DONE statuses, quantities, totals and detail links. Mobile horizontal overflow measured 0 px.</x:v>
+      </x:c>
+      <x:c r="G215" s="7" t="str">
+        <x:v>Playwright browser smoke PASS; desktop/mobile screenshots inspected; zero console errors and zero page errors.</x:v>
+      </x:c>
+      <x:c r="H215" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I215" s="7" t="str">
+        <x:v>P1 - Browser runtime + responsive geometry + visual inspection</x:v>
+      </x:c>
+      <x:c r="J215" s="7" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="K215" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L215" s="7" t="str">
+        <x:v>Browser responses used synthetic owned-order fixtures; no production or local customer order records were changed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="108" customHeight="1">
+      <x:c r="A216" s="7" t="str">
+        <x:v>E2E-236</x:v>
+      </x:c>
+      <x:c r="B216" s="7" t="str">
+        <x:v>Cart</x:v>
+      </x:c>
+      <x:c r="C216" s="7" t="str">
+        <x:v>Customer cart persists draft references safely</x:v>
+      </x:c>
+      <x:c r="D216" s="7" t="str">
+        <x:v>Add an owned draft to Cart, open Cart, verify preview and checkout/edit/remove actions, then reload the page.</x:v>
+      </x:c>
+      <x:c r="E216" s="7" t="str">
+        <x:v>The cart count and item remain available after navigation. Cart storage contains draft IDs only, and draft content is reloaded through the owner-scoped API.</x:v>
+      </x:c>
+      <x:c r="F216" s="7" t="str">
+        <x:v>Cart count, preview, checkout/edit/remove actions and reload behavior passed. Stale or inaccessible IDs are removed automatically.</x:v>
+      </x:c>
+      <x:c r="G216" s="7" t="str">
+        <x:v>Frontend build/typecheck PASS; XSS guard PASS; Playwright cart smoke PASS with zero runtime errors.</x:v>
+      </x:c>
+      <x:c r="H216" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I216" s="7" t="str">
+        <x:v>P1 - Vue build + XSS guard + browser persistence/interaction checks</x:v>
+      </x:c>
+      <x:c r="J216" s="7" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="K216" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L216" s="7" t="str">
+        <x:v>Only numeric design IDs are stored in localStorage. Design content and ownership are always resolved by the backend.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="108" customHeight="1">
+      <x:c r="A217" s="7" t="str">
+        <x:v>E2E-237</x:v>
+      </x:c>
+      <x:c r="B217" s="7" t="str">
+        <x:v>Drafts / Delete</x:v>
+      </x:c>
+      <x:c r="C217" s="7" t="str">
+        <x:v>Owned draft deletion requires explicit confirmation</x:v>
+      </x:c>
+      <x:c r="D217" s="7" t="str">
+        <x:v>Click Delete on a draft, choose Cancel, then repeat and choose Delete draft in the warning dialog.</x:v>
+      </x:c>
+      <x:c r="E217" s="7" t="str">
+        <x:v>Cancel closes the dialog without a DELETE request. Confirm sends one DELETE request and removes the card from My drafts.</x:v>
+      </x:c>
+      <x:c r="F217" s="7" t="str">
+        <x:v>Cancel produced 0 DELETE requests and kept the draft visible; confirmation produced exactly 1 DELETE request and removed it.</x:v>
+      </x:c>
+      <x:c r="G217" s="7" t="str">
+        <x:v>Playwright destructive-action smoke PASS; dialog keyboard/backdrop behavior and desktop screenshot inspected.</x:v>
+      </x:c>
+      <x:c r="H217" s="7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I217" s="7" t="str">
+        <x:v>P0 - Browser network assertion + confirmation modal interaction + existing backend ownership enforcement</x:v>
+      </x:c>
+      <x:c r="J217" s="7" t="str">
+        <x:v>2026-07-24</x:v>
+      </x:c>
+      <x:c r="K217" s="7" t="str">
+        <x:v>localhost FE5176 / BE18080</x:v>
+      </x:c>
+      <x:c r="L217" s="7" t="str">
+        <x:v>The browser smoke intercepted DELETE and did not remove a real draft. Public templates are not customer-deletable.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9758,7 +9986,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>2026-07-21</x:v>
+        <x:v>2026-07-24</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="40" customHeight="1">
@@ -9766,7 +9994,7 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Local login Failed to fetch caused by missing CORS origins for FE port 5176</x:v>
+        <x:v>Customer cart, owner-scoped order tracking, order statuses and confirmed draft deletion</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
@@ -9774,7 +10002,7 @@
         <x:v>Frontend</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>http://127.0.0.1:5176/account</x:v>
+        <x:v>http://127.0.0.1:5176/orders and /cart</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -9782,7 +10010,7 @@
         <x:v>Backend</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>http://127.0.0.1:18080; local PostgreSQL 127.0.0.1:55432</x:v>
+        <x:v>Spring Boot http://127.0.0.1:18080</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
@@ -9790,23 +10018,23 @@
         <x:v>Health</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>CORS/API PASS; invalid login returns normal 401; 3 fixture ADMIN logins PASS; frontend build and backend 108/108 PASS</x:v>
+        <x:v>Frontend build/typecheck and XSS guard PASS; full backend 129/129 PASS; customer commerce browser smoke PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Source</x:v>
+        <x:v>Security</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>application.properties app.cors.allowed-origins default now includes localhost:5176 and 127.0.0.1:5176</x:v>
+        <x:v>Orders and drafts are owner-scoped; anonymous order history returns 401; cart stores numeric draft IDs only</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Test case</x:v>
+        <x:v>Browser</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>E2E-231</x:v>
+        <x:v>Orders/status/detail, cart persistence/actions, delete cancel/confirm and mobile 0px overflow all PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
@@ -9814,7 +10042,7 @@
         <x:v>Retest PASS</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>E2E-231</x:v>
+        <x:v>E2E-234 - E2E-237</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -9822,7 +10050,7 @@
         <x:v>Retest FAIL</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>None after fix</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" customHeight="1">
@@ -9830,7 +10058,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>login-network-smoke.cjs; direct CSRF/CORS check; local-admin-login-smoke.cjs; npm run build; mvnw test</x:v>
+        <x:v>Spring focused/full suites; live HTTP check; Playwright network/runtime/responsive assertions; screenshots</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -9838,7 +10066,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Clean browser context used for login verification; no credentials, tokens or personal data recorded</x:v>
+        <x:v>Browser fixtures were synthetic; no real orders, drafts, credentials, secrets or personal data were changed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>